<commit_message>
baseline Run1 complete: 4 datasets reproduced (F1 CDD 97.75 / LEVIR 91.95 / SYSU 82.48 / WHU 94.84)
</commit_message>
<xml_diff>
--- a/docs/experiment_metrics.xlsx
+++ b/docs/experiment_metrics.xlsx
@@ -10,7 +10,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="metrics" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'metrics'!$A$1:$N$1</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'metrics'!$A$1:$N$5</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -51,9 +51,10 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="2" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -419,7 +420,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N1"/>
+  <dimension ref="A1:N5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -510,8 +511,208 @@
         </is>
       </c>
     </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>baseline</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>Run1</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr"/>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>CDD-CD-256</t>
+        </is>
+      </c>
+      <c r="E2" s="2" t="n">
+        <v>97.72</v>
+      </c>
+      <c r="F2" s="2" t="n">
+        <v>97.78</v>
+      </c>
+      <c r="G2" s="2" t="n">
+        <v>99.44</v>
+      </c>
+      <c r="H2" s="2" t="n">
+        <v>97.75</v>
+      </c>
+      <c r="I2" s="2" t="n">
+        <v>95.59999999999999</v>
+      </c>
+      <c r="J2" s="2" t="n">
+        <v>97.43000000000001</v>
+      </c>
+      <c r="K2" s="2" t="n">
+        <v>11.754</v>
+      </c>
+      <c r="L2" s="2" t="n">
+        <v>20.661</v>
+      </c>
+      <c r="M2" s="2" t="n">
+        <v>26.3246</v>
+      </c>
+      <c r="N2" t="inlineStr">
+        <is>
+          <t>baseline</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>baseline</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>Run1</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr"/>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>LEVIR-CD-256</t>
+        </is>
+      </c>
+      <c r="E3" s="2" t="n">
+        <v>91.56999999999999</v>
+      </c>
+      <c r="F3" s="2" t="n">
+        <v>92.33</v>
+      </c>
+      <c r="G3" s="2" t="n">
+        <v>99.18000000000001</v>
+      </c>
+      <c r="H3" s="2" t="n">
+        <v>91.95</v>
+      </c>
+      <c r="I3" s="2" t="n">
+        <v>85.09999999999999</v>
+      </c>
+      <c r="J3" s="2" t="n">
+        <v>91.52</v>
+      </c>
+      <c r="K3" s="2" t="n">
+        <v>11.754</v>
+      </c>
+      <c r="L3" s="2" t="n">
+        <v>20.661</v>
+      </c>
+      <c r="M3" s="2" t="n">
+        <v>26.3246</v>
+      </c>
+      <c r="N3" t="inlineStr">
+        <is>
+          <t>baseline</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>baseline</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>Run1</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr"/>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>SYSU-CD-256</t>
+        </is>
+      </c>
+      <c r="E4" s="2" t="n">
+        <v>80.77</v>
+      </c>
+      <c r="F4" s="2" t="n">
+        <v>84.27</v>
+      </c>
+      <c r="G4" s="2" t="n">
+        <v>91.91</v>
+      </c>
+      <c r="H4" s="2" t="n">
+        <v>82.48</v>
+      </c>
+      <c r="I4" s="2" t="n">
+        <v>70.19</v>
+      </c>
+      <c r="J4" s="2" t="n">
+        <v>77.23</v>
+      </c>
+      <c r="K4" s="2" t="n">
+        <v>11.754</v>
+      </c>
+      <c r="L4" s="2" t="n">
+        <v>20.661</v>
+      </c>
+      <c r="M4" s="2" t="n">
+        <v>26.3246</v>
+      </c>
+      <c r="N4" t="inlineStr">
+        <is>
+          <t>baseline</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>baseline</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>Run1</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr"/>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>WHU-CD-256</t>
+        </is>
+      </c>
+      <c r="E5" s="2" t="n">
+        <v>93.62</v>
+      </c>
+      <c r="F5" s="2" t="n">
+        <v>96.09</v>
+      </c>
+      <c r="G5" s="2" t="n">
+        <v>99.59999999999999</v>
+      </c>
+      <c r="H5" s="2" t="n">
+        <v>94.84</v>
+      </c>
+      <c r="I5" s="2" t="n">
+        <v>90.18000000000001</v>
+      </c>
+      <c r="J5" s="2" t="n">
+        <v>94.63</v>
+      </c>
+      <c r="K5" s="2" t="n">
+        <v>11.754</v>
+      </c>
+      <c r="L5" s="2" t="n">
+        <v>20.661</v>
+      </c>
+      <c r="M5" s="2" t="n">
+        <v>26.3246</v>
+      </c>
+      <c r="N5" t="inlineStr">
+        <is>
+          <t>baseline</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:N1"/>
+  <autoFilter ref="A1:N5"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Run2 complete: 12/12 results + D1/D2 zero-cost diagnostics; LEVIR +0.07~+0.22 / SYSU -0.34~-0.62 (targets not met, mechanism evidence self-consistent); report/json/snapshot/xlsx
</commit_message>
<xml_diff>
--- a/docs/experiment_metrics.xlsx
+++ b/docs/experiment_metrics.xlsx
@@ -10,7 +10,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="metrics" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'metrics'!$A$1:$N$59</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'metrics'!$A$1:$N$71</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -420,7 +420,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N59"/>
+  <dimension ref="A1:N71"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -2242,223 +2242,223 @@
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>CASAA</t>
+          <t>CASA-TViM</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>Run1</t>
+          <t>Run2</t>
         </is>
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>A1_SAA</t>
+          <t>E1_CP_CAACP</t>
         </is>
       </c>
       <c r="D34" t="inlineStr">
         <is>
-          <t>LEVIR-CD-256</t>
+          <t>CDD-CD-256</t>
         </is>
       </c>
       <c r="E34" s="2" t="n">
-        <v>91.09</v>
+        <v>97.02</v>
       </c>
       <c r="F34" s="2" t="n">
-        <v>92.8</v>
+        <v>97.27</v>
       </c>
       <c r="G34" s="2" t="n">
-        <v>99.19</v>
+        <v>99.3</v>
       </c>
       <c r="H34" s="2" t="n">
-        <v>91.94</v>
+        <v>97.14</v>
       </c>
       <c r="I34" s="2" t="n">
-        <v>85.08</v>
+        <v>94.45</v>
       </c>
       <c r="J34" s="2" t="n">
-        <v>91.51000000000001</v>
+        <v>96.73999999999999</v>
       </c>
       <c r="K34" s="2" t="n">
-        <v>11.754</v>
+        <v>4.88</v>
       </c>
       <c r="L34" s="2" t="n">
-        <v>20.661</v>
+        <v>4.88</v>
       </c>
       <c r="M34" s="2" t="n">
-        <v>26.3183</v>
+        <v>2.6747</v>
       </c>
       <c r="N34" t="inlineStr">
         <is>
-          <t>saa</t>
+          <t>casa_tvim_str</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>CASAA</t>
+          <t>CASA-TViM</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>Run1</t>
+          <t>Run2</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>A1_SAA</t>
+          <t>E1_CP_CAACP</t>
         </is>
       </c>
       <c r="D35" t="inlineStr">
         <is>
-          <t>SYSU-CD-256</t>
+          <t>LEVIR-CD-256</t>
         </is>
       </c>
       <c r="E35" s="2" t="n">
-        <v>80.3</v>
+        <v>90.64</v>
       </c>
       <c r="F35" s="2" t="n">
-        <v>84.81</v>
+        <v>91.64</v>
       </c>
       <c r="G35" s="2" t="n">
-        <v>91.95999999999999</v>
+        <v>99.09999999999999</v>
       </c>
       <c r="H35" s="2" t="n">
-        <v>82.5</v>
+        <v>91.14</v>
       </c>
       <c r="I35" s="2" t="n">
-        <v>70.20999999999999</v>
+        <v>83.72</v>
       </c>
       <c r="J35" s="2" t="n">
-        <v>77.29000000000001</v>
+        <v>90.66</v>
       </c>
       <c r="K35" s="2" t="n">
-        <v>11.754</v>
+        <v>4.88</v>
       </c>
       <c r="L35" s="2" t="n">
-        <v>20.661</v>
+        <v>4.88</v>
       </c>
       <c r="M35" s="2" t="n">
-        <v>26.3183</v>
+        <v>2.6747</v>
       </c>
       <c r="N35" t="inlineStr">
         <is>
-          <t>saa</t>
+          <t>casa_tvim_str</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>CASAA</t>
+          <t>CASA-TViM</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>Run1</t>
+          <t>Run2</t>
         </is>
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>A2_CASAA</t>
+          <t>E1_CP_CAACP</t>
         </is>
       </c>
       <c r="D36" t="inlineStr">
         <is>
-          <t>LEVIR-CD-256</t>
+          <t>SYSU-CD-256</t>
         </is>
       </c>
       <c r="E36" s="2" t="n">
-        <v>90.98999999999999</v>
+        <v>80.94</v>
       </c>
       <c r="F36" s="2" t="n">
-        <v>92.75</v>
+        <v>85.43000000000001</v>
       </c>
       <c r="G36" s="2" t="n">
-        <v>99.18000000000001</v>
+        <v>92.25</v>
       </c>
       <c r="H36" s="2" t="n">
-        <v>91.86</v>
+        <v>83.13</v>
       </c>
       <c r="I36" s="2" t="n">
-        <v>84.94</v>
+        <v>71.12</v>
       </c>
       <c r="J36" s="2" t="n">
-        <v>91.43000000000001</v>
+        <v>78.09999999999999</v>
       </c>
       <c r="K36" s="2" t="n">
-        <v>11.754</v>
+        <v>4.88</v>
       </c>
       <c r="L36" s="2" t="n">
-        <v>20.661</v>
+        <v>4.88</v>
       </c>
       <c r="M36" s="2" t="n">
-        <v>26.2593</v>
+        <v>2.6747</v>
       </c>
       <c r="N36" t="inlineStr">
         <is>
-          <t>casaa</t>
+          <t>casa_tvim_str</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>CASAA</t>
+          <t>CASA-TViM</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>Run1</t>
+          <t>Run2</t>
         </is>
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>A2_CASAA</t>
+          <t>E1_CP_CAACP</t>
         </is>
       </c>
       <c r="D37" t="inlineStr">
         <is>
-          <t>SYSU-CD-256</t>
+          <t>WHU-CD-256</t>
         </is>
       </c>
       <c r="E37" s="2" t="n">
-        <v>80.55</v>
+        <v>93.73999999999999</v>
       </c>
       <c r="F37" s="2" t="n">
-        <v>84.23</v>
+        <v>96.67</v>
       </c>
       <c r="G37" s="2" t="n">
-        <v>91.86</v>
+        <v>99.62</v>
       </c>
       <c r="H37" s="2" t="n">
-        <v>82.34999999999999</v>
+        <v>95.18000000000001</v>
       </c>
       <c r="I37" s="2" t="n">
-        <v>70</v>
+        <v>90.81</v>
       </c>
       <c r="J37" s="2" t="n">
-        <v>77.06</v>
+        <v>94.98999999999999</v>
       </c>
       <c r="K37" s="2" t="n">
-        <v>11.754</v>
+        <v>4.88</v>
       </c>
       <c r="L37" s="2" t="n">
-        <v>20.661</v>
+        <v>4.88</v>
       </c>
       <c r="M37" s="2" t="n">
-        <v>26.2593</v>
+        <v>2.6747</v>
       </c>
       <c r="N37" t="inlineStr">
         <is>
-          <t>casaa</t>
+          <t>casa_tvim_str</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>CASAA</t>
+          <t>CASA-TViM</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
@@ -2468,51 +2468,51 @@
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>A1_SAA_FROZEN</t>
+          <t>E2_FRH</t>
         </is>
       </c>
       <c r="D38" t="inlineStr">
         <is>
-          <t>LEVIR-CD-256</t>
+          <t>CDD-CD-256</t>
         </is>
       </c>
       <c r="E38" s="2" t="n">
-        <v>91.38</v>
+        <v>97.02</v>
       </c>
       <c r="F38" s="2" t="n">
-        <v>92.3</v>
+        <v>97.33</v>
       </c>
       <c r="G38" s="2" t="n">
-        <v>99.17</v>
+        <v>99.3</v>
       </c>
       <c r="H38" s="2" t="n">
-        <v>91.84</v>
+        <v>97.17</v>
       </c>
       <c r="I38" s="2" t="n">
-        <v>84.91</v>
+        <v>94.5</v>
       </c>
       <c r="J38" s="2" t="n">
-        <v>91.40000000000001</v>
+        <v>96.78</v>
       </c>
       <c r="K38" s="2" t="n">
-        <v>11.754</v>
+        <v>4.881</v>
       </c>
       <c r="L38" s="2" t="n">
-        <v>15.125</v>
+        <v>4.881</v>
       </c>
       <c r="M38" s="2" t="n">
-        <v>26.1484</v>
+        <v>2.6947</v>
       </c>
       <c r="N38" t="inlineStr">
         <is>
-          <t>saa</t>
+          <t>casa_tvim_str</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>CASAA</t>
+          <t>CASA-TViM</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
@@ -2522,51 +2522,51 @@
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>A1_SAA_FROZEN</t>
+          <t>E2_FRH</t>
         </is>
       </c>
       <c r="D39" t="inlineStr">
         <is>
-          <t>SYSU-CD-256</t>
+          <t>LEVIR-CD-256</t>
         </is>
       </c>
       <c r="E39" s="2" t="n">
-        <v>78.40000000000001</v>
+        <v>90.22</v>
       </c>
       <c r="F39" s="2" t="n">
-        <v>86.03</v>
+        <v>92.22</v>
       </c>
       <c r="G39" s="2" t="n">
-        <v>91.90000000000001</v>
+        <v>99.11</v>
       </c>
       <c r="H39" s="2" t="n">
-        <v>82.04000000000001</v>
+        <v>91.20999999999999</v>
       </c>
       <c r="I39" s="2" t="n">
-        <v>69.55</v>
+        <v>83.83</v>
       </c>
       <c r="J39" s="2" t="n">
-        <v>76.83</v>
+        <v>90.73999999999999</v>
       </c>
       <c r="K39" s="2" t="n">
-        <v>11.754</v>
+        <v>4.881</v>
       </c>
       <c r="L39" s="2" t="n">
-        <v>15.125</v>
+        <v>4.881</v>
       </c>
       <c r="M39" s="2" t="n">
-        <v>26.1484</v>
+        <v>2.6947</v>
       </c>
       <c r="N39" t="inlineStr">
         <is>
-          <t>saa</t>
+          <t>casa_tvim_str</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>CASAA</t>
+          <t>CASA-TViM</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
@@ -2576,51 +2576,51 @@
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>A3_ORACLE_FROZEN</t>
+          <t>E2_FRH</t>
         </is>
       </c>
       <c r="D40" t="inlineStr">
         <is>
-          <t>LEVIR-CD-256</t>
+          <t>SYSU-CD-256</t>
         </is>
       </c>
       <c r="E40" s="2" t="n">
-        <v>91.13</v>
+        <v>80.09999999999999</v>
       </c>
       <c r="F40" s="2" t="n">
-        <v>92.65000000000001</v>
+        <v>86.05</v>
       </c>
       <c r="G40" s="2" t="n">
-        <v>99.18000000000001</v>
+        <v>92.23999999999999</v>
       </c>
       <c r="H40" s="2" t="n">
-        <v>91.88</v>
+        <v>82.97</v>
       </c>
       <c r="I40" s="2" t="n">
-        <v>84.98</v>
+        <v>70.89</v>
       </c>
       <c r="J40" s="2" t="n">
-        <v>91.45</v>
+        <v>77.95999999999999</v>
       </c>
       <c r="K40" s="2" t="n">
-        <v>11.754</v>
+        <v>4.881</v>
       </c>
       <c r="L40" s="2" t="n">
-        <v>15.125</v>
+        <v>4.881</v>
       </c>
       <c r="M40" s="2" t="n">
-        <v>26.0894</v>
+        <v>2.6947</v>
       </c>
       <c r="N40" t="inlineStr">
         <is>
-          <t>casaa</t>
+          <t>casa_tvim_str</t>
         </is>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>CASAA</t>
+          <t>CASA-TViM</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
@@ -2630,385 +2630,385 @@
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>A3_ORACLE_FROZEN</t>
+          <t>E2_FRH</t>
         </is>
       </c>
       <c r="D41" t="inlineStr">
         <is>
-          <t>SYSU-CD-256</t>
+          <t>WHU-CD-256</t>
         </is>
       </c>
       <c r="E41" s="2" t="n">
-        <v>82.04000000000001</v>
+        <v>93.45999999999999</v>
       </c>
       <c r="F41" s="2" t="n">
-        <v>85.05</v>
+        <v>96</v>
       </c>
       <c r="G41" s="2" t="n">
-        <v>92.36</v>
+        <v>99.59</v>
       </c>
       <c r="H41" s="2" t="n">
-        <v>83.52</v>
+        <v>94.70999999999999</v>
       </c>
       <c r="I41" s="2" t="n">
-        <v>71.7</v>
+        <v>89.95</v>
       </c>
       <c r="J41" s="2" t="n">
-        <v>78.55</v>
+        <v>94.48999999999999</v>
       </c>
       <c r="K41" s="2" t="n">
-        <v>11.754</v>
+        <v>4.881</v>
       </c>
       <c r="L41" s="2" t="n">
-        <v>15.125</v>
+        <v>4.881</v>
       </c>
       <c r="M41" s="2" t="n">
-        <v>26.0894</v>
+        <v>2.6947</v>
       </c>
       <c r="N41" t="inlineStr">
         <is>
-          <t>casaa</t>
+          <t>casa_tvim_str</t>
         </is>
       </c>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>CASAA</t>
+          <t>CASA-TViM</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>Run3</t>
+          <t>Run2</t>
         </is>
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>A4_DETAIL_FROZEN</t>
+          <t>E3_CP_FRH</t>
         </is>
       </c>
       <c r="D42" t="inlineStr">
         <is>
-          <t>SYSU-CD-256</t>
+          <t>CDD-CD-256</t>
         </is>
       </c>
       <c r="E42" s="2" t="n">
-        <v>79.68000000000001</v>
+        <v>97.02</v>
       </c>
       <c r="F42" s="2" t="n">
-        <v>84.28</v>
+        <v>97.34</v>
       </c>
       <c r="G42" s="2" t="n">
-        <v>91.7</v>
+        <v>99.3</v>
       </c>
       <c r="H42" s="2" t="n">
-        <v>81.92</v>
+        <v>97.18000000000001</v>
       </c>
       <c r="I42" s="2" t="n">
-        <v>69.37</v>
+        <v>94.51000000000001</v>
       </c>
       <c r="J42" s="2" t="n">
-        <v>76.54000000000001</v>
+        <v>96.78</v>
       </c>
       <c r="K42" s="2" t="n">
-        <v>11.754</v>
+        <v>4.881</v>
       </c>
       <c r="L42" s="2" t="n">
-        <v>15.125</v>
+        <v>4.881</v>
       </c>
       <c r="M42" s="2" t="n">
-        <v>26.0894</v>
+        <v>2.6947</v>
       </c>
       <c r="N42" t="inlineStr">
         <is>
-          <t>casaa</t>
+          <t>casa_tvim_str</t>
         </is>
       </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>STR-Fusion</t>
+          <t>CASA-TViM</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>Run2_TASS</t>
+          <t>Run2</t>
         </is>
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>C0_TOKEN</t>
+          <t>E3_CP_FRH</t>
         </is>
       </c>
       <c r="D43" t="inlineStr">
         <is>
-          <t>CDD-CD-256</t>
+          <t>LEVIR-CD-256</t>
         </is>
       </c>
       <c r="E43" s="2" t="n">
-        <v>93.13</v>
+        <v>90.20999999999999</v>
       </c>
       <c r="F43" s="2" t="n">
-        <v>95.16</v>
+        <v>92.41</v>
       </c>
       <c r="G43" s="2" t="n">
-        <v>98.56999999999999</v>
+        <v>99.12</v>
       </c>
       <c r="H43" s="2" t="n">
-        <v>94.13</v>
+        <v>91.29000000000001</v>
       </c>
       <c r="I43" s="2" t="n">
-        <v>88.91</v>
+        <v>83.98</v>
       </c>
       <c r="J43" s="2" t="n">
-        <v>93.31999999999999</v>
+        <v>90.83</v>
       </c>
       <c r="K43" s="2" t="n">
-        <v>2.596</v>
+        <v>4.881</v>
       </c>
       <c r="L43" s="2" t="n">
-        <v>0.62</v>
+        <v>4.881</v>
       </c>
       <c r="M43" s="2" t="n">
-        <v>2.2136</v>
+        <v>2.6947</v>
       </c>
       <c r="N43" t="inlineStr">
         <is>
-          <t>str_tass</t>
+          <t>casa_tvim_str</t>
         </is>
       </c>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>STR-Fusion</t>
+          <t>CASA-TViM</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>Run2_TASS</t>
+          <t>Run2</t>
         </is>
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>C0_TOKEN</t>
+          <t>E3_CP_FRH</t>
         </is>
       </c>
       <c r="D44" t="inlineStr">
         <is>
-          <t>LEVIR-CD-256</t>
+          <t>SYSU-CD-256</t>
         </is>
       </c>
       <c r="E44" s="2" t="n">
-        <v>86.37</v>
+        <v>80.69</v>
       </c>
       <c r="F44" s="2" t="n">
-        <v>89.25</v>
+        <v>85.12</v>
       </c>
       <c r="G44" s="2" t="n">
-        <v>98.78</v>
+        <v>92.12</v>
       </c>
       <c r="H44" s="2" t="n">
-        <v>87.79000000000001</v>
+        <v>82.84999999999999</v>
       </c>
       <c r="I44" s="2" t="n">
-        <v>78.23999999999999</v>
+        <v>70.72</v>
       </c>
       <c r="J44" s="2" t="n">
-        <v>87.14</v>
+        <v>77.73999999999999</v>
       </c>
       <c r="K44" s="2" t="n">
-        <v>2.596</v>
+        <v>4.881</v>
       </c>
       <c r="L44" s="2" t="n">
-        <v>0.62</v>
+        <v>4.881</v>
       </c>
       <c r="M44" s="2" t="n">
-        <v>2.2136</v>
+        <v>2.6947</v>
       </c>
       <c r="N44" t="inlineStr">
         <is>
-          <t>str_tass</t>
+          <t>casa_tvim_str</t>
         </is>
       </c>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>STR-Fusion</t>
+          <t>CASA-TViM</t>
         </is>
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>Run2_TASS</t>
+          <t>Run2</t>
         </is>
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>C0_TOKEN</t>
+          <t>E3_CP_FRH</t>
         </is>
       </c>
       <c r="D45" t="inlineStr">
         <is>
-          <t>SYSU-CD-256</t>
+          <t>WHU-CD-256</t>
         </is>
       </c>
       <c r="E45" s="2" t="n">
-        <v>79.93000000000001</v>
+        <v>93.8</v>
       </c>
       <c r="F45" s="2" t="n">
-        <v>84.5</v>
+        <v>96.18000000000001</v>
       </c>
       <c r="G45" s="2" t="n">
-        <v>91.81</v>
+        <v>99.61</v>
       </c>
       <c r="H45" s="2" t="n">
-        <v>82.15000000000001</v>
+        <v>94.98</v>
       </c>
       <c r="I45" s="2" t="n">
-        <v>69.70999999999999</v>
+        <v>90.44</v>
       </c>
       <c r="J45" s="2" t="n">
-        <v>76.84</v>
+        <v>94.77</v>
       </c>
       <c r="K45" s="2" t="n">
-        <v>2.596</v>
+        <v>4.881</v>
       </c>
       <c r="L45" s="2" t="n">
-        <v>0.62</v>
+        <v>4.881</v>
       </c>
       <c r="M45" s="2" t="n">
-        <v>2.2136</v>
+        <v>2.6947</v>
       </c>
       <c r="N45" t="inlineStr">
         <is>
-          <t>str_tass</t>
+          <t>casa_tvim_str</t>
         </is>
       </c>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>STR-Fusion</t>
+          <t>CASAA</t>
         </is>
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>Run2_TASS</t>
+          <t>Run1</t>
         </is>
       </c>
       <c r="C46" t="inlineStr">
         <is>
-          <t>C0_TOKEN</t>
+          <t>A1_SAA</t>
         </is>
       </c>
       <c r="D46" t="inlineStr">
         <is>
-          <t>WHU-CD-256</t>
+          <t>LEVIR-CD-256</t>
         </is>
       </c>
       <c r="E46" s="2" t="n">
-        <v>90.16</v>
+        <v>91.09</v>
       </c>
       <c r="F46" s="2" t="n">
-        <v>93.97</v>
+        <v>92.8</v>
       </c>
       <c r="G46" s="2" t="n">
-        <v>99.38</v>
+        <v>99.19</v>
       </c>
       <c r="H46" s="2" t="n">
-        <v>92.02</v>
+        <v>91.94</v>
       </c>
       <c r="I46" s="2" t="n">
-        <v>85.23</v>
+        <v>85.08</v>
       </c>
       <c r="J46" s="2" t="n">
-        <v>91.7</v>
+        <v>91.51000000000001</v>
       </c>
       <c r="K46" s="2" t="n">
-        <v>2.596</v>
+        <v>11.754</v>
       </c>
       <c r="L46" s="2" t="n">
-        <v>0.62</v>
+        <v>20.661</v>
       </c>
       <c r="M46" s="2" t="n">
-        <v>2.2136</v>
+        <v>26.3183</v>
       </c>
       <c r="N46" t="inlineStr">
         <is>
-          <t>str_tass</t>
+          <t>saa</t>
         </is>
       </c>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>STR-Fusion</t>
+          <t>CASAA</t>
         </is>
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>Run2_TASS</t>
+          <t>Run1</t>
         </is>
       </c>
       <c r="C47" t="inlineStr">
         <is>
-          <t>M1_TASS</t>
+          <t>A1_SAA</t>
         </is>
       </c>
       <c r="D47" t="inlineStr">
         <is>
-          <t>CDD-CD-256</t>
+          <t>SYSU-CD-256</t>
         </is>
       </c>
       <c r="E47" s="2" t="n">
-        <v>94.7</v>
+        <v>80.3</v>
       </c>
       <c r="F47" s="2" t="n">
-        <v>96.13</v>
+        <v>84.81</v>
       </c>
       <c r="G47" s="2" t="n">
-        <v>98.88</v>
+        <v>91.95999999999999</v>
       </c>
       <c r="H47" s="2" t="n">
-        <v>95.41</v>
+        <v>82.5</v>
       </c>
       <c r="I47" s="2" t="n">
-        <v>91.22</v>
+        <v>70.20999999999999</v>
       </c>
       <c r="J47" s="2" t="n">
-        <v>94.77</v>
+        <v>77.29000000000001</v>
       </c>
       <c r="K47" s="2" t="n">
-        <v>3.455</v>
+        <v>11.754</v>
       </c>
       <c r="L47" s="2" t="n">
-        <v>1.478</v>
+        <v>20.661</v>
       </c>
       <c r="M47" s="2" t="n">
-        <v>3.5459</v>
+        <v>26.3183</v>
       </c>
       <c r="N47" t="inlineStr">
         <is>
-          <t>str_tass</t>
+          <t>saa</t>
         </is>
       </c>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>STR-Fusion</t>
+          <t>CASAA</t>
         </is>
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>Run2_TASS</t>
+          <t>Run1</t>
         </is>
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>M1_TASS</t>
+          <t>A2_CASAA</t>
         </is>
       </c>
       <c r="D48" t="inlineStr">
@@ -3017,52 +3017,52 @@
         </is>
       </c>
       <c r="E48" s="2" t="n">
-        <v>88.42</v>
+        <v>90.98999999999999</v>
       </c>
       <c r="F48" s="2" t="n">
-        <v>91.97</v>
+        <v>92.75</v>
       </c>
       <c r="G48" s="2" t="n">
-        <v>99.02</v>
+        <v>99.18000000000001</v>
       </c>
       <c r="H48" s="2" t="n">
-        <v>90.16</v>
+        <v>91.86</v>
       </c>
       <c r="I48" s="2" t="n">
-        <v>82.08</v>
+        <v>84.94</v>
       </c>
       <c r="J48" s="2" t="n">
-        <v>89.64</v>
+        <v>91.43000000000001</v>
       </c>
       <c r="K48" s="2" t="n">
-        <v>3.455</v>
+        <v>11.754</v>
       </c>
       <c r="L48" s="2" t="n">
-        <v>1.478</v>
+        <v>20.661</v>
       </c>
       <c r="M48" s="2" t="n">
-        <v>3.5459</v>
+        <v>26.2593</v>
       </c>
       <c r="N48" t="inlineStr">
         <is>
-          <t>str_tass</t>
+          <t>casaa</t>
         </is>
       </c>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>STR-Fusion</t>
+          <t>CASAA</t>
         </is>
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>Run2_TASS</t>
+          <t>Run1</t>
         </is>
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>M1_TASS</t>
+          <t>A2_CASAA</t>
         </is>
       </c>
       <c r="D49" t="inlineStr">
@@ -3071,106 +3071,106 @@
         </is>
       </c>
       <c r="E49" s="2" t="n">
-        <v>78.73</v>
+        <v>80.55</v>
       </c>
       <c r="F49" s="2" t="n">
-        <v>84.98</v>
+        <v>84.23</v>
       </c>
       <c r="G49" s="2" t="n">
-        <v>91.7</v>
+        <v>91.86</v>
       </c>
       <c r="H49" s="2" t="n">
-        <v>81.73999999999999</v>
+        <v>82.34999999999999</v>
       </c>
       <c r="I49" s="2" t="n">
-        <v>69.11</v>
+        <v>70</v>
       </c>
       <c r="J49" s="2" t="n">
-        <v>76.38</v>
+        <v>77.06</v>
       </c>
       <c r="K49" s="2" t="n">
-        <v>3.455</v>
+        <v>11.754</v>
       </c>
       <c r="L49" s="2" t="n">
-        <v>1.478</v>
+        <v>20.661</v>
       </c>
       <c r="M49" s="2" t="n">
-        <v>3.5459</v>
+        <v>26.2593</v>
       </c>
       <c r="N49" t="inlineStr">
         <is>
-          <t>str_tass</t>
+          <t>casaa</t>
         </is>
       </c>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>STR-Fusion</t>
+          <t>CASAA</t>
         </is>
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>Run2_TASS</t>
+          <t>Run2</t>
         </is>
       </c>
       <c r="C50" t="inlineStr">
         <is>
-          <t>M1_TASS</t>
+          <t>A1_SAA_FROZEN</t>
         </is>
       </c>
       <c r="D50" t="inlineStr">
         <is>
-          <t>WHU-CD-256</t>
+          <t>LEVIR-CD-256</t>
         </is>
       </c>
       <c r="E50" s="2" t="n">
-        <v>91.64</v>
+        <v>91.38</v>
       </c>
       <c r="F50" s="2" t="n">
-        <v>94.81999999999999</v>
+        <v>92.3</v>
       </c>
       <c r="G50" s="2" t="n">
-        <v>99.47</v>
+        <v>99.17</v>
       </c>
       <c r="H50" s="2" t="n">
-        <v>93.2</v>
+        <v>91.84</v>
       </c>
       <c r="I50" s="2" t="n">
-        <v>87.27</v>
+        <v>84.91</v>
       </c>
       <c r="J50" s="2" t="n">
-        <v>92.93000000000001</v>
+        <v>91.40000000000001</v>
       </c>
       <c r="K50" s="2" t="n">
-        <v>3.455</v>
+        <v>11.754</v>
       </c>
       <c r="L50" s="2" t="n">
-        <v>1.478</v>
+        <v>15.125</v>
       </c>
       <c r="M50" s="2" t="n">
-        <v>3.5459</v>
+        <v>26.1484</v>
       </c>
       <c r="N50" t="inlineStr">
         <is>
-          <t>str_tass</t>
+          <t>saa</t>
         </is>
       </c>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>UltraLight</t>
+          <t>CASAA</t>
         </is>
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>Run4</t>
+          <t>Run2</t>
         </is>
       </c>
       <c r="C51" t="inlineStr">
         <is>
-          <t>R4_0_A0_FULL12_FROZEN</t>
+          <t>A1_SAA_FROZEN</t>
         </is>
       </c>
       <c r="D51" t="inlineStr">
@@ -3179,22 +3179,22 @@
         </is>
       </c>
       <c r="E51" s="2" t="n">
-        <v>82.42</v>
+        <v>78.40000000000001</v>
       </c>
       <c r="F51" s="2" t="n">
-        <v>83.87</v>
+        <v>86.03</v>
       </c>
       <c r="G51" s="2" t="n">
-        <v>92.12</v>
+        <v>91.90000000000001</v>
       </c>
       <c r="H51" s="2" t="n">
-        <v>83.14</v>
+        <v>82.04000000000001</v>
       </c>
       <c r="I51" s="2" t="n">
-        <v>71.14</v>
+        <v>69.55</v>
       </c>
       <c r="J51" s="2" t="n">
-        <v>77.98999999999999</v>
+        <v>76.83</v>
       </c>
       <c r="K51" s="2" t="n">
         <v>11.754</v>
@@ -3203,82 +3203,82 @@
         <v>15.125</v>
       </c>
       <c r="M51" s="2" t="n">
-        <v>26.3246</v>
+        <v>26.1484</v>
       </c>
       <c r="N51" t="inlineStr">
         <is>
-          <t>baseline</t>
+          <t>saa</t>
         </is>
       </c>
     </row>
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>UltraLight</t>
+          <t>CASAA</t>
         </is>
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t>Run4</t>
+          <t>Run2</t>
         </is>
       </c>
       <c r="C52" t="inlineStr">
         <is>
-          <t>R4_1_VIT4_OLDHEAD</t>
+          <t>A3_ORACLE_FROZEN</t>
         </is>
       </c>
       <c r="D52" t="inlineStr">
         <is>
-          <t>SYSU-CD-256</t>
+          <t>LEVIR-CD-256</t>
         </is>
       </c>
       <c r="E52" s="2" t="n">
-        <v>82.15000000000001</v>
+        <v>91.13</v>
       </c>
       <c r="F52" s="2" t="n">
-        <v>83.40000000000001</v>
+        <v>92.65000000000001</v>
       </c>
       <c r="G52" s="2" t="n">
-        <v>91.94</v>
+        <v>99.18000000000001</v>
       </c>
       <c r="H52" s="2" t="n">
-        <v>82.77</v>
+        <v>91.88</v>
       </c>
       <c r="I52" s="2" t="n">
-        <v>70.61</v>
+        <v>84.98</v>
       </c>
       <c r="J52" s="2" t="n">
-        <v>77.51000000000001</v>
+        <v>91.45</v>
       </c>
       <c r="K52" s="2" t="n">
-        <v>8.195</v>
+        <v>11.754</v>
       </c>
       <c r="L52" s="2" t="n">
         <v>15.125</v>
       </c>
       <c r="M52" s="2" t="n">
-        <v>24.1021</v>
+        <v>26.0894</v>
       </c>
       <c r="N52" t="inlineStr">
         <is>
-          <t>baseline</t>
+          <t>casaa</t>
         </is>
       </c>
     </row>
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>UltraLight</t>
+          <t>CASAA</t>
         </is>
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>Run4</t>
+          <t>Run2</t>
         </is>
       </c>
       <c r="C53" t="inlineStr">
         <is>
-          <t>R4_2_VIT4_LIGHTDETAIL</t>
+          <t>A3_ORACLE_FROZEN</t>
         </is>
       </c>
       <c r="D53" t="inlineStr">
@@ -3287,52 +3287,52 @@
         </is>
       </c>
       <c r="E53" s="2" t="n">
-        <v>79.94</v>
+        <v>82.04000000000001</v>
       </c>
       <c r="F53" s="2" t="n">
-        <v>84.79000000000001</v>
+        <v>85.05</v>
       </c>
       <c r="G53" s="2" t="n">
-        <v>91.89</v>
+        <v>92.36</v>
       </c>
       <c r="H53" s="2" t="n">
-        <v>82.3</v>
+        <v>83.52</v>
       </c>
       <c r="I53" s="2" t="n">
-        <v>69.92</v>
+        <v>71.7</v>
       </c>
       <c r="J53" s="2" t="n">
-        <v>77.04000000000001</v>
+        <v>78.55</v>
       </c>
       <c r="K53" s="2" t="n">
-        <v>5.492</v>
+        <v>11.754</v>
       </c>
       <c r="L53" s="2" t="n">
-        <v>3.515</v>
+        <v>15.125</v>
       </c>
       <c r="M53" s="2" t="n">
-        <v>10.7311</v>
+        <v>26.0894</v>
       </c>
       <c r="N53" t="inlineStr">
         <is>
-          <t>baseline</t>
+          <t>casaa</t>
         </is>
       </c>
     </row>
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>UltraLight</t>
+          <t>CASAA</t>
         </is>
       </c>
       <c r="B54" t="inlineStr">
         <is>
-          <t>Run4</t>
+          <t>Run3</t>
         </is>
       </c>
       <c r="C54" t="inlineStr">
         <is>
-          <t>R4_2b_VIT4_LIGHTDETAIL48</t>
+          <t>A4_DETAIL_FROZEN</t>
         </is>
       </c>
       <c r="D54" t="inlineStr">
@@ -3341,294 +3341,942 @@
         </is>
       </c>
       <c r="E54" s="2" t="n">
-        <v>80.87</v>
+        <v>79.68000000000001</v>
       </c>
       <c r="F54" s="2" t="n">
-        <v>83.81</v>
+        <v>84.28</v>
       </c>
       <c r="G54" s="2" t="n">
-        <v>91.81</v>
+        <v>91.7</v>
       </c>
       <c r="H54" s="2" t="n">
-        <v>82.31999999999999</v>
+        <v>81.92</v>
       </c>
       <c r="I54" s="2" t="n">
-        <v>69.95</v>
+        <v>69.37</v>
       </c>
       <c r="J54" s="2" t="n">
-        <v>76.98999999999999</v>
+        <v>76.54000000000001</v>
       </c>
       <c r="K54" s="2" t="n">
-        <v>5.533</v>
+        <v>11.754</v>
       </c>
       <c r="L54" s="2" t="n">
-        <v>3.556</v>
+        <v>15.125</v>
       </c>
       <c r="M54" s="2" t="n">
-        <v>10.9824</v>
+        <v>26.0894</v>
       </c>
       <c r="N54" t="inlineStr">
         <is>
-          <t>baseline</t>
+          <t>casaa</t>
         </is>
       </c>
     </row>
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>UltraLight</t>
+          <t>STR-Fusion</t>
         </is>
       </c>
       <c r="B55" t="inlineStr">
         <is>
-          <t>Run4</t>
+          <t>Run2_TASS</t>
         </is>
       </c>
       <c r="C55" t="inlineStr">
         <is>
-          <t>R4_2d_PSD_DETAIL</t>
+          <t>C0_TOKEN</t>
         </is>
       </c>
       <c r="D55" t="inlineStr">
         <is>
-          <t>SYSU-CD-256</t>
+          <t>CDD-CD-256</t>
         </is>
       </c>
       <c r="E55" s="2" t="n">
-        <v>79.78</v>
+        <v>93.13</v>
       </c>
       <c r="F55" s="2" t="n">
-        <v>84.39</v>
+        <v>95.16</v>
       </c>
       <c r="G55" s="2" t="n">
-        <v>91.75</v>
+        <v>98.56999999999999</v>
       </c>
       <c r="H55" s="2" t="n">
-        <v>82.02</v>
+        <v>94.13</v>
       </c>
       <c r="I55" s="2" t="n">
-        <v>69.52</v>
+        <v>88.91</v>
       </c>
       <c r="J55" s="2" t="n">
-        <v>76.68000000000001</v>
+        <v>93.31999999999999</v>
       </c>
       <c r="K55" s="2" t="n">
-        <v>5.491</v>
+        <v>2.596</v>
       </c>
       <c r="L55" s="2" t="n">
-        <v>3.514</v>
+        <v>0.62</v>
       </c>
       <c r="M55" s="2" t="n">
-        <v>11.5239</v>
+        <v>2.2136</v>
       </c>
       <c r="N55" t="inlineStr">
         <is>
-          <t>baseline</t>
+          <t>str_tass</t>
         </is>
       </c>
     </row>
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>baseline</t>
+          <t>STR-Fusion</t>
         </is>
       </c>
       <c r="B56" t="inlineStr">
         <is>
-          <t>Run1</t>
-        </is>
-      </c>
-      <c r="C56" t="inlineStr"/>
+          <t>Run2_TASS</t>
+        </is>
+      </c>
+      <c r="C56" t="inlineStr">
+        <is>
+          <t>C0_TOKEN</t>
+        </is>
+      </c>
       <c r="D56" t="inlineStr">
         <is>
-          <t>CDD-CD-256</t>
+          <t>LEVIR-CD-256</t>
         </is>
       </c>
       <c r="E56" s="2" t="n">
-        <v>97.72</v>
+        <v>86.37</v>
       </c>
       <c r="F56" s="2" t="n">
-        <v>97.78</v>
+        <v>89.25</v>
       </c>
       <c r="G56" s="2" t="n">
-        <v>99.44</v>
+        <v>98.78</v>
       </c>
       <c r="H56" s="2" t="n">
-        <v>97.75</v>
+        <v>87.79000000000001</v>
       </c>
       <c r="I56" s="2" t="n">
-        <v>95.59999999999999</v>
+        <v>78.23999999999999</v>
       </c>
       <c r="J56" s="2" t="n">
-        <v>97.43000000000001</v>
+        <v>87.14</v>
       </c>
       <c r="K56" s="2" t="n">
-        <v>11.754</v>
+        <v>2.596</v>
       </c>
       <c r="L56" s="2" t="n">
-        <v>20.661</v>
+        <v>0.62</v>
       </c>
       <c r="M56" s="2" t="n">
-        <v>26.3246</v>
+        <v>2.2136</v>
       </c>
       <c r="N56" t="inlineStr">
         <is>
-          <t>baseline</t>
+          <t>str_tass</t>
         </is>
       </c>
     </row>
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>baseline</t>
+          <t>STR-Fusion</t>
         </is>
       </c>
       <c r="B57" t="inlineStr">
         <is>
-          <t>Run1</t>
-        </is>
-      </c>
-      <c r="C57" t="inlineStr"/>
+          <t>Run2_TASS</t>
+        </is>
+      </c>
+      <c r="C57" t="inlineStr">
+        <is>
+          <t>C0_TOKEN</t>
+        </is>
+      </c>
       <c r="D57" t="inlineStr">
         <is>
-          <t>LEVIR-CD-256</t>
+          <t>SYSU-CD-256</t>
         </is>
       </c>
       <c r="E57" s="2" t="n">
-        <v>91.56999999999999</v>
+        <v>79.93000000000001</v>
       </c>
       <c r="F57" s="2" t="n">
-        <v>92.33</v>
+        <v>84.5</v>
       </c>
       <c r="G57" s="2" t="n">
-        <v>99.18000000000001</v>
+        <v>91.81</v>
       </c>
       <c r="H57" s="2" t="n">
-        <v>91.95</v>
+        <v>82.15000000000001</v>
       </c>
       <c r="I57" s="2" t="n">
-        <v>85.09999999999999</v>
+        <v>69.70999999999999</v>
       </c>
       <c r="J57" s="2" t="n">
-        <v>91.52</v>
+        <v>76.84</v>
       </c>
       <c r="K57" s="2" t="n">
-        <v>11.754</v>
+        <v>2.596</v>
       </c>
       <c r="L57" s="2" t="n">
-        <v>20.661</v>
+        <v>0.62</v>
       </c>
       <c r="M57" s="2" t="n">
-        <v>26.3246</v>
+        <v>2.2136</v>
       </c>
       <c r="N57" t="inlineStr">
         <is>
-          <t>baseline</t>
+          <t>str_tass</t>
         </is>
       </c>
     </row>
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t>baseline</t>
+          <t>STR-Fusion</t>
         </is>
       </c>
       <c r="B58" t="inlineStr">
         <is>
-          <t>Run1</t>
-        </is>
-      </c>
-      <c r="C58" t="inlineStr"/>
+          <t>Run2_TASS</t>
+        </is>
+      </c>
+      <c r="C58" t="inlineStr">
+        <is>
+          <t>C0_TOKEN</t>
+        </is>
+      </c>
       <c r="D58" t="inlineStr">
         <is>
-          <t>SYSU-CD-256</t>
+          <t>WHU-CD-256</t>
         </is>
       </c>
       <c r="E58" s="2" t="n">
-        <v>80.77</v>
+        <v>90.16</v>
       </c>
       <c r="F58" s="2" t="n">
-        <v>84.27</v>
+        <v>93.97</v>
       </c>
       <c r="G58" s="2" t="n">
-        <v>91.91</v>
+        <v>99.38</v>
       </c>
       <c r="H58" s="2" t="n">
-        <v>82.48</v>
+        <v>92.02</v>
       </c>
       <c r="I58" s="2" t="n">
-        <v>70.19</v>
+        <v>85.23</v>
       </c>
       <c r="J58" s="2" t="n">
-        <v>77.23</v>
+        <v>91.7</v>
       </c>
       <c r="K58" s="2" t="n">
-        <v>11.754</v>
+        <v>2.596</v>
       </c>
       <c r="L58" s="2" t="n">
-        <v>20.661</v>
+        <v>0.62</v>
       </c>
       <c r="M58" s="2" t="n">
-        <v>26.3246</v>
+        <v>2.2136</v>
       </c>
       <c r="N58" t="inlineStr">
         <is>
-          <t>baseline</t>
+          <t>str_tass</t>
         </is>
       </c>
     </row>
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
+          <t>STR-Fusion</t>
+        </is>
+      </c>
+      <c r="B59" t="inlineStr">
+        <is>
+          <t>Run2_TASS</t>
+        </is>
+      </c>
+      <c r="C59" t="inlineStr">
+        <is>
+          <t>M1_TASS</t>
+        </is>
+      </c>
+      <c r="D59" t="inlineStr">
+        <is>
+          <t>CDD-CD-256</t>
+        </is>
+      </c>
+      <c r="E59" s="2" t="n">
+        <v>94.7</v>
+      </c>
+      <c r="F59" s="2" t="n">
+        <v>96.13</v>
+      </c>
+      <c r="G59" s="2" t="n">
+        <v>98.88</v>
+      </c>
+      <c r="H59" s="2" t="n">
+        <v>95.41</v>
+      </c>
+      <c r="I59" s="2" t="n">
+        <v>91.22</v>
+      </c>
+      <c r="J59" s="2" t="n">
+        <v>94.77</v>
+      </c>
+      <c r="K59" s="2" t="n">
+        <v>3.455</v>
+      </c>
+      <c r="L59" s="2" t="n">
+        <v>1.478</v>
+      </c>
+      <c r="M59" s="2" t="n">
+        <v>3.5459</v>
+      </c>
+      <c r="N59" t="inlineStr">
+        <is>
+          <t>str_tass</t>
+        </is>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" t="inlineStr">
+        <is>
+          <t>STR-Fusion</t>
+        </is>
+      </c>
+      <c r="B60" t="inlineStr">
+        <is>
+          <t>Run2_TASS</t>
+        </is>
+      </c>
+      <c r="C60" t="inlineStr">
+        <is>
+          <t>M1_TASS</t>
+        </is>
+      </c>
+      <c r="D60" t="inlineStr">
+        <is>
+          <t>LEVIR-CD-256</t>
+        </is>
+      </c>
+      <c r="E60" s="2" t="n">
+        <v>88.42</v>
+      </c>
+      <c r="F60" s="2" t="n">
+        <v>91.97</v>
+      </c>
+      <c r="G60" s="2" t="n">
+        <v>99.02</v>
+      </c>
+      <c r="H60" s="2" t="n">
+        <v>90.16</v>
+      </c>
+      <c r="I60" s="2" t="n">
+        <v>82.08</v>
+      </c>
+      <c r="J60" s="2" t="n">
+        <v>89.64</v>
+      </c>
+      <c r="K60" s="2" t="n">
+        <v>3.455</v>
+      </c>
+      <c r="L60" s="2" t="n">
+        <v>1.478</v>
+      </c>
+      <c r="M60" s="2" t="n">
+        <v>3.5459</v>
+      </c>
+      <c r="N60" t="inlineStr">
+        <is>
+          <t>str_tass</t>
+        </is>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" t="inlineStr">
+        <is>
+          <t>STR-Fusion</t>
+        </is>
+      </c>
+      <c r="B61" t="inlineStr">
+        <is>
+          <t>Run2_TASS</t>
+        </is>
+      </c>
+      <c r="C61" t="inlineStr">
+        <is>
+          <t>M1_TASS</t>
+        </is>
+      </c>
+      <c r="D61" t="inlineStr">
+        <is>
+          <t>SYSU-CD-256</t>
+        </is>
+      </c>
+      <c r="E61" s="2" t="n">
+        <v>78.73</v>
+      </c>
+      <c r="F61" s="2" t="n">
+        <v>84.98</v>
+      </c>
+      <c r="G61" s="2" t="n">
+        <v>91.7</v>
+      </c>
+      <c r="H61" s="2" t="n">
+        <v>81.73999999999999</v>
+      </c>
+      <c r="I61" s="2" t="n">
+        <v>69.11</v>
+      </c>
+      <c r="J61" s="2" t="n">
+        <v>76.38</v>
+      </c>
+      <c r="K61" s="2" t="n">
+        <v>3.455</v>
+      </c>
+      <c r="L61" s="2" t="n">
+        <v>1.478</v>
+      </c>
+      <c r="M61" s="2" t="n">
+        <v>3.5459</v>
+      </c>
+      <c r="N61" t="inlineStr">
+        <is>
+          <t>str_tass</t>
+        </is>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" t="inlineStr">
+        <is>
+          <t>STR-Fusion</t>
+        </is>
+      </c>
+      <c r="B62" t="inlineStr">
+        <is>
+          <t>Run2_TASS</t>
+        </is>
+      </c>
+      <c r="C62" t="inlineStr">
+        <is>
+          <t>M1_TASS</t>
+        </is>
+      </c>
+      <c r="D62" t="inlineStr">
+        <is>
+          <t>WHU-CD-256</t>
+        </is>
+      </c>
+      <c r="E62" s="2" t="n">
+        <v>91.64</v>
+      </c>
+      <c r="F62" s="2" t="n">
+        <v>94.81999999999999</v>
+      </c>
+      <c r="G62" s="2" t="n">
+        <v>99.47</v>
+      </c>
+      <c r="H62" s="2" t="n">
+        <v>93.2</v>
+      </c>
+      <c r="I62" s="2" t="n">
+        <v>87.27</v>
+      </c>
+      <c r="J62" s="2" t="n">
+        <v>92.93000000000001</v>
+      </c>
+      <c r="K62" s="2" t="n">
+        <v>3.455</v>
+      </c>
+      <c r="L62" s="2" t="n">
+        <v>1.478</v>
+      </c>
+      <c r="M62" s="2" t="n">
+        <v>3.5459</v>
+      </c>
+      <c r="N62" t="inlineStr">
+        <is>
+          <t>str_tass</t>
+        </is>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" t="inlineStr">
+        <is>
+          <t>UltraLight</t>
+        </is>
+      </c>
+      <c r="B63" t="inlineStr">
+        <is>
+          <t>Run4</t>
+        </is>
+      </c>
+      <c r="C63" t="inlineStr">
+        <is>
+          <t>R4_0_A0_FULL12_FROZEN</t>
+        </is>
+      </c>
+      <c r="D63" t="inlineStr">
+        <is>
+          <t>SYSU-CD-256</t>
+        </is>
+      </c>
+      <c r="E63" s="2" t="n">
+        <v>82.42</v>
+      </c>
+      <c r="F63" s="2" t="n">
+        <v>83.87</v>
+      </c>
+      <c r="G63" s="2" t="n">
+        <v>92.12</v>
+      </c>
+      <c r="H63" s="2" t="n">
+        <v>83.14</v>
+      </c>
+      <c r="I63" s="2" t="n">
+        <v>71.14</v>
+      </c>
+      <c r="J63" s="2" t="n">
+        <v>77.98999999999999</v>
+      </c>
+      <c r="K63" s="2" t="n">
+        <v>11.754</v>
+      </c>
+      <c r="L63" s="2" t="n">
+        <v>15.125</v>
+      </c>
+      <c r="M63" s="2" t="n">
+        <v>26.3246</v>
+      </c>
+      <c r="N63" t="inlineStr">
+        <is>
           <t>baseline</t>
         </is>
       </c>
-      <c r="B59" t="inlineStr">
+    </row>
+    <row r="64">
+      <c r="A64" t="inlineStr">
+        <is>
+          <t>UltraLight</t>
+        </is>
+      </c>
+      <c r="B64" t="inlineStr">
+        <is>
+          <t>Run4</t>
+        </is>
+      </c>
+      <c r="C64" t="inlineStr">
+        <is>
+          <t>R4_1_VIT4_OLDHEAD</t>
+        </is>
+      </c>
+      <c r="D64" t="inlineStr">
+        <is>
+          <t>SYSU-CD-256</t>
+        </is>
+      </c>
+      <c r="E64" s="2" t="n">
+        <v>82.15000000000001</v>
+      </c>
+      <c r="F64" s="2" t="n">
+        <v>83.40000000000001</v>
+      </c>
+      <c r="G64" s="2" t="n">
+        <v>91.94</v>
+      </c>
+      <c r="H64" s="2" t="n">
+        <v>82.77</v>
+      </c>
+      <c r="I64" s="2" t="n">
+        <v>70.61</v>
+      </c>
+      <c r="J64" s="2" t="n">
+        <v>77.51000000000001</v>
+      </c>
+      <c r="K64" s="2" t="n">
+        <v>8.195</v>
+      </c>
+      <c r="L64" s="2" t="n">
+        <v>15.125</v>
+      </c>
+      <c r="M64" s="2" t="n">
+        <v>24.1021</v>
+      </c>
+      <c r="N64" t="inlineStr">
+        <is>
+          <t>baseline</t>
+        </is>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" t="inlineStr">
+        <is>
+          <t>UltraLight</t>
+        </is>
+      </c>
+      <c r="B65" t="inlineStr">
+        <is>
+          <t>Run4</t>
+        </is>
+      </c>
+      <c r="C65" t="inlineStr">
+        <is>
+          <t>R4_2_VIT4_LIGHTDETAIL</t>
+        </is>
+      </c>
+      <c r="D65" t="inlineStr">
+        <is>
+          <t>SYSU-CD-256</t>
+        </is>
+      </c>
+      <c r="E65" s="2" t="n">
+        <v>79.94</v>
+      </c>
+      <c r="F65" s="2" t="n">
+        <v>84.79000000000001</v>
+      </c>
+      <c r="G65" s="2" t="n">
+        <v>91.89</v>
+      </c>
+      <c r="H65" s="2" t="n">
+        <v>82.3</v>
+      </c>
+      <c r="I65" s="2" t="n">
+        <v>69.92</v>
+      </c>
+      <c r="J65" s="2" t="n">
+        <v>77.04000000000001</v>
+      </c>
+      <c r="K65" s="2" t="n">
+        <v>5.492</v>
+      </c>
+      <c r="L65" s="2" t="n">
+        <v>3.515</v>
+      </c>
+      <c r="M65" s="2" t="n">
+        <v>10.7311</v>
+      </c>
+      <c r="N65" t="inlineStr">
+        <is>
+          <t>baseline</t>
+        </is>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" t="inlineStr">
+        <is>
+          <t>UltraLight</t>
+        </is>
+      </c>
+      <c r="B66" t="inlineStr">
+        <is>
+          <t>Run4</t>
+        </is>
+      </c>
+      <c r="C66" t="inlineStr">
+        <is>
+          <t>R4_2b_VIT4_LIGHTDETAIL48</t>
+        </is>
+      </c>
+      <c r="D66" t="inlineStr">
+        <is>
+          <t>SYSU-CD-256</t>
+        </is>
+      </c>
+      <c r="E66" s="2" t="n">
+        <v>80.87</v>
+      </c>
+      <c r="F66" s="2" t="n">
+        <v>83.81</v>
+      </c>
+      <c r="G66" s="2" t="n">
+        <v>91.81</v>
+      </c>
+      <c r="H66" s="2" t="n">
+        <v>82.31999999999999</v>
+      </c>
+      <c r="I66" s="2" t="n">
+        <v>69.95</v>
+      </c>
+      <c r="J66" s="2" t="n">
+        <v>76.98999999999999</v>
+      </c>
+      <c r="K66" s="2" t="n">
+        <v>5.533</v>
+      </c>
+      <c r="L66" s="2" t="n">
+        <v>3.556</v>
+      </c>
+      <c r="M66" s="2" t="n">
+        <v>10.9824</v>
+      </c>
+      <c r="N66" t="inlineStr">
+        <is>
+          <t>baseline</t>
+        </is>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" t="inlineStr">
+        <is>
+          <t>UltraLight</t>
+        </is>
+      </c>
+      <c r="B67" t="inlineStr">
+        <is>
+          <t>Run4</t>
+        </is>
+      </c>
+      <c r="C67" t="inlineStr">
+        <is>
+          <t>R4_2d_PSD_DETAIL</t>
+        </is>
+      </c>
+      <c r="D67" t="inlineStr">
+        <is>
+          <t>SYSU-CD-256</t>
+        </is>
+      </c>
+      <c r="E67" s="2" t="n">
+        <v>79.78</v>
+      </c>
+      <c r="F67" s="2" t="n">
+        <v>84.39</v>
+      </c>
+      <c r="G67" s="2" t="n">
+        <v>91.75</v>
+      </c>
+      <c r="H67" s="2" t="n">
+        <v>82.02</v>
+      </c>
+      <c r="I67" s="2" t="n">
+        <v>69.52</v>
+      </c>
+      <c r="J67" s="2" t="n">
+        <v>76.68000000000001</v>
+      </c>
+      <c r="K67" s="2" t="n">
+        <v>5.491</v>
+      </c>
+      <c r="L67" s="2" t="n">
+        <v>3.514</v>
+      </c>
+      <c r="M67" s="2" t="n">
+        <v>11.5239</v>
+      </c>
+      <c r="N67" t="inlineStr">
+        <is>
+          <t>baseline</t>
+        </is>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" t="inlineStr">
+        <is>
+          <t>baseline</t>
+        </is>
+      </c>
+      <c r="B68" t="inlineStr">
         <is>
           <t>Run1</t>
         </is>
       </c>
-      <c r="C59" t="inlineStr"/>
-      <c r="D59" t="inlineStr">
+      <c r="C68" t="inlineStr"/>
+      <c r="D68" t="inlineStr">
+        <is>
+          <t>CDD-CD-256</t>
+        </is>
+      </c>
+      <c r="E68" s="2" t="n">
+        <v>97.72</v>
+      </c>
+      <c r="F68" s="2" t="n">
+        <v>97.78</v>
+      </c>
+      <c r="G68" s="2" t="n">
+        <v>99.44</v>
+      </c>
+      <c r="H68" s="2" t="n">
+        <v>97.75</v>
+      </c>
+      <c r="I68" s="2" t="n">
+        <v>95.59999999999999</v>
+      </c>
+      <c r="J68" s="2" t="n">
+        <v>97.43000000000001</v>
+      </c>
+      <c r="K68" s="2" t="n">
+        <v>11.754</v>
+      </c>
+      <c r="L68" s="2" t="n">
+        <v>20.661</v>
+      </c>
+      <c r="M68" s="2" t="n">
+        <v>26.3246</v>
+      </c>
+      <c r="N68" t="inlineStr">
+        <is>
+          <t>baseline</t>
+        </is>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" t="inlineStr">
+        <is>
+          <t>baseline</t>
+        </is>
+      </c>
+      <c r="B69" t="inlineStr">
+        <is>
+          <t>Run1</t>
+        </is>
+      </c>
+      <c r="C69" t="inlineStr"/>
+      <c r="D69" t="inlineStr">
+        <is>
+          <t>LEVIR-CD-256</t>
+        </is>
+      </c>
+      <c r="E69" s="2" t="n">
+        <v>91.56999999999999</v>
+      </c>
+      <c r="F69" s="2" t="n">
+        <v>92.33</v>
+      </c>
+      <c r="G69" s="2" t="n">
+        <v>99.18000000000001</v>
+      </c>
+      <c r="H69" s="2" t="n">
+        <v>91.95</v>
+      </c>
+      <c r="I69" s="2" t="n">
+        <v>85.09999999999999</v>
+      </c>
+      <c r="J69" s="2" t="n">
+        <v>91.52</v>
+      </c>
+      <c r="K69" s="2" t="n">
+        <v>11.754</v>
+      </c>
+      <c r="L69" s="2" t="n">
+        <v>20.661</v>
+      </c>
+      <c r="M69" s="2" t="n">
+        <v>26.3246</v>
+      </c>
+      <c r="N69" t="inlineStr">
+        <is>
+          <t>baseline</t>
+        </is>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" t="inlineStr">
+        <is>
+          <t>baseline</t>
+        </is>
+      </c>
+      <c r="B70" t="inlineStr">
+        <is>
+          <t>Run1</t>
+        </is>
+      </c>
+      <c r="C70" t="inlineStr"/>
+      <c r="D70" t="inlineStr">
+        <is>
+          <t>SYSU-CD-256</t>
+        </is>
+      </c>
+      <c r="E70" s="2" t="n">
+        <v>80.77</v>
+      </c>
+      <c r="F70" s="2" t="n">
+        <v>84.27</v>
+      </c>
+      <c r="G70" s="2" t="n">
+        <v>91.91</v>
+      </c>
+      <c r="H70" s="2" t="n">
+        <v>82.48</v>
+      </c>
+      <c r="I70" s="2" t="n">
+        <v>70.19</v>
+      </c>
+      <c r="J70" s="2" t="n">
+        <v>77.23</v>
+      </c>
+      <c r="K70" s="2" t="n">
+        <v>11.754</v>
+      </c>
+      <c r="L70" s="2" t="n">
+        <v>20.661</v>
+      </c>
+      <c r="M70" s="2" t="n">
+        <v>26.3246</v>
+      </c>
+      <c r="N70" t="inlineStr">
+        <is>
+          <t>baseline</t>
+        </is>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" t="inlineStr">
+        <is>
+          <t>baseline</t>
+        </is>
+      </c>
+      <c r="B71" t="inlineStr">
+        <is>
+          <t>Run1</t>
+        </is>
+      </c>
+      <c r="C71" t="inlineStr"/>
+      <c r="D71" t="inlineStr">
         <is>
           <t>WHU-CD-256</t>
         </is>
       </c>
-      <c r="E59" s="2" t="n">
+      <c r="E71" s="2" t="n">
         <v>93.62</v>
       </c>
-      <c r="F59" s="2" t="n">
+      <c r="F71" s="2" t="n">
         <v>96.09</v>
       </c>
-      <c r="G59" s="2" t="n">
+      <c r="G71" s="2" t="n">
         <v>99.59999999999999</v>
       </c>
-      <c r="H59" s="2" t="n">
+      <c r="H71" s="2" t="n">
         <v>94.84</v>
       </c>
-      <c r="I59" s="2" t="n">
+      <c r="I71" s="2" t="n">
         <v>90.18000000000001</v>
       </c>
-      <c r="J59" s="2" t="n">
+      <c r="J71" s="2" t="n">
         <v>94.63</v>
       </c>
-      <c r="K59" s="2" t="n">
+      <c r="K71" s="2" t="n">
         <v>11.754</v>
       </c>
-      <c r="L59" s="2" t="n">
+      <c r="L71" s="2" t="n">
         <v>20.661</v>
       </c>
-      <c r="M59" s="2" t="n">
+      <c r="M71" s="2" t="n">
         <v>26.3246</v>
       </c>
-      <c r="N59" t="inlineStr">
+      <c r="N71" t="inlineStr">
         <is>
           <t>baseline</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:N59"/>
+  <autoFilter ref="A1:N71"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Run3 complete: E4/E5 both FAIL pre-registered conditions; D2 retest (E4 small 0.1842 best-of-five, E5 small R lowest); decision tree -> S2-HCAACP/SP-DCR; report/README/xlsx/snapshot
</commit_message>
<xml_diff>
--- a/docs/experiment_metrics.xlsx
+++ b/docs/experiment_metrics.xlsx
@@ -10,7 +10,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="metrics" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'metrics'!$A$1:$N$71</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'metrics'!$A$1:$N$79</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -420,7 +420,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N71"/>
+  <dimension ref="A1:N79"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -2890,432 +2890,432 @@
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>CASAA</t>
+          <t>CASA-TViM</t>
         </is>
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>Run1</t>
+          <t>Run3</t>
         </is>
       </c>
       <c r="C46" t="inlineStr">
         <is>
-          <t>A1_SAA</t>
+          <t>E4_RA_CAACP</t>
         </is>
       </c>
       <c r="D46" t="inlineStr">
         <is>
-          <t>LEVIR-CD-256</t>
+          <t>CDD-CD-256</t>
         </is>
       </c>
       <c r="E46" s="2" t="n">
-        <v>91.09</v>
+        <v>97.02</v>
       </c>
       <c r="F46" s="2" t="n">
-        <v>92.8</v>
+        <v>97.25</v>
       </c>
       <c r="G46" s="2" t="n">
-        <v>99.19</v>
+        <v>99.29000000000001</v>
       </c>
       <c r="H46" s="2" t="n">
-        <v>91.94</v>
+        <v>97.13</v>
       </c>
       <c r="I46" s="2" t="n">
-        <v>85.08</v>
+        <v>94.42</v>
       </c>
       <c r="J46" s="2" t="n">
-        <v>91.51000000000001</v>
+        <v>96.73</v>
       </c>
       <c r="K46" s="2" t="n">
-        <v>11.754</v>
+        <v>4.88</v>
       </c>
       <c r="L46" s="2" t="n">
-        <v>20.661</v>
+        <v>4.88</v>
       </c>
       <c r="M46" s="2" t="n">
-        <v>26.3183</v>
+        <v>2.6747</v>
       </c>
       <c r="N46" t="inlineStr">
         <is>
-          <t>saa</t>
+          <t>casa_tvim_str</t>
         </is>
       </c>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>CASAA</t>
+          <t>CASA-TViM</t>
         </is>
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>Run1</t>
+          <t>Run3</t>
         </is>
       </c>
       <c r="C47" t="inlineStr">
         <is>
-          <t>A1_SAA</t>
+          <t>E4_RA_CAACP</t>
         </is>
       </c>
       <c r="D47" t="inlineStr">
         <is>
-          <t>SYSU-CD-256</t>
+          <t>LEVIR-CD-256</t>
         </is>
       </c>
       <c r="E47" s="2" t="n">
-        <v>80.3</v>
+        <v>90.05</v>
       </c>
       <c r="F47" s="2" t="n">
-        <v>84.81</v>
+        <v>92.12</v>
       </c>
       <c r="G47" s="2" t="n">
-        <v>91.95999999999999</v>
+        <v>99.09999999999999</v>
       </c>
       <c r="H47" s="2" t="n">
-        <v>82.5</v>
+        <v>91.06999999999999</v>
       </c>
       <c r="I47" s="2" t="n">
-        <v>70.20999999999999</v>
+        <v>83.59999999999999</v>
       </c>
       <c r="J47" s="2" t="n">
-        <v>77.29000000000001</v>
+        <v>90.59999999999999</v>
       </c>
       <c r="K47" s="2" t="n">
-        <v>11.754</v>
+        <v>4.88</v>
       </c>
       <c r="L47" s="2" t="n">
-        <v>20.661</v>
+        <v>4.88</v>
       </c>
       <c r="M47" s="2" t="n">
-        <v>26.3183</v>
+        <v>2.6747</v>
       </c>
       <c r="N47" t="inlineStr">
         <is>
-          <t>saa</t>
+          <t>casa_tvim_str</t>
         </is>
       </c>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>CASAA</t>
+          <t>CASA-TViM</t>
         </is>
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>Run1</t>
+          <t>Run3</t>
         </is>
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>A2_CASAA</t>
+          <t>E4_RA_CAACP</t>
         </is>
       </c>
       <c r="D48" t="inlineStr">
         <is>
-          <t>LEVIR-CD-256</t>
+          <t>SYSU-CD-256</t>
         </is>
       </c>
       <c r="E48" s="2" t="n">
-        <v>90.98999999999999</v>
+        <v>81.44</v>
       </c>
       <c r="F48" s="2" t="n">
-        <v>92.75</v>
+        <v>84.94</v>
       </c>
       <c r="G48" s="2" t="n">
-        <v>99.18000000000001</v>
+        <v>92.22</v>
       </c>
       <c r="H48" s="2" t="n">
-        <v>91.86</v>
+        <v>83.16</v>
       </c>
       <c r="I48" s="2" t="n">
-        <v>84.94</v>
+        <v>71.17</v>
       </c>
       <c r="J48" s="2" t="n">
-        <v>91.43000000000001</v>
+        <v>78.09999999999999</v>
       </c>
       <c r="K48" s="2" t="n">
-        <v>11.754</v>
+        <v>4.88</v>
       </c>
       <c r="L48" s="2" t="n">
-        <v>20.661</v>
+        <v>4.88</v>
       </c>
       <c r="M48" s="2" t="n">
-        <v>26.2593</v>
+        <v>2.6747</v>
       </c>
       <c r="N48" t="inlineStr">
         <is>
-          <t>casaa</t>
+          <t>casa_tvim_str</t>
         </is>
       </c>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>CASAA</t>
+          <t>CASA-TViM</t>
         </is>
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>Run1</t>
+          <t>Run3</t>
         </is>
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>A2_CASAA</t>
+          <t>E4_RA_CAACP</t>
         </is>
       </c>
       <c r="D49" t="inlineStr">
         <is>
-          <t>SYSU-CD-256</t>
+          <t>WHU-CD-256</t>
         </is>
       </c>
       <c r="E49" s="2" t="n">
-        <v>80.55</v>
+        <v>93.42</v>
       </c>
       <c r="F49" s="2" t="n">
-        <v>84.23</v>
+        <v>96.66</v>
       </c>
       <c r="G49" s="2" t="n">
-        <v>91.86</v>
+        <v>99.61</v>
       </c>
       <c r="H49" s="2" t="n">
-        <v>82.34999999999999</v>
+        <v>95.02</v>
       </c>
       <c r="I49" s="2" t="n">
-        <v>70</v>
+        <v>90.5</v>
       </c>
       <c r="J49" s="2" t="n">
-        <v>77.06</v>
+        <v>94.81</v>
       </c>
       <c r="K49" s="2" t="n">
-        <v>11.754</v>
+        <v>4.88</v>
       </c>
       <c r="L49" s="2" t="n">
-        <v>20.661</v>
+        <v>4.88</v>
       </c>
       <c r="M49" s="2" t="n">
-        <v>26.2593</v>
+        <v>2.6747</v>
       </c>
       <c r="N49" t="inlineStr">
         <is>
-          <t>casaa</t>
+          <t>casa_tvim_str</t>
         </is>
       </c>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>CASAA</t>
+          <t>CASA-TViM</t>
         </is>
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>Run2</t>
+          <t>Run3</t>
         </is>
       </c>
       <c r="C50" t="inlineStr">
         <is>
-          <t>A1_SAA_FROZEN</t>
+          <t>E5_FS_TAR</t>
         </is>
       </c>
       <c r="D50" t="inlineStr">
         <is>
-          <t>LEVIR-CD-256</t>
+          <t>CDD-CD-256</t>
         </is>
       </c>
       <c r="E50" s="2" t="n">
-        <v>91.38</v>
+        <v>97.03</v>
       </c>
       <c r="F50" s="2" t="n">
-        <v>92.3</v>
+        <v>97.23999999999999</v>
       </c>
       <c r="G50" s="2" t="n">
-        <v>99.17</v>
+        <v>99.29000000000001</v>
       </c>
       <c r="H50" s="2" t="n">
-        <v>91.84</v>
+        <v>97.13</v>
       </c>
       <c r="I50" s="2" t="n">
-        <v>84.91</v>
+        <v>94.43000000000001</v>
       </c>
       <c r="J50" s="2" t="n">
-        <v>91.40000000000001</v>
+        <v>96.73</v>
       </c>
       <c r="K50" s="2" t="n">
-        <v>11.754</v>
+        <v>4.954</v>
       </c>
       <c r="L50" s="2" t="n">
-        <v>15.125</v>
+        <v>4.954</v>
       </c>
       <c r="M50" s="2" t="n">
-        <v>26.1484</v>
+        <v>2.9767</v>
       </c>
       <c r="N50" t="inlineStr">
         <is>
-          <t>saa</t>
+          <t>casa_tvim_str</t>
         </is>
       </c>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>CASAA</t>
+          <t>CASA-TViM</t>
         </is>
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>Run2</t>
+          <t>Run3</t>
         </is>
       </c>
       <c r="C51" t="inlineStr">
         <is>
-          <t>A1_SAA_FROZEN</t>
+          <t>E5_FS_TAR</t>
         </is>
       </c>
       <c r="D51" t="inlineStr">
         <is>
-          <t>SYSU-CD-256</t>
+          <t>LEVIR-CD-256</t>
         </is>
       </c>
       <c r="E51" s="2" t="n">
-        <v>78.40000000000001</v>
+        <v>90.25</v>
       </c>
       <c r="F51" s="2" t="n">
-        <v>86.03</v>
+        <v>92.12</v>
       </c>
       <c r="G51" s="2" t="n">
-        <v>91.90000000000001</v>
+        <v>99.11</v>
       </c>
       <c r="H51" s="2" t="n">
-        <v>82.04000000000001</v>
+        <v>91.18000000000001</v>
       </c>
       <c r="I51" s="2" t="n">
-        <v>69.55</v>
+        <v>83.78</v>
       </c>
       <c r="J51" s="2" t="n">
-        <v>76.83</v>
+        <v>90.70999999999999</v>
       </c>
       <c r="K51" s="2" t="n">
-        <v>11.754</v>
+        <v>4.954</v>
       </c>
       <c r="L51" s="2" t="n">
-        <v>15.125</v>
+        <v>4.954</v>
       </c>
       <c r="M51" s="2" t="n">
-        <v>26.1484</v>
+        <v>2.9767</v>
       </c>
       <c r="N51" t="inlineStr">
         <is>
-          <t>saa</t>
+          <t>casa_tvim_str</t>
         </is>
       </c>
     </row>
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>CASAA</t>
+          <t>CASA-TViM</t>
         </is>
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t>Run2</t>
+          <t>Run3</t>
         </is>
       </c>
       <c r="C52" t="inlineStr">
         <is>
-          <t>A3_ORACLE_FROZEN</t>
+          <t>E5_FS_TAR</t>
         </is>
       </c>
       <c r="D52" t="inlineStr">
         <is>
-          <t>LEVIR-CD-256</t>
+          <t>SYSU-CD-256</t>
         </is>
       </c>
       <c r="E52" s="2" t="n">
-        <v>91.13</v>
+        <v>81.26000000000001</v>
       </c>
       <c r="F52" s="2" t="n">
-        <v>92.65000000000001</v>
+        <v>85.31</v>
       </c>
       <c r="G52" s="2" t="n">
-        <v>99.18000000000001</v>
+        <v>92.28</v>
       </c>
       <c r="H52" s="2" t="n">
-        <v>91.88</v>
+        <v>83.23999999999999</v>
       </c>
       <c r="I52" s="2" t="n">
-        <v>84.98</v>
+        <v>71.29000000000001</v>
       </c>
       <c r="J52" s="2" t="n">
-        <v>91.45</v>
+        <v>78.23</v>
       </c>
       <c r="K52" s="2" t="n">
-        <v>11.754</v>
+        <v>4.954</v>
       </c>
       <c r="L52" s="2" t="n">
-        <v>15.125</v>
+        <v>4.954</v>
       </c>
       <c r="M52" s="2" t="n">
-        <v>26.0894</v>
+        <v>2.9767</v>
       </c>
       <c r="N52" t="inlineStr">
         <is>
-          <t>casaa</t>
+          <t>casa_tvim_str</t>
         </is>
       </c>
     </row>
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>CASAA</t>
+          <t>CASA-TViM</t>
         </is>
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>Run2</t>
+          <t>Run3</t>
         </is>
       </c>
       <c r="C53" t="inlineStr">
         <is>
-          <t>A3_ORACLE_FROZEN</t>
+          <t>E5_FS_TAR</t>
         </is>
       </c>
       <c r="D53" t="inlineStr">
         <is>
-          <t>SYSU-CD-256</t>
+          <t>WHU-CD-256</t>
         </is>
       </c>
       <c r="E53" s="2" t="n">
-        <v>82.04000000000001</v>
+        <v>93.11</v>
       </c>
       <c r="F53" s="2" t="n">
-        <v>85.05</v>
+        <v>96.78</v>
       </c>
       <c r="G53" s="2" t="n">
-        <v>92.36</v>
+        <v>99.59999999999999</v>
       </c>
       <c r="H53" s="2" t="n">
-        <v>83.52</v>
+        <v>94.91</v>
       </c>
       <c r="I53" s="2" t="n">
-        <v>71.7</v>
+        <v>90.31</v>
       </c>
       <c r="J53" s="2" t="n">
-        <v>78.55</v>
+        <v>94.7</v>
       </c>
       <c r="K53" s="2" t="n">
-        <v>11.754</v>
+        <v>4.954</v>
       </c>
       <c r="L53" s="2" t="n">
-        <v>15.125</v>
+        <v>4.954</v>
       </c>
       <c r="M53" s="2" t="n">
-        <v>26.0894</v>
+        <v>2.9767</v>
       </c>
       <c r="N53" t="inlineStr">
         <is>
-          <t>casaa</t>
+          <t>casa_tvim_str</t>
         </is>
       </c>
     </row>
@@ -3327,120 +3327,120 @@
       </c>
       <c r="B54" t="inlineStr">
         <is>
-          <t>Run3</t>
+          <t>Run1</t>
         </is>
       </c>
       <c r="C54" t="inlineStr">
         <is>
-          <t>A4_DETAIL_FROZEN</t>
+          <t>A1_SAA</t>
         </is>
       </c>
       <c r="D54" t="inlineStr">
         <is>
-          <t>SYSU-CD-256</t>
+          <t>LEVIR-CD-256</t>
         </is>
       </c>
       <c r="E54" s="2" t="n">
-        <v>79.68000000000001</v>
+        <v>91.09</v>
       </c>
       <c r="F54" s="2" t="n">
-        <v>84.28</v>
+        <v>92.8</v>
       </c>
       <c r="G54" s="2" t="n">
-        <v>91.7</v>
+        <v>99.19</v>
       </c>
       <c r="H54" s="2" t="n">
-        <v>81.92</v>
+        <v>91.94</v>
       </c>
       <c r="I54" s="2" t="n">
-        <v>69.37</v>
+        <v>85.08</v>
       </c>
       <c r="J54" s="2" t="n">
-        <v>76.54000000000001</v>
+        <v>91.51000000000001</v>
       </c>
       <c r="K54" s="2" t="n">
         <v>11.754</v>
       </c>
       <c r="L54" s="2" t="n">
-        <v>15.125</v>
+        <v>20.661</v>
       </c>
       <c r="M54" s="2" t="n">
-        <v>26.0894</v>
+        <v>26.3183</v>
       </c>
       <c r="N54" t="inlineStr">
         <is>
-          <t>casaa</t>
+          <t>saa</t>
         </is>
       </c>
     </row>
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>STR-Fusion</t>
+          <t>CASAA</t>
         </is>
       </c>
       <c r="B55" t="inlineStr">
         <is>
-          <t>Run2_TASS</t>
+          <t>Run1</t>
         </is>
       </c>
       <c r="C55" t="inlineStr">
         <is>
-          <t>C0_TOKEN</t>
+          <t>A1_SAA</t>
         </is>
       </c>
       <c r="D55" t="inlineStr">
         <is>
-          <t>CDD-CD-256</t>
+          <t>SYSU-CD-256</t>
         </is>
       </c>
       <c r="E55" s="2" t="n">
-        <v>93.13</v>
+        <v>80.3</v>
       </c>
       <c r="F55" s="2" t="n">
-        <v>95.16</v>
+        <v>84.81</v>
       </c>
       <c r="G55" s="2" t="n">
-        <v>98.56999999999999</v>
+        <v>91.95999999999999</v>
       </c>
       <c r="H55" s="2" t="n">
-        <v>94.13</v>
+        <v>82.5</v>
       </c>
       <c r="I55" s="2" t="n">
-        <v>88.91</v>
+        <v>70.20999999999999</v>
       </c>
       <c r="J55" s="2" t="n">
-        <v>93.31999999999999</v>
+        <v>77.29000000000001</v>
       </c>
       <c r="K55" s="2" t="n">
-        <v>2.596</v>
+        <v>11.754</v>
       </c>
       <c r="L55" s="2" t="n">
-        <v>0.62</v>
+        <v>20.661</v>
       </c>
       <c r="M55" s="2" t="n">
-        <v>2.2136</v>
+        <v>26.3183</v>
       </c>
       <c r="N55" t="inlineStr">
         <is>
-          <t>str_tass</t>
+          <t>saa</t>
         </is>
       </c>
     </row>
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>STR-Fusion</t>
+          <t>CASAA</t>
         </is>
       </c>
       <c r="B56" t="inlineStr">
         <is>
-          <t>Run2_TASS</t>
+          <t>Run1</t>
         </is>
       </c>
       <c r="C56" t="inlineStr">
         <is>
-          <t>C0_TOKEN</t>
+          <t>A2_CASAA</t>
         </is>
       </c>
       <c r="D56" t="inlineStr">
@@ -3449,52 +3449,52 @@
         </is>
       </c>
       <c r="E56" s="2" t="n">
-        <v>86.37</v>
+        <v>90.98999999999999</v>
       </c>
       <c r="F56" s="2" t="n">
-        <v>89.25</v>
+        <v>92.75</v>
       </c>
       <c r="G56" s="2" t="n">
-        <v>98.78</v>
+        <v>99.18000000000001</v>
       </c>
       <c r="H56" s="2" t="n">
-        <v>87.79000000000001</v>
+        <v>91.86</v>
       </c>
       <c r="I56" s="2" t="n">
-        <v>78.23999999999999</v>
+        <v>84.94</v>
       </c>
       <c r="J56" s="2" t="n">
-        <v>87.14</v>
+        <v>91.43000000000001</v>
       </c>
       <c r="K56" s="2" t="n">
-        <v>2.596</v>
+        <v>11.754</v>
       </c>
       <c r="L56" s="2" t="n">
-        <v>0.62</v>
+        <v>20.661</v>
       </c>
       <c r="M56" s="2" t="n">
-        <v>2.2136</v>
+        <v>26.2593</v>
       </c>
       <c r="N56" t="inlineStr">
         <is>
-          <t>str_tass</t>
+          <t>casaa</t>
         </is>
       </c>
     </row>
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>STR-Fusion</t>
+          <t>CASAA</t>
         </is>
       </c>
       <c r="B57" t="inlineStr">
         <is>
-          <t>Run2_TASS</t>
+          <t>Run1</t>
         </is>
       </c>
       <c r="C57" t="inlineStr">
         <is>
-          <t>C0_TOKEN</t>
+          <t>A2_CASAA</t>
         </is>
       </c>
       <c r="D57" t="inlineStr">
@@ -3503,160 +3503,160 @@
         </is>
       </c>
       <c r="E57" s="2" t="n">
-        <v>79.93000000000001</v>
+        <v>80.55</v>
       </c>
       <c r="F57" s="2" t="n">
-        <v>84.5</v>
+        <v>84.23</v>
       </c>
       <c r="G57" s="2" t="n">
-        <v>91.81</v>
+        <v>91.86</v>
       </c>
       <c r="H57" s="2" t="n">
-        <v>82.15000000000001</v>
+        <v>82.34999999999999</v>
       </c>
       <c r="I57" s="2" t="n">
-        <v>69.70999999999999</v>
+        <v>70</v>
       </c>
       <c r="J57" s="2" t="n">
-        <v>76.84</v>
+        <v>77.06</v>
       </c>
       <c r="K57" s="2" t="n">
-        <v>2.596</v>
+        <v>11.754</v>
       </c>
       <c r="L57" s="2" t="n">
-        <v>0.62</v>
+        <v>20.661</v>
       </c>
       <c r="M57" s="2" t="n">
-        <v>2.2136</v>
+        <v>26.2593</v>
       </c>
       <c r="N57" t="inlineStr">
         <is>
-          <t>str_tass</t>
+          <t>casaa</t>
         </is>
       </c>
     </row>
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t>STR-Fusion</t>
+          <t>CASAA</t>
         </is>
       </c>
       <c r="B58" t="inlineStr">
         <is>
-          <t>Run2_TASS</t>
+          <t>Run2</t>
         </is>
       </c>
       <c r="C58" t="inlineStr">
         <is>
-          <t>C0_TOKEN</t>
+          <t>A1_SAA_FROZEN</t>
         </is>
       </c>
       <c r="D58" t="inlineStr">
         <is>
-          <t>WHU-CD-256</t>
+          <t>LEVIR-CD-256</t>
         </is>
       </c>
       <c r="E58" s="2" t="n">
-        <v>90.16</v>
+        <v>91.38</v>
       </c>
       <c r="F58" s="2" t="n">
-        <v>93.97</v>
+        <v>92.3</v>
       </c>
       <c r="G58" s="2" t="n">
-        <v>99.38</v>
+        <v>99.17</v>
       </c>
       <c r="H58" s="2" t="n">
-        <v>92.02</v>
+        <v>91.84</v>
       </c>
       <c r="I58" s="2" t="n">
-        <v>85.23</v>
+        <v>84.91</v>
       </c>
       <c r="J58" s="2" t="n">
-        <v>91.7</v>
+        <v>91.40000000000001</v>
       </c>
       <c r="K58" s="2" t="n">
-        <v>2.596</v>
+        <v>11.754</v>
       </c>
       <c r="L58" s="2" t="n">
-        <v>0.62</v>
+        <v>15.125</v>
       </c>
       <c r="M58" s="2" t="n">
-        <v>2.2136</v>
+        <v>26.1484</v>
       </c>
       <c r="N58" t="inlineStr">
         <is>
-          <t>str_tass</t>
+          <t>saa</t>
         </is>
       </c>
     </row>
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>STR-Fusion</t>
+          <t>CASAA</t>
         </is>
       </c>
       <c r="B59" t="inlineStr">
         <is>
-          <t>Run2_TASS</t>
+          <t>Run2</t>
         </is>
       </c>
       <c r="C59" t="inlineStr">
         <is>
-          <t>M1_TASS</t>
+          <t>A1_SAA_FROZEN</t>
         </is>
       </c>
       <c r="D59" t="inlineStr">
         <is>
-          <t>CDD-CD-256</t>
+          <t>SYSU-CD-256</t>
         </is>
       </c>
       <c r="E59" s="2" t="n">
-        <v>94.7</v>
+        <v>78.40000000000001</v>
       </c>
       <c r="F59" s="2" t="n">
-        <v>96.13</v>
+        <v>86.03</v>
       </c>
       <c r="G59" s="2" t="n">
-        <v>98.88</v>
+        <v>91.90000000000001</v>
       </c>
       <c r="H59" s="2" t="n">
-        <v>95.41</v>
+        <v>82.04000000000001</v>
       </c>
       <c r="I59" s="2" t="n">
-        <v>91.22</v>
+        <v>69.55</v>
       </c>
       <c r="J59" s="2" t="n">
-        <v>94.77</v>
+        <v>76.83</v>
       </c>
       <c r="K59" s="2" t="n">
-        <v>3.455</v>
+        <v>11.754</v>
       </c>
       <c r="L59" s="2" t="n">
-        <v>1.478</v>
+        <v>15.125</v>
       </c>
       <c r="M59" s="2" t="n">
-        <v>3.5459</v>
+        <v>26.1484</v>
       </c>
       <c r="N59" t="inlineStr">
         <is>
-          <t>str_tass</t>
+          <t>saa</t>
         </is>
       </c>
     </row>
     <row r="60">
       <c r="A60" t="inlineStr">
         <is>
-          <t>STR-Fusion</t>
+          <t>CASAA</t>
         </is>
       </c>
       <c r="B60" t="inlineStr">
         <is>
-          <t>Run2_TASS</t>
+          <t>Run2</t>
         </is>
       </c>
       <c r="C60" t="inlineStr">
         <is>
-          <t>M1_TASS</t>
+          <t>A3_ORACLE_FROZEN</t>
         </is>
       </c>
       <c r="D60" t="inlineStr">
@@ -3665,52 +3665,52 @@
         </is>
       </c>
       <c r="E60" s="2" t="n">
-        <v>88.42</v>
+        <v>91.13</v>
       </c>
       <c r="F60" s="2" t="n">
-        <v>91.97</v>
+        <v>92.65000000000001</v>
       </c>
       <c r="G60" s="2" t="n">
-        <v>99.02</v>
+        <v>99.18000000000001</v>
       </c>
       <c r="H60" s="2" t="n">
-        <v>90.16</v>
+        <v>91.88</v>
       </c>
       <c r="I60" s="2" t="n">
-        <v>82.08</v>
+        <v>84.98</v>
       </c>
       <c r="J60" s="2" t="n">
-        <v>89.64</v>
+        <v>91.45</v>
       </c>
       <c r="K60" s="2" t="n">
-        <v>3.455</v>
+        <v>11.754</v>
       </c>
       <c r="L60" s="2" t="n">
-        <v>1.478</v>
+        <v>15.125</v>
       </c>
       <c r="M60" s="2" t="n">
-        <v>3.5459</v>
+        <v>26.0894</v>
       </c>
       <c r="N60" t="inlineStr">
         <is>
-          <t>str_tass</t>
+          <t>casaa</t>
         </is>
       </c>
     </row>
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t>STR-Fusion</t>
+          <t>CASAA</t>
         </is>
       </c>
       <c r="B61" t="inlineStr">
         <is>
-          <t>Run2_TASS</t>
+          <t>Run2</t>
         </is>
       </c>
       <c r="C61" t="inlineStr">
         <is>
-          <t>M1_TASS</t>
+          <t>A3_ORACLE_FROZEN</t>
         </is>
       </c>
       <c r="D61" t="inlineStr">
@@ -3719,214 +3719,214 @@
         </is>
       </c>
       <c r="E61" s="2" t="n">
-        <v>78.73</v>
+        <v>82.04000000000001</v>
       </c>
       <c r="F61" s="2" t="n">
-        <v>84.98</v>
+        <v>85.05</v>
       </c>
       <c r="G61" s="2" t="n">
-        <v>91.7</v>
+        <v>92.36</v>
       </c>
       <c r="H61" s="2" t="n">
-        <v>81.73999999999999</v>
+        <v>83.52</v>
       </c>
       <c r="I61" s="2" t="n">
-        <v>69.11</v>
+        <v>71.7</v>
       </c>
       <c r="J61" s="2" t="n">
-        <v>76.38</v>
+        <v>78.55</v>
       </c>
       <c r="K61" s="2" t="n">
-        <v>3.455</v>
+        <v>11.754</v>
       </c>
       <c r="L61" s="2" t="n">
-        <v>1.478</v>
+        <v>15.125</v>
       </c>
       <c r="M61" s="2" t="n">
-        <v>3.5459</v>
+        <v>26.0894</v>
       </c>
       <c r="N61" t="inlineStr">
         <is>
-          <t>str_tass</t>
+          <t>casaa</t>
         </is>
       </c>
     </row>
     <row r="62">
       <c r="A62" t="inlineStr">
         <is>
-          <t>STR-Fusion</t>
+          <t>CASAA</t>
         </is>
       </c>
       <c r="B62" t="inlineStr">
         <is>
-          <t>Run2_TASS</t>
+          <t>Run3</t>
         </is>
       </c>
       <c r="C62" t="inlineStr">
         <is>
-          <t>M1_TASS</t>
+          <t>A4_DETAIL_FROZEN</t>
         </is>
       </c>
       <c r="D62" t="inlineStr">
         <is>
-          <t>WHU-CD-256</t>
+          <t>SYSU-CD-256</t>
         </is>
       </c>
       <c r="E62" s="2" t="n">
-        <v>91.64</v>
+        <v>79.68000000000001</v>
       </c>
       <c r="F62" s="2" t="n">
-        <v>94.81999999999999</v>
+        <v>84.28</v>
       </c>
       <c r="G62" s="2" t="n">
-        <v>99.47</v>
+        <v>91.7</v>
       </c>
       <c r="H62" s="2" t="n">
-        <v>93.2</v>
+        <v>81.92</v>
       </c>
       <c r="I62" s="2" t="n">
-        <v>87.27</v>
+        <v>69.37</v>
       </c>
       <c r="J62" s="2" t="n">
-        <v>92.93000000000001</v>
+        <v>76.54000000000001</v>
       </c>
       <c r="K62" s="2" t="n">
-        <v>3.455</v>
+        <v>11.754</v>
       </c>
       <c r="L62" s="2" t="n">
-        <v>1.478</v>
+        <v>15.125</v>
       </c>
       <c r="M62" s="2" t="n">
-        <v>3.5459</v>
+        <v>26.0894</v>
       </c>
       <c r="N62" t="inlineStr">
         <is>
-          <t>str_tass</t>
+          <t>casaa</t>
         </is>
       </c>
     </row>
     <row r="63">
       <c r="A63" t="inlineStr">
         <is>
-          <t>UltraLight</t>
+          <t>STR-Fusion</t>
         </is>
       </c>
       <c r="B63" t="inlineStr">
         <is>
-          <t>Run4</t>
+          <t>Run2_TASS</t>
         </is>
       </c>
       <c r="C63" t="inlineStr">
         <is>
-          <t>R4_0_A0_FULL12_FROZEN</t>
+          <t>C0_TOKEN</t>
         </is>
       </c>
       <c r="D63" t="inlineStr">
         <is>
-          <t>SYSU-CD-256</t>
+          <t>CDD-CD-256</t>
         </is>
       </c>
       <c r="E63" s="2" t="n">
-        <v>82.42</v>
+        <v>93.13</v>
       </c>
       <c r="F63" s="2" t="n">
-        <v>83.87</v>
+        <v>95.16</v>
       </c>
       <c r="G63" s="2" t="n">
-        <v>92.12</v>
+        <v>98.56999999999999</v>
       </c>
       <c r="H63" s="2" t="n">
-        <v>83.14</v>
+        <v>94.13</v>
       </c>
       <c r="I63" s="2" t="n">
-        <v>71.14</v>
+        <v>88.91</v>
       </c>
       <c r="J63" s="2" t="n">
-        <v>77.98999999999999</v>
+        <v>93.31999999999999</v>
       </c>
       <c r="K63" s="2" t="n">
-        <v>11.754</v>
+        <v>2.596</v>
       </c>
       <c r="L63" s="2" t="n">
-        <v>15.125</v>
+        <v>0.62</v>
       </c>
       <c r="M63" s="2" t="n">
-        <v>26.3246</v>
+        <v>2.2136</v>
       </c>
       <c r="N63" t="inlineStr">
         <is>
-          <t>baseline</t>
+          <t>str_tass</t>
         </is>
       </c>
     </row>
     <row r="64">
       <c r="A64" t="inlineStr">
         <is>
-          <t>UltraLight</t>
+          <t>STR-Fusion</t>
         </is>
       </c>
       <c r="B64" t="inlineStr">
         <is>
-          <t>Run4</t>
+          <t>Run2_TASS</t>
         </is>
       </c>
       <c r="C64" t="inlineStr">
         <is>
-          <t>R4_1_VIT4_OLDHEAD</t>
+          <t>C0_TOKEN</t>
         </is>
       </c>
       <c r="D64" t="inlineStr">
         <is>
-          <t>SYSU-CD-256</t>
+          <t>LEVIR-CD-256</t>
         </is>
       </c>
       <c r="E64" s="2" t="n">
-        <v>82.15000000000001</v>
+        <v>86.37</v>
       </c>
       <c r="F64" s="2" t="n">
-        <v>83.40000000000001</v>
+        <v>89.25</v>
       </c>
       <c r="G64" s="2" t="n">
-        <v>91.94</v>
+        <v>98.78</v>
       </c>
       <c r="H64" s="2" t="n">
-        <v>82.77</v>
+        <v>87.79000000000001</v>
       </c>
       <c r="I64" s="2" t="n">
-        <v>70.61</v>
+        <v>78.23999999999999</v>
       </c>
       <c r="J64" s="2" t="n">
-        <v>77.51000000000001</v>
+        <v>87.14</v>
       </c>
       <c r="K64" s="2" t="n">
-        <v>8.195</v>
+        <v>2.596</v>
       </c>
       <c r="L64" s="2" t="n">
-        <v>15.125</v>
+        <v>0.62</v>
       </c>
       <c r="M64" s="2" t="n">
-        <v>24.1021</v>
+        <v>2.2136</v>
       </c>
       <c r="N64" t="inlineStr">
         <is>
-          <t>baseline</t>
+          <t>str_tass</t>
         </is>
       </c>
     </row>
     <row r="65">
       <c r="A65" t="inlineStr">
         <is>
-          <t>UltraLight</t>
+          <t>STR-Fusion</t>
         </is>
       </c>
       <c r="B65" t="inlineStr">
         <is>
-          <t>Run4</t>
+          <t>Run2_TASS</t>
         </is>
       </c>
       <c r="C65" t="inlineStr">
         <is>
-          <t>R4_2_VIT4_LIGHTDETAIL</t>
+          <t>C0_TOKEN</t>
         </is>
       </c>
       <c r="D65" t="inlineStr">
@@ -3935,336 +3935,352 @@
         </is>
       </c>
       <c r="E65" s="2" t="n">
-        <v>79.94</v>
+        <v>79.93000000000001</v>
       </c>
       <c r="F65" s="2" t="n">
-        <v>84.79000000000001</v>
+        <v>84.5</v>
       </c>
       <c r="G65" s="2" t="n">
-        <v>91.89</v>
+        <v>91.81</v>
       </c>
       <c r="H65" s="2" t="n">
-        <v>82.3</v>
+        <v>82.15000000000001</v>
       </c>
       <c r="I65" s="2" t="n">
-        <v>69.92</v>
+        <v>69.70999999999999</v>
       </c>
       <c r="J65" s="2" t="n">
-        <v>77.04000000000001</v>
+        <v>76.84</v>
       </c>
       <c r="K65" s="2" t="n">
-        <v>5.492</v>
+        <v>2.596</v>
       </c>
       <c r="L65" s="2" t="n">
-        <v>3.515</v>
+        <v>0.62</v>
       </c>
       <c r="M65" s="2" t="n">
-        <v>10.7311</v>
+        <v>2.2136</v>
       </c>
       <c r="N65" t="inlineStr">
         <is>
-          <t>baseline</t>
+          <t>str_tass</t>
         </is>
       </c>
     </row>
     <row r="66">
       <c r="A66" t="inlineStr">
         <is>
-          <t>UltraLight</t>
+          <t>STR-Fusion</t>
         </is>
       </c>
       <c r="B66" t="inlineStr">
         <is>
-          <t>Run4</t>
+          <t>Run2_TASS</t>
         </is>
       </c>
       <c r="C66" t="inlineStr">
         <is>
-          <t>R4_2b_VIT4_LIGHTDETAIL48</t>
+          <t>C0_TOKEN</t>
         </is>
       </c>
       <c r="D66" t="inlineStr">
         <is>
-          <t>SYSU-CD-256</t>
+          <t>WHU-CD-256</t>
         </is>
       </c>
       <c r="E66" s="2" t="n">
-        <v>80.87</v>
+        <v>90.16</v>
       </c>
       <c r="F66" s="2" t="n">
-        <v>83.81</v>
+        <v>93.97</v>
       </c>
       <c r="G66" s="2" t="n">
-        <v>91.81</v>
+        <v>99.38</v>
       </c>
       <c r="H66" s="2" t="n">
-        <v>82.31999999999999</v>
+        <v>92.02</v>
       </c>
       <c r="I66" s="2" t="n">
-        <v>69.95</v>
+        <v>85.23</v>
       </c>
       <c r="J66" s="2" t="n">
-        <v>76.98999999999999</v>
+        <v>91.7</v>
       </c>
       <c r="K66" s="2" t="n">
-        <v>5.533</v>
+        <v>2.596</v>
       </c>
       <c r="L66" s="2" t="n">
-        <v>3.556</v>
+        <v>0.62</v>
       </c>
       <c r="M66" s="2" t="n">
-        <v>10.9824</v>
+        <v>2.2136</v>
       </c>
       <c r="N66" t="inlineStr">
         <is>
-          <t>baseline</t>
+          <t>str_tass</t>
         </is>
       </c>
     </row>
     <row r="67">
       <c r="A67" t="inlineStr">
         <is>
-          <t>UltraLight</t>
+          <t>STR-Fusion</t>
         </is>
       </c>
       <c r="B67" t="inlineStr">
         <is>
-          <t>Run4</t>
+          <t>Run2_TASS</t>
         </is>
       </c>
       <c r="C67" t="inlineStr">
         <is>
-          <t>R4_2d_PSD_DETAIL</t>
+          <t>M1_TASS</t>
         </is>
       </c>
       <c r="D67" t="inlineStr">
         <is>
-          <t>SYSU-CD-256</t>
+          <t>CDD-CD-256</t>
         </is>
       </c>
       <c r="E67" s="2" t="n">
-        <v>79.78</v>
+        <v>94.7</v>
       </c>
       <c r="F67" s="2" t="n">
-        <v>84.39</v>
+        <v>96.13</v>
       </c>
       <c r="G67" s="2" t="n">
-        <v>91.75</v>
+        <v>98.88</v>
       </c>
       <c r="H67" s="2" t="n">
-        <v>82.02</v>
+        <v>95.41</v>
       </c>
       <c r="I67" s="2" t="n">
-        <v>69.52</v>
+        <v>91.22</v>
       </c>
       <c r="J67" s="2" t="n">
-        <v>76.68000000000001</v>
+        <v>94.77</v>
       </c>
       <c r="K67" s="2" t="n">
-        <v>5.491</v>
+        <v>3.455</v>
       </c>
       <c r="L67" s="2" t="n">
-        <v>3.514</v>
+        <v>1.478</v>
       </c>
       <c r="M67" s="2" t="n">
-        <v>11.5239</v>
+        <v>3.5459</v>
       </c>
       <c r="N67" t="inlineStr">
         <is>
-          <t>baseline</t>
+          <t>str_tass</t>
         </is>
       </c>
     </row>
     <row r="68">
       <c r="A68" t="inlineStr">
         <is>
-          <t>baseline</t>
+          <t>STR-Fusion</t>
         </is>
       </c>
       <c r="B68" t="inlineStr">
         <is>
-          <t>Run1</t>
-        </is>
-      </c>
-      <c r="C68" t="inlineStr"/>
+          <t>Run2_TASS</t>
+        </is>
+      </c>
+      <c r="C68" t="inlineStr">
+        <is>
+          <t>M1_TASS</t>
+        </is>
+      </c>
       <c r="D68" t="inlineStr">
         <is>
-          <t>CDD-CD-256</t>
+          <t>LEVIR-CD-256</t>
         </is>
       </c>
       <c r="E68" s="2" t="n">
-        <v>97.72</v>
+        <v>88.42</v>
       </c>
       <c r="F68" s="2" t="n">
-        <v>97.78</v>
+        <v>91.97</v>
       </c>
       <c r="G68" s="2" t="n">
-        <v>99.44</v>
+        <v>99.02</v>
       </c>
       <c r="H68" s="2" t="n">
-        <v>97.75</v>
+        <v>90.16</v>
       </c>
       <c r="I68" s="2" t="n">
-        <v>95.59999999999999</v>
+        <v>82.08</v>
       </c>
       <c r="J68" s="2" t="n">
-        <v>97.43000000000001</v>
+        <v>89.64</v>
       </c>
       <c r="K68" s="2" t="n">
-        <v>11.754</v>
+        <v>3.455</v>
       </c>
       <c r="L68" s="2" t="n">
-        <v>20.661</v>
+        <v>1.478</v>
       </c>
       <c r="M68" s="2" t="n">
-        <v>26.3246</v>
+        <v>3.5459</v>
       </c>
       <c r="N68" t="inlineStr">
         <is>
-          <t>baseline</t>
+          <t>str_tass</t>
         </is>
       </c>
     </row>
     <row r="69">
       <c r="A69" t="inlineStr">
         <is>
-          <t>baseline</t>
+          <t>STR-Fusion</t>
         </is>
       </c>
       <c r="B69" t="inlineStr">
         <is>
-          <t>Run1</t>
-        </is>
-      </c>
-      <c r="C69" t="inlineStr"/>
+          <t>Run2_TASS</t>
+        </is>
+      </c>
+      <c r="C69" t="inlineStr">
+        <is>
+          <t>M1_TASS</t>
+        </is>
+      </c>
       <c r="D69" t="inlineStr">
         <is>
-          <t>LEVIR-CD-256</t>
+          <t>SYSU-CD-256</t>
         </is>
       </c>
       <c r="E69" s="2" t="n">
-        <v>91.56999999999999</v>
+        <v>78.73</v>
       </c>
       <c r="F69" s="2" t="n">
-        <v>92.33</v>
+        <v>84.98</v>
       </c>
       <c r="G69" s="2" t="n">
-        <v>99.18000000000001</v>
+        <v>91.7</v>
       </c>
       <c r="H69" s="2" t="n">
-        <v>91.95</v>
+        <v>81.73999999999999</v>
       </c>
       <c r="I69" s="2" t="n">
-        <v>85.09999999999999</v>
+        <v>69.11</v>
       </c>
       <c r="J69" s="2" t="n">
-        <v>91.52</v>
+        <v>76.38</v>
       </c>
       <c r="K69" s="2" t="n">
-        <v>11.754</v>
+        <v>3.455</v>
       </c>
       <c r="L69" s="2" t="n">
-        <v>20.661</v>
+        <v>1.478</v>
       </c>
       <c r="M69" s="2" t="n">
-        <v>26.3246</v>
+        <v>3.5459</v>
       </c>
       <c r="N69" t="inlineStr">
         <is>
-          <t>baseline</t>
+          <t>str_tass</t>
         </is>
       </c>
     </row>
     <row r="70">
       <c r="A70" t="inlineStr">
         <is>
-          <t>baseline</t>
+          <t>STR-Fusion</t>
         </is>
       </c>
       <c r="B70" t="inlineStr">
         <is>
-          <t>Run1</t>
-        </is>
-      </c>
-      <c r="C70" t="inlineStr"/>
+          <t>Run2_TASS</t>
+        </is>
+      </c>
+      <c r="C70" t="inlineStr">
+        <is>
+          <t>M1_TASS</t>
+        </is>
+      </c>
       <c r="D70" t="inlineStr">
         <is>
-          <t>SYSU-CD-256</t>
+          <t>WHU-CD-256</t>
         </is>
       </c>
       <c r="E70" s="2" t="n">
-        <v>80.77</v>
+        <v>91.64</v>
       </c>
       <c r="F70" s="2" t="n">
-        <v>84.27</v>
+        <v>94.81999999999999</v>
       </c>
       <c r="G70" s="2" t="n">
-        <v>91.91</v>
+        <v>99.47</v>
       </c>
       <c r="H70" s="2" t="n">
-        <v>82.48</v>
+        <v>93.2</v>
       </c>
       <c r="I70" s="2" t="n">
-        <v>70.19</v>
+        <v>87.27</v>
       </c>
       <c r="J70" s="2" t="n">
-        <v>77.23</v>
+        <v>92.93000000000001</v>
       </c>
       <c r="K70" s="2" t="n">
-        <v>11.754</v>
+        <v>3.455</v>
       </c>
       <c r="L70" s="2" t="n">
-        <v>20.661</v>
+        <v>1.478</v>
       </c>
       <c r="M70" s="2" t="n">
-        <v>26.3246</v>
+        <v>3.5459</v>
       </c>
       <c r="N70" t="inlineStr">
         <is>
-          <t>baseline</t>
+          <t>str_tass</t>
         </is>
       </c>
     </row>
     <row r="71">
       <c r="A71" t="inlineStr">
         <is>
-          <t>baseline</t>
+          <t>UltraLight</t>
         </is>
       </c>
       <c r="B71" t="inlineStr">
         <is>
-          <t>Run1</t>
-        </is>
-      </c>
-      <c r="C71" t="inlineStr"/>
+          <t>Run4</t>
+        </is>
+      </c>
+      <c r="C71" t="inlineStr">
+        <is>
+          <t>R4_0_A0_FULL12_FROZEN</t>
+        </is>
+      </c>
       <c r="D71" t="inlineStr">
         <is>
-          <t>WHU-CD-256</t>
+          <t>SYSU-CD-256</t>
         </is>
       </c>
       <c r="E71" s="2" t="n">
-        <v>93.62</v>
+        <v>82.42</v>
       </c>
       <c r="F71" s="2" t="n">
-        <v>96.09</v>
+        <v>83.87</v>
       </c>
       <c r="G71" s="2" t="n">
-        <v>99.59999999999999</v>
+        <v>92.12</v>
       </c>
       <c r="H71" s="2" t="n">
-        <v>94.84</v>
+        <v>83.14</v>
       </c>
       <c r="I71" s="2" t="n">
-        <v>90.18000000000001</v>
+        <v>71.14</v>
       </c>
       <c r="J71" s="2" t="n">
-        <v>94.63</v>
+        <v>77.98999999999999</v>
       </c>
       <c r="K71" s="2" t="n">
         <v>11.754</v>
       </c>
       <c r="L71" s="2" t="n">
-        <v>20.661</v>
+        <v>15.125</v>
       </c>
       <c r="M71" s="2" t="n">
         <v>26.3246</v>
@@ -4275,8 +4291,424 @@
         </is>
       </c>
     </row>
+    <row r="72">
+      <c r="A72" t="inlineStr">
+        <is>
+          <t>UltraLight</t>
+        </is>
+      </c>
+      <c r="B72" t="inlineStr">
+        <is>
+          <t>Run4</t>
+        </is>
+      </c>
+      <c r="C72" t="inlineStr">
+        <is>
+          <t>R4_1_VIT4_OLDHEAD</t>
+        </is>
+      </c>
+      <c r="D72" t="inlineStr">
+        <is>
+          <t>SYSU-CD-256</t>
+        </is>
+      </c>
+      <c r="E72" s="2" t="n">
+        <v>82.15000000000001</v>
+      </c>
+      <c r="F72" s="2" t="n">
+        <v>83.40000000000001</v>
+      </c>
+      <c r="G72" s="2" t="n">
+        <v>91.94</v>
+      </c>
+      <c r="H72" s="2" t="n">
+        <v>82.77</v>
+      </c>
+      <c r="I72" s="2" t="n">
+        <v>70.61</v>
+      </c>
+      <c r="J72" s="2" t="n">
+        <v>77.51000000000001</v>
+      </c>
+      <c r="K72" s="2" t="n">
+        <v>8.195</v>
+      </c>
+      <c r="L72" s="2" t="n">
+        <v>15.125</v>
+      </c>
+      <c r="M72" s="2" t="n">
+        <v>24.1021</v>
+      </c>
+      <c r="N72" t="inlineStr">
+        <is>
+          <t>baseline</t>
+        </is>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" t="inlineStr">
+        <is>
+          <t>UltraLight</t>
+        </is>
+      </c>
+      <c r="B73" t="inlineStr">
+        <is>
+          <t>Run4</t>
+        </is>
+      </c>
+      <c r="C73" t="inlineStr">
+        <is>
+          <t>R4_2_VIT4_LIGHTDETAIL</t>
+        </is>
+      </c>
+      <c r="D73" t="inlineStr">
+        <is>
+          <t>SYSU-CD-256</t>
+        </is>
+      </c>
+      <c r="E73" s="2" t="n">
+        <v>79.94</v>
+      </c>
+      <c r="F73" s="2" t="n">
+        <v>84.79000000000001</v>
+      </c>
+      <c r="G73" s="2" t="n">
+        <v>91.89</v>
+      </c>
+      <c r="H73" s="2" t="n">
+        <v>82.3</v>
+      </c>
+      <c r="I73" s="2" t="n">
+        <v>69.92</v>
+      </c>
+      <c r="J73" s="2" t="n">
+        <v>77.04000000000001</v>
+      </c>
+      <c r="K73" s="2" t="n">
+        <v>5.492</v>
+      </c>
+      <c r="L73" s="2" t="n">
+        <v>3.515</v>
+      </c>
+      <c r="M73" s="2" t="n">
+        <v>10.7311</v>
+      </c>
+      <c r="N73" t="inlineStr">
+        <is>
+          <t>baseline</t>
+        </is>
+      </c>
+    </row>
+    <row r="74">
+      <c r="A74" t="inlineStr">
+        <is>
+          <t>UltraLight</t>
+        </is>
+      </c>
+      <c r="B74" t="inlineStr">
+        <is>
+          <t>Run4</t>
+        </is>
+      </c>
+      <c r="C74" t="inlineStr">
+        <is>
+          <t>R4_2b_VIT4_LIGHTDETAIL48</t>
+        </is>
+      </c>
+      <c r="D74" t="inlineStr">
+        <is>
+          <t>SYSU-CD-256</t>
+        </is>
+      </c>
+      <c r="E74" s="2" t="n">
+        <v>80.87</v>
+      </c>
+      <c r="F74" s="2" t="n">
+        <v>83.81</v>
+      </c>
+      <c r="G74" s="2" t="n">
+        <v>91.81</v>
+      </c>
+      <c r="H74" s="2" t="n">
+        <v>82.31999999999999</v>
+      </c>
+      <c r="I74" s="2" t="n">
+        <v>69.95</v>
+      </c>
+      <c r="J74" s="2" t="n">
+        <v>76.98999999999999</v>
+      </c>
+      <c r="K74" s="2" t="n">
+        <v>5.533</v>
+      </c>
+      <c r="L74" s="2" t="n">
+        <v>3.556</v>
+      </c>
+      <c r="M74" s="2" t="n">
+        <v>10.9824</v>
+      </c>
+      <c r="N74" t="inlineStr">
+        <is>
+          <t>baseline</t>
+        </is>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75" t="inlineStr">
+        <is>
+          <t>UltraLight</t>
+        </is>
+      </c>
+      <c r="B75" t="inlineStr">
+        <is>
+          <t>Run4</t>
+        </is>
+      </c>
+      <c r="C75" t="inlineStr">
+        <is>
+          <t>R4_2d_PSD_DETAIL</t>
+        </is>
+      </c>
+      <c r="D75" t="inlineStr">
+        <is>
+          <t>SYSU-CD-256</t>
+        </is>
+      </c>
+      <c r="E75" s="2" t="n">
+        <v>79.78</v>
+      </c>
+      <c r="F75" s="2" t="n">
+        <v>84.39</v>
+      </c>
+      <c r="G75" s="2" t="n">
+        <v>91.75</v>
+      </c>
+      <c r="H75" s="2" t="n">
+        <v>82.02</v>
+      </c>
+      <c r="I75" s="2" t="n">
+        <v>69.52</v>
+      </c>
+      <c r="J75" s="2" t="n">
+        <v>76.68000000000001</v>
+      </c>
+      <c r="K75" s="2" t="n">
+        <v>5.491</v>
+      </c>
+      <c r="L75" s="2" t="n">
+        <v>3.514</v>
+      </c>
+      <c r="M75" s="2" t="n">
+        <v>11.5239</v>
+      </c>
+      <c r="N75" t="inlineStr">
+        <is>
+          <t>baseline</t>
+        </is>
+      </c>
+    </row>
+    <row r="76">
+      <c r="A76" t="inlineStr">
+        <is>
+          <t>baseline</t>
+        </is>
+      </c>
+      <c r="B76" t="inlineStr">
+        <is>
+          <t>Run1</t>
+        </is>
+      </c>
+      <c r="C76" t="inlineStr"/>
+      <c r="D76" t="inlineStr">
+        <is>
+          <t>CDD-CD-256</t>
+        </is>
+      </c>
+      <c r="E76" s="2" t="n">
+        <v>97.72</v>
+      </c>
+      <c r="F76" s="2" t="n">
+        <v>97.78</v>
+      </c>
+      <c r="G76" s="2" t="n">
+        <v>99.44</v>
+      </c>
+      <c r="H76" s="2" t="n">
+        <v>97.75</v>
+      </c>
+      <c r="I76" s="2" t="n">
+        <v>95.59999999999999</v>
+      </c>
+      <c r="J76" s="2" t="n">
+        <v>97.43000000000001</v>
+      </c>
+      <c r="K76" s="2" t="n">
+        <v>11.754</v>
+      </c>
+      <c r="L76" s="2" t="n">
+        <v>20.661</v>
+      </c>
+      <c r="M76" s="2" t="n">
+        <v>26.3246</v>
+      </c>
+      <c r="N76" t="inlineStr">
+        <is>
+          <t>baseline</t>
+        </is>
+      </c>
+    </row>
+    <row r="77">
+      <c r="A77" t="inlineStr">
+        <is>
+          <t>baseline</t>
+        </is>
+      </c>
+      <c r="B77" t="inlineStr">
+        <is>
+          <t>Run1</t>
+        </is>
+      </c>
+      <c r="C77" t="inlineStr"/>
+      <c r="D77" t="inlineStr">
+        <is>
+          <t>LEVIR-CD-256</t>
+        </is>
+      </c>
+      <c r="E77" s="2" t="n">
+        <v>91.56999999999999</v>
+      </c>
+      <c r="F77" s="2" t="n">
+        <v>92.33</v>
+      </c>
+      <c r="G77" s="2" t="n">
+        <v>99.18000000000001</v>
+      </c>
+      <c r="H77" s="2" t="n">
+        <v>91.95</v>
+      </c>
+      <c r="I77" s="2" t="n">
+        <v>85.09999999999999</v>
+      </c>
+      <c r="J77" s="2" t="n">
+        <v>91.52</v>
+      </c>
+      <c r="K77" s="2" t="n">
+        <v>11.754</v>
+      </c>
+      <c r="L77" s="2" t="n">
+        <v>20.661</v>
+      </c>
+      <c r="M77" s="2" t="n">
+        <v>26.3246</v>
+      </c>
+      <c r="N77" t="inlineStr">
+        <is>
+          <t>baseline</t>
+        </is>
+      </c>
+    </row>
+    <row r="78">
+      <c r="A78" t="inlineStr">
+        <is>
+          <t>baseline</t>
+        </is>
+      </c>
+      <c r="B78" t="inlineStr">
+        <is>
+          <t>Run1</t>
+        </is>
+      </c>
+      <c r="C78" t="inlineStr"/>
+      <c r="D78" t="inlineStr">
+        <is>
+          <t>SYSU-CD-256</t>
+        </is>
+      </c>
+      <c r="E78" s="2" t="n">
+        <v>80.77</v>
+      </c>
+      <c r="F78" s="2" t="n">
+        <v>84.27</v>
+      </c>
+      <c r="G78" s="2" t="n">
+        <v>91.91</v>
+      </c>
+      <c r="H78" s="2" t="n">
+        <v>82.48</v>
+      </c>
+      <c r="I78" s="2" t="n">
+        <v>70.19</v>
+      </c>
+      <c r="J78" s="2" t="n">
+        <v>77.23</v>
+      </c>
+      <c r="K78" s="2" t="n">
+        <v>11.754</v>
+      </c>
+      <c r="L78" s="2" t="n">
+        <v>20.661</v>
+      </c>
+      <c r="M78" s="2" t="n">
+        <v>26.3246</v>
+      </c>
+      <c r="N78" t="inlineStr">
+        <is>
+          <t>baseline</t>
+        </is>
+      </c>
+    </row>
+    <row r="79">
+      <c r="A79" t="inlineStr">
+        <is>
+          <t>baseline</t>
+        </is>
+      </c>
+      <c r="B79" t="inlineStr">
+        <is>
+          <t>Run1</t>
+        </is>
+      </c>
+      <c r="C79" t="inlineStr"/>
+      <c r="D79" t="inlineStr">
+        <is>
+          <t>WHU-CD-256</t>
+        </is>
+      </c>
+      <c r="E79" s="2" t="n">
+        <v>93.62</v>
+      </c>
+      <c r="F79" s="2" t="n">
+        <v>96.09</v>
+      </c>
+      <c r="G79" s="2" t="n">
+        <v>99.59999999999999</v>
+      </c>
+      <c r="H79" s="2" t="n">
+        <v>94.84</v>
+      </c>
+      <c r="I79" s="2" t="n">
+        <v>90.18000000000001</v>
+      </c>
+      <c r="J79" s="2" t="n">
+        <v>94.63</v>
+      </c>
+      <c r="K79" s="2" t="n">
+        <v>11.754</v>
+      </c>
+      <c r="L79" s="2" t="n">
+        <v>20.661</v>
+      </c>
+      <c r="M79" s="2" t="n">
+        <v>26.3246</v>
+      </c>
+      <c r="N79" t="inlineStr">
+        <is>
+          <t>baseline</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:N71"/>
+  <autoFilter ref="A1:N79"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Run9: record 3 valid results after stop
CDD CTRL F1=0.9777, HSAM F1=0.9765 (delta=-0.0012).
LEVIR CTRL F1=0.9114; HSAM failed without a final TEST block.
Preserve 98 historical workbook rows, add Run9 snapshot, and guard tools against lost history.
</commit_message>
<xml_diff>
--- a/docs/experiment_metrics.xlsx
+++ b/docs/experiment_metrics.xlsx
@@ -10,7 +10,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="metrics" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'metrics'!$A$1:$N$99</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'metrics'!$A$1:$N$102</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -420,7 +420,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N99"/>
+  <dimension ref="A1:N102"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -1381,6 +1381,7 @@
           <t>CASA-TViM</t>
         </is>
       </c>
+      <c r="B18" t="inlineStr"/>
       <c r="C18" t="inlineStr">
         <is>
           <t>Exploration/Exp1/STG_INJ</t>
@@ -1424,6 +1425,7 @@
           <t>CASA-TViM</t>
         </is>
       </c>
+      <c r="B19" t="inlineStr"/>
       <c r="C19" t="inlineStr">
         <is>
           <t>Exploration/Exp1/STG_INJ</t>
@@ -1467,6 +1469,7 @@
           <t>CASA-TViM</t>
         </is>
       </c>
+      <c r="B20" t="inlineStr"/>
       <c r="C20" t="inlineStr">
         <is>
           <t>Exploration/Exp1/STG_SUP</t>
@@ -1512,6 +1515,7 @@
           <t>CASA-TViM</t>
         </is>
       </c>
+      <c r="B21" t="inlineStr"/>
       <c r="C21" t="inlineStr">
         <is>
           <t>Exploration/Exp1/STG_SUP</t>
@@ -1557,6 +1561,7 @@
           <t>CASA-TViM</t>
         </is>
       </c>
+      <c r="B22" t="inlineStr"/>
       <c r="C22" t="inlineStr">
         <is>
           <t>Exploration/Exp1/STG_V2</t>
@@ -1600,6 +1605,7 @@
           <t>CASA-TViM</t>
         </is>
       </c>
+      <c r="B23" t="inlineStr"/>
       <c r="C23" t="inlineStr">
         <is>
           <t>Exploration/Exp1/STG_V2</t>
@@ -4340,162 +4346,162 @@
     <row r="74">
       <c r="A74" t="inlineStr">
         <is>
-          <t>CASAA</t>
+          <t>CASA-TViM</t>
         </is>
       </c>
       <c r="B74" t="inlineStr">
         <is>
-          <t>Run1</t>
+          <t>Run9</t>
         </is>
       </c>
       <c r="C74" t="inlineStr">
         <is>
-          <t>A1_SAA</t>
+          <t>S0_CTRL</t>
         </is>
       </c>
       <c r="D74" t="inlineStr">
         <is>
-          <t>LEVIR-CD-256</t>
+          <t>CDD-CD-256</t>
         </is>
       </c>
       <c r="E74" s="2" t="n">
-        <v>91.09</v>
+        <v>97.77</v>
       </c>
       <c r="F74" s="2" t="n">
-        <v>92.8</v>
+        <v>97.77</v>
       </c>
       <c r="G74" s="2" t="n">
-        <v>99.19</v>
+        <v>99.45</v>
       </c>
       <c r="H74" s="2" t="n">
-        <v>91.94</v>
+        <v>97.77</v>
       </c>
       <c r="I74" s="2" t="n">
-        <v>85.08</v>
+        <v>95.65000000000001</v>
       </c>
       <c r="J74" s="2" t="n">
-        <v>91.51000000000001</v>
+        <v>97.45999999999999</v>
       </c>
       <c r="K74" s="2" t="n">
-        <v>11.754</v>
+        <v>31.977</v>
       </c>
       <c r="L74" s="2" t="n">
-        <v>20.661</v>
+        <v>31.977</v>
       </c>
       <c r="M74" s="2" t="n">
-        <v>26.3183</v>
+        <v>14.6841</v>
       </c>
       <c r="N74" t="inlineStr">
         <is>
-          <t>saa</t>
+          <t>baseline</t>
         </is>
       </c>
     </row>
     <row r="75">
       <c r="A75" t="inlineStr">
         <is>
-          <t>CASAA</t>
+          <t>CASA-TViM</t>
         </is>
       </c>
       <c r="B75" t="inlineStr">
         <is>
-          <t>Run1</t>
+          <t>Run9</t>
         </is>
       </c>
       <c r="C75" t="inlineStr">
         <is>
-          <t>A1_SAA</t>
+          <t>S0_CTRL</t>
         </is>
       </c>
       <c r="D75" t="inlineStr">
         <is>
-          <t>SYSU-CD-256</t>
+          <t>LEVIR-CD-256</t>
         </is>
       </c>
       <c r="E75" s="2" t="n">
-        <v>80.3</v>
+        <v>89.79000000000001</v>
       </c>
       <c r="F75" s="2" t="n">
-        <v>84.81</v>
+        <v>92.53</v>
       </c>
       <c r="G75" s="2" t="n">
-        <v>91.95999999999999</v>
+        <v>99.11</v>
       </c>
       <c r="H75" s="2" t="n">
-        <v>82.5</v>
+        <v>91.14</v>
       </c>
       <c r="I75" s="2" t="n">
-        <v>70.20999999999999</v>
+        <v>83.72</v>
       </c>
       <c r="J75" s="2" t="n">
-        <v>77.29000000000001</v>
+        <v>90.67</v>
       </c>
       <c r="K75" s="2" t="n">
-        <v>11.754</v>
+        <v>31.977</v>
       </c>
       <c r="L75" s="2" t="n">
-        <v>20.661</v>
+        <v>31.977</v>
       </c>
       <c r="M75" s="2" t="n">
-        <v>26.3183</v>
+        <v>14.6841</v>
       </c>
       <c r="N75" t="inlineStr">
         <is>
-          <t>saa</t>
+          <t>baseline</t>
         </is>
       </c>
     </row>
     <row r="76">
       <c r="A76" t="inlineStr">
         <is>
-          <t>CASAA</t>
+          <t>CASA-TViM</t>
         </is>
       </c>
       <c r="B76" t="inlineStr">
         <is>
-          <t>Run1</t>
+          <t>Run9</t>
         </is>
       </c>
       <c r="C76" t="inlineStr">
         <is>
-          <t>A2_CASAA</t>
+          <t>S1_HSAM</t>
         </is>
       </c>
       <c r="D76" t="inlineStr">
         <is>
-          <t>LEVIR-CD-256</t>
+          <t>CDD-CD-256</t>
         </is>
       </c>
       <c r="E76" s="2" t="n">
-        <v>90.98999999999999</v>
+        <v>97.66</v>
       </c>
       <c r="F76" s="2" t="n">
-        <v>92.75</v>
+        <v>97.65000000000001</v>
       </c>
       <c r="G76" s="2" t="n">
-        <v>99.18000000000001</v>
+        <v>99.42</v>
       </c>
       <c r="H76" s="2" t="n">
-        <v>91.86</v>
+        <v>97.65000000000001</v>
       </c>
       <c r="I76" s="2" t="n">
-        <v>84.94</v>
+        <v>95.42</v>
       </c>
       <c r="J76" s="2" t="n">
-        <v>91.43000000000001</v>
+        <v>97.31999999999999</v>
       </c>
       <c r="K76" s="2" t="n">
-        <v>11.754</v>
+        <v>31.977</v>
       </c>
       <c r="L76" s="2" t="n">
-        <v>20.661</v>
+        <v>31.977</v>
       </c>
       <c r="M76" s="2" t="n">
-        <v>26.2593</v>
+        <v>14.769</v>
       </c>
       <c r="N76" t="inlineStr">
         <is>
-          <t>casaa</t>
+          <t>baseline</t>
         </is>
       </c>
     </row>
@@ -4512,31 +4518,31 @@
       </c>
       <c r="C77" t="inlineStr">
         <is>
-          <t>A2_CASAA</t>
+          <t>A1_SAA</t>
         </is>
       </c>
       <c r="D77" t="inlineStr">
         <is>
-          <t>SYSU-CD-256</t>
+          <t>LEVIR-CD-256</t>
         </is>
       </c>
       <c r="E77" s="2" t="n">
-        <v>80.55</v>
+        <v>91.09</v>
       </c>
       <c r="F77" s="2" t="n">
-        <v>84.23</v>
+        <v>92.8</v>
       </c>
       <c r="G77" s="2" t="n">
-        <v>91.86</v>
+        <v>99.19</v>
       </c>
       <c r="H77" s="2" t="n">
-        <v>82.34999999999999</v>
+        <v>91.94</v>
       </c>
       <c r="I77" s="2" t="n">
-        <v>70</v>
+        <v>85.08</v>
       </c>
       <c r="J77" s="2" t="n">
-        <v>77.06</v>
+        <v>91.51000000000001</v>
       </c>
       <c r="K77" s="2" t="n">
         <v>11.754</v>
@@ -4545,11 +4551,11 @@
         <v>20.661</v>
       </c>
       <c r="M77" s="2" t="n">
-        <v>26.2593</v>
+        <v>26.3183</v>
       </c>
       <c r="N77" t="inlineStr">
         <is>
-          <t>casaa</t>
+          <t>saa</t>
         </is>
       </c>
     </row>
@@ -4561,45 +4567,45 @@
       </c>
       <c r="B78" t="inlineStr">
         <is>
-          <t>Run2</t>
+          <t>Run1</t>
         </is>
       </c>
       <c r="C78" t="inlineStr">
         <is>
-          <t>A1_SAA_FROZEN</t>
+          <t>A1_SAA</t>
         </is>
       </c>
       <c r="D78" t="inlineStr">
         <is>
-          <t>LEVIR-CD-256</t>
+          <t>SYSU-CD-256</t>
         </is>
       </c>
       <c r="E78" s="2" t="n">
-        <v>91.38</v>
+        <v>80.3</v>
       </c>
       <c r="F78" s="2" t="n">
-        <v>92.3</v>
+        <v>84.81</v>
       </c>
       <c r="G78" s="2" t="n">
-        <v>99.17</v>
+        <v>91.95999999999999</v>
       </c>
       <c r="H78" s="2" t="n">
-        <v>91.84</v>
+        <v>82.5</v>
       </c>
       <c r="I78" s="2" t="n">
-        <v>84.91</v>
+        <v>70.20999999999999</v>
       </c>
       <c r="J78" s="2" t="n">
-        <v>91.40000000000001</v>
+        <v>77.29000000000001</v>
       </c>
       <c r="K78" s="2" t="n">
         <v>11.754</v>
       </c>
       <c r="L78" s="2" t="n">
-        <v>15.125</v>
+        <v>20.661</v>
       </c>
       <c r="M78" s="2" t="n">
-        <v>26.1484</v>
+        <v>26.3183</v>
       </c>
       <c r="N78" t="inlineStr">
         <is>
@@ -4615,49 +4621,49 @@
       </c>
       <c r="B79" t="inlineStr">
         <is>
-          <t>Run2</t>
+          <t>Run1</t>
         </is>
       </c>
       <c r="C79" t="inlineStr">
         <is>
-          <t>A1_SAA_FROZEN</t>
+          <t>A2_CASAA</t>
         </is>
       </c>
       <c r="D79" t="inlineStr">
         <is>
-          <t>SYSU-CD-256</t>
+          <t>LEVIR-CD-256</t>
         </is>
       </c>
       <c r="E79" s="2" t="n">
-        <v>78.40000000000001</v>
+        <v>90.98999999999999</v>
       </c>
       <c r="F79" s="2" t="n">
-        <v>86.03</v>
+        <v>92.75</v>
       </c>
       <c r="G79" s="2" t="n">
-        <v>91.90000000000001</v>
+        <v>99.18000000000001</v>
       </c>
       <c r="H79" s="2" t="n">
-        <v>82.04000000000001</v>
+        <v>91.86</v>
       </c>
       <c r="I79" s="2" t="n">
-        <v>69.55</v>
+        <v>84.94</v>
       </c>
       <c r="J79" s="2" t="n">
-        <v>76.83</v>
+        <v>91.43000000000001</v>
       </c>
       <c r="K79" s="2" t="n">
         <v>11.754</v>
       </c>
       <c r="L79" s="2" t="n">
-        <v>15.125</v>
+        <v>20.661</v>
       </c>
       <c r="M79" s="2" t="n">
-        <v>26.1484</v>
+        <v>26.2593</v>
       </c>
       <c r="N79" t="inlineStr">
         <is>
-          <t>saa</t>
+          <t>casaa</t>
         </is>
       </c>
     </row>
@@ -4669,45 +4675,45 @@
       </c>
       <c r="B80" t="inlineStr">
         <is>
-          <t>Run2</t>
+          <t>Run1</t>
         </is>
       </c>
       <c r="C80" t="inlineStr">
         <is>
-          <t>A3_ORACLE_FROZEN</t>
+          <t>A2_CASAA</t>
         </is>
       </c>
       <c r="D80" t="inlineStr">
         <is>
-          <t>LEVIR-CD-256</t>
+          <t>SYSU-CD-256</t>
         </is>
       </c>
       <c r="E80" s="2" t="n">
-        <v>91.13</v>
+        <v>80.55</v>
       </c>
       <c r="F80" s="2" t="n">
-        <v>92.65000000000001</v>
+        <v>84.23</v>
       </c>
       <c r="G80" s="2" t="n">
-        <v>99.18000000000001</v>
+        <v>91.86</v>
       </c>
       <c r="H80" s="2" t="n">
-        <v>91.88</v>
+        <v>82.34999999999999</v>
       </c>
       <c r="I80" s="2" t="n">
-        <v>84.98</v>
+        <v>70</v>
       </c>
       <c r="J80" s="2" t="n">
-        <v>91.45</v>
+        <v>77.06</v>
       </c>
       <c r="K80" s="2" t="n">
         <v>11.754</v>
       </c>
       <c r="L80" s="2" t="n">
-        <v>15.125</v>
+        <v>20.661</v>
       </c>
       <c r="M80" s="2" t="n">
-        <v>26.0894</v>
+        <v>26.2593</v>
       </c>
       <c r="N80" t="inlineStr">
         <is>
@@ -4728,31 +4734,31 @@
       </c>
       <c r="C81" t="inlineStr">
         <is>
-          <t>A3_ORACLE_FROZEN</t>
+          <t>A1_SAA_FROZEN</t>
         </is>
       </c>
       <c r="D81" t="inlineStr">
         <is>
-          <t>SYSU-CD-256</t>
+          <t>LEVIR-CD-256</t>
         </is>
       </c>
       <c r="E81" s="2" t="n">
-        <v>82.04000000000001</v>
+        <v>91.38</v>
       </c>
       <c r="F81" s="2" t="n">
-        <v>85.05</v>
+        <v>92.3</v>
       </c>
       <c r="G81" s="2" t="n">
-        <v>92.36</v>
+        <v>99.17</v>
       </c>
       <c r="H81" s="2" t="n">
-        <v>83.52</v>
+        <v>91.84</v>
       </c>
       <c r="I81" s="2" t="n">
-        <v>71.7</v>
+        <v>84.91</v>
       </c>
       <c r="J81" s="2" t="n">
-        <v>78.55</v>
+        <v>91.40000000000001</v>
       </c>
       <c r="K81" s="2" t="n">
         <v>11.754</v>
@@ -4761,11 +4767,11 @@
         <v>15.125</v>
       </c>
       <c r="M81" s="2" t="n">
-        <v>26.0894</v>
+        <v>26.1484</v>
       </c>
       <c r="N81" t="inlineStr">
         <is>
-          <t>casaa</t>
+          <t>saa</t>
         </is>
       </c>
     </row>
@@ -4777,12 +4783,12 @@
       </c>
       <c r="B82" t="inlineStr">
         <is>
-          <t>Run3</t>
+          <t>Run2</t>
         </is>
       </c>
       <c r="C82" t="inlineStr">
         <is>
-          <t>A4_DETAIL_FROZEN</t>
+          <t>A1_SAA_FROZEN</t>
         </is>
       </c>
       <c r="D82" t="inlineStr">
@@ -4791,22 +4797,22 @@
         </is>
       </c>
       <c r="E82" s="2" t="n">
-        <v>79.68000000000001</v>
+        <v>78.40000000000001</v>
       </c>
       <c r="F82" s="2" t="n">
-        <v>84.28</v>
+        <v>86.03</v>
       </c>
       <c r="G82" s="2" t="n">
-        <v>91.7</v>
+        <v>91.90000000000001</v>
       </c>
       <c r="H82" s="2" t="n">
-        <v>81.92</v>
+        <v>82.04000000000001</v>
       </c>
       <c r="I82" s="2" t="n">
-        <v>69.37</v>
+        <v>69.55</v>
       </c>
       <c r="J82" s="2" t="n">
-        <v>76.54000000000001</v>
+        <v>76.83</v>
       </c>
       <c r="K82" s="2" t="n">
         <v>11.754</v>
@@ -4815,136 +4821,136 @@
         <v>15.125</v>
       </c>
       <c r="M82" s="2" t="n">
-        <v>26.0894</v>
+        <v>26.1484</v>
       </c>
       <c r="N82" t="inlineStr">
         <is>
-          <t>casaa</t>
+          <t>saa</t>
         </is>
       </c>
     </row>
     <row r="83">
       <c r="A83" t="inlineStr">
         <is>
-          <t>STR-Fusion</t>
+          <t>CASAA</t>
         </is>
       </c>
       <c r="B83" t="inlineStr">
         <is>
-          <t>Run2_TASS</t>
+          <t>Run2</t>
         </is>
       </c>
       <c r="C83" t="inlineStr">
         <is>
-          <t>C0_TOKEN</t>
+          <t>A3_ORACLE_FROZEN</t>
         </is>
       </c>
       <c r="D83" t="inlineStr">
         <is>
-          <t>CDD-CD-256</t>
+          <t>LEVIR-CD-256</t>
         </is>
       </c>
       <c r="E83" s="2" t="n">
-        <v>93.13</v>
+        <v>91.13</v>
       </c>
       <c r="F83" s="2" t="n">
-        <v>95.16</v>
+        <v>92.65000000000001</v>
       </c>
       <c r="G83" s="2" t="n">
-        <v>98.56999999999999</v>
+        <v>99.18000000000001</v>
       </c>
       <c r="H83" s="2" t="n">
-        <v>94.13</v>
+        <v>91.88</v>
       </c>
       <c r="I83" s="2" t="n">
-        <v>88.91</v>
+        <v>84.98</v>
       </c>
       <c r="J83" s="2" t="n">
-        <v>93.31999999999999</v>
+        <v>91.45</v>
       </c>
       <c r="K83" s="2" t="n">
-        <v>2.596</v>
+        <v>11.754</v>
       </c>
       <c r="L83" s="2" t="n">
-        <v>0.62</v>
+        <v>15.125</v>
       </c>
       <c r="M83" s="2" t="n">
-        <v>2.2136</v>
+        <v>26.0894</v>
       </c>
       <c r="N83" t="inlineStr">
         <is>
-          <t>str_tass</t>
+          <t>casaa</t>
         </is>
       </c>
     </row>
     <row r="84">
       <c r="A84" t="inlineStr">
         <is>
-          <t>STR-Fusion</t>
+          <t>CASAA</t>
         </is>
       </c>
       <c r="B84" t="inlineStr">
         <is>
-          <t>Run2_TASS</t>
+          <t>Run2</t>
         </is>
       </c>
       <c r="C84" t="inlineStr">
         <is>
-          <t>C0_TOKEN</t>
+          <t>A3_ORACLE_FROZEN</t>
         </is>
       </c>
       <c r="D84" t="inlineStr">
         <is>
-          <t>LEVIR-CD-256</t>
+          <t>SYSU-CD-256</t>
         </is>
       </c>
       <c r="E84" s="2" t="n">
-        <v>86.37</v>
+        <v>82.04000000000001</v>
       </c>
       <c r="F84" s="2" t="n">
-        <v>89.25</v>
+        <v>85.05</v>
       </c>
       <c r="G84" s="2" t="n">
-        <v>98.78</v>
+        <v>92.36</v>
       </c>
       <c r="H84" s="2" t="n">
-        <v>87.79000000000001</v>
+        <v>83.52</v>
       </c>
       <c r="I84" s="2" t="n">
-        <v>78.23999999999999</v>
+        <v>71.7</v>
       </c>
       <c r="J84" s="2" t="n">
-        <v>87.14</v>
+        <v>78.55</v>
       </c>
       <c r="K84" s="2" t="n">
-        <v>2.596</v>
+        <v>11.754</v>
       </c>
       <c r="L84" s="2" t="n">
-        <v>0.62</v>
+        <v>15.125</v>
       </c>
       <c r="M84" s="2" t="n">
-        <v>2.2136</v>
+        <v>26.0894</v>
       </c>
       <c r="N84" t="inlineStr">
         <is>
-          <t>str_tass</t>
+          <t>casaa</t>
         </is>
       </c>
     </row>
     <row r="85">
       <c r="A85" t="inlineStr">
         <is>
-          <t>STR-Fusion</t>
+          <t>CASAA</t>
         </is>
       </c>
       <c r="B85" t="inlineStr">
         <is>
-          <t>Run2_TASS</t>
+          <t>Run3</t>
         </is>
       </c>
       <c r="C85" t="inlineStr">
         <is>
-          <t>C0_TOKEN</t>
+          <t>A4_DETAIL_FROZEN</t>
         </is>
       </c>
       <c r="D85" t="inlineStr">
@@ -4953,35 +4959,35 @@
         </is>
       </c>
       <c r="E85" s="2" t="n">
-        <v>79.93000000000001</v>
+        <v>79.68000000000001</v>
       </c>
       <c r="F85" s="2" t="n">
-        <v>84.5</v>
+        <v>84.28</v>
       </c>
       <c r="G85" s="2" t="n">
-        <v>91.81</v>
+        <v>91.7</v>
       </c>
       <c r="H85" s="2" t="n">
-        <v>82.15000000000001</v>
+        <v>81.92</v>
       </c>
       <c r="I85" s="2" t="n">
-        <v>69.70999999999999</v>
+        <v>69.37</v>
       </c>
       <c r="J85" s="2" t="n">
-        <v>76.84</v>
+        <v>76.54000000000001</v>
       </c>
       <c r="K85" s="2" t="n">
-        <v>2.596</v>
+        <v>11.754</v>
       </c>
       <c r="L85" s="2" t="n">
-        <v>0.62</v>
+        <v>15.125</v>
       </c>
       <c r="M85" s="2" t="n">
-        <v>2.2136</v>
+        <v>26.0894</v>
       </c>
       <c r="N85" t="inlineStr">
         <is>
-          <t>str_tass</t>
+          <t>casaa</t>
         </is>
       </c>
     </row>
@@ -5003,26 +5009,26 @@
       </c>
       <c r="D86" t="inlineStr">
         <is>
-          <t>WHU-CD-256</t>
+          <t>CDD-CD-256</t>
         </is>
       </c>
       <c r="E86" s="2" t="n">
-        <v>90.16</v>
+        <v>93.13</v>
       </c>
       <c r="F86" s="2" t="n">
-        <v>93.97</v>
+        <v>95.16</v>
       </c>
       <c r="G86" s="2" t="n">
-        <v>99.38</v>
+        <v>98.56999999999999</v>
       </c>
       <c r="H86" s="2" t="n">
-        <v>92.02</v>
+        <v>94.13</v>
       </c>
       <c r="I86" s="2" t="n">
-        <v>85.23</v>
+        <v>88.91</v>
       </c>
       <c r="J86" s="2" t="n">
-        <v>91.7</v>
+        <v>93.31999999999999</v>
       </c>
       <c r="K86" s="2" t="n">
         <v>2.596</v>
@@ -5052,40 +5058,40 @@
       </c>
       <c r="C87" t="inlineStr">
         <is>
-          <t>M1_TASS</t>
+          <t>C0_TOKEN</t>
         </is>
       </c>
       <c r="D87" t="inlineStr">
         <is>
-          <t>CDD-CD-256</t>
+          <t>LEVIR-CD-256</t>
         </is>
       </c>
       <c r="E87" s="2" t="n">
-        <v>94.7</v>
+        <v>86.37</v>
       </c>
       <c r="F87" s="2" t="n">
-        <v>96.13</v>
+        <v>89.25</v>
       </c>
       <c r="G87" s="2" t="n">
-        <v>98.88</v>
+        <v>98.78</v>
       </c>
       <c r="H87" s="2" t="n">
-        <v>95.41</v>
+        <v>87.79000000000001</v>
       </c>
       <c r="I87" s="2" t="n">
-        <v>91.22</v>
+        <v>78.23999999999999</v>
       </c>
       <c r="J87" s="2" t="n">
-        <v>94.77</v>
+        <v>87.14</v>
       </c>
       <c r="K87" s="2" t="n">
-        <v>3.455</v>
+        <v>2.596</v>
       </c>
       <c r="L87" s="2" t="n">
-        <v>1.478</v>
+        <v>0.62</v>
       </c>
       <c r="M87" s="2" t="n">
-        <v>3.5459</v>
+        <v>2.2136</v>
       </c>
       <c r="N87" t="inlineStr">
         <is>
@@ -5106,40 +5112,40 @@
       </c>
       <c r="C88" t="inlineStr">
         <is>
-          <t>M1_TASS</t>
+          <t>C0_TOKEN</t>
         </is>
       </c>
       <c r="D88" t="inlineStr">
         <is>
-          <t>LEVIR-CD-256</t>
+          <t>SYSU-CD-256</t>
         </is>
       </c>
       <c r="E88" s="2" t="n">
-        <v>88.42</v>
+        <v>79.93000000000001</v>
       </c>
       <c r="F88" s="2" t="n">
-        <v>91.97</v>
+        <v>84.5</v>
       </c>
       <c r="G88" s="2" t="n">
-        <v>99.02</v>
+        <v>91.81</v>
       </c>
       <c r="H88" s="2" t="n">
-        <v>90.16</v>
+        <v>82.15000000000001</v>
       </c>
       <c r="I88" s="2" t="n">
-        <v>82.08</v>
+        <v>69.70999999999999</v>
       </c>
       <c r="J88" s="2" t="n">
-        <v>89.64</v>
+        <v>76.84</v>
       </c>
       <c r="K88" s="2" t="n">
-        <v>3.455</v>
+        <v>2.596</v>
       </c>
       <c r="L88" s="2" t="n">
-        <v>1.478</v>
+        <v>0.62</v>
       </c>
       <c r="M88" s="2" t="n">
-        <v>3.5459</v>
+        <v>2.2136</v>
       </c>
       <c r="N88" t="inlineStr">
         <is>
@@ -5160,40 +5166,40 @@
       </c>
       <c r="C89" t="inlineStr">
         <is>
-          <t>M1_TASS</t>
+          <t>C0_TOKEN</t>
         </is>
       </c>
       <c r="D89" t="inlineStr">
         <is>
-          <t>SYSU-CD-256</t>
+          <t>WHU-CD-256</t>
         </is>
       </c>
       <c r="E89" s="2" t="n">
-        <v>78.73</v>
+        <v>90.16</v>
       </c>
       <c r="F89" s="2" t="n">
-        <v>84.98</v>
+        <v>93.97</v>
       </c>
       <c r="G89" s="2" t="n">
+        <v>99.38</v>
+      </c>
+      <c r="H89" s="2" t="n">
+        <v>92.02</v>
+      </c>
+      <c r="I89" s="2" t="n">
+        <v>85.23</v>
+      </c>
+      <c r="J89" s="2" t="n">
         <v>91.7</v>
       </c>
-      <c r="H89" s="2" t="n">
-        <v>81.73999999999999</v>
-      </c>
-      <c r="I89" s="2" t="n">
-        <v>69.11</v>
-      </c>
-      <c r="J89" s="2" t="n">
-        <v>76.38</v>
-      </c>
       <c r="K89" s="2" t="n">
-        <v>3.455</v>
+        <v>2.596</v>
       </c>
       <c r="L89" s="2" t="n">
-        <v>1.478</v>
+        <v>0.62</v>
       </c>
       <c r="M89" s="2" t="n">
-        <v>3.5459</v>
+        <v>2.2136</v>
       </c>
       <c r="N89" t="inlineStr">
         <is>
@@ -5219,26 +5225,26 @@
       </c>
       <c r="D90" t="inlineStr">
         <is>
-          <t>WHU-CD-256</t>
+          <t>CDD-CD-256</t>
         </is>
       </c>
       <c r="E90" s="2" t="n">
-        <v>91.64</v>
+        <v>94.7</v>
       </c>
       <c r="F90" s="2" t="n">
-        <v>94.81999999999999</v>
+        <v>96.13</v>
       </c>
       <c r="G90" s="2" t="n">
-        <v>99.47</v>
+        <v>98.88</v>
       </c>
       <c r="H90" s="2" t="n">
-        <v>93.2</v>
+        <v>95.41</v>
       </c>
       <c r="I90" s="2" t="n">
-        <v>87.27</v>
+        <v>91.22</v>
       </c>
       <c r="J90" s="2" t="n">
-        <v>92.93000000000001</v>
+        <v>94.77</v>
       </c>
       <c r="K90" s="2" t="n">
         <v>3.455</v>
@@ -5258,71 +5264,71 @@
     <row r="91">
       <c r="A91" t="inlineStr">
         <is>
-          <t>UltraLight</t>
+          <t>STR-Fusion</t>
         </is>
       </c>
       <c r="B91" t="inlineStr">
         <is>
-          <t>Run4</t>
+          <t>Run2_TASS</t>
         </is>
       </c>
       <c r="C91" t="inlineStr">
         <is>
-          <t>R4_0_A0_FULL12_FROZEN</t>
+          <t>M1_TASS</t>
         </is>
       </c>
       <c r="D91" t="inlineStr">
         <is>
-          <t>SYSU-CD-256</t>
+          <t>LEVIR-CD-256</t>
         </is>
       </c>
       <c r="E91" s="2" t="n">
-        <v>82.42</v>
+        <v>88.42</v>
       </c>
       <c r="F91" s="2" t="n">
-        <v>83.87</v>
+        <v>91.97</v>
       </c>
       <c r="G91" s="2" t="n">
-        <v>92.12</v>
+        <v>99.02</v>
       </c>
       <c r="H91" s="2" t="n">
-        <v>83.14</v>
+        <v>90.16</v>
       </c>
       <c r="I91" s="2" t="n">
-        <v>71.14</v>
+        <v>82.08</v>
       </c>
       <c r="J91" s="2" t="n">
-        <v>77.98999999999999</v>
+        <v>89.64</v>
       </c>
       <c r="K91" s="2" t="n">
-        <v>11.754</v>
+        <v>3.455</v>
       </c>
       <c r="L91" s="2" t="n">
-        <v>15.125</v>
+        <v>1.478</v>
       </c>
       <c r="M91" s="2" t="n">
-        <v>26.3246</v>
+        <v>3.5459</v>
       </c>
       <c r="N91" t="inlineStr">
         <is>
-          <t>baseline</t>
+          <t>str_tass</t>
         </is>
       </c>
     </row>
     <row r="92">
       <c r="A92" t="inlineStr">
         <is>
-          <t>UltraLight</t>
+          <t>STR-Fusion</t>
         </is>
       </c>
       <c r="B92" t="inlineStr">
         <is>
-          <t>Run4</t>
+          <t>Run2_TASS</t>
         </is>
       </c>
       <c r="C92" t="inlineStr">
         <is>
-          <t>R4_1_VIT4_OLDHEAD</t>
+          <t>M1_TASS</t>
         </is>
       </c>
       <c r="D92" t="inlineStr">
@@ -5331,89 +5337,89 @@
         </is>
       </c>
       <c r="E92" s="2" t="n">
-        <v>82.15000000000001</v>
+        <v>78.73</v>
       </c>
       <c r="F92" s="2" t="n">
-        <v>83.40000000000001</v>
+        <v>84.98</v>
       </c>
       <c r="G92" s="2" t="n">
-        <v>91.94</v>
+        <v>91.7</v>
       </c>
       <c r="H92" s="2" t="n">
-        <v>82.77</v>
+        <v>81.73999999999999</v>
       </c>
       <c r="I92" s="2" t="n">
-        <v>70.61</v>
+        <v>69.11</v>
       </c>
       <c r="J92" s="2" t="n">
-        <v>77.51000000000001</v>
+        <v>76.38</v>
       </c>
       <c r="K92" s="2" t="n">
-        <v>8.195</v>
+        <v>3.455</v>
       </c>
       <c r="L92" s="2" t="n">
-        <v>15.125</v>
+        <v>1.478</v>
       </c>
       <c r="M92" s="2" t="n">
-        <v>24.1021</v>
+        <v>3.5459</v>
       </c>
       <c r="N92" t="inlineStr">
         <is>
-          <t>baseline</t>
+          <t>str_tass</t>
         </is>
       </c>
     </row>
     <row r="93">
       <c r="A93" t="inlineStr">
         <is>
-          <t>UltraLight</t>
+          <t>STR-Fusion</t>
         </is>
       </c>
       <c r="B93" t="inlineStr">
         <is>
-          <t>Run4</t>
+          <t>Run2_TASS</t>
         </is>
       </c>
       <c r="C93" t="inlineStr">
         <is>
-          <t>R4_2_VIT4_LIGHTDETAIL</t>
+          <t>M1_TASS</t>
         </is>
       </c>
       <c r="D93" t="inlineStr">
         <is>
-          <t>SYSU-CD-256</t>
+          <t>WHU-CD-256</t>
         </is>
       </c>
       <c r="E93" s="2" t="n">
-        <v>79.94</v>
+        <v>91.64</v>
       </c>
       <c r="F93" s="2" t="n">
-        <v>84.79000000000001</v>
+        <v>94.81999999999999</v>
       </c>
       <c r="G93" s="2" t="n">
-        <v>91.89</v>
+        <v>99.47</v>
       </c>
       <c r="H93" s="2" t="n">
-        <v>82.3</v>
+        <v>93.2</v>
       </c>
       <c r="I93" s="2" t="n">
-        <v>69.92</v>
+        <v>87.27</v>
       </c>
       <c r="J93" s="2" t="n">
-        <v>77.04000000000001</v>
+        <v>92.93000000000001</v>
       </c>
       <c r="K93" s="2" t="n">
-        <v>5.492</v>
+        <v>3.455</v>
       </c>
       <c r="L93" s="2" t="n">
-        <v>3.515</v>
+        <v>1.478</v>
       </c>
       <c r="M93" s="2" t="n">
-        <v>10.7311</v>
+        <v>3.5459</v>
       </c>
       <c r="N93" t="inlineStr">
         <is>
-          <t>baseline</t>
+          <t>str_tass</t>
         </is>
       </c>
     </row>
@@ -5430,7 +5436,7 @@
       </c>
       <c r="C94" t="inlineStr">
         <is>
-          <t>R4_2b_VIT4_LIGHTDETAIL48</t>
+          <t>R4_0_A0_FULL12_FROZEN</t>
         </is>
       </c>
       <c r="D94" t="inlineStr">
@@ -5439,31 +5445,31 @@
         </is>
       </c>
       <c r="E94" s="2" t="n">
-        <v>80.87</v>
+        <v>82.42</v>
       </c>
       <c r="F94" s="2" t="n">
-        <v>83.81</v>
+        <v>83.87</v>
       </c>
       <c r="G94" s="2" t="n">
-        <v>91.81</v>
+        <v>92.12</v>
       </c>
       <c r="H94" s="2" t="n">
-        <v>82.31999999999999</v>
+        <v>83.14</v>
       </c>
       <c r="I94" s="2" t="n">
-        <v>69.95</v>
+        <v>71.14</v>
       </c>
       <c r="J94" s="2" t="n">
-        <v>76.98999999999999</v>
+        <v>77.98999999999999</v>
       </c>
       <c r="K94" s="2" t="n">
-        <v>5.533</v>
+        <v>11.754</v>
       </c>
       <c r="L94" s="2" t="n">
-        <v>3.556</v>
+        <v>15.125</v>
       </c>
       <c r="M94" s="2" t="n">
-        <v>10.9824</v>
+        <v>26.3246</v>
       </c>
       <c r="N94" t="inlineStr">
         <is>
@@ -5484,7 +5490,7 @@
       </c>
       <c r="C95" t="inlineStr">
         <is>
-          <t>R4_2d_PSD_DETAIL</t>
+          <t>R4_1_VIT4_OLDHEAD</t>
         </is>
       </c>
       <c r="D95" t="inlineStr">
@@ -5493,31 +5499,31 @@
         </is>
       </c>
       <c r="E95" s="2" t="n">
-        <v>79.78</v>
+        <v>82.15000000000001</v>
       </c>
       <c r="F95" s="2" t="n">
-        <v>84.39</v>
+        <v>83.40000000000001</v>
       </c>
       <c r="G95" s="2" t="n">
-        <v>91.75</v>
+        <v>91.94</v>
       </c>
       <c r="H95" s="2" t="n">
-        <v>82.02</v>
+        <v>82.77</v>
       </c>
       <c r="I95" s="2" t="n">
-        <v>69.52</v>
+        <v>70.61</v>
       </c>
       <c r="J95" s="2" t="n">
-        <v>76.68000000000001</v>
+        <v>77.51000000000001</v>
       </c>
       <c r="K95" s="2" t="n">
-        <v>5.491</v>
+        <v>8.195</v>
       </c>
       <c r="L95" s="2" t="n">
-        <v>3.514</v>
+        <v>15.125</v>
       </c>
       <c r="M95" s="2" t="n">
-        <v>11.5239</v>
+        <v>24.1021</v>
       </c>
       <c r="N95" t="inlineStr">
         <is>
@@ -5528,45 +5534,50 @@
     <row r="96">
       <c r="A96" t="inlineStr">
         <is>
-          <t>baseline</t>
+          <t>UltraLight</t>
         </is>
       </c>
       <c r="B96" t="inlineStr">
         <is>
-          <t>Run1</t>
+          <t>Run4</t>
+        </is>
+      </c>
+      <c r="C96" t="inlineStr">
+        <is>
+          <t>R4_2_VIT4_LIGHTDETAIL</t>
         </is>
       </c>
       <c r="D96" t="inlineStr">
         <is>
-          <t>CDD-CD-256</t>
+          <t>SYSU-CD-256</t>
         </is>
       </c>
       <c r="E96" s="2" t="n">
-        <v>97.72</v>
+        <v>79.94</v>
       </c>
       <c r="F96" s="2" t="n">
-        <v>97.78</v>
+        <v>84.79000000000001</v>
       </c>
       <c r="G96" s="2" t="n">
-        <v>99.44</v>
+        <v>91.89</v>
       </c>
       <c r="H96" s="2" t="n">
-        <v>97.75</v>
+        <v>82.3</v>
       </c>
       <c r="I96" s="2" t="n">
-        <v>95.59999999999999</v>
+        <v>69.92</v>
       </c>
       <c r="J96" s="2" t="n">
-        <v>97.43000000000001</v>
+        <v>77.04000000000001</v>
       </c>
       <c r="K96" s="2" t="n">
-        <v>11.754</v>
+        <v>5.492</v>
       </c>
       <c r="L96" s="2" t="n">
-        <v>20.661</v>
+        <v>3.515</v>
       </c>
       <c r="M96" s="2" t="n">
-        <v>26.3246</v>
+        <v>10.7311</v>
       </c>
       <c r="N96" t="inlineStr">
         <is>
@@ -5577,45 +5588,50 @@
     <row r="97">
       <c r="A97" t="inlineStr">
         <is>
-          <t>baseline</t>
+          <t>UltraLight</t>
         </is>
       </c>
       <c r="B97" t="inlineStr">
         <is>
-          <t>Run1</t>
+          <t>Run4</t>
+        </is>
+      </c>
+      <c r="C97" t="inlineStr">
+        <is>
+          <t>R4_2b_VIT4_LIGHTDETAIL48</t>
         </is>
       </c>
       <c r="D97" t="inlineStr">
         <is>
-          <t>LEVIR-CD-256</t>
+          <t>SYSU-CD-256</t>
         </is>
       </c>
       <c r="E97" s="2" t="n">
-        <v>91.56999999999999</v>
+        <v>80.87</v>
       </c>
       <c r="F97" s="2" t="n">
-        <v>92.33</v>
+        <v>83.81</v>
       </c>
       <c r="G97" s="2" t="n">
-        <v>99.18000000000001</v>
+        <v>91.81</v>
       </c>
       <c r="H97" s="2" t="n">
-        <v>91.95</v>
+        <v>82.31999999999999</v>
       </c>
       <c r="I97" s="2" t="n">
-        <v>85.09999999999999</v>
+        <v>69.95</v>
       </c>
       <c r="J97" s="2" t="n">
-        <v>91.52</v>
+        <v>76.98999999999999</v>
       </c>
       <c r="K97" s="2" t="n">
-        <v>11.754</v>
+        <v>5.533</v>
       </c>
       <c r="L97" s="2" t="n">
-        <v>20.661</v>
+        <v>3.556</v>
       </c>
       <c r="M97" s="2" t="n">
-        <v>26.3246</v>
+        <v>10.9824</v>
       </c>
       <c r="N97" t="inlineStr">
         <is>
@@ -5626,12 +5642,17 @@
     <row r="98">
       <c r="A98" t="inlineStr">
         <is>
-          <t>baseline</t>
+          <t>UltraLight</t>
         </is>
       </c>
       <c r="B98" t="inlineStr">
         <is>
-          <t>Run1</t>
+          <t>Run4</t>
+        </is>
+      </c>
+      <c r="C98" t="inlineStr">
+        <is>
+          <t>R4_2d_PSD_DETAIL</t>
         </is>
       </c>
       <c r="D98" t="inlineStr">
@@ -5640,31 +5661,31 @@
         </is>
       </c>
       <c r="E98" s="2" t="n">
-        <v>80.77</v>
+        <v>79.78</v>
       </c>
       <c r="F98" s="2" t="n">
-        <v>84.27</v>
+        <v>84.39</v>
       </c>
       <c r="G98" s="2" t="n">
-        <v>91.91</v>
+        <v>91.75</v>
       </c>
       <c r="H98" s="2" t="n">
-        <v>82.48</v>
+        <v>82.02</v>
       </c>
       <c r="I98" s="2" t="n">
-        <v>70.19</v>
+        <v>69.52</v>
       </c>
       <c r="J98" s="2" t="n">
-        <v>77.23</v>
+        <v>76.68000000000001</v>
       </c>
       <c r="K98" s="2" t="n">
-        <v>11.754</v>
+        <v>5.491</v>
       </c>
       <c r="L98" s="2" t="n">
-        <v>20.661</v>
+        <v>3.514</v>
       </c>
       <c r="M98" s="2" t="n">
-        <v>26.3246</v>
+        <v>11.5239</v>
       </c>
       <c r="N98" t="inlineStr">
         <is>
@@ -5683,28 +5704,29 @@
           <t>Run1</t>
         </is>
       </c>
+      <c r="C99" t="inlineStr"/>
       <c r="D99" t="inlineStr">
         <is>
-          <t>WHU-CD-256</t>
+          <t>CDD-CD-256</t>
         </is>
       </c>
       <c r="E99" s="2" t="n">
-        <v>93.62</v>
+        <v>97.72</v>
       </c>
       <c r="F99" s="2" t="n">
-        <v>96.09</v>
+        <v>97.78</v>
       </c>
       <c r="G99" s="2" t="n">
-        <v>99.59999999999999</v>
+        <v>99.44</v>
       </c>
       <c r="H99" s="2" t="n">
-        <v>94.84</v>
+        <v>97.75</v>
       </c>
       <c r="I99" s="2" t="n">
-        <v>90.18000000000001</v>
+        <v>95.59999999999999</v>
       </c>
       <c r="J99" s="2" t="n">
-        <v>94.63</v>
+        <v>97.43000000000001</v>
       </c>
       <c r="K99" s="2" t="n">
         <v>11.754</v>
@@ -5721,8 +5743,158 @@
         </is>
       </c>
     </row>
+    <row r="100">
+      <c r="A100" t="inlineStr">
+        <is>
+          <t>baseline</t>
+        </is>
+      </c>
+      <c r="B100" t="inlineStr">
+        <is>
+          <t>Run1</t>
+        </is>
+      </c>
+      <c r="C100" t="inlineStr"/>
+      <c r="D100" t="inlineStr">
+        <is>
+          <t>LEVIR-CD-256</t>
+        </is>
+      </c>
+      <c r="E100" s="2" t="n">
+        <v>91.56999999999999</v>
+      </c>
+      <c r="F100" s="2" t="n">
+        <v>92.33</v>
+      </c>
+      <c r="G100" s="2" t="n">
+        <v>99.18000000000001</v>
+      </c>
+      <c r="H100" s="2" t="n">
+        <v>91.95</v>
+      </c>
+      <c r="I100" s="2" t="n">
+        <v>85.09999999999999</v>
+      </c>
+      <c r="J100" s="2" t="n">
+        <v>91.52</v>
+      </c>
+      <c r="K100" s="2" t="n">
+        <v>11.754</v>
+      </c>
+      <c r="L100" s="2" t="n">
+        <v>20.661</v>
+      </c>
+      <c r="M100" s="2" t="n">
+        <v>26.3246</v>
+      </c>
+      <c r="N100" t="inlineStr">
+        <is>
+          <t>baseline</t>
+        </is>
+      </c>
+    </row>
+    <row r="101">
+      <c r="A101" t="inlineStr">
+        <is>
+          <t>baseline</t>
+        </is>
+      </c>
+      <c r="B101" t="inlineStr">
+        <is>
+          <t>Run1</t>
+        </is>
+      </c>
+      <c r="C101" t="inlineStr"/>
+      <c r="D101" t="inlineStr">
+        <is>
+          <t>SYSU-CD-256</t>
+        </is>
+      </c>
+      <c r="E101" s="2" t="n">
+        <v>80.77</v>
+      </c>
+      <c r="F101" s="2" t="n">
+        <v>84.27</v>
+      </c>
+      <c r="G101" s="2" t="n">
+        <v>91.91</v>
+      </c>
+      <c r="H101" s="2" t="n">
+        <v>82.48</v>
+      </c>
+      <c r="I101" s="2" t="n">
+        <v>70.19</v>
+      </c>
+      <c r="J101" s="2" t="n">
+        <v>77.23</v>
+      </c>
+      <c r="K101" s="2" t="n">
+        <v>11.754</v>
+      </c>
+      <c r="L101" s="2" t="n">
+        <v>20.661</v>
+      </c>
+      <c r="M101" s="2" t="n">
+        <v>26.3246</v>
+      </c>
+      <c r="N101" t="inlineStr">
+        <is>
+          <t>baseline</t>
+        </is>
+      </c>
+    </row>
+    <row r="102">
+      <c r="A102" t="inlineStr">
+        <is>
+          <t>baseline</t>
+        </is>
+      </c>
+      <c r="B102" t="inlineStr">
+        <is>
+          <t>Run1</t>
+        </is>
+      </c>
+      <c r="C102" t="inlineStr"/>
+      <c r="D102" t="inlineStr">
+        <is>
+          <t>WHU-CD-256</t>
+        </is>
+      </c>
+      <c r="E102" s="2" t="n">
+        <v>93.62</v>
+      </c>
+      <c r="F102" s="2" t="n">
+        <v>96.09</v>
+      </c>
+      <c r="G102" s="2" t="n">
+        <v>99.59999999999999</v>
+      </c>
+      <c r="H102" s="2" t="n">
+        <v>94.84</v>
+      </c>
+      <c r="I102" s="2" t="n">
+        <v>90.18000000000001</v>
+      </c>
+      <c r="J102" s="2" t="n">
+        <v>94.63</v>
+      </c>
+      <c r="K102" s="2" t="n">
+        <v>11.754</v>
+      </c>
+      <c r="L102" s="2" t="n">
+        <v>20.661</v>
+      </c>
+      <c r="M102" s="2" t="n">
+        <v>26.3246</v>
+      </c>
+      <c r="N102" t="inlineStr">
+        <is>
+          <t>baseline</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:N99"/>
+  <autoFilter ref="A1:N102"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Record WDMF SYSU control test results
</commit_message>
<xml_diff>
--- a/docs/experiment_metrics.xlsx
+++ b/docs/experiment_metrics.xlsx
@@ -10,7 +10,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="metrics" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'metrics'!$A$1:$N$102</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'metrics'!$A$1:$N$103</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -420,7 +420,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N102"/>
+  <dimension ref="A1:N103"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -4508,7 +4508,7 @@
     <row r="77">
       <c r="A77" t="inlineStr">
         <is>
-          <t>CASAA</t>
+          <t>CASA-WDMF</t>
         </is>
       </c>
       <c r="B77" t="inlineStr">
@@ -4518,44 +4518,42 @@
       </c>
       <c r="C77" t="inlineStr">
         <is>
-          <t>A1_SAA</t>
+          <t>M0_CTRL</t>
         </is>
       </c>
       <c r="D77" t="inlineStr">
         <is>
-          <t>LEVIR-CD-256</t>
+          <t>SYSU-CD-256</t>
         </is>
       </c>
       <c r="E77" s="2" t="n">
-        <v>91.09</v>
+        <v>80.27</v>
       </c>
       <c r="F77" s="2" t="n">
-        <v>92.8</v>
+        <v>85.19</v>
       </c>
       <c r="G77" s="2" t="n">
-        <v>99.19</v>
+        <v>92.06</v>
       </c>
       <c r="H77" s="2" t="n">
-        <v>91.94</v>
+        <v>82.65000000000001</v>
       </c>
       <c r="I77" s="2" t="n">
-        <v>85.08</v>
+        <v>70.44</v>
       </c>
       <c r="J77" s="2" t="n">
-        <v>91.51000000000001</v>
+        <v>77.51000000000001</v>
       </c>
       <c r="K77" s="2" t="n">
-        <v>11.754</v>
+        <v>3.016737</v>
       </c>
       <c r="L77" s="2" t="n">
-        <v>20.661</v>
-      </c>
-      <c r="M77" s="2" t="n">
-        <v>26.3183</v>
-      </c>
+        <v>3.100404</v>
+      </c>
+      <c r="M77" s="2" t="n"/>
       <c r="N77" t="inlineStr">
         <is>
-          <t>saa</t>
+          <t>casa_wdmf_str_none</t>
         </is>
       </c>
     </row>
@@ -4577,26 +4575,26 @@
       </c>
       <c r="D78" t="inlineStr">
         <is>
-          <t>SYSU-CD-256</t>
+          <t>LEVIR-CD-256</t>
         </is>
       </c>
       <c r="E78" s="2" t="n">
-        <v>80.3</v>
+        <v>91.09</v>
       </c>
       <c r="F78" s="2" t="n">
-        <v>84.81</v>
+        <v>92.8</v>
       </c>
       <c r="G78" s="2" t="n">
-        <v>91.95999999999999</v>
+        <v>99.19</v>
       </c>
       <c r="H78" s="2" t="n">
-        <v>82.5</v>
+        <v>91.94</v>
       </c>
       <c r="I78" s="2" t="n">
-        <v>70.20999999999999</v>
+        <v>85.08</v>
       </c>
       <c r="J78" s="2" t="n">
-        <v>77.29000000000001</v>
+        <v>91.51000000000001</v>
       </c>
       <c r="K78" s="2" t="n">
         <v>11.754</v>
@@ -4626,31 +4624,31 @@
       </c>
       <c r="C79" t="inlineStr">
         <is>
-          <t>A2_CASAA</t>
+          <t>A1_SAA</t>
         </is>
       </c>
       <c r="D79" t="inlineStr">
         <is>
-          <t>LEVIR-CD-256</t>
+          <t>SYSU-CD-256</t>
         </is>
       </c>
       <c r="E79" s="2" t="n">
-        <v>90.98999999999999</v>
+        <v>80.3</v>
       </c>
       <c r="F79" s="2" t="n">
-        <v>92.75</v>
+        <v>84.81</v>
       </c>
       <c r="G79" s="2" t="n">
-        <v>99.18000000000001</v>
+        <v>91.95999999999999</v>
       </c>
       <c r="H79" s="2" t="n">
-        <v>91.86</v>
+        <v>82.5</v>
       </c>
       <c r="I79" s="2" t="n">
-        <v>84.94</v>
+        <v>70.20999999999999</v>
       </c>
       <c r="J79" s="2" t="n">
-        <v>91.43000000000001</v>
+        <v>77.29000000000001</v>
       </c>
       <c r="K79" s="2" t="n">
         <v>11.754</v>
@@ -4659,11 +4657,11 @@
         <v>20.661</v>
       </c>
       <c r="M79" s="2" t="n">
-        <v>26.2593</v>
+        <v>26.3183</v>
       </c>
       <c r="N79" t="inlineStr">
         <is>
-          <t>casaa</t>
+          <t>saa</t>
         </is>
       </c>
     </row>
@@ -4685,26 +4683,26 @@
       </c>
       <c r="D80" t="inlineStr">
         <is>
-          <t>SYSU-CD-256</t>
+          <t>LEVIR-CD-256</t>
         </is>
       </c>
       <c r="E80" s="2" t="n">
-        <v>80.55</v>
+        <v>90.98999999999999</v>
       </c>
       <c r="F80" s="2" t="n">
-        <v>84.23</v>
+        <v>92.75</v>
       </c>
       <c r="G80" s="2" t="n">
+        <v>99.18000000000001</v>
+      </c>
+      <c r="H80" s="2" t="n">
         <v>91.86</v>
       </c>
-      <c r="H80" s="2" t="n">
-        <v>82.34999999999999</v>
-      </c>
       <c r="I80" s="2" t="n">
-        <v>70</v>
+        <v>84.94</v>
       </c>
       <c r="J80" s="2" t="n">
-        <v>77.06</v>
+        <v>91.43000000000001</v>
       </c>
       <c r="K80" s="2" t="n">
         <v>11.754</v>
@@ -4729,49 +4727,49 @@
       </c>
       <c r="B81" t="inlineStr">
         <is>
-          <t>Run2</t>
+          <t>Run1</t>
         </is>
       </c>
       <c r="C81" t="inlineStr">
         <is>
-          <t>A1_SAA_FROZEN</t>
+          <t>A2_CASAA</t>
         </is>
       </c>
       <c r="D81" t="inlineStr">
         <is>
-          <t>LEVIR-CD-256</t>
+          <t>SYSU-CD-256</t>
         </is>
       </c>
       <c r="E81" s="2" t="n">
-        <v>91.38</v>
+        <v>80.55</v>
       </c>
       <c r="F81" s="2" t="n">
-        <v>92.3</v>
+        <v>84.23</v>
       </c>
       <c r="G81" s="2" t="n">
-        <v>99.17</v>
+        <v>91.86</v>
       </c>
       <c r="H81" s="2" t="n">
-        <v>91.84</v>
+        <v>82.34999999999999</v>
       </c>
       <c r="I81" s="2" t="n">
-        <v>84.91</v>
+        <v>70</v>
       </c>
       <c r="J81" s="2" t="n">
-        <v>91.40000000000001</v>
+        <v>77.06</v>
       </c>
       <c r="K81" s="2" t="n">
         <v>11.754</v>
       </c>
       <c r="L81" s="2" t="n">
-        <v>15.125</v>
+        <v>20.661</v>
       </c>
       <c r="M81" s="2" t="n">
-        <v>26.1484</v>
+        <v>26.2593</v>
       </c>
       <c r="N81" t="inlineStr">
         <is>
-          <t>saa</t>
+          <t>casaa</t>
         </is>
       </c>
     </row>
@@ -4793,26 +4791,26 @@
       </c>
       <c r="D82" t="inlineStr">
         <is>
-          <t>SYSU-CD-256</t>
+          <t>LEVIR-CD-256</t>
         </is>
       </c>
       <c r="E82" s="2" t="n">
-        <v>78.40000000000001</v>
+        <v>91.38</v>
       </c>
       <c r="F82" s="2" t="n">
-        <v>86.03</v>
+        <v>92.3</v>
       </c>
       <c r="G82" s="2" t="n">
-        <v>91.90000000000001</v>
+        <v>99.17</v>
       </c>
       <c r="H82" s="2" t="n">
-        <v>82.04000000000001</v>
+        <v>91.84</v>
       </c>
       <c r="I82" s="2" t="n">
-        <v>69.55</v>
+        <v>84.91</v>
       </c>
       <c r="J82" s="2" t="n">
-        <v>76.83</v>
+        <v>91.40000000000001</v>
       </c>
       <c r="K82" s="2" t="n">
         <v>11.754</v>
@@ -4842,31 +4840,31 @@
       </c>
       <c r="C83" t="inlineStr">
         <is>
-          <t>A3_ORACLE_FROZEN</t>
+          <t>A1_SAA_FROZEN</t>
         </is>
       </c>
       <c r="D83" t="inlineStr">
         <is>
-          <t>LEVIR-CD-256</t>
+          <t>SYSU-CD-256</t>
         </is>
       </c>
       <c r="E83" s="2" t="n">
-        <v>91.13</v>
+        <v>78.40000000000001</v>
       </c>
       <c r="F83" s="2" t="n">
-        <v>92.65000000000001</v>
+        <v>86.03</v>
       </c>
       <c r="G83" s="2" t="n">
-        <v>99.18000000000001</v>
+        <v>91.90000000000001</v>
       </c>
       <c r="H83" s="2" t="n">
-        <v>91.88</v>
+        <v>82.04000000000001</v>
       </c>
       <c r="I83" s="2" t="n">
-        <v>84.98</v>
+        <v>69.55</v>
       </c>
       <c r="J83" s="2" t="n">
-        <v>91.45</v>
+        <v>76.83</v>
       </c>
       <c r="K83" s="2" t="n">
         <v>11.754</v>
@@ -4875,11 +4873,11 @@
         <v>15.125</v>
       </c>
       <c r="M83" s="2" t="n">
-        <v>26.0894</v>
+        <v>26.1484</v>
       </c>
       <c r="N83" t="inlineStr">
         <is>
-          <t>casaa</t>
+          <t>saa</t>
         </is>
       </c>
     </row>
@@ -4901,26 +4899,26 @@
       </c>
       <c r="D84" t="inlineStr">
         <is>
-          <t>SYSU-CD-256</t>
+          <t>LEVIR-CD-256</t>
         </is>
       </c>
       <c r="E84" s="2" t="n">
-        <v>82.04000000000001</v>
+        <v>91.13</v>
       </c>
       <c r="F84" s="2" t="n">
-        <v>85.05</v>
+        <v>92.65000000000001</v>
       </c>
       <c r="G84" s="2" t="n">
-        <v>92.36</v>
+        <v>99.18000000000001</v>
       </c>
       <c r="H84" s="2" t="n">
-        <v>83.52</v>
+        <v>91.88</v>
       </c>
       <c r="I84" s="2" t="n">
-        <v>71.7</v>
+        <v>84.98</v>
       </c>
       <c r="J84" s="2" t="n">
-        <v>78.55</v>
+        <v>91.45</v>
       </c>
       <c r="K84" s="2" t="n">
         <v>11.754</v>
@@ -4945,12 +4943,12 @@
       </c>
       <c r="B85" t="inlineStr">
         <is>
-          <t>Run3</t>
+          <t>Run2</t>
         </is>
       </c>
       <c r="C85" t="inlineStr">
         <is>
-          <t>A4_DETAIL_FROZEN</t>
+          <t>A3_ORACLE_FROZEN</t>
         </is>
       </c>
       <c r="D85" t="inlineStr">
@@ -4959,22 +4957,22 @@
         </is>
       </c>
       <c r="E85" s="2" t="n">
-        <v>79.68000000000001</v>
+        <v>82.04000000000001</v>
       </c>
       <c r="F85" s="2" t="n">
-        <v>84.28</v>
+        <v>85.05</v>
       </c>
       <c r="G85" s="2" t="n">
-        <v>91.7</v>
+        <v>92.36</v>
       </c>
       <c r="H85" s="2" t="n">
-        <v>81.92</v>
+        <v>83.52</v>
       </c>
       <c r="I85" s="2" t="n">
-        <v>69.37</v>
+        <v>71.7</v>
       </c>
       <c r="J85" s="2" t="n">
-        <v>76.54000000000001</v>
+        <v>78.55</v>
       </c>
       <c r="K85" s="2" t="n">
         <v>11.754</v>
@@ -4994,54 +4992,54 @@
     <row r="86">
       <c r="A86" t="inlineStr">
         <is>
-          <t>STR-Fusion</t>
+          <t>CASAA</t>
         </is>
       </c>
       <c r="B86" t="inlineStr">
         <is>
-          <t>Run2_TASS</t>
+          <t>Run3</t>
         </is>
       </c>
       <c r="C86" t="inlineStr">
         <is>
-          <t>C0_TOKEN</t>
+          <t>A4_DETAIL_FROZEN</t>
         </is>
       </c>
       <c r="D86" t="inlineStr">
         <is>
-          <t>CDD-CD-256</t>
+          <t>SYSU-CD-256</t>
         </is>
       </c>
       <c r="E86" s="2" t="n">
-        <v>93.13</v>
+        <v>79.68000000000001</v>
       </c>
       <c r="F86" s="2" t="n">
-        <v>95.16</v>
+        <v>84.28</v>
       </c>
       <c r="G86" s="2" t="n">
-        <v>98.56999999999999</v>
+        <v>91.7</v>
       </c>
       <c r="H86" s="2" t="n">
-        <v>94.13</v>
+        <v>81.92</v>
       </c>
       <c r="I86" s="2" t="n">
-        <v>88.91</v>
+        <v>69.37</v>
       </c>
       <c r="J86" s="2" t="n">
-        <v>93.31999999999999</v>
+        <v>76.54000000000001</v>
       </c>
       <c r="K86" s="2" t="n">
-        <v>2.596</v>
+        <v>11.754</v>
       </c>
       <c r="L86" s="2" t="n">
-        <v>0.62</v>
+        <v>15.125</v>
       </c>
       <c r="M86" s="2" t="n">
-        <v>2.2136</v>
+        <v>26.0894</v>
       </c>
       <c r="N86" t="inlineStr">
         <is>
-          <t>str_tass</t>
+          <t>casaa</t>
         </is>
       </c>
     </row>
@@ -5063,26 +5061,26 @@
       </c>
       <c r="D87" t="inlineStr">
         <is>
-          <t>LEVIR-CD-256</t>
+          <t>CDD-CD-256</t>
         </is>
       </c>
       <c r="E87" s="2" t="n">
-        <v>86.37</v>
+        <v>93.13</v>
       </c>
       <c r="F87" s="2" t="n">
-        <v>89.25</v>
+        <v>95.16</v>
       </c>
       <c r="G87" s="2" t="n">
-        <v>98.78</v>
+        <v>98.56999999999999</v>
       </c>
       <c r="H87" s="2" t="n">
-        <v>87.79000000000001</v>
+        <v>94.13</v>
       </c>
       <c r="I87" s="2" t="n">
-        <v>78.23999999999999</v>
+        <v>88.91</v>
       </c>
       <c r="J87" s="2" t="n">
-        <v>87.14</v>
+        <v>93.31999999999999</v>
       </c>
       <c r="K87" s="2" t="n">
         <v>2.596</v>
@@ -5117,26 +5115,26 @@
       </c>
       <c r="D88" t="inlineStr">
         <is>
-          <t>SYSU-CD-256</t>
+          <t>LEVIR-CD-256</t>
         </is>
       </c>
       <c r="E88" s="2" t="n">
-        <v>79.93000000000001</v>
+        <v>86.37</v>
       </c>
       <c r="F88" s="2" t="n">
-        <v>84.5</v>
+        <v>89.25</v>
       </c>
       <c r="G88" s="2" t="n">
-        <v>91.81</v>
+        <v>98.78</v>
       </c>
       <c r="H88" s="2" t="n">
-        <v>82.15000000000001</v>
+        <v>87.79000000000001</v>
       </c>
       <c r="I88" s="2" t="n">
-        <v>69.70999999999999</v>
+        <v>78.23999999999999</v>
       </c>
       <c r="J88" s="2" t="n">
-        <v>76.84</v>
+        <v>87.14</v>
       </c>
       <c r="K88" s="2" t="n">
         <v>2.596</v>
@@ -5171,26 +5169,26 @@
       </c>
       <c r="D89" t="inlineStr">
         <is>
-          <t>WHU-CD-256</t>
+          <t>SYSU-CD-256</t>
         </is>
       </c>
       <c r="E89" s="2" t="n">
-        <v>90.16</v>
+        <v>79.93000000000001</v>
       </c>
       <c r="F89" s="2" t="n">
-        <v>93.97</v>
+        <v>84.5</v>
       </c>
       <c r="G89" s="2" t="n">
-        <v>99.38</v>
+        <v>91.81</v>
       </c>
       <c r="H89" s="2" t="n">
-        <v>92.02</v>
+        <v>82.15000000000001</v>
       </c>
       <c r="I89" s="2" t="n">
-        <v>85.23</v>
+        <v>69.70999999999999</v>
       </c>
       <c r="J89" s="2" t="n">
-        <v>91.7</v>
+        <v>76.84</v>
       </c>
       <c r="K89" s="2" t="n">
         <v>2.596</v>
@@ -5220,40 +5218,40 @@
       </c>
       <c r="C90" t="inlineStr">
         <is>
-          <t>M1_TASS</t>
+          <t>C0_TOKEN</t>
         </is>
       </c>
       <c r="D90" t="inlineStr">
         <is>
-          <t>CDD-CD-256</t>
+          <t>WHU-CD-256</t>
         </is>
       </c>
       <c r="E90" s="2" t="n">
-        <v>94.7</v>
+        <v>90.16</v>
       </c>
       <c r="F90" s="2" t="n">
-        <v>96.13</v>
+        <v>93.97</v>
       </c>
       <c r="G90" s="2" t="n">
-        <v>98.88</v>
+        <v>99.38</v>
       </c>
       <c r="H90" s="2" t="n">
-        <v>95.41</v>
+        <v>92.02</v>
       </c>
       <c r="I90" s="2" t="n">
-        <v>91.22</v>
+        <v>85.23</v>
       </c>
       <c r="J90" s="2" t="n">
-        <v>94.77</v>
+        <v>91.7</v>
       </c>
       <c r="K90" s="2" t="n">
-        <v>3.455</v>
+        <v>2.596</v>
       </c>
       <c r="L90" s="2" t="n">
-        <v>1.478</v>
+        <v>0.62</v>
       </c>
       <c r="M90" s="2" t="n">
-        <v>3.5459</v>
+        <v>2.2136</v>
       </c>
       <c r="N90" t="inlineStr">
         <is>
@@ -5279,26 +5277,26 @@
       </c>
       <c r="D91" t="inlineStr">
         <is>
-          <t>LEVIR-CD-256</t>
+          <t>CDD-CD-256</t>
         </is>
       </c>
       <c r="E91" s="2" t="n">
-        <v>88.42</v>
+        <v>94.7</v>
       </c>
       <c r="F91" s="2" t="n">
-        <v>91.97</v>
+        <v>96.13</v>
       </c>
       <c r="G91" s="2" t="n">
-        <v>99.02</v>
+        <v>98.88</v>
       </c>
       <c r="H91" s="2" t="n">
-        <v>90.16</v>
+        <v>95.41</v>
       </c>
       <c r="I91" s="2" t="n">
-        <v>82.08</v>
+        <v>91.22</v>
       </c>
       <c r="J91" s="2" t="n">
-        <v>89.64</v>
+        <v>94.77</v>
       </c>
       <c r="K91" s="2" t="n">
         <v>3.455</v>
@@ -5333,26 +5331,26 @@
       </c>
       <c r="D92" t="inlineStr">
         <is>
-          <t>SYSU-CD-256</t>
+          <t>LEVIR-CD-256</t>
         </is>
       </c>
       <c r="E92" s="2" t="n">
-        <v>78.73</v>
+        <v>88.42</v>
       </c>
       <c r="F92" s="2" t="n">
-        <v>84.98</v>
+        <v>91.97</v>
       </c>
       <c r="G92" s="2" t="n">
-        <v>91.7</v>
+        <v>99.02</v>
       </c>
       <c r="H92" s="2" t="n">
-        <v>81.73999999999999</v>
+        <v>90.16</v>
       </c>
       <c r="I92" s="2" t="n">
-        <v>69.11</v>
+        <v>82.08</v>
       </c>
       <c r="J92" s="2" t="n">
-        <v>76.38</v>
+        <v>89.64</v>
       </c>
       <c r="K92" s="2" t="n">
         <v>3.455</v>
@@ -5387,26 +5385,26 @@
       </c>
       <c r="D93" t="inlineStr">
         <is>
-          <t>WHU-CD-256</t>
+          <t>SYSU-CD-256</t>
         </is>
       </c>
       <c r="E93" s="2" t="n">
-        <v>91.64</v>
+        <v>78.73</v>
       </c>
       <c r="F93" s="2" t="n">
-        <v>94.81999999999999</v>
+        <v>84.98</v>
       </c>
       <c r="G93" s="2" t="n">
-        <v>99.47</v>
+        <v>91.7</v>
       </c>
       <c r="H93" s="2" t="n">
-        <v>93.2</v>
+        <v>81.73999999999999</v>
       </c>
       <c r="I93" s="2" t="n">
-        <v>87.27</v>
+        <v>69.11</v>
       </c>
       <c r="J93" s="2" t="n">
-        <v>92.93000000000001</v>
+        <v>76.38</v>
       </c>
       <c r="K93" s="2" t="n">
         <v>3.455</v>
@@ -5426,54 +5424,54 @@
     <row r="94">
       <c r="A94" t="inlineStr">
         <is>
-          <t>UltraLight</t>
+          <t>STR-Fusion</t>
         </is>
       </c>
       <c r="B94" t="inlineStr">
         <is>
-          <t>Run4</t>
+          <t>Run2_TASS</t>
         </is>
       </c>
       <c r="C94" t="inlineStr">
         <is>
-          <t>R4_0_A0_FULL12_FROZEN</t>
+          <t>M1_TASS</t>
         </is>
       </c>
       <c r="D94" t="inlineStr">
         <is>
-          <t>SYSU-CD-256</t>
+          <t>WHU-CD-256</t>
         </is>
       </c>
       <c r="E94" s="2" t="n">
-        <v>82.42</v>
+        <v>91.64</v>
       </c>
       <c r="F94" s="2" t="n">
-        <v>83.87</v>
+        <v>94.81999999999999</v>
       </c>
       <c r="G94" s="2" t="n">
-        <v>92.12</v>
+        <v>99.47</v>
       </c>
       <c r="H94" s="2" t="n">
-        <v>83.14</v>
+        <v>93.2</v>
       </c>
       <c r="I94" s="2" t="n">
-        <v>71.14</v>
+        <v>87.27</v>
       </c>
       <c r="J94" s="2" t="n">
-        <v>77.98999999999999</v>
+        <v>92.93000000000001</v>
       </c>
       <c r="K94" s="2" t="n">
-        <v>11.754</v>
+        <v>3.455</v>
       </c>
       <c r="L94" s="2" t="n">
-        <v>15.125</v>
+        <v>1.478</v>
       </c>
       <c r="M94" s="2" t="n">
-        <v>26.3246</v>
+        <v>3.5459</v>
       </c>
       <c r="N94" t="inlineStr">
         <is>
-          <t>baseline</t>
+          <t>str_tass</t>
         </is>
       </c>
     </row>
@@ -5490,7 +5488,7 @@
       </c>
       <c r="C95" t="inlineStr">
         <is>
-          <t>R4_1_VIT4_OLDHEAD</t>
+          <t>R4_0_A0_FULL12_FROZEN</t>
         </is>
       </c>
       <c r="D95" t="inlineStr">
@@ -5499,31 +5497,31 @@
         </is>
       </c>
       <c r="E95" s="2" t="n">
-        <v>82.15000000000001</v>
+        <v>82.42</v>
       </c>
       <c r="F95" s="2" t="n">
-        <v>83.40000000000001</v>
+        <v>83.87</v>
       </c>
       <c r="G95" s="2" t="n">
-        <v>91.94</v>
+        <v>92.12</v>
       </c>
       <c r="H95" s="2" t="n">
-        <v>82.77</v>
+        <v>83.14</v>
       </c>
       <c r="I95" s="2" t="n">
-        <v>70.61</v>
+        <v>71.14</v>
       </c>
       <c r="J95" s="2" t="n">
-        <v>77.51000000000001</v>
+        <v>77.98999999999999</v>
       </c>
       <c r="K95" s="2" t="n">
-        <v>8.195</v>
+        <v>11.754</v>
       </c>
       <c r="L95" s="2" t="n">
         <v>15.125</v>
       </c>
       <c r="M95" s="2" t="n">
-        <v>24.1021</v>
+        <v>26.3246</v>
       </c>
       <c r="N95" t="inlineStr">
         <is>
@@ -5544,7 +5542,7 @@
       </c>
       <c r="C96" t="inlineStr">
         <is>
-          <t>R4_2_VIT4_LIGHTDETAIL</t>
+          <t>R4_1_VIT4_OLDHEAD</t>
         </is>
       </c>
       <c r="D96" t="inlineStr">
@@ -5553,31 +5551,31 @@
         </is>
       </c>
       <c r="E96" s="2" t="n">
-        <v>79.94</v>
+        <v>82.15000000000001</v>
       </c>
       <c r="F96" s="2" t="n">
-        <v>84.79000000000001</v>
+        <v>83.40000000000001</v>
       </c>
       <c r="G96" s="2" t="n">
-        <v>91.89</v>
+        <v>91.94</v>
       </c>
       <c r="H96" s="2" t="n">
-        <v>82.3</v>
+        <v>82.77</v>
       </c>
       <c r="I96" s="2" t="n">
-        <v>69.92</v>
+        <v>70.61</v>
       </c>
       <c r="J96" s="2" t="n">
-        <v>77.04000000000001</v>
+        <v>77.51000000000001</v>
       </c>
       <c r="K96" s="2" t="n">
-        <v>5.492</v>
+        <v>8.195</v>
       </c>
       <c r="L96" s="2" t="n">
-        <v>3.515</v>
+        <v>15.125</v>
       </c>
       <c r="M96" s="2" t="n">
-        <v>10.7311</v>
+        <v>24.1021</v>
       </c>
       <c r="N96" t="inlineStr">
         <is>
@@ -5598,7 +5596,7 @@
       </c>
       <c r="C97" t="inlineStr">
         <is>
-          <t>R4_2b_VIT4_LIGHTDETAIL48</t>
+          <t>R4_2_VIT4_LIGHTDETAIL</t>
         </is>
       </c>
       <c r="D97" t="inlineStr">
@@ -5607,31 +5605,31 @@
         </is>
       </c>
       <c r="E97" s="2" t="n">
-        <v>80.87</v>
+        <v>79.94</v>
       </c>
       <c r="F97" s="2" t="n">
-        <v>83.81</v>
+        <v>84.79000000000001</v>
       </c>
       <c r="G97" s="2" t="n">
-        <v>91.81</v>
+        <v>91.89</v>
       </c>
       <c r="H97" s="2" t="n">
-        <v>82.31999999999999</v>
+        <v>82.3</v>
       </c>
       <c r="I97" s="2" t="n">
-        <v>69.95</v>
+        <v>69.92</v>
       </c>
       <c r="J97" s="2" t="n">
-        <v>76.98999999999999</v>
+        <v>77.04000000000001</v>
       </c>
       <c r="K97" s="2" t="n">
-        <v>5.533</v>
+        <v>5.492</v>
       </c>
       <c r="L97" s="2" t="n">
-        <v>3.556</v>
+        <v>3.515</v>
       </c>
       <c r="M97" s="2" t="n">
-        <v>10.9824</v>
+        <v>10.7311</v>
       </c>
       <c r="N97" t="inlineStr">
         <is>
@@ -5652,7 +5650,7 @@
       </c>
       <c r="C98" t="inlineStr">
         <is>
-          <t>R4_2d_PSD_DETAIL</t>
+          <t>R4_2b_VIT4_LIGHTDETAIL48</t>
         </is>
       </c>
       <c r="D98" t="inlineStr">
@@ -5661,31 +5659,31 @@
         </is>
       </c>
       <c r="E98" s="2" t="n">
-        <v>79.78</v>
+        <v>80.87</v>
       </c>
       <c r="F98" s="2" t="n">
-        <v>84.39</v>
+        <v>83.81</v>
       </c>
       <c r="G98" s="2" t="n">
-        <v>91.75</v>
+        <v>91.81</v>
       </c>
       <c r="H98" s="2" t="n">
-        <v>82.02</v>
+        <v>82.31999999999999</v>
       </c>
       <c r="I98" s="2" t="n">
-        <v>69.52</v>
+        <v>69.95</v>
       </c>
       <c r="J98" s="2" t="n">
-        <v>76.68000000000001</v>
+        <v>76.98999999999999</v>
       </c>
       <c r="K98" s="2" t="n">
-        <v>5.491</v>
+        <v>5.533</v>
       </c>
       <c r="L98" s="2" t="n">
-        <v>3.514</v>
+        <v>3.556</v>
       </c>
       <c r="M98" s="2" t="n">
-        <v>11.5239</v>
+        <v>10.9824</v>
       </c>
       <c r="N98" t="inlineStr">
         <is>
@@ -5696,46 +5694,50 @@
     <row r="99">
       <c r="A99" t="inlineStr">
         <is>
-          <t>baseline</t>
+          <t>UltraLight</t>
         </is>
       </c>
       <c r="B99" t="inlineStr">
         <is>
-          <t>Run1</t>
-        </is>
-      </c>
-      <c r="C99" t="inlineStr"/>
+          <t>Run4</t>
+        </is>
+      </c>
+      <c r="C99" t="inlineStr">
+        <is>
+          <t>R4_2d_PSD_DETAIL</t>
+        </is>
+      </c>
       <c r="D99" t="inlineStr">
         <is>
-          <t>CDD-CD-256</t>
+          <t>SYSU-CD-256</t>
         </is>
       </c>
       <c r="E99" s="2" t="n">
-        <v>97.72</v>
+        <v>79.78</v>
       </c>
       <c r="F99" s="2" t="n">
-        <v>97.78</v>
+        <v>84.39</v>
       </c>
       <c r="G99" s="2" t="n">
-        <v>99.44</v>
+        <v>91.75</v>
       </c>
       <c r="H99" s="2" t="n">
-        <v>97.75</v>
+        <v>82.02</v>
       </c>
       <c r="I99" s="2" t="n">
-        <v>95.59999999999999</v>
+        <v>69.52</v>
       </c>
       <c r="J99" s="2" t="n">
-        <v>97.43000000000001</v>
+        <v>76.68000000000001</v>
       </c>
       <c r="K99" s="2" t="n">
-        <v>11.754</v>
+        <v>5.491</v>
       </c>
       <c r="L99" s="2" t="n">
-        <v>20.661</v>
+        <v>3.514</v>
       </c>
       <c r="M99" s="2" t="n">
-        <v>26.3246</v>
+        <v>11.5239</v>
       </c>
       <c r="N99" t="inlineStr">
         <is>
@@ -5757,26 +5759,26 @@
       <c r="C100" t="inlineStr"/>
       <c r="D100" t="inlineStr">
         <is>
-          <t>LEVIR-CD-256</t>
+          <t>CDD-CD-256</t>
         </is>
       </c>
       <c r="E100" s="2" t="n">
-        <v>91.56999999999999</v>
+        <v>97.72</v>
       </c>
       <c r="F100" s="2" t="n">
-        <v>92.33</v>
+        <v>97.78</v>
       </c>
       <c r="G100" s="2" t="n">
-        <v>99.18000000000001</v>
+        <v>99.44</v>
       </c>
       <c r="H100" s="2" t="n">
-        <v>91.95</v>
+        <v>97.75</v>
       </c>
       <c r="I100" s="2" t="n">
-        <v>85.09999999999999</v>
+        <v>95.59999999999999</v>
       </c>
       <c r="J100" s="2" t="n">
-        <v>91.52</v>
+        <v>97.43000000000001</v>
       </c>
       <c r="K100" s="2" t="n">
         <v>11.754</v>
@@ -5807,26 +5809,26 @@
       <c r="C101" t="inlineStr"/>
       <c r="D101" t="inlineStr">
         <is>
-          <t>SYSU-CD-256</t>
+          <t>LEVIR-CD-256</t>
         </is>
       </c>
       <c r="E101" s="2" t="n">
-        <v>80.77</v>
+        <v>91.56999999999999</v>
       </c>
       <c r="F101" s="2" t="n">
-        <v>84.27</v>
+        <v>92.33</v>
       </c>
       <c r="G101" s="2" t="n">
-        <v>91.91</v>
+        <v>99.18000000000001</v>
       </c>
       <c r="H101" s="2" t="n">
-        <v>82.48</v>
+        <v>91.95</v>
       </c>
       <c r="I101" s="2" t="n">
-        <v>70.19</v>
+        <v>85.09999999999999</v>
       </c>
       <c r="J101" s="2" t="n">
-        <v>77.23</v>
+        <v>91.52</v>
       </c>
       <c r="K101" s="2" t="n">
         <v>11.754</v>
@@ -5857,26 +5859,26 @@
       <c r="C102" t="inlineStr"/>
       <c r="D102" t="inlineStr">
         <is>
-          <t>WHU-CD-256</t>
+          <t>SYSU-CD-256</t>
         </is>
       </c>
       <c r="E102" s="2" t="n">
-        <v>93.62</v>
+        <v>80.77</v>
       </c>
       <c r="F102" s="2" t="n">
-        <v>96.09</v>
+        <v>84.27</v>
       </c>
       <c r="G102" s="2" t="n">
-        <v>99.59999999999999</v>
+        <v>91.91</v>
       </c>
       <c r="H102" s="2" t="n">
-        <v>94.84</v>
+        <v>82.48</v>
       </c>
       <c r="I102" s="2" t="n">
-        <v>90.18000000000001</v>
+        <v>70.19</v>
       </c>
       <c r="J102" s="2" t="n">
-        <v>94.63</v>
+        <v>77.23</v>
       </c>
       <c r="K102" s="2" t="n">
         <v>11.754</v>
@@ -5893,8 +5895,58 @@
         </is>
       </c>
     </row>
+    <row r="103">
+      <c r="A103" t="inlineStr">
+        <is>
+          <t>baseline</t>
+        </is>
+      </c>
+      <c r="B103" t="inlineStr">
+        <is>
+          <t>Run1</t>
+        </is>
+      </c>
+      <c r="C103" t="inlineStr"/>
+      <c r="D103" t="inlineStr">
+        <is>
+          <t>WHU-CD-256</t>
+        </is>
+      </c>
+      <c r="E103" s="2" t="n">
+        <v>93.62</v>
+      </c>
+      <c r="F103" s="2" t="n">
+        <v>96.09</v>
+      </c>
+      <c r="G103" s="2" t="n">
+        <v>99.59999999999999</v>
+      </c>
+      <c r="H103" s="2" t="n">
+        <v>94.84</v>
+      </c>
+      <c r="I103" s="2" t="n">
+        <v>90.18000000000001</v>
+      </c>
+      <c r="J103" s="2" t="n">
+        <v>94.63</v>
+      </c>
+      <c r="K103" s="2" t="n">
+        <v>11.754</v>
+      </c>
+      <c r="L103" s="2" t="n">
+        <v>20.661</v>
+      </c>
+      <c r="M103" s="2" t="n">
+        <v>26.3246</v>
+      </c>
+      <c r="N103" t="inlineStr">
+        <is>
+          <t>baseline</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:N102"/>
+  <autoFilter ref="A1:N103"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Record SYSU hyperbolic QKV test and training diagnostics
</commit_message>
<xml_diff>
--- a/docs/experiment_metrics.xlsx
+++ b/docs/experiment_metrics.xlsx
@@ -10,7 +10,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="metrics" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'metrics'!$A$1:$N$103</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'metrics'!$A$1:$N$104</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -420,7 +420,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N103"/>
+  <dimension ref="A1:N104"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -4560,54 +4560,52 @@
     <row r="78">
       <c r="A78" t="inlineStr">
         <is>
-          <t>CASAA</t>
+          <t>CASA-WDMF</t>
         </is>
       </c>
       <c r="B78" t="inlineStr">
         <is>
-          <t>Run1</t>
+          <t>Run2</t>
         </is>
       </c>
       <c r="C78" t="inlineStr">
         <is>
-          <t>A1_SAA</t>
+          <t>M1_HYPER_QKV</t>
         </is>
       </c>
       <c r="D78" t="inlineStr">
         <is>
-          <t>LEVIR-CD-256</t>
+          <t>SYSU-CD-256</t>
         </is>
       </c>
       <c r="E78" s="2" t="n">
-        <v>91.09</v>
+        <v>78.67</v>
       </c>
       <c r="F78" s="2" t="n">
-        <v>92.8</v>
+        <v>85.08</v>
       </c>
       <c r="G78" s="2" t="n">
-        <v>99.19</v>
+        <v>91.72</v>
       </c>
       <c r="H78" s="2" t="n">
-        <v>91.94</v>
+        <v>81.75</v>
       </c>
       <c r="I78" s="2" t="n">
-        <v>85.08</v>
+        <v>69.13</v>
       </c>
       <c r="J78" s="2" t="n">
-        <v>91.51000000000001</v>
+        <v>76.40000000000001</v>
       </c>
       <c r="K78" s="2" t="n">
-        <v>11.754</v>
+        <v>3.049509</v>
       </c>
       <c r="L78" s="2" t="n">
-        <v>20.661</v>
-      </c>
-      <c r="M78" s="2" t="n">
-        <v>26.3183</v>
-      </c>
+        <v>3.133176</v>
+      </c>
+      <c r="M78" s="2" t="n"/>
       <c r="N78" t="inlineStr">
         <is>
-          <t>saa</t>
+          <t>casa_wdmf_str_hyperbolic</t>
         </is>
       </c>
     </row>
@@ -4629,26 +4627,26 @@
       </c>
       <c r="D79" t="inlineStr">
         <is>
-          <t>SYSU-CD-256</t>
+          <t>LEVIR-CD-256</t>
         </is>
       </c>
       <c r="E79" s="2" t="n">
-        <v>80.3</v>
+        <v>91.09</v>
       </c>
       <c r="F79" s="2" t="n">
-        <v>84.81</v>
+        <v>92.8</v>
       </c>
       <c r="G79" s="2" t="n">
-        <v>91.95999999999999</v>
+        <v>99.19</v>
       </c>
       <c r="H79" s="2" t="n">
-        <v>82.5</v>
+        <v>91.94</v>
       </c>
       <c r="I79" s="2" t="n">
-        <v>70.20999999999999</v>
+        <v>85.08</v>
       </c>
       <c r="J79" s="2" t="n">
-        <v>77.29000000000001</v>
+        <v>91.51000000000001</v>
       </c>
       <c r="K79" s="2" t="n">
         <v>11.754</v>
@@ -4678,31 +4676,31 @@
       </c>
       <c r="C80" t="inlineStr">
         <is>
-          <t>A2_CASAA</t>
+          <t>A1_SAA</t>
         </is>
       </c>
       <c r="D80" t="inlineStr">
         <is>
-          <t>LEVIR-CD-256</t>
+          <t>SYSU-CD-256</t>
         </is>
       </c>
       <c r="E80" s="2" t="n">
-        <v>90.98999999999999</v>
+        <v>80.3</v>
       </c>
       <c r="F80" s="2" t="n">
-        <v>92.75</v>
+        <v>84.81</v>
       </c>
       <c r="G80" s="2" t="n">
-        <v>99.18000000000001</v>
+        <v>91.95999999999999</v>
       </c>
       <c r="H80" s="2" t="n">
-        <v>91.86</v>
+        <v>82.5</v>
       </c>
       <c r="I80" s="2" t="n">
-        <v>84.94</v>
+        <v>70.20999999999999</v>
       </c>
       <c r="J80" s="2" t="n">
-        <v>91.43000000000001</v>
+        <v>77.29000000000001</v>
       </c>
       <c r="K80" s="2" t="n">
         <v>11.754</v>
@@ -4711,11 +4709,11 @@
         <v>20.661</v>
       </c>
       <c r="M80" s="2" t="n">
-        <v>26.2593</v>
+        <v>26.3183</v>
       </c>
       <c r="N80" t="inlineStr">
         <is>
-          <t>casaa</t>
+          <t>saa</t>
         </is>
       </c>
     </row>
@@ -4737,26 +4735,26 @@
       </c>
       <c r="D81" t="inlineStr">
         <is>
-          <t>SYSU-CD-256</t>
+          <t>LEVIR-CD-256</t>
         </is>
       </c>
       <c r="E81" s="2" t="n">
-        <v>80.55</v>
+        <v>90.98999999999999</v>
       </c>
       <c r="F81" s="2" t="n">
-        <v>84.23</v>
+        <v>92.75</v>
       </c>
       <c r="G81" s="2" t="n">
+        <v>99.18000000000001</v>
+      </c>
+      <c r="H81" s="2" t="n">
         <v>91.86</v>
       </c>
-      <c r="H81" s="2" t="n">
-        <v>82.34999999999999</v>
-      </c>
       <c r="I81" s="2" t="n">
-        <v>70</v>
+        <v>84.94</v>
       </c>
       <c r="J81" s="2" t="n">
-        <v>77.06</v>
+        <v>91.43000000000001</v>
       </c>
       <c r="K81" s="2" t="n">
         <v>11.754</v>
@@ -4781,49 +4779,49 @@
       </c>
       <c r="B82" t="inlineStr">
         <is>
-          <t>Run2</t>
+          <t>Run1</t>
         </is>
       </c>
       <c r="C82" t="inlineStr">
         <is>
-          <t>A1_SAA_FROZEN</t>
+          <t>A2_CASAA</t>
         </is>
       </c>
       <c r="D82" t="inlineStr">
         <is>
-          <t>LEVIR-CD-256</t>
+          <t>SYSU-CD-256</t>
         </is>
       </c>
       <c r="E82" s="2" t="n">
-        <v>91.38</v>
+        <v>80.55</v>
       </c>
       <c r="F82" s="2" t="n">
-        <v>92.3</v>
+        <v>84.23</v>
       </c>
       <c r="G82" s="2" t="n">
-        <v>99.17</v>
+        <v>91.86</v>
       </c>
       <c r="H82" s="2" t="n">
-        <v>91.84</v>
+        <v>82.34999999999999</v>
       </c>
       <c r="I82" s="2" t="n">
-        <v>84.91</v>
+        <v>70</v>
       </c>
       <c r="J82" s="2" t="n">
-        <v>91.40000000000001</v>
+        <v>77.06</v>
       </c>
       <c r="K82" s="2" t="n">
         <v>11.754</v>
       </c>
       <c r="L82" s="2" t="n">
-        <v>15.125</v>
+        <v>20.661</v>
       </c>
       <c r="M82" s="2" t="n">
-        <v>26.1484</v>
+        <v>26.2593</v>
       </c>
       <c r="N82" t="inlineStr">
         <is>
-          <t>saa</t>
+          <t>casaa</t>
         </is>
       </c>
     </row>
@@ -4845,26 +4843,26 @@
       </c>
       <c r="D83" t="inlineStr">
         <is>
-          <t>SYSU-CD-256</t>
+          <t>LEVIR-CD-256</t>
         </is>
       </c>
       <c r="E83" s="2" t="n">
-        <v>78.40000000000001</v>
+        <v>91.38</v>
       </c>
       <c r="F83" s="2" t="n">
-        <v>86.03</v>
+        <v>92.3</v>
       </c>
       <c r="G83" s="2" t="n">
-        <v>91.90000000000001</v>
+        <v>99.17</v>
       </c>
       <c r="H83" s="2" t="n">
-        <v>82.04000000000001</v>
+        <v>91.84</v>
       </c>
       <c r="I83" s="2" t="n">
-        <v>69.55</v>
+        <v>84.91</v>
       </c>
       <c r="J83" s="2" t="n">
-        <v>76.83</v>
+        <v>91.40000000000001</v>
       </c>
       <c r="K83" s="2" t="n">
         <v>11.754</v>
@@ -4894,31 +4892,31 @@
       </c>
       <c r="C84" t="inlineStr">
         <is>
-          <t>A3_ORACLE_FROZEN</t>
+          <t>A1_SAA_FROZEN</t>
         </is>
       </c>
       <c r="D84" t="inlineStr">
         <is>
-          <t>LEVIR-CD-256</t>
+          <t>SYSU-CD-256</t>
         </is>
       </c>
       <c r="E84" s="2" t="n">
-        <v>91.13</v>
+        <v>78.40000000000001</v>
       </c>
       <c r="F84" s="2" t="n">
-        <v>92.65000000000001</v>
+        <v>86.03</v>
       </c>
       <c r="G84" s="2" t="n">
-        <v>99.18000000000001</v>
+        <v>91.90000000000001</v>
       </c>
       <c r="H84" s="2" t="n">
-        <v>91.88</v>
+        <v>82.04000000000001</v>
       </c>
       <c r="I84" s="2" t="n">
-        <v>84.98</v>
+        <v>69.55</v>
       </c>
       <c r="J84" s="2" t="n">
-        <v>91.45</v>
+        <v>76.83</v>
       </c>
       <c r="K84" s="2" t="n">
         <v>11.754</v>
@@ -4927,11 +4925,11 @@
         <v>15.125</v>
       </c>
       <c r="M84" s="2" t="n">
-        <v>26.0894</v>
+        <v>26.1484</v>
       </c>
       <c r="N84" t="inlineStr">
         <is>
-          <t>casaa</t>
+          <t>saa</t>
         </is>
       </c>
     </row>
@@ -4953,26 +4951,26 @@
       </c>
       <c r="D85" t="inlineStr">
         <is>
-          <t>SYSU-CD-256</t>
+          <t>LEVIR-CD-256</t>
         </is>
       </c>
       <c r="E85" s="2" t="n">
-        <v>82.04000000000001</v>
+        <v>91.13</v>
       </c>
       <c r="F85" s="2" t="n">
-        <v>85.05</v>
+        <v>92.65000000000001</v>
       </c>
       <c r="G85" s="2" t="n">
-        <v>92.36</v>
+        <v>99.18000000000001</v>
       </c>
       <c r="H85" s="2" t="n">
-        <v>83.52</v>
+        <v>91.88</v>
       </c>
       <c r="I85" s="2" t="n">
-        <v>71.7</v>
+        <v>84.98</v>
       </c>
       <c r="J85" s="2" t="n">
-        <v>78.55</v>
+        <v>91.45</v>
       </c>
       <c r="K85" s="2" t="n">
         <v>11.754</v>
@@ -4997,12 +4995,12 @@
       </c>
       <c r="B86" t="inlineStr">
         <is>
-          <t>Run3</t>
+          <t>Run2</t>
         </is>
       </c>
       <c r="C86" t="inlineStr">
         <is>
-          <t>A4_DETAIL_FROZEN</t>
+          <t>A3_ORACLE_FROZEN</t>
         </is>
       </c>
       <c r="D86" t="inlineStr">
@@ -5011,22 +5009,22 @@
         </is>
       </c>
       <c r="E86" s="2" t="n">
-        <v>79.68000000000001</v>
+        <v>82.04000000000001</v>
       </c>
       <c r="F86" s="2" t="n">
-        <v>84.28</v>
+        <v>85.05</v>
       </c>
       <c r="G86" s="2" t="n">
-        <v>91.7</v>
+        <v>92.36</v>
       </c>
       <c r="H86" s="2" t="n">
-        <v>81.92</v>
+        <v>83.52</v>
       </c>
       <c r="I86" s="2" t="n">
-        <v>69.37</v>
+        <v>71.7</v>
       </c>
       <c r="J86" s="2" t="n">
-        <v>76.54000000000001</v>
+        <v>78.55</v>
       </c>
       <c r="K86" s="2" t="n">
         <v>11.754</v>
@@ -5046,54 +5044,54 @@
     <row r="87">
       <c r="A87" t="inlineStr">
         <is>
-          <t>STR-Fusion</t>
+          <t>CASAA</t>
         </is>
       </c>
       <c r="B87" t="inlineStr">
         <is>
-          <t>Run2_TASS</t>
+          <t>Run3</t>
         </is>
       </c>
       <c r="C87" t="inlineStr">
         <is>
-          <t>C0_TOKEN</t>
+          <t>A4_DETAIL_FROZEN</t>
         </is>
       </c>
       <c r="D87" t="inlineStr">
         <is>
-          <t>CDD-CD-256</t>
+          <t>SYSU-CD-256</t>
         </is>
       </c>
       <c r="E87" s="2" t="n">
-        <v>93.13</v>
+        <v>79.68000000000001</v>
       </c>
       <c r="F87" s="2" t="n">
-        <v>95.16</v>
+        <v>84.28</v>
       </c>
       <c r="G87" s="2" t="n">
-        <v>98.56999999999999</v>
+        <v>91.7</v>
       </c>
       <c r="H87" s="2" t="n">
-        <v>94.13</v>
+        <v>81.92</v>
       </c>
       <c r="I87" s="2" t="n">
-        <v>88.91</v>
+        <v>69.37</v>
       </c>
       <c r="J87" s="2" t="n">
-        <v>93.31999999999999</v>
+        <v>76.54000000000001</v>
       </c>
       <c r="K87" s="2" t="n">
-        <v>2.596</v>
+        <v>11.754</v>
       </c>
       <c r="L87" s="2" t="n">
-        <v>0.62</v>
+        <v>15.125</v>
       </c>
       <c r="M87" s="2" t="n">
-        <v>2.2136</v>
+        <v>26.0894</v>
       </c>
       <c r="N87" t="inlineStr">
         <is>
-          <t>str_tass</t>
+          <t>casaa</t>
         </is>
       </c>
     </row>
@@ -5115,26 +5113,26 @@
       </c>
       <c r="D88" t="inlineStr">
         <is>
-          <t>LEVIR-CD-256</t>
+          <t>CDD-CD-256</t>
         </is>
       </c>
       <c r="E88" s="2" t="n">
-        <v>86.37</v>
+        <v>93.13</v>
       </c>
       <c r="F88" s="2" t="n">
-        <v>89.25</v>
+        <v>95.16</v>
       </c>
       <c r="G88" s="2" t="n">
-        <v>98.78</v>
+        <v>98.56999999999999</v>
       </c>
       <c r="H88" s="2" t="n">
-        <v>87.79000000000001</v>
+        <v>94.13</v>
       </c>
       <c r="I88" s="2" t="n">
-        <v>78.23999999999999</v>
+        <v>88.91</v>
       </c>
       <c r="J88" s="2" t="n">
-        <v>87.14</v>
+        <v>93.31999999999999</v>
       </c>
       <c r="K88" s="2" t="n">
         <v>2.596</v>
@@ -5169,26 +5167,26 @@
       </c>
       <c r="D89" t="inlineStr">
         <is>
-          <t>SYSU-CD-256</t>
+          <t>LEVIR-CD-256</t>
         </is>
       </c>
       <c r="E89" s="2" t="n">
-        <v>79.93000000000001</v>
+        <v>86.37</v>
       </c>
       <c r="F89" s="2" t="n">
-        <v>84.5</v>
+        <v>89.25</v>
       </c>
       <c r="G89" s="2" t="n">
-        <v>91.81</v>
+        <v>98.78</v>
       </c>
       <c r="H89" s="2" t="n">
-        <v>82.15000000000001</v>
+        <v>87.79000000000001</v>
       </c>
       <c r="I89" s="2" t="n">
-        <v>69.70999999999999</v>
+        <v>78.23999999999999</v>
       </c>
       <c r="J89" s="2" t="n">
-        <v>76.84</v>
+        <v>87.14</v>
       </c>
       <c r="K89" s="2" t="n">
         <v>2.596</v>
@@ -5223,26 +5221,26 @@
       </c>
       <c r="D90" t="inlineStr">
         <is>
-          <t>WHU-CD-256</t>
+          <t>SYSU-CD-256</t>
         </is>
       </c>
       <c r="E90" s="2" t="n">
-        <v>90.16</v>
+        <v>79.93000000000001</v>
       </c>
       <c r="F90" s="2" t="n">
-        <v>93.97</v>
+        <v>84.5</v>
       </c>
       <c r="G90" s="2" t="n">
-        <v>99.38</v>
+        <v>91.81</v>
       </c>
       <c r="H90" s="2" t="n">
-        <v>92.02</v>
+        <v>82.15000000000001</v>
       </c>
       <c r="I90" s="2" t="n">
-        <v>85.23</v>
+        <v>69.70999999999999</v>
       </c>
       <c r="J90" s="2" t="n">
-        <v>91.7</v>
+        <v>76.84</v>
       </c>
       <c r="K90" s="2" t="n">
         <v>2.596</v>
@@ -5272,40 +5270,40 @@
       </c>
       <c r="C91" t="inlineStr">
         <is>
-          <t>M1_TASS</t>
+          <t>C0_TOKEN</t>
         </is>
       </c>
       <c r="D91" t="inlineStr">
         <is>
-          <t>CDD-CD-256</t>
+          <t>WHU-CD-256</t>
         </is>
       </c>
       <c r="E91" s="2" t="n">
-        <v>94.7</v>
+        <v>90.16</v>
       </c>
       <c r="F91" s="2" t="n">
-        <v>96.13</v>
+        <v>93.97</v>
       </c>
       <c r="G91" s="2" t="n">
-        <v>98.88</v>
+        <v>99.38</v>
       </c>
       <c r="H91" s="2" t="n">
-        <v>95.41</v>
+        <v>92.02</v>
       </c>
       <c r="I91" s="2" t="n">
-        <v>91.22</v>
+        <v>85.23</v>
       </c>
       <c r="J91" s="2" t="n">
-        <v>94.77</v>
+        <v>91.7</v>
       </c>
       <c r="K91" s="2" t="n">
-        <v>3.455</v>
+        <v>2.596</v>
       </c>
       <c r="L91" s="2" t="n">
-        <v>1.478</v>
+        <v>0.62</v>
       </c>
       <c r="M91" s="2" t="n">
-        <v>3.5459</v>
+        <v>2.2136</v>
       </c>
       <c r="N91" t="inlineStr">
         <is>
@@ -5331,26 +5329,26 @@
       </c>
       <c r="D92" t="inlineStr">
         <is>
-          <t>LEVIR-CD-256</t>
+          <t>CDD-CD-256</t>
         </is>
       </c>
       <c r="E92" s="2" t="n">
-        <v>88.42</v>
+        <v>94.7</v>
       </c>
       <c r="F92" s="2" t="n">
-        <v>91.97</v>
+        <v>96.13</v>
       </c>
       <c r="G92" s="2" t="n">
-        <v>99.02</v>
+        <v>98.88</v>
       </c>
       <c r="H92" s="2" t="n">
-        <v>90.16</v>
+        <v>95.41</v>
       </c>
       <c r="I92" s="2" t="n">
-        <v>82.08</v>
+        <v>91.22</v>
       </c>
       <c r="J92" s="2" t="n">
-        <v>89.64</v>
+        <v>94.77</v>
       </c>
       <c r="K92" s="2" t="n">
         <v>3.455</v>
@@ -5385,26 +5383,26 @@
       </c>
       <c r="D93" t="inlineStr">
         <is>
-          <t>SYSU-CD-256</t>
+          <t>LEVIR-CD-256</t>
         </is>
       </c>
       <c r="E93" s="2" t="n">
-        <v>78.73</v>
+        <v>88.42</v>
       </c>
       <c r="F93" s="2" t="n">
-        <v>84.98</v>
+        <v>91.97</v>
       </c>
       <c r="G93" s="2" t="n">
-        <v>91.7</v>
+        <v>99.02</v>
       </c>
       <c r="H93" s="2" t="n">
-        <v>81.73999999999999</v>
+        <v>90.16</v>
       </c>
       <c r="I93" s="2" t="n">
-        <v>69.11</v>
+        <v>82.08</v>
       </c>
       <c r="J93" s="2" t="n">
-        <v>76.38</v>
+        <v>89.64</v>
       </c>
       <c r="K93" s="2" t="n">
         <v>3.455</v>
@@ -5439,26 +5437,26 @@
       </c>
       <c r="D94" t="inlineStr">
         <is>
-          <t>WHU-CD-256</t>
+          <t>SYSU-CD-256</t>
         </is>
       </c>
       <c r="E94" s="2" t="n">
-        <v>91.64</v>
+        <v>78.73</v>
       </c>
       <c r="F94" s="2" t="n">
-        <v>94.81999999999999</v>
+        <v>84.98</v>
       </c>
       <c r="G94" s="2" t="n">
-        <v>99.47</v>
+        <v>91.7</v>
       </c>
       <c r="H94" s="2" t="n">
-        <v>93.2</v>
+        <v>81.73999999999999</v>
       </c>
       <c r="I94" s="2" t="n">
-        <v>87.27</v>
+        <v>69.11</v>
       </c>
       <c r="J94" s="2" t="n">
-        <v>92.93000000000001</v>
+        <v>76.38</v>
       </c>
       <c r="K94" s="2" t="n">
         <v>3.455</v>
@@ -5478,54 +5476,54 @@
     <row r="95">
       <c r="A95" t="inlineStr">
         <is>
-          <t>UltraLight</t>
+          <t>STR-Fusion</t>
         </is>
       </c>
       <c r="B95" t="inlineStr">
         <is>
-          <t>Run4</t>
+          <t>Run2_TASS</t>
         </is>
       </c>
       <c r="C95" t="inlineStr">
         <is>
-          <t>R4_0_A0_FULL12_FROZEN</t>
+          <t>M1_TASS</t>
         </is>
       </c>
       <c r="D95" t="inlineStr">
         <is>
-          <t>SYSU-CD-256</t>
+          <t>WHU-CD-256</t>
         </is>
       </c>
       <c r="E95" s="2" t="n">
-        <v>82.42</v>
+        <v>91.64</v>
       </c>
       <c r="F95" s="2" t="n">
-        <v>83.87</v>
+        <v>94.81999999999999</v>
       </c>
       <c r="G95" s="2" t="n">
-        <v>92.12</v>
+        <v>99.47</v>
       </c>
       <c r="H95" s="2" t="n">
-        <v>83.14</v>
+        <v>93.2</v>
       </c>
       <c r="I95" s="2" t="n">
-        <v>71.14</v>
+        <v>87.27</v>
       </c>
       <c r="J95" s="2" t="n">
-        <v>77.98999999999999</v>
+        <v>92.93000000000001</v>
       </c>
       <c r="K95" s="2" t="n">
-        <v>11.754</v>
+        <v>3.455</v>
       </c>
       <c r="L95" s="2" t="n">
-        <v>15.125</v>
+        <v>1.478</v>
       </c>
       <c r="M95" s="2" t="n">
-        <v>26.3246</v>
+        <v>3.5459</v>
       </c>
       <c r="N95" t="inlineStr">
         <is>
-          <t>baseline</t>
+          <t>str_tass</t>
         </is>
       </c>
     </row>
@@ -5542,7 +5540,7 @@
       </c>
       <c r="C96" t="inlineStr">
         <is>
-          <t>R4_1_VIT4_OLDHEAD</t>
+          <t>R4_0_A0_FULL12_FROZEN</t>
         </is>
       </c>
       <c r="D96" t="inlineStr">
@@ -5551,31 +5549,31 @@
         </is>
       </c>
       <c r="E96" s="2" t="n">
-        <v>82.15000000000001</v>
+        <v>82.42</v>
       </c>
       <c r="F96" s="2" t="n">
-        <v>83.40000000000001</v>
+        <v>83.87</v>
       </c>
       <c r="G96" s="2" t="n">
-        <v>91.94</v>
+        <v>92.12</v>
       </c>
       <c r="H96" s="2" t="n">
-        <v>82.77</v>
+        <v>83.14</v>
       </c>
       <c r="I96" s="2" t="n">
-        <v>70.61</v>
+        <v>71.14</v>
       </c>
       <c r="J96" s="2" t="n">
-        <v>77.51000000000001</v>
+        <v>77.98999999999999</v>
       </c>
       <c r="K96" s="2" t="n">
-        <v>8.195</v>
+        <v>11.754</v>
       </c>
       <c r="L96" s="2" t="n">
         <v>15.125</v>
       </c>
       <c r="M96" s="2" t="n">
-        <v>24.1021</v>
+        <v>26.3246</v>
       </c>
       <c r="N96" t="inlineStr">
         <is>
@@ -5596,7 +5594,7 @@
       </c>
       <c r="C97" t="inlineStr">
         <is>
-          <t>R4_2_VIT4_LIGHTDETAIL</t>
+          <t>R4_1_VIT4_OLDHEAD</t>
         </is>
       </c>
       <c r="D97" t="inlineStr">
@@ -5605,31 +5603,31 @@
         </is>
       </c>
       <c r="E97" s="2" t="n">
-        <v>79.94</v>
+        <v>82.15000000000001</v>
       </c>
       <c r="F97" s="2" t="n">
-        <v>84.79000000000001</v>
+        <v>83.40000000000001</v>
       </c>
       <c r="G97" s="2" t="n">
-        <v>91.89</v>
+        <v>91.94</v>
       </c>
       <c r="H97" s="2" t="n">
-        <v>82.3</v>
+        <v>82.77</v>
       </c>
       <c r="I97" s="2" t="n">
-        <v>69.92</v>
+        <v>70.61</v>
       </c>
       <c r="J97" s="2" t="n">
-        <v>77.04000000000001</v>
+        <v>77.51000000000001</v>
       </c>
       <c r="K97" s="2" t="n">
-        <v>5.492</v>
+        <v>8.195</v>
       </c>
       <c r="L97" s="2" t="n">
-        <v>3.515</v>
+        <v>15.125</v>
       </c>
       <c r="M97" s="2" t="n">
-        <v>10.7311</v>
+        <v>24.1021</v>
       </c>
       <c r="N97" t="inlineStr">
         <is>
@@ -5650,7 +5648,7 @@
       </c>
       <c r="C98" t="inlineStr">
         <is>
-          <t>R4_2b_VIT4_LIGHTDETAIL48</t>
+          <t>R4_2_VIT4_LIGHTDETAIL</t>
         </is>
       </c>
       <c r="D98" t="inlineStr">
@@ -5659,31 +5657,31 @@
         </is>
       </c>
       <c r="E98" s="2" t="n">
-        <v>80.87</v>
+        <v>79.94</v>
       </c>
       <c r="F98" s="2" t="n">
-        <v>83.81</v>
+        <v>84.79000000000001</v>
       </c>
       <c r="G98" s="2" t="n">
-        <v>91.81</v>
+        <v>91.89</v>
       </c>
       <c r="H98" s="2" t="n">
-        <v>82.31999999999999</v>
+        <v>82.3</v>
       </c>
       <c r="I98" s="2" t="n">
-        <v>69.95</v>
+        <v>69.92</v>
       </c>
       <c r="J98" s="2" t="n">
-        <v>76.98999999999999</v>
+        <v>77.04000000000001</v>
       </c>
       <c r="K98" s="2" t="n">
-        <v>5.533</v>
+        <v>5.492</v>
       </c>
       <c r="L98" s="2" t="n">
-        <v>3.556</v>
+        <v>3.515</v>
       </c>
       <c r="M98" s="2" t="n">
-        <v>10.9824</v>
+        <v>10.7311</v>
       </c>
       <c r="N98" t="inlineStr">
         <is>
@@ -5704,7 +5702,7 @@
       </c>
       <c r="C99" t="inlineStr">
         <is>
-          <t>R4_2d_PSD_DETAIL</t>
+          <t>R4_2b_VIT4_LIGHTDETAIL48</t>
         </is>
       </c>
       <c r="D99" t="inlineStr">
@@ -5713,31 +5711,31 @@
         </is>
       </c>
       <c r="E99" s="2" t="n">
-        <v>79.78</v>
+        <v>80.87</v>
       </c>
       <c r="F99" s="2" t="n">
-        <v>84.39</v>
+        <v>83.81</v>
       </c>
       <c r="G99" s="2" t="n">
-        <v>91.75</v>
+        <v>91.81</v>
       </c>
       <c r="H99" s="2" t="n">
-        <v>82.02</v>
+        <v>82.31999999999999</v>
       </c>
       <c r="I99" s="2" t="n">
-        <v>69.52</v>
+        <v>69.95</v>
       </c>
       <c r="J99" s="2" t="n">
-        <v>76.68000000000001</v>
+        <v>76.98999999999999</v>
       </c>
       <c r="K99" s="2" t="n">
-        <v>5.491</v>
+        <v>5.533</v>
       </c>
       <c r="L99" s="2" t="n">
-        <v>3.514</v>
+        <v>3.556</v>
       </c>
       <c r="M99" s="2" t="n">
-        <v>11.5239</v>
+        <v>10.9824</v>
       </c>
       <c r="N99" t="inlineStr">
         <is>
@@ -5748,46 +5746,50 @@
     <row r="100">
       <c r="A100" t="inlineStr">
         <is>
-          <t>baseline</t>
+          <t>UltraLight</t>
         </is>
       </c>
       <c r="B100" t="inlineStr">
         <is>
-          <t>Run1</t>
-        </is>
-      </c>
-      <c r="C100" t="inlineStr"/>
+          <t>Run4</t>
+        </is>
+      </c>
+      <c r="C100" t="inlineStr">
+        <is>
+          <t>R4_2d_PSD_DETAIL</t>
+        </is>
+      </c>
       <c r="D100" t="inlineStr">
         <is>
-          <t>CDD-CD-256</t>
+          <t>SYSU-CD-256</t>
         </is>
       </c>
       <c r="E100" s="2" t="n">
-        <v>97.72</v>
+        <v>79.78</v>
       </c>
       <c r="F100" s="2" t="n">
-        <v>97.78</v>
+        <v>84.39</v>
       </c>
       <c r="G100" s="2" t="n">
-        <v>99.44</v>
+        <v>91.75</v>
       </c>
       <c r="H100" s="2" t="n">
-        <v>97.75</v>
+        <v>82.02</v>
       </c>
       <c r="I100" s="2" t="n">
-        <v>95.59999999999999</v>
+        <v>69.52</v>
       </c>
       <c r="J100" s="2" t="n">
-        <v>97.43000000000001</v>
+        <v>76.68000000000001</v>
       </c>
       <c r="K100" s="2" t="n">
-        <v>11.754</v>
+        <v>5.491</v>
       </c>
       <c r="L100" s="2" t="n">
-        <v>20.661</v>
+        <v>3.514</v>
       </c>
       <c r="M100" s="2" t="n">
-        <v>26.3246</v>
+        <v>11.5239</v>
       </c>
       <c r="N100" t="inlineStr">
         <is>
@@ -5809,26 +5811,26 @@
       <c r="C101" t="inlineStr"/>
       <c r="D101" t="inlineStr">
         <is>
-          <t>LEVIR-CD-256</t>
+          <t>CDD-CD-256</t>
         </is>
       </c>
       <c r="E101" s="2" t="n">
-        <v>91.56999999999999</v>
+        <v>97.72</v>
       </c>
       <c r="F101" s="2" t="n">
-        <v>92.33</v>
+        <v>97.78</v>
       </c>
       <c r="G101" s="2" t="n">
-        <v>99.18000000000001</v>
+        <v>99.44</v>
       </c>
       <c r="H101" s="2" t="n">
-        <v>91.95</v>
+        <v>97.75</v>
       </c>
       <c r="I101" s="2" t="n">
-        <v>85.09999999999999</v>
+        <v>95.59999999999999</v>
       </c>
       <c r="J101" s="2" t="n">
-        <v>91.52</v>
+        <v>97.43000000000001</v>
       </c>
       <c r="K101" s="2" t="n">
         <v>11.754</v>
@@ -5859,26 +5861,26 @@
       <c r="C102" t="inlineStr"/>
       <c r="D102" t="inlineStr">
         <is>
-          <t>SYSU-CD-256</t>
+          <t>LEVIR-CD-256</t>
         </is>
       </c>
       <c r="E102" s="2" t="n">
-        <v>80.77</v>
+        <v>91.56999999999999</v>
       </c>
       <c r="F102" s="2" t="n">
-        <v>84.27</v>
+        <v>92.33</v>
       </c>
       <c r="G102" s="2" t="n">
-        <v>91.91</v>
+        <v>99.18000000000001</v>
       </c>
       <c r="H102" s="2" t="n">
-        <v>82.48</v>
+        <v>91.95</v>
       </c>
       <c r="I102" s="2" t="n">
-        <v>70.19</v>
+        <v>85.09999999999999</v>
       </c>
       <c r="J102" s="2" t="n">
-        <v>77.23</v>
+        <v>91.52</v>
       </c>
       <c r="K102" s="2" t="n">
         <v>11.754</v>
@@ -5909,26 +5911,26 @@
       <c r="C103" t="inlineStr"/>
       <c r="D103" t="inlineStr">
         <is>
-          <t>WHU-CD-256</t>
+          <t>SYSU-CD-256</t>
         </is>
       </c>
       <c r="E103" s="2" t="n">
-        <v>93.62</v>
+        <v>80.77</v>
       </c>
       <c r="F103" s="2" t="n">
-        <v>96.09</v>
+        <v>84.27</v>
       </c>
       <c r="G103" s="2" t="n">
-        <v>99.59999999999999</v>
+        <v>91.91</v>
       </c>
       <c r="H103" s="2" t="n">
-        <v>94.84</v>
+        <v>82.48</v>
       </c>
       <c r="I103" s="2" t="n">
-        <v>90.18000000000001</v>
+        <v>70.19</v>
       </c>
       <c r="J103" s="2" t="n">
-        <v>94.63</v>
+        <v>77.23</v>
       </c>
       <c r="K103" s="2" t="n">
         <v>11.754</v>
@@ -5945,8 +5947,58 @@
         </is>
       </c>
     </row>
+    <row r="104">
+      <c r="A104" t="inlineStr">
+        <is>
+          <t>baseline</t>
+        </is>
+      </c>
+      <c r="B104" t="inlineStr">
+        <is>
+          <t>Run1</t>
+        </is>
+      </c>
+      <c r="C104" t="inlineStr"/>
+      <c r="D104" t="inlineStr">
+        <is>
+          <t>WHU-CD-256</t>
+        </is>
+      </c>
+      <c r="E104" s="2" t="n">
+        <v>93.62</v>
+      </c>
+      <c r="F104" s="2" t="n">
+        <v>96.09</v>
+      </c>
+      <c r="G104" s="2" t="n">
+        <v>99.59999999999999</v>
+      </c>
+      <c r="H104" s="2" t="n">
+        <v>94.84</v>
+      </c>
+      <c r="I104" s="2" t="n">
+        <v>90.18000000000001</v>
+      </c>
+      <c r="J104" s="2" t="n">
+        <v>94.63</v>
+      </c>
+      <c r="K104" s="2" t="n">
+        <v>11.754</v>
+      </c>
+      <c r="L104" s="2" t="n">
+        <v>20.661</v>
+      </c>
+      <c r="M104" s="2" t="n">
+        <v>26.3246</v>
+      </c>
+      <c r="N104" t="inlineStr">
+        <is>
+          <t>baseline</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:N103"/>
+  <autoFilter ref="A1:N104"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Record SYSU change-aware QKV test results
</commit_message>
<xml_diff>
--- a/docs/experiment_metrics.xlsx
+++ b/docs/experiment_metrics.xlsx
@@ -10,7 +10,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="metrics" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'metrics'!$A$1:$N$104</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'metrics'!$A$1:$N$105</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -420,7 +420,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N104"/>
+  <dimension ref="A1:N105"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -4612,54 +4612,52 @@
     <row r="79">
       <c r="A79" t="inlineStr">
         <is>
-          <t>CASAA</t>
+          <t>CASA-WDMF</t>
         </is>
       </c>
       <c r="B79" t="inlineStr">
         <is>
-          <t>Run1</t>
+          <t>Run2</t>
         </is>
       </c>
       <c r="C79" t="inlineStr">
         <is>
-          <t>A1_SAA</t>
+          <t>M2_CA_QKV</t>
         </is>
       </c>
       <c r="D79" t="inlineStr">
         <is>
-          <t>LEVIR-CD-256</t>
+          <t>SYSU-CD-256</t>
         </is>
       </c>
       <c r="E79" s="2" t="n">
-        <v>91.09</v>
+        <v>82.83</v>
       </c>
       <c r="F79" s="2" t="n">
-        <v>92.8</v>
+        <v>82.86</v>
       </c>
       <c r="G79" s="2" t="n">
-        <v>99.19</v>
+        <v>91.91</v>
       </c>
       <c r="H79" s="2" t="n">
-        <v>91.94</v>
+        <v>82.84999999999999</v>
       </c>
       <c r="I79" s="2" t="n">
-        <v>85.08</v>
+        <v>70.72</v>
       </c>
       <c r="J79" s="2" t="n">
-        <v>91.51000000000001</v>
+        <v>77.56</v>
       </c>
       <c r="K79" s="2" t="n">
-        <v>11.754</v>
+        <v>3.049509</v>
       </c>
       <c r="L79" s="2" t="n">
-        <v>20.661</v>
-      </c>
-      <c r="M79" s="2" t="n">
-        <v>26.3183</v>
-      </c>
+        <v>3.133176</v>
+      </c>
+      <c r="M79" s="2" t="n"/>
       <c r="N79" t="inlineStr">
         <is>
-          <t>saa</t>
+          <t>casa_wdmf_str_qkv</t>
         </is>
       </c>
     </row>
@@ -4681,26 +4679,26 @@
       </c>
       <c r="D80" t="inlineStr">
         <is>
-          <t>SYSU-CD-256</t>
+          <t>LEVIR-CD-256</t>
         </is>
       </c>
       <c r="E80" s="2" t="n">
-        <v>80.3</v>
+        <v>91.09</v>
       </c>
       <c r="F80" s="2" t="n">
-        <v>84.81</v>
+        <v>92.8</v>
       </c>
       <c r="G80" s="2" t="n">
-        <v>91.95999999999999</v>
+        <v>99.19</v>
       </c>
       <c r="H80" s="2" t="n">
-        <v>82.5</v>
+        <v>91.94</v>
       </c>
       <c r="I80" s="2" t="n">
-        <v>70.20999999999999</v>
+        <v>85.08</v>
       </c>
       <c r="J80" s="2" t="n">
-        <v>77.29000000000001</v>
+        <v>91.51000000000001</v>
       </c>
       <c r="K80" s="2" t="n">
         <v>11.754</v>
@@ -4730,31 +4728,31 @@
       </c>
       <c r="C81" t="inlineStr">
         <is>
-          <t>A2_CASAA</t>
+          <t>A1_SAA</t>
         </is>
       </c>
       <c r="D81" t="inlineStr">
         <is>
-          <t>LEVIR-CD-256</t>
+          <t>SYSU-CD-256</t>
         </is>
       </c>
       <c r="E81" s="2" t="n">
-        <v>90.98999999999999</v>
+        <v>80.3</v>
       </c>
       <c r="F81" s="2" t="n">
-        <v>92.75</v>
+        <v>84.81</v>
       </c>
       <c r="G81" s="2" t="n">
-        <v>99.18000000000001</v>
+        <v>91.95999999999999</v>
       </c>
       <c r="H81" s="2" t="n">
-        <v>91.86</v>
+        <v>82.5</v>
       </c>
       <c r="I81" s="2" t="n">
-        <v>84.94</v>
+        <v>70.20999999999999</v>
       </c>
       <c r="J81" s="2" t="n">
-        <v>91.43000000000001</v>
+        <v>77.29000000000001</v>
       </c>
       <c r="K81" s="2" t="n">
         <v>11.754</v>
@@ -4763,11 +4761,11 @@
         <v>20.661</v>
       </c>
       <c r="M81" s="2" t="n">
-        <v>26.2593</v>
+        <v>26.3183</v>
       </c>
       <c r="N81" t="inlineStr">
         <is>
-          <t>casaa</t>
+          <t>saa</t>
         </is>
       </c>
     </row>
@@ -4789,26 +4787,26 @@
       </c>
       <c r="D82" t="inlineStr">
         <is>
-          <t>SYSU-CD-256</t>
+          <t>LEVIR-CD-256</t>
         </is>
       </c>
       <c r="E82" s="2" t="n">
-        <v>80.55</v>
+        <v>90.98999999999999</v>
       </c>
       <c r="F82" s="2" t="n">
-        <v>84.23</v>
+        <v>92.75</v>
       </c>
       <c r="G82" s="2" t="n">
+        <v>99.18000000000001</v>
+      </c>
+      <c r="H82" s="2" t="n">
         <v>91.86</v>
       </c>
-      <c r="H82" s="2" t="n">
-        <v>82.34999999999999</v>
-      </c>
       <c r="I82" s="2" t="n">
-        <v>70</v>
+        <v>84.94</v>
       </c>
       <c r="J82" s="2" t="n">
-        <v>77.06</v>
+        <v>91.43000000000001</v>
       </c>
       <c r="K82" s="2" t="n">
         <v>11.754</v>
@@ -4833,49 +4831,49 @@
       </c>
       <c r="B83" t="inlineStr">
         <is>
-          <t>Run2</t>
+          <t>Run1</t>
         </is>
       </c>
       <c r="C83" t="inlineStr">
         <is>
-          <t>A1_SAA_FROZEN</t>
+          <t>A2_CASAA</t>
         </is>
       </c>
       <c r="D83" t="inlineStr">
         <is>
-          <t>LEVIR-CD-256</t>
+          <t>SYSU-CD-256</t>
         </is>
       </c>
       <c r="E83" s="2" t="n">
-        <v>91.38</v>
+        <v>80.55</v>
       </c>
       <c r="F83" s="2" t="n">
-        <v>92.3</v>
+        <v>84.23</v>
       </c>
       <c r="G83" s="2" t="n">
-        <v>99.17</v>
+        <v>91.86</v>
       </c>
       <c r="H83" s="2" t="n">
-        <v>91.84</v>
+        <v>82.34999999999999</v>
       </c>
       <c r="I83" s="2" t="n">
-        <v>84.91</v>
+        <v>70</v>
       </c>
       <c r="J83" s="2" t="n">
-        <v>91.40000000000001</v>
+        <v>77.06</v>
       </c>
       <c r="K83" s="2" t="n">
         <v>11.754</v>
       </c>
       <c r="L83" s="2" t="n">
-        <v>15.125</v>
+        <v>20.661</v>
       </c>
       <c r="M83" s="2" t="n">
-        <v>26.1484</v>
+        <v>26.2593</v>
       </c>
       <c r="N83" t="inlineStr">
         <is>
-          <t>saa</t>
+          <t>casaa</t>
         </is>
       </c>
     </row>
@@ -4897,26 +4895,26 @@
       </c>
       <c r="D84" t="inlineStr">
         <is>
-          <t>SYSU-CD-256</t>
+          <t>LEVIR-CD-256</t>
         </is>
       </c>
       <c r="E84" s="2" t="n">
-        <v>78.40000000000001</v>
+        <v>91.38</v>
       </c>
       <c r="F84" s="2" t="n">
-        <v>86.03</v>
+        <v>92.3</v>
       </c>
       <c r="G84" s="2" t="n">
-        <v>91.90000000000001</v>
+        <v>99.17</v>
       </c>
       <c r="H84" s="2" t="n">
-        <v>82.04000000000001</v>
+        <v>91.84</v>
       </c>
       <c r="I84" s="2" t="n">
-        <v>69.55</v>
+        <v>84.91</v>
       </c>
       <c r="J84" s="2" t="n">
-        <v>76.83</v>
+        <v>91.40000000000001</v>
       </c>
       <c r="K84" s="2" t="n">
         <v>11.754</v>
@@ -4946,31 +4944,31 @@
       </c>
       <c r="C85" t="inlineStr">
         <is>
-          <t>A3_ORACLE_FROZEN</t>
+          <t>A1_SAA_FROZEN</t>
         </is>
       </c>
       <c r="D85" t="inlineStr">
         <is>
-          <t>LEVIR-CD-256</t>
+          <t>SYSU-CD-256</t>
         </is>
       </c>
       <c r="E85" s="2" t="n">
-        <v>91.13</v>
+        <v>78.40000000000001</v>
       </c>
       <c r="F85" s="2" t="n">
-        <v>92.65000000000001</v>
+        <v>86.03</v>
       </c>
       <c r="G85" s="2" t="n">
-        <v>99.18000000000001</v>
+        <v>91.90000000000001</v>
       </c>
       <c r="H85" s="2" t="n">
-        <v>91.88</v>
+        <v>82.04000000000001</v>
       </c>
       <c r="I85" s="2" t="n">
-        <v>84.98</v>
+        <v>69.55</v>
       </c>
       <c r="J85" s="2" t="n">
-        <v>91.45</v>
+        <v>76.83</v>
       </c>
       <c r="K85" s="2" t="n">
         <v>11.754</v>
@@ -4979,11 +4977,11 @@
         <v>15.125</v>
       </c>
       <c r="M85" s="2" t="n">
-        <v>26.0894</v>
+        <v>26.1484</v>
       </c>
       <c r="N85" t="inlineStr">
         <is>
-          <t>casaa</t>
+          <t>saa</t>
         </is>
       </c>
     </row>
@@ -5005,26 +5003,26 @@
       </c>
       <c r="D86" t="inlineStr">
         <is>
-          <t>SYSU-CD-256</t>
+          <t>LEVIR-CD-256</t>
         </is>
       </c>
       <c r="E86" s="2" t="n">
-        <v>82.04000000000001</v>
+        <v>91.13</v>
       </c>
       <c r="F86" s="2" t="n">
-        <v>85.05</v>
+        <v>92.65000000000001</v>
       </c>
       <c r="G86" s="2" t="n">
-        <v>92.36</v>
+        <v>99.18000000000001</v>
       </c>
       <c r="H86" s="2" t="n">
-        <v>83.52</v>
+        <v>91.88</v>
       </c>
       <c r="I86" s="2" t="n">
-        <v>71.7</v>
+        <v>84.98</v>
       </c>
       <c r="J86" s="2" t="n">
-        <v>78.55</v>
+        <v>91.45</v>
       </c>
       <c r="K86" s="2" t="n">
         <v>11.754</v>
@@ -5049,12 +5047,12 @@
       </c>
       <c r="B87" t="inlineStr">
         <is>
-          <t>Run3</t>
+          <t>Run2</t>
         </is>
       </c>
       <c r="C87" t="inlineStr">
         <is>
-          <t>A4_DETAIL_FROZEN</t>
+          <t>A3_ORACLE_FROZEN</t>
         </is>
       </c>
       <c r="D87" t="inlineStr">
@@ -5063,22 +5061,22 @@
         </is>
       </c>
       <c r="E87" s="2" t="n">
-        <v>79.68000000000001</v>
+        <v>82.04000000000001</v>
       </c>
       <c r="F87" s="2" t="n">
-        <v>84.28</v>
+        <v>85.05</v>
       </c>
       <c r="G87" s="2" t="n">
-        <v>91.7</v>
+        <v>92.36</v>
       </c>
       <c r="H87" s="2" t="n">
-        <v>81.92</v>
+        <v>83.52</v>
       </c>
       <c r="I87" s="2" t="n">
-        <v>69.37</v>
+        <v>71.7</v>
       </c>
       <c r="J87" s="2" t="n">
-        <v>76.54000000000001</v>
+        <v>78.55</v>
       </c>
       <c r="K87" s="2" t="n">
         <v>11.754</v>
@@ -5098,54 +5096,54 @@
     <row r="88">
       <c r="A88" t="inlineStr">
         <is>
-          <t>STR-Fusion</t>
+          <t>CASAA</t>
         </is>
       </c>
       <c r="B88" t="inlineStr">
         <is>
-          <t>Run2_TASS</t>
+          <t>Run3</t>
         </is>
       </c>
       <c r="C88" t="inlineStr">
         <is>
-          <t>C0_TOKEN</t>
+          <t>A4_DETAIL_FROZEN</t>
         </is>
       </c>
       <c r="D88" t="inlineStr">
         <is>
-          <t>CDD-CD-256</t>
+          <t>SYSU-CD-256</t>
         </is>
       </c>
       <c r="E88" s="2" t="n">
-        <v>93.13</v>
+        <v>79.68000000000001</v>
       </c>
       <c r="F88" s="2" t="n">
-        <v>95.16</v>
+        <v>84.28</v>
       </c>
       <c r="G88" s="2" t="n">
-        <v>98.56999999999999</v>
+        <v>91.7</v>
       </c>
       <c r="H88" s="2" t="n">
-        <v>94.13</v>
+        <v>81.92</v>
       </c>
       <c r="I88" s="2" t="n">
-        <v>88.91</v>
+        <v>69.37</v>
       </c>
       <c r="J88" s="2" t="n">
-        <v>93.31999999999999</v>
+        <v>76.54000000000001</v>
       </c>
       <c r="K88" s="2" t="n">
-        <v>2.596</v>
+        <v>11.754</v>
       </c>
       <c r="L88" s="2" t="n">
-        <v>0.62</v>
+        <v>15.125</v>
       </c>
       <c r="M88" s="2" t="n">
-        <v>2.2136</v>
+        <v>26.0894</v>
       </c>
       <c r="N88" t="inlineStr">
         <is>
-          <t>str_tass</t>
+          <t>casaa</t>
         </is>
       </c>
     </row>
@@ -5167,26 +5165,26 @@
       </c>
       <c r="D89" t="inlineStr">
         <is>
-          <t>LEVIR-CD-256</t>
+          <t>CDD-CD-256</t>
         </is>
       </c>
       <c r="E89" s="2" t="n">
-        <v>86.37</v>
+        <v>93.13</v>
       </c>
       <c r="F89" s="2" t="n">
-        <v>89.25</v>
+        <v>95.16</v>
       </c>
       <c r="G89" s="2" t="n">
-        <v>98.78</v>
+        <v>98.56999999999999</v>
       </c>
       <c r="H89" s="2" t="n">
-        <v>87.79000000000001</v>
+        <v>94.13</v>
       </c>
       <c r="I89" s="2" t="n">
-        <v>78.23999999999999</v>
+        <v>88.91</v>
       </c>
       <c r="J89" s="2" t="n">
-        <v>87.14</v>
+        <v>93.31999999999999</v>
       </c>
       <c r="K89" s="2" t="n">
         <v>2.596</v>
@@ -5221,26 +5219,26 @@
       </c>
       <c r="D90" t="inlineStr">
         <is>
-          <t>SYSU-CD-256</t>
+          <t>LEVIR-CD-256</t>
         </is>
       </c>
       <c r="E90" s="2" t="n">
-        <v>79.93000000000001</v>
+        <v>86.37</v>
       </c>
       <c r="F90" s="2" t="n">
-        <v>84.5</v>
+        <v>89.25</v>
       </c>
       <c r="G90" s="2" t="n">
-        <v>91.81</v>
+        <v>98.78</v>
       </c>
       <c r="H90" s="2" t="n">
-        <v>82.15000000000001</v>
+        <v>87.79000000000001</v>
       </c>
       <c r="I90" s="2" t="n">
-        <v>69.70999999999999</v>
+        <v>78.23999999999999</v>
       </c>
       <c r="J90" s="2" t="n">
-        <v>76.84</v>
+        <v>87.14</v>
       </c>
       <c r="K90" s="2" t="n">
         <v>2.596</v>
@@ -5275,26 +5273,26 @@
       </c>
       <c r="D91" t="inlineStr">
         <is>
-          <t>WHU-CD-256</t>
+          <t>SYSU-CD-256</t>
         </is>
       </c>
       <c r="E91" s="2" t="n">
-        <v>90.16</v>
+        <v>79.93000000000001</v>
       </c>
       <c r="F91" s="2" t="n">
-        <v>93.97</v>
+        <v>84.5</v>
       </c>
       <c r="G91" s="2" t="n">
-        <v>99.38</v>
+        <v>91.81</v>
       </c>
       <c r="H91" s="2" t="n">
-        <v>92.02</v>
+        <v>82.15000000000001</v>
       </c>
       <c r="I91" s="2" t="n">
-        <v>85.23</v>
+        <v>69.70999999999999</v>
       </c>
       <c r="J91" s="2" t="n">
-        <v>91.7</v>
+        <v>76.84</v>
       </c>
       <c r="K91" s="2" t="n">
         <v>2.596</v>
@@ -5324,40 +5322,40 @@
       </c>
       <c r="C92" t="inlineStr">
         <is>
-          <t>M1_TASS</t>
+          <t>C0_TOKEN</t>
         </is>
       </c>
       <c r="D92" t="inlineStr">
         <is>
-          <t>CDD-CD-256</t>
+          <t>WHU-CD-256</t>
         </is>
       </c>
       <c r="E92" s="2" t="n">
-        <v>94.7</v>
+        <v>90.16</v>
       </c>
       <c r="F92" s="2" t="n">
-        <v>96.13</v>
+        <v>93.97</v>
       </c>
       <c r="G92" s="2" t="n">
-        <v>98.88</v>
+        <v>99.38</v>
       </c>
       <c r="H92" s="2" t="n">
-        <v>95.41</v>
+        <v>92.02</v>
       </c>
       <c r="I92" s="2" t="n">
-        <v>91.22</v>
+        <v>85.23</v>
       </c>
       <c r="J92" s="2" t="n">
-        <v>94.77</v>
+        <v>91.7</v>
       </c>
       <c r="K92" s="2" t="n">
-        <v>3.455</v>
+        <v>2.596</v>
       </c>
       <c r="L92" s="2" t="n">
-        <v>1.478</v>
+        <v>0.62</v>
       </c>
       <c r="M92" s="2" t="n">
-        <v>3.5459</v>
+        <v>2.2136</v>
       </c>
       <c r="N92" t="inlineStr">
         <is>
@@ -5383,26 +5381,26 @@
       </c>
       <c r="D93" t="inlineStr">
         <is>
-          <t>LEVIR-CD-256</t>
+          <t>CDD-CD-256</t>
         </is>
       </c>
       <c r="E93" s="2" t="n">
-        <v>88.42</v>
+        <v>94.7</v>
       </c>
       <c r="F93" s="2" t="n">
-        <v>91.97</v>
+        <v>96.13</v>
       </c>
       <c r="G93" s="2" t="n">
-        <v>99.02</v>
+        <v>98.88</v>
       </c>
       <c r="H93" s="2" t="n">
-        <v>90.16</v>
+        <v>95.41</v>
       </c>
       <c r="I93" s="2" t="n">
-        <v>82.08</v>
+        <v>91.22</v>
       </c>
       <c r="J93" s="2" t="n">
-        <v>89.64</v>
+        <v>94.77</v>
       </c>
       <c r="K93" s="2" t="n">
         <v>3.455</v>
@@ -5437,26 +5435,26 @@
       </c>
       <c r="D94" t="inlineStr">
         <is>
-          <t>SYSU-CD-256</t>
+          <t>LEVIR-CD-256</t>
         </is>
       </c>
       <c r="E94" s="2" t="n">
-        <v>78.73</v>
+        <v>88.42</v>
       </c>
       <c r="F94" s="2" t="n">
-        <v>84.98</v>
+        <v>91.97</v>
       </c>
       <c r="G94" s="2" t="n">
-        <v>91.7</v>
+        <v>99.02</v>
       </c>
       <c r="H94" s="2" t="n">
-        <v>81.73999999999999</v>
+        <v>90.16</v>
       </c>
       <c r="I94" s="2" t="n">
-        <v>69.11</v>
+        <v>82.08</v>
       </c>
       <c r="J94" s="2" t="n">
-        <v>76.38</v>
+        <v>89.64</v>
       </c>
       <c r="K94" s="2" t="n">
         <v>3.455</v>
@@ -5491,26 +5489,26 @@
       </c>
       <c r="D95" t="inlineStr">
         <is>
-          <t>WHU-CD-256</t>
+          <t>SYSU-CD-256</t>
         </is>
       </c>
       <c r="E95" s="2" t="n">
-        <v>91.64</v>
+        <v>78.73</v>
       </c>
       <c r="F95" s="2" t="n">
-        <v>94.81999999999999</v>
+        <v>84.98</v>
       </c>
       <c r="G95" s="2" t="n">
-        <v>99.47</v>
+        <v>91.7</v>
       </c>
       <c r="H95" s="2" t="n">
-        <v>93.2</v>
+        <v>81.73999999999999</v>
       </c>
       <c r="I95" s="2" t="n">
-        <v>87.27</v>
+        <v>69.11</v>
       </c>
       <c r="J95" s="2" t="n">
-        <v>92.93000000000001</v>
+        <v>76.38</v>
       </c>
       <c r="K95" s="2" t="n">
         <v>3.455</v>
@@ -5530,54 +5528,54 @@
     <row r="96">
       <c r="A96" t="inlineStr">
         <is>
-          <t>UltraLight</t>
+          <t>STR-Fusion</t>
         </is>
       </c>
       <c r="B96" t="inlineStr">
         <is>
-          <t>Run4</t>
+          <t>Run2_TASS</t>
         </is>
       </c>
       <c r="C96" t="inlineStr">
         <is>
-          <t>R4_0_A0_FULL12_FROZEN</t>
+          <t>M1_TASS</t>
         </is>
       </c>
       <c r="D96" t="inlineStr">
         <is>
-          <t>SYSU-CD-256</t>
+          <t>WHU-CD-256</t>
         </is>
       </c>
       <c r="E96" s="2" t="n">
-        <v>82.42</v>
+        <v>91.64</v>
       </c>
       <c r="F96" s="2" t="n">
-        <v>83.87</v>
+        <v>94.81999999999999</v>
       </c>
       <c r="G96" s="2" t="n">
-        <v>92.12</v>
+        <v>99.47</v>
       </c>
       <c r="H96" s="2" t="n">
-        <v>83.14</v>
+        <v>93.2</v>
       </c>
       <c r="I96" s="2" t="n">
-        <v>71.14</v>
+        <v>87.27</v>
       </c>
       <c r="J96" s="2" t="n">
-        <v>77.98999999999999</v>
+        <v>92.93000000000001</v>
       </c>
       <c r="K96" s="2" t="n">
-        <v>11.754</v>
+        <v>3.455</v>
       </c>
       <c r="L96" s="2" t="n">
-        <v>15.125</v>
+        <v>1.478</v>
       </c>
       <c r="M96" s="2" t="n">
-        <v>26.3246</v>
+        <v>3.5459</v>
       </c>
       <c r="N96" t="inlineStr">
         <is>
-          <t>baseline</t>
+          <t>str_tass</t>
         </is>
       </c>
     </row>
@@ -5594,7 +5592,7 @@
       </c>
       <c r="C97" t="inlineStr">
         <is>
-          <t>R4_1_VIT4_OLDHEAD</t>
+          <t>R4_0_A0_FULL12_FROZEN</t>
         </is>
       </c>
       <c r="D97" t="inlineStr">
@@ -5603,31 +5601,31 @@
         </is>
       </c>
       <c r="E97" s="2" t="n">
-        <v>82.15000000000001</v>
+        <v>82.42</v>
       </c>
       <c r="F97" s="2" t="n">
-        <v>83.40000000000001</v>
+        <v>83.87</v>
       </c>
       <c r="G97" s="2" t="n">
-        <v>91.94</v>
+        <v>92.12</v>
       </c>
       <c r="H97" s="2" t="n">
-        <v>82.77</v>
+        <v>83.14</v>
       </c>
       <c r="I97" s="2" t="n">
-        <v>70.61</v>
+        <v>71.14</v>
       </c>
       <c r="J97" s="2" t="n">
-        <v>77.51000000000001</v>
+        <v>77.98999999999999</v>
       </c>
       <c r="K97" s="2" t="n">
-        <v>8.195</v>
+        <v>11.754</v>
       </c>
       <c r="L97" s="2" t="n">
         <v>15.125</v>
       </c>
       <c r="M97" s="2" t="n">
-        <v>24.1021</v>
+        <v>26.3246</v>
       </c>
       <c r="N97" t="inlineStr">
         <is>
@@ -5648,7 +5646,7 @@
       </c>
       <c r="C98" t="inlineStr">
         <is>
-          <t>R4_2_VIT4_LIGHTDETAIL</t>
+          <t>R4_1_VIT4_OLDHEAD</t>
         </is>
       </c>
       <c r="D98" t="inlineStr">
@@ -5657,31 +5655,31 @@
         </is>
       </c>
       <c r="E98" s="2" t="n">
-        <v>79.94</v>
+        <v>82.15000000000001</v>
       </c>
       <c r="F98" s="2" t="n">
-        <v>84.79000000000001</v>
+        <v>83.40000000000001</v>
       </c>
       <c r="G98" s="2" t="n">
-        <v>91.89</v>
+        <v>91.94</v>
       </c>
       <c r="H98" s="2" t="n">
-        <v>82.3</v>
+        <v>82.77</v>
       </c>
       <c r="I98" s="2" t="n">
-        <v>69.92</v>
+        <v>70.61</v>
       </c>
       <c r="J98" s="2" t="n">
-        <v>77.04000000000001</v>
+        <v>77.51000000000001</v>
       </c>
       <c r="K98" s="2" t="n">
-        <v>5.492</v>
+        <v>8.195</v>
       </c>
       <c r="L98" s="2" t="n">
-        <v>3.515</v>
+        <v>15.125</v>
       </c>
       <c r="M98" s="2" t="n">
-        <v>10.7311</v>
+        <v>24.1021</v>
       </c>
       <c r="N98" t="inlineStr">
         <is>
@@ -5702,7 +5700,7 @@
       </c>
       <c r="C99" t="inlineStr">
         <is>
-          <t>R4_2b_VIT4_LIGHTDETAIL48</t>
+          <t>R4_2_VIT4_LIGHTDETAIL</t>
         </is>
       </c>
       <c r="D99" t="inlineStr">
@@ -5711,31 +5709,31 @@
         </is>
       </c>
       <c r="E99" s="2" t="n">
-        <v>80.87</v>
+        <v>79.94</v>
       </c>
       <c r="F99" s="2" t="n">
-        <v>83.81</v>
+        <v>84.79000000000001</v>
       </c>
       <c r="G99" s="2" t="n">
-        <v>91.81</v>
+        <v>91.89</v>
       </c>
       <c r="H99" s="2" t="n">
-        <v>82.31999999999999</v>
+        <v>82.3</v>
       </c>
       <c r="I99" s="2" t="n">
-        <v>69.95</v>
+        <v>69.92</v>
       </c>
       <c r="J99" s="2" t="n">
-        <v>76.98999999999999</v>
+        <v>77.04000000000001</v>
       </c>
       <c r="K99" s="2" t="n">
-        <v>5.533</v>
+        <v>5.492</v>
       </c>
       <c r="L99" s="2" t="n">
-        <v>3.556</v>
+        <v>3.515</v>
       </c>
       <c r="M99" s="2" t="n">
-        <v>10.9824</v>
+        <v>10.7311</v>
       </c>
       <c r="N99" t="inlineStr">
         <is>
@@ -5756,7 +5754,7 @@
       </c>
       <c r="C100" t="inlineStr">
         <is>
-          <t>R4_2d_PSD_DETAIL</t>
+          <t>R4_2b_VIT4_LIGHTDETAIL48</t>
         </is>
       </c>
       <c r="D100" t="inlineStr">
@@ -5765,31 +5763,31 @@
         </is>
       </c>
       <c r="E100" s="2" t="n">
-        <v>79.78</v>
+        <v>80.87</v>
       </c>
       <c r="F100" s="2" t="n">
-        <v>84.39</v>
+        <v>83.81</v>
       </c>
       <c r="G100" s="2" t="n">
-        <v>91.75</v>
+        <v>91.81</v>
       </c>
       <c r="H100" s="2" t="n">
-        <v>82.02</v>
+        <v>82.31999999999999</v>
       </c>
       <c r="I100" s="2" t="n">
-        <v>69.52</v>
+        <v>69.95</v>
       </c>
       <c r="J100" s="2" t="n">
-        <v>76.68000000000001</v>
+        <v>76.98999999999999</v>
       </c>
       <c r="K100" s="2" t="n">
-        <v>5.491</v>
+        <v>5.533</v>
       </c>
       <c r="L100" s="2" t="n">
-        <v>3.514</v>
+        <v>3.556</v>
       </c>
       <c r="M100" s="2" t="n">
-        <v>11.5239</v>
+        <v>10.9824</v>
       </c>
       <c r="N100" t="inlineStr">
         <is>
@@ -5800,46 +5798,50 @@
     <row r="101">
       <c r="A101" t="inlineStr">
         <is>
-          <t>baseline</t>
+          <t>UltraLight</t>
         </is>
       </c>
       <c r="B101" t="inlineStr">
         <is>
-          <t>Run1</t>
-        </is>
-      </c>
-      <c r="C101" t="inlineStr"/>
+          <t>Run4</t>
+        </is>
+      </c>
+      <c r="C101" t="inlineStr">
+        <is>
+          <t>R4_2d_PSD_DETAIL</t>
+        </is>
+      </c>
       <c r="D101" t="inlineStr">
         <is>
-          <t>CDD-CD-256</t>
+          <t>SYSU-CD-256</t>
         </is>
       </c>
       <c r="E101" s="2" t="n">
-        <v>97.72</v>
+        <v>79.78</v>
       </c>
       <c r="F101" s="2" t="n">
-        <v>97.78</v>
+        <v>84.39</v>
       </c>
       <c r="G101" s="2" t="n">
-        <v>99.44</v>
+        <v>91.75</v>
       </c>
       <c r="H101" s="2" t="n">
-        <v>97.75</v>
+        <v>82.02</v>
       </c>
       <c r="I101" s="2" t="n">
-        <v>95.59999999999999</v>
+        <v>69.52</v>
       </c>
       <c r="J101" s="2" t="n">
-        <v>97.43000000000001</v>
+        <v>76.68000000000001</v>
       </c>
       <c r="K101" s="2" t="n">
-        <v>11.754</v>
+        <v>5.491</v>
       </c>
       <c r="L101" s="2" t="n">
-        <v>20.661</v>
+        <v>3.514</v>
       </c>
       <c r="M101" s="2" t="n">
-        <v>26.3246</v>
+        <v>11.5239</v>
       </c>
       <c r="N101" t="inlineStr">
         <is>
@@ -5861,26 +5863,26 @@
       <c r="C102" t="inlineStr"/>
       <c r="D102" t="inlineStr">
         <is>
-          <t>LEVIR-CD-256</t>
+          <t>CDD-CD-256</t>
         </is>
       </c>
       <c r="E102" s="2" t="n">
-        <v>91.56999999999999</v>
+        <v>97.72</v>
       </c>
       <c r="F102" s="2" t="n">
-        <v>92.33</v>
+        <v>97.78</v>
       </c>
       <c r="G102" s="2" t="n">
-        <v>99.18000000000001</v>
+        <v>99.44</v>
       </c>
       <c r="H102" s="2" t="n">
-        <v>91.95</v>
+        <v>97.75</v>
       </c>
       <c r="I102" s="2" t="n">
-        <v>85.09999999999999</v>
+        <v>95.59999999999999</v>
       </c>
       <c r="J102" s="2" t="n">
-        <v>91.52</v>
+        <v>97.43000000000001</v>
       </c>
       <c r="K102" s="2" t="n">
         <v>11.754</v>
@@ -5911,26 +5913,26 @@
       <c r="C103" t="inlineStr"/>
       <c r="D103" t="inlineStr">
         <is>
-          <t>SYSU-CD-256</t>
+          <t>LEVIR-CD-256</t>
         </is>
       </c>
       <c r="E103" s="2" t="n">
-        <v>80.77</v>
+        <v>91.56999999999999</v>
       </c>
       <c r="F103" s="2" t="n">
-        <v>84.27</v>
+        <v>92.33</v>
       </c>
       <c r="G103" s="2" t="n">
-        <v>91.91</v>
+        <v>99.18000000000001</v>
       </c>
       <c r="H103" s="2" t="n">
-        <v>82.48</v>
+        <v>91.95</v>
       </c>
       <c r="I103" s="2" t="n">
-        <v>70.19</v>
+        <v>85.09999999999999</v>
       </c>
       <c r="J103" s="2" t="n">
-        <v>77.23</v>
+        <v>91.52</v>
       </c>
       <c r="K103" s="2" t="n">
         <v>11.754</v>
@@ -5961,26 +5963,26 @@
       <c r="C104" t="inlineStr"/>
       <c r="D104" t="inlineStr">
         <is>
-          <t>WHU-CD-256</t>
+          <t>SYSU-CD-256</t>
         </is>
       </c>
       <c r="E104" s="2" t="n">
-        <v>93.62</v>
+        <v>80.77</v>
       </c>
       <c r="F104" s="2" t="n">
-        <v>96.09</v>
+        <v>84.27</v>
       </c>
       <c r="G104" s="2" t="n">
-        <v>99.59999999999999</v>
+        <v>91.91</v>
       </c>
       <c r="H104" s="2" t="n">
-        <v>94.84</v>
+        <v>82.48</v>
       </c>
       <c r="I104" s="2" t="n">
-        <v>90.18000000000001</v>
+        <v>70.19</v>
       </c>
       <c r="J104" s="2" t="n">
-        <v>94.63</v>
+        <v>77.23</v>
       </c>
       <c r="K104" s="2" t="n">
         <v>11.754</v>
@@ -5997,8 +5999,58 @@
         </is>
       </c>
     </row>
+    <row r="105">
+      <c r="A105" t="inlineStr">
+        <is>
+          <t>baseline</t>
+        </is>
+      </c>
+      <c r="B105" t="inlineStr">
+        <is>
+          <t>Run1</t>
+        </is>
+      </c>
+      <c r="C105" t="inlineStr"/>
+      <c r="D105" t="inlineStr">
+        <is>
+          <t>WHU-CD-256</t>
+        </is>
+      </c>
+      <c r="E105" s="2" t="n">
+        <v>93.62</v>
+      </c>
+      <c r="F105" s="2" t="n">
+        <v>96.09</v>
+      </c>
+      <c r="G105" s="2" t="n">
+        <v>99.59999999999999</v>
+      </c>
+      <c r="H105" s="2" t="n">
+        <v>94.84</v>
+      </c>
+      <c r="I105" s="2" t="n">
+        <v>90.18000000000001</v>
+      </c>
+      <c r="J105" s="2" t="n">
+        <v>94.63</v>
+      </c>
+      <c r="K105" s="2" t="n">
+        <v>11.754</v>
+      </c>
+      <c r="L105" s="2" t="n">
+        <v>20.661</v>
+      </c>
+      <c r="M105" s="2" t="n">
+        <v>26.3246</v>
+      </c>
+      <c r="N105" t="inlineStr">
+        <is>
+          <t>baseline</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:N104"/>
+  <autoFilter ref="A1:N105"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Complete SYSU ablation results and comparison
</commit_message>
<xml_diff>
--- a/docs/experiment_metrics.xlsx
+++ b/docs/experiment_metrics.xlsx
@@ -10,7 +10,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="metrics" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'metrics'!$A$1:$N$105</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'metrics'!$A$1:$N$106</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -420,7 +420,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N105"/>
+  <dimension ref="A1:N106"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -4570,7 +4570,7 @@
       </c>
       <c r="C78" t="inlineStr">
         <is>
-          <t>M1_HYPER_QKV</t>
+          <t>M0_CTRL</t>
         </is>
       </c>
       <c r="D78" t="inlineStr">
@@ -4579,33 +4579,33 @@
         </is>
       </c>
       <c r="E78" s="2" t="n">
-        <v>78.67</v>
+        <v>80.39</v>
       </c>
       <c r="F78" s="2" t="n">
-        <v>85.08</v>
+        <v>82.89</v>
       </c>
       <c r="G78" s="2" t="n">
-        <v>91.72</v>
+        <v>91.45999999999999</v>
       </c>
       <c r="H78" s="2" t="n">
-        <v>81.75</v>
+        <v>81.62</v>
       </c>
       <c r="I78" s="2" t="n">
-        <v>69.13</v>
+        <v>68.95</v>
       </c>
       <c r="J78" s="2" t="n">
-        <v>76.40000000000001</v>
+        <v>76.06999999999999</v>
       </c>
       <c r="K78" s="2" t="n">
-        <v>3.049509</v>
+        <v>3.016737</v>
       </c>
       <c r="L78" s="2" t="n">
-        <v>3.133176</v>
+        <v>3.100404</v>
       </c>
       <c r="M78" s="2" t="n"/>
       <c r="N78" t="inlineStr">
         <is>
-          <t>casa_wdmf_str_hyperbolic</t>
+          <t>casa_wdmf_str_none</t>
         </is>
       </c>
     </row>
@@ -4622,7 +4622,7 @@
       </c>
       <c r="C79" t="inlineStr">
         <is>
-          <t>M2_CA_QKV</t>
+          <t>M1_HYPER_QKV</t>
         </is>
       </c>
       <c r="D79" t="inlineStr">
@@ -4631,22 +4631,22 @@
         </is>
       </c>
       <c r="E79" s="2" t="n">
-        <v>82.83</v>
+        <v>78.67</v>
       </c>
       <c r="F79" s="2" t="n">
-        <v>82.86</v>
+        <v>85.08</v>
       </c>
       <c r="G79" s="2" t="n">
-        <v>91.91</v>
+        <v>91.72</v>
       </c>
       <c r="H79" s="2" t="n">
-        <v>82.84999999999999</v>
+        <v>81.75</v>
       </c>
       <c r="I79" s="2" t="n">
-        <v>70.72</v>
+        <v>69.13</v>
       </c>
       <c r="J79" s="2" t="n">
-        <v>77.56</v>
+        <v>76.40000000000001</v>
       </c>
       <c r="K79" s="2" t="n">
         <v>3.049509</v>
@@ -4657,61 +4657,59 @@
       <c r="M79" s="2" t="n"/>
       <c r="N79" t="inlineStr">
         <is>
-          <t>casa_wdmf_str_qkv</t>
+          <t>casa_wdmf_str_hyperbolic</t>
         </is>
       </c>
     </row>
     <row r="80">
       <c r="A80" t="inlineStr">
         <is>
-          <t>CASAA</t>
+          <t>CASA-WDMF</t>
         </is>
       </c>
       <c r="B80" t="inlineStr">
         <is>
-          <t>Run1</t>
+          <t>Run2</t>
         </is>
       </c>
       <c r="C80" t="inlineStr">
         <is>
-          <t>A1_SAA</t>
+          <t>M2_CA_QKV</t>
         </is>
       </c>
       <c r="D80" t="inlineStr">
         <is>
-          <t>LEVIR-CD-256</t>
+          <t>SYSU-CD-256</t>
         </is>
       </c>
       <c r="E80" s="2" t="n">
-        <v>91.09</v>
+        <v>82.83</v>
       </c>
       <c r="F80" s="2" t="n">
-        <v>92.8</v>
+        <v>82.86</v>
       </c>
       <c r="G80" s="2" t="n">
-        <v>99.19</v>
+        <v>91.91</v>
       </c>
       <c r="H80" s="2" t="n">
-        <v>91.94</v>
+        <v>82.84999999999999</v>
       </c>
       <c r="I80" s="2" t="n">
-        <v>85.08</v>
+        <v>70.72</v>
       </c>
       <c r="J80" s="2" t="n">
-        <v>91.51000000000001</v>
+        <v>77.56</v>
       </c>
       <c r="K80" s="2" t="n">
-        <v>11.754</v>
+        <v>3.049509</v>
       </c>
       <c r="L80" s="2" t="n">
-        <v>20.661</v>
-      </c>
-      <c r="M80" s="2" t="n">
-        <v>26.3183</v>
-      </c>
+        <v>3.133176</v>
+      </c>
+      <c r="M80" s="2" t="n"/>
       <c r="N80" t="inlineStr">
         <is>
-          <t>saa</t>
+          <t>casa_wdmf_str_qkv</t>
         </is>
       </c>
     </row>
@@ -4733,26 +4731,26 @@
       </c>
       <c r="D81" t="inlineStr">
         <is>
-          <t>SYSU-CD-256</t>
+          <t>LEVIR-CD-256</t>
         </is>
       </c>
       <c r="E81" s="2" t="n">
-        <v>80.3</v>
+        <v>91.09</v>
       </c>
       <c r="F81" s="2" t="n">
-        <v>84.81</v>
+        <v>92.8</v>
       </c>
       <c r="G81" s="2" t="n">
-        <v>91.95999999999999</v>
+        <v>99.19</v>
       </c>
       <c r="H81" s="2" t="n">
-        <v>82.5</v>
+        <v>91.94</v>
       </c>
       <c r="I81" s="2" t="n">
-        <v>70.20999999999999</v>
+        <v>85.08</v>
       </c>
       <c r="J81" s="2" t="n">
-        <v>77.29000000000001</v>
+        <v>91.51000000000001</v>
       </c>
       <c r="K81" s="2" t="n">
         <v>11.754</v>
@@ -4782,31 +4780,31 @@
       </c>
       <c r="C82" t="inlineStr">
         <is>
-          <t>A2_CASAA</t>
+          <t>A1_SAA</t>
         </is>
       </c>
       <c r="D82" t="inlineStr">
         <is>
-          <t>LEVIR-CD-256</t>
+          <t>SYSU-CD-256</t>
         </is>
       </c>
       <c r="E82" s="2" t="n">
-        <v>90.98999999999999</v>
+        <v>80.3</v>
       </c>
       <c r="F82" s="2" t="n">
-        <v>92.75</v>
+        <v>84.81</v>
       </c>
       <c r="G82" s="2" t="n">
-        <v>99.18000000000001</v>
+        <v>91.95999999999999</v>
       </c>
       <c r="H82" s="2" t="n">
-        <v>91.86</v>
+        <v>82.5</v>
       </c>
       <c r="I82" s="2" t="n">
-        <v>84.94</v>
+        <v>70.20999999999999</v>
       </c>
       <c r="J82" s="2" t="n">
-        <v>91.43000000000001</v>
+        <v>77.29000000000001</v>
       </c>
       <c r="K82" s="2" t="n">
         <v>11.754</v>
@@ -4815,11 +4813,11 @@
         <v>20.661</v>
       </c>
       <c r="M82" s="2" t="n">
-        <v>26.2593</v>
+        <v>26.3183</v>
       </c>
       <c r="N82" t="inlineStr">
         <is>
-          <t>casaa</t>
+          <t>saa</t>
         </is>
       </c>
     </row>
@@ -4841,26 +4839,26 @@
       </c>
       <c r="D83" t="inlineStr">
         <is>
-          <t>SYSU-CD-256</t>
+          <t>LEVIR-CD-256</t>
         </is>
       </c>
       <c r="E83" s="2" t="n">
-        <v>80.55</v>
+        <v>90.98999999999999</v>
       </c>
       <c r="F83" s="2" t="n">
-        <v>84.23</v>
+        <v>92.75</v>
       </c>
       <c r="G83" s="2" t="n">
+        <v>99.18000000000001</v>
+      </c>
+      <c r="H83" s="2" t="n">
         <v>91.86</v>
       </c>
-      <c r="H83" s="2" t="n">
-        <v>82.34999999999999</v>
-      </c>
       <c r="I83" s="2" t="n">
-        <v>70</v>
+        <v>84.94</v>
       </c>
       <c r="J83" s="2" t="n">
-        <v>77.06</v>
+        <v>91.43000000000001</v>
       </c>
       <c r="K83" s="2" t="n">
         <v>11.754</v>
@@ -4885,49 +4883,49 @@
       </c>
       <c r="B84" t="inlineStr">
         <is>
-          <t>Run2</t>
+          <t>Run1</t>
         </is>
       </c>
       <c r="C84" t="inlineStr">
         <is>
-          <t>A1_SAA_FROZEN</t>
+          <t>A2_CASAA</t>
         </is>
       </c>
       <c r="D84" t="inlineStr">
         <is>
-          <t>LEVIR-CD-256</t>
+          <t>SYSU-CD-256</t>
         </is>
       </c>
       <c r="E84" s="2" t="n">
-        <v>91.38</v>
+        <v>80.55</v>
       </c>
       <c r="F84" s="2" t="n">
-        <v>92.3</v>
+        <v>84.23</v>
       </c>
       <c r="G84" s="2" t="n">
-        <v>99.17</v>
+        <v>91.86</v>
       </c>
       <c r="H84" s="2" t="n">
-        <v>91.84</v>
+        <v>82.34999999999999</v>
       </c>
       <c r="I84" s="2" t="n">
-        <v>84.91</v>
+        <v>70</v>
       </c>
       <c r="J84" s="2" t="n">
-        <v>91.40000000000001</v>
+        <v>77.06</v>
       </c>
       <c r="K84" s="2" t="n">
         <v>11.754</v>
       </c>
       <c r="L84" s="2" t="n">
-        <v>15.125</v>
+        <v>20.661</v>
       </c>
       <c r="M84" s="2" t="n">
-        <v>26.1484</v>
+        <v>26.2593</v>
       </c>
       <c r="N84" t="inlineStr">
         <is>
-          <t>saa</t>
+          <t>casaa</t>
         </is>
       </c>
     </row>
@@ -4949,26 +4947,26 @@
       </c>
       <c r="D85" t="inlineStr">
         <is>
-          <t>SYSU-CD-256</t>
+          <t>LEVIR-CD-256</t>
         </is>
       </c>
       <c r="E85" s="2" t="n">
-        <v>78.40000000000001</v>
+        <v>91.38</v>
       </c>
       <c r="F85" s="2" t="n">
-        <v>86.03</v>
+        <v>92.3</v>
       </c>
       <c r="G85" s="2" t="n">
-        <v>91.90000000000001</v>
+        <v>99.17</v>
       </c>
       <c r="H85" s="2" t="n">
-        <v>82.04000000000001</v>
+        <v>91.84</v>
       </c>
       <c r="I85" s="2" t="n">
-        <v>69.55</v>
+        <v>84.91</v>
       </c>
       <c r="J85" s="2" t="n">
-        <v>76.83</v>
+        <v>91.40000000000001</v>
       </c>
       <c r="K85" s="2" t="n">
         <v>11.754</v>
@@ -4998,31 +4996,31 @@
       </c>
       <c r="C86" t="inlineStr">
         <is>
-          <t>A3_ORACLE_FROZEN</t>
+          <t>A1_SAA_FROZEN</t>
         </is>
       </c>
       <c r="D86" t="inlineStr">
         <is>
-          <t>LEVIR-CD-256</t>
+          <t>SYSU-CD-256</t>
         </is>
       </c>
       <c r="E86" s="2" t="n">
-        <v>91.13</v>
+        <v>78.40000000000001</v>
       </c>
       <c r="F86" s="2" t="n">
-        <v>92.65000000000001</v>
+        <v>86.03</v>
       </c>
       <c r="G86" s="2" t="n">
-        <v>99.18000000000001</v>
+        <v>91.90000000000001</v>
       </c>
       <c r="H86" s="2" t="n">
-        <v>91.88</v>
+        <v>82.04000000000001</v>
       </c>
       <c r="I86" s="2" t="n">
-        <v>84.98</v>
+        <v>69.55</v>
       </c>
       <c r="J86" s="2" t="n">
-        <v>91.45</v>
+        <v>76.83</v>
       </c>
       <c r="K86" s="2" t="n">
         <v>11.754</v>
@@ -5031,11 +5029,11 @@
         <v>15.125</v>
       </c>
       <c r="M86" s="2" t="n">
-        <v>26.0894</v>
+        <v>26.1484</v>
       </c>
       <c r="N86" t="inlineStr">
         <is>
-          <t>casaa</t>
+          <t>saa</t>
         </is>
       </c>
     </row>
@@ -5057,26 +5055,26 @@
       </c>
       <c r="D87" t="inlineStr">
         <is>
-          <t>SYSU-CD-256</t>
+          <t>LEVIR-CD-256</t>
         </is>
       </c>
       <c r="E87" s="2" t="n">
-        <v>82.04000000000001</v>
+        <v>91.13</v>
       </c>
       <c r="F87" s="2" t="n">
-        <v>85.05</v>
+        <v>92.65000000000001</v>
       </c>
       <c r="G87" s="2" t="n">
-        <v>92.36</v>
+        <v>99.18000000000001</v>
       </c>
       <c r="H87" s="2" t="n">
-        <v>83.52</v>
+        <v>91.88</v>
       </c>
       <c r="I87" s="2" t="n">
-        <v>71.7</v>
+        <v>84.98</v>
       </c>
       <c r="J87" s="2" t="n">
-        <v>78.55</v>
+        <v>91.45</v>
       </c>
       <c r="K87" s="2" t="n">
         <v>11.754</v>
@@ -5101,12 +5099,12 @@
       </c>
       <c r="B88" t="inlineStr">
         <is>
-          <t>Run3</t>
+          <t>Run2</t>
         </is>
       </c>
       <c r="C88" t="inlineStr">
         <is>
-          <t>A4_DETAIL_FROZEN</t>
+          <t>A3_ORACLE_FROZEN</t>
         </is>
       </c>
       <c r="D88" t="inlineStr">
@@ -5115,22 +5113,22 @@
         </is>
       </c>
       <c r="E88" s="2" t="n">
-        <v>79.68000000000001</v>
+        <v>82.04000000000001</v>
       </c>
       <c r="F88" s="2" t="n">
-        <v>84.28</v>
+        <v>85.05</v>
       </c>
       <c r="G88" s="2" t="n">
-        <v>91.7</v>
+        <v>92.36</v>
       </c>
       <c r="H88" s="2" t="n">
-        <v>81.92</v>
+        <v>83.52</v>
       </c>
       <c r="I88" s="2" t="n">
-        <v>69.37</v>
+        <v>71.7</v>
       </c>
       <c r="J88" s="2" t="n">
-        <v>76.54000000000001</v>
+        <v>78.55</v>
       </c>
       <c r="K88" s="2" t="n">
         <v>11.754</v>
@@ -5150,54 +5148,54 @@
     <row r="89">
       <c r="A89" t="inlineStr">
         <is>
-          <t>STR-Fusion</t>
+          <t>CASAA</t>
         </is>
       </c>
       <c r="B89" t="inlineStr">
         <is>
-          <t>Run2_TASS</t>
+          <t>Run3</t>
         </is>
       </c>
       <c r="C89" t="inlineStr">
         <is>
-          <t>C0_TOKEN</t>
+          <t>A4_DETAIL_FROZEN</t>
         </is>
       </c>
       <c r="D89" t="inlineStr">
         <is>
-          <t>CDD-CD-256</t>
+          <t>SYSU-CD-256</t>
         </is>
       </c>
       <c r="E89" s="2" t="n">
-        <v>93.13</v>
+        <v>79.68000000000001</v>
       </c>
       <c r="F89" s="2" t="n">
-        <v>95.16</v>
+        <v>84.28</v>
       </c>
       <c r="G89" s="2" t="n">
-        <v>98.56999999999999</v>
+        <v>91.7</v>
       </c>
       <c r="H89" s="2" t="n">
-        <v>94.13</v>
+        <v>81.92</v>
       </c>
       <c r="I89" s="2" t="n">
-        <v>88.91</v>
+        <v>69.37</v>
       </c>
       <c r="J89" s="2" t="n">
-        <v>93.31999999999999</v>
+        <v>76.54000000000001</v>
       </c>
       <c r="K89" s="2" t="n">
-        <v>2.596</v>
+        <v>11.754</v>
       </c>
       <c r="L89" s="2" t="n">
-        <v>0.62</v>
+        <v>15.125</v>
       </c>
       <c r="M89" s="2" t="n">
-        <v>2.2136</v>
+        <v>26.0894</v>
       </c>
       <c r="N89" t="inlineStr">
         <is>
-          <t>str_tass</t>
+          <t>casaa</t>
         </is>
       </c>
     </row>
@@ -5219,26 +5217,26 @@
       </c>
       <c r="D90" t="inlineStr">
         <is>
-          <t>LEVIR-CD-256</t>
+          <t>CDD-CD-256</t>
         </is>
       </c>
       <c r="E90" s="2" t="n">
-        <v>86.37</v>
+        <v>93.13</v>
       </c>
       <c r="F90" s="2" t="n">
-        <v>89.25</v>
+        <v>95.16</v>
       </c>
       <c r="G90" s="2" t="n">
-        <v>98.78</v>
+        <v>98.56999999999999</v>
       </c>
       <c r="H90" s="2" t="n">
-        <v>87.79000000000001</v>
+        <v>94.13</v>
       </c>
       <c r="I90" s="2" t="n">
-        <v>78.23999999999999</v>
+        <v>88.91</v>
       </c>
       <c r="J90" s="2" t="n">
-        <v>87.14</v>
+        <v>93.31999999999999</v>
       </c>
       <c r="K90" s="2" t="n">
         <v>2.596</v>
@@ -5273,26 +5271,26 @@
       </c>
       <c r="D91" t="inlineStr">
         <is>
-          <t>SYSU-CD-256</t>
+          <t>LEVIR-CD-256</t>
         </is>
       </c>
       <c r="E91" s="2" t="n">
-        <v>79.93000000000001</v>
+        <v>86.37</v>
       </c>
       <c r="F91" s="2" t="n">
-        <v>84.5</v>
+        <v>89.25</v>
       </c>
       <c r="G91" s="2" t="n">
-        <v>91.81</v>
+        <v>98.78</v>
       </c>
       <c r="H91" s="2" t="n">
-        <v>82.15000000000001</v>
+        <v>87.79000000000001</v>
       </c>
       <c r="I91" s="2" t="n">
-        <v>69.70999999999999</v>
+        <v>78.23999999999999</v>
       </c>
       <c r="J91" s="2" t="n">
-        <v>76.84</v>
+        <v>87.14</v>
       </c>
       <c r="K91" s="2" t="n">
         <v>2.596</v>
@@ -5327,26 +5325,26 @@
       </c>
       <c r="D92" t="inlineStr">
         <is>
-          <t>WHU-CD-256</t>
+          <t>SYSU-CD-256</t>
         </is>
       </c>
       <c r="E92" s="2" t="n">
-        <v>90.16</v>
+        <v>79.93000000000001</v>
       </c>
       <c r="F92" s="2" t="n">
-        <v>93.97</v>
+        <v>84.5</v>
       </c>
       <c r="G92" s="2" t="n">
-        <v>99.38</v>
+        <v>91.81</v>
       </c>
       <c r="H92" s="2" t="n">
-        <v>92.02</v>
+        <v>82.15000000000001</v>
       </c>
       <c r="I92" s="2" t="n">
-        <v>85.23</v>
+        <v>69.70999999999999</v>
       </c>
       <c r="J92" s="2" t="n">
-        <v>91.7</v>
+        <v>76.84</v>
       </c>
       <c r="K92" s="2" t="n">
         <v>2.596</v>
@@ -5376,40 +5374,40 @@
       </c>
       <c r="C93" t="inlineStr">
         <is>
-          <t>M1_TASS</t>
+          <t>C0_TOKEN</t>
         </is>
       </c>
       <c r="D93" t="inlineStr">
         <is>
-          <t>CDD-CD-256</t>
+          <t>WHU-CD-256</t>
         </is>
       </c>
       <c r="E93" s="2" t="n">
-        <v>94.7</v>
+        <v>90.16</v>
       </c>
       <c r="F93" s="2" t="n">
-        <v>96.13</v>
+        <v>93.97</v>
       </c>
       <c r="G93" s="2" t="n">
-        <v>98.88</v>
+        <v>99.38</v>
       </c>
       <c r="H93" s="2" t="n">
-        <v>95.41</v>
+        <v>92.02</v>
       </c>
       <c r="I93" s="2" t="n">
-        <v>91.22</v>
+        <v>85.23</v>
       </c>
       <c r="J93" s="2" t="n">
-        <v>94.77</v>
+        <v>91.7</v>
       </c>
       <c r="K93" s="2" t="n">
-        <v>3.455</v>
+        <v>2.596</v>
       </c>
       <c r="L93" s="2" t="n">
-        <v>1.478</v>
+        <v>0.62</v>
       </c>
       <c r="M93" s="2" t="n">
-        <v>3.5459</v>
+        <v>2.2136</v>
       </c>
       <c r="N93" t="inlineStr">
         <is>
@@ -5435,26 +5433,26 @@
       </c>
       <c r="D94" t="inlineStr">
         <is>
-          <t>LEVIR-CD-256</t>
+          <t>CDD-CD-256</t>
         </is>
       </c>
       <c r="E94" s="2" t="n">
-        <v>88.42</v>
+        <v>94.7</v>
       </c>
       <c r="F94" s="2" t="n">
-        <v>91.97</v>
+        <v>96.13</v>
       </c>
       <c r="G94" s="2" t="n">
-        <v>99.02</v>
+        <v>98.88</v>
       </c>
       <c r="H94" s="2" t="n">
-        <v>90.16</v>
+        <v>95.41</v>
       </c>
       <c r="I94" s="2" t="n">
-        <v>82.08</v>
+        <v>91.22</v>
       </c>
       <c r="J94" s="2" t="n">
-        <v>89.64</v>
+        <v>94.77</v>
       </c>
       <c r="K94" s="2" t="n">
         <v>3.455</v>
@@ -5489,26 +5487,26 @@
       </c>
       <c r="D95" t="inlineStr">
         <is>
-          <t>SYSU-CD-256</t>
+          <t>LEVIR-CD-256</t>
         </is>
       </c>
       <c r="E95" s="2" t="n">
-        <v>78.73</v>
+        <v>88.42</v>
       </c>
       <c r="F95" s="2" t="n">
-        <v>84.98</v>
+        <v>91.97</v>
       </c>
       <c r="G95" s="2" t="n">
-        <v>91.7</v>
+        <v>99.02</v>
       </c>
       <c r="H95" s="2" t="n">
-        <v>81.73999999999999</v>
+        <v>90.16</v>
       </c>
       <c r="I95" s="2" t="n">
-        <v>69.11</v>
+        <v>82.08</v>
       </c>
       <c r="J95" s="2" t="n">
-        <v>76.38</v>
+        <v>89.64</v>
       </c>
       <c r="K95" s="2" t="n">
         <v>3.455</v>
@@ -5543,26 +5541,26 @@
       </c>
       <c r="D96" t="inlineStr">
         <is>
-          <t>WHU-CD-256</t>
+          <t>SYSU-CD-256</t>
         </is>
       </c>
       <c r="E96" s="2" t="n">
-        <v>91.64</v>
+        <v>78.73</v>
       </c>
       <c r="F96" s="2" t="n">
-        <v>94.81999999999999</v>
+        <v>84.98</v>
       </c>
       <c r="G96" s="2" t="n">
-        <v>99.47</v>
+        <v>91.7</v>
       </c>
       <c r="H96" s="2" t="n">
-        <v>93.2</v>
+        <v>81.73999999999999</v>
       </c>
       <c r="I96" s="2" t="n">
-        <v>87.27</v>
+        <v>69.11</v>
       </c>
       <c r="J96" s="2" t="n">
-        <v>92.93000000000001</v>
+        <v>76.38</v>
       </c>
       <c r="K96" s="2" t="n">
         <v>3.455</v>
@@ -5582,54 +5580,54 @@
     <row r="97">
       <c r="A97" t="inlineStr">
         <is>
-          <t>UltraLight</t>
+          <t>STR-Fusion</t>
         </is>
       </c>
       <c r="B97" t="inlineStr">
         <is>
-          <t>Run4</t>
+          <t>Run2_TASS</t>
         </is>
       </c>
       <c r="C97" t="inlineStr">
         <is>
-          <t>R4_0_A0_FULL12_FROZEN</t>
+          <t>M1_TASS</t>
         </is>
       </c>
       <c r="D97" t="inlineStr">
         <is>
-          <t>SYSU-CD-256</t>
+          <t>WHU-CD-256</t>
         </is>
       </c>
       <c r="E97" s="2" t="n">
-        <v>82.42</v>
+        <v>91.64</v>
       </c>
       <c r="F97" s="2" t="n">
-        <v>83.87</v>
+        <v>94.81999999999999</v>
       </c>
       <c r="G97" s="2" t="n">
-        <v>92.12</v>
+        <v>99.47</v>
       </c>
       <c r="H97" s="2" t="n">
-        <v>83.14</v>
+        <v>93.2</v>
       </c>
       <c r="I97" s="2" t="n">
-        <v>71.14</v>
+        <v>87.27</v>
       </c>
       <c r="J97" s="2" t="n">
-        <v>77.98999999999999</v>
+        <v>92.93000000000001</v>
       </c>
       <c r="K97" s="2" t="n">
-        <v>11.754</v>
+        <v>3.455</v>
       </c>
       <c r="L97" s="2" t="n">
-        <v>15.125</v>
+        <v>1.478</v>
       </c>
       <c r="M97" s="2" t="n">
-        <v>26.3246</v>
+        <v>3.5459</v>
       </c>
       <c r="N97" t="inlineStr">
         <is>
-          <t>baseline</t>
+          <t>str_tass</t>
         </is>
       </c>
     </row>
@@ -5646,7 +5644,7 @@
       </c>
       <c r="C98" t="inlineStr">
         <is>
-          <t>R4_1_VIT4_OLDHEAD</t>
+          <t>R4_0_A0_FULL12_FROZEN</t>
         </is>
       </c>
       <c r="D98" t="inlineStr">
@@ -5655,31 +5653,31 @@
         </is>
       </c>
       <c r="E98" s="2" t="n">
-        <v>82.15000000000001</v>
+        <v>82.42</v>
       </c>
       <c r="F98" s="2" t="n">
-        <v>83.40000000000001</v>
+        <v>83.87</v>
       </c>
       <c r="G98" s="2" t="n">
-        <v>91.94</v>
+        <v>92.12</v>
       </c>
       <c r="H98" s="2" t="n">
-        <v>82.77</v>
+        <v>83.14</v>
       </c>
       <c r="I98" s="2" t="n">
-        <v>70.61</v>
+        <v>71.14</v>
       </c>
       <c r="J98" s="2" t="n">
-        <v>77.51000000000001</v>
+        <v>77.98999999999999</v>
       </c>
       <c r="K98" s="2" t="n">
-        <v>8.195</v>
+        <v>11.754</v>
       </c>
       <c r="L98" s="2" t="n">
         <v>15.125</v>
       </c>
       <c r="M98" s="2" t="n">
-        <v>24.1021</v>
+        <v>26.3246</v>
       </c>
       <c r="N98" t="inlineStr">
         <is>
@@ -5700,7 +5698,7 @@
       </c>
       <c r="C99" t="inlineStr">
         <is>
-          <t>R4_2_VIT4_LIGHTDETAIL</t>
+          <t>R4_1_VIT4_OLDHEAD</t>
         </is>
       </c>
       <c r="D99" t="inlineStr">
@@ -5709,31 +5707,31 @@
         </is>
       </c>
       <c r="E99" s="2" t="n">
-        <v>79.94</v>
+        <v>82.15000000000001</v>
       </c>
       <c r="F99" s="2" t="n">
-        <v>84.79000000000001</v>
+        <v>83.40000000000001</v>
       </c>
       <c r="G99" s="2" t="n">
-        <v>91.89</v>
+        <v>91.94</v>
       </c>
       <c r="H99" s="2" t="n">
-        <v>82.3</v>
+        <v>82.77</v>
       </c>
       <c r="I99" s="2" t="n">
-        <v>69.92</v>
+        <v>70.61</v>
       </c>
       <c r="J99" s="2" t="n">
-        <v>77.04000000000001</v>
+        <v>77.51000000000001</v>
       </c>
       <c r="K99" s="2" t="n">
-        <v>5.492</v>
+        <v>8.195</v>
       </c>
       <c r="L99" s="2" t="n">
-        <v>3.515</v>
+        <v>15.125</v>
       </c>
       <c r="M99" s="2" t="n">
-        <v>10.7311</v>
+        <v>24.1021</v>
       </c>
       <c r="N99" t="inlineStr">
         <is>
@@ -5754,7 +5752,7 @@
       </c>
       <c r="C100" t="inlineStr">
         <is>
-          <t>R4_2b_VIT4_LIGHTDETAIL48</t>
+          <t>R4_2_VIT4_LIGHTDETAIL</t>
         </is>
       </c>
       <c r="D100" t="inlineStr">
@@ -5763,31 +5761,31 @@
         </is>
       </c>
       <c r="E100" s="2" t="n">
-        <v>80.87</v>
+        <v>79.94</v>
       </c>
       <c r="F100" s="2" t="n">
-        <v>83.81</v>
+        <v>84.79000000000001</v>
       </c>
       <c r="G100" s="2" t="n">
-        <v>91.81</v>
+        <v>91.89</v>
       </c>
       <c r="H100" s="2" t="n">
-        <v>82.31999999999999</v>
+        <v>82.3</v>
       </c>
       <c r="I100" s="2" t="n">
-        <v>69.95</v>
+        <v>69.92</v>
       </c>
       <c r="J100" s="2" t="n">
-        <v>76.98999999999999</v>
+        <v>77.04000000000001</v>
       </c>
       <c r="K100" s="2" t="n">
-        <v>5.533</v>
+        <v>5.492</v>
       </c>
       <c r="L100" s="2" t="n">
-        <v>3.556</v>
+        <v>3.515</v>
       </c>
       <c r="M100" s="2" t="n">
-        <v>10.9824</v>
+        <v>10.7311</v>
       </c>
       <c r="N100" t="inlineStr">
         <is>
@@ -5808,7 +5806,7 @@
       </c>
       <c r="C101" t="inlineStr">
         <is>
-          <t>R4_2d_PSD_DETAIL</t>
+          <t>R4_2b_VIT4_LIGHTDETAIL48</t>
         </is>
       </c>
       <c r="D101" t="inlineStr">
@@ -5817,31 +5815,31 @@
         </is>
       </c>
       <c r="E101" s="2" t="n">
-        <v>79.78</v>
+        <v>80.87</v>
       </c>
       <c r="F101" s="2" t="n">
-        <v>84.39</v>
+        <v>83.81</v>
       </c>
       <c r="G101" s="2" t="n">
-        <v>91.75</v>
+        <v>91.81</v>
       </c>
       <c r="H101" s="2" t="n">
-        <v>82.02</v>
+        <v>82.31999999999999</v>
       </c>
       <c r="I101" s="2" t="n">
-        <v>69.52</v>
+        <v>69.95</v>
       </c>
       <c r="J101" s="2" t="n">
-        <v>76.68000000000001</v>
+        <v>76.98999999999999</v>
       </c>
       <c r="K101" s="2" t="n">
-        <v>5.491</v>
+        <v>5.533</v>
       </c>
       <c r="L101" s="2" t="n">
-        <v>3.514</v>
+        <v>3.556</v>
       </c>
       <c r="M101" s="2" t="n">
-        <v>11.5239</v>
+        <v>10.9824</v>
       </c>
       <c r="N101" t="inlineStr">
         <is>
@@ -5852,46 +5850,50 @@
     <row r="102">
       <c r="A102" t="inlineStr">
         <is>
-          <t>baseline</t>
+          <t>UltraLight</t>
         </is>
       </c>
       <c r="B102" t="inlineStr">
         <is>
-          <t>Run1</t>
-        </is>
-      </c>
-      <c r="C102" t="inlineStr"/>
+          <t>Run4</t>
+        </is>
+      </c>
+      <c r="C102" t="inlineStr">
+        <is>
+          <t>R4_2d_PSD_DETAIL</t>
+        </is>
+      </c>
       <c r="D102" t="inlineStr">
         <is>
-          <t>CDD-CD-256</t>
+          <t>SYSU-CD-256</t>
         </is>
       </c>
       <c r="E102" s="2" t="n">
-        <v>97.72</v>
+        <v>79.78</v>
       </c>
       <c r="F102" s="2" t="n">
-        <v>97.78</v>
+        <v>84.39</v>
       </c>
       <c r="G102" s="2" t="n">
-        <v>99.44</v>
+        <v>91.75</v>
       </c>
       <c r="H102" s="2" t="n">
-        <v>97.75</v>
+        <v>82.02</v>
       </c>
       <c r="I102" s="2" t="n">
-        <v>95.59999999999999</v>
+        <v>69.52</v>
       </c>
       <c r="J102" s="2" t="n">
-        <v>97.43000000000001</v>
+        <v>76.68000000000001</v>
       </c>
       <c r="K102" s="2" t="n">
-        <v>11.754</v>
+        <v>5.491</v>
       </c>
       <c r="L102" s="2" t="n">
-        <v>20.661</v>
+        <v>3.514</v>
       </c>
       <c r="M102" s="2" t="n">
-        <v>26.3246</v>
+        <v>11.5239</v>
       </c>
       <c r="N102" t="inlineStr">
         <is>
@@ -5913,26 +5915,26 @@
       <c r="C103" t="inlineStr"/>
       <c r="D103" t="inlineStr">
         <is>
-          <t>LEVIR-CD-256</t>
+          <t>CDD-CD-256</t>
         </is>
       </c>
       <c r="E103" s="2" t="n">
-        <v>91.56999999999999</v>
+        <v>97.72</v>
       </c>
       <c r="F103" s="2" t="n">
-        <v>92.33</v>
+        <v>97.78</v>
       </c>
       <c r="G103" s="2" t="n">
-        <v>99.18000000000001</v>
+        <v>99.44</v>
       </c>
       <c r="H103" s="2" t="n">
-        <v>91.95</v>
+        <v>97.75</v>
       </c>
       <c r="I103" s="2" t="n">
-        <v>85.09999999999999</v>
+        <v>95.59999999999999</v>
       </c>
       <c r="J103" s="2" t="n">
-        <v>91.52</v>
+        <v>97.43000000000001</v>
       </c>
       <c r="K103" s="2" t="n">
         <v>11.754</v>
@@ -5963,26 +5965,26 @@
       <c r="C104" t="inlineStr"/>
       <c r="D104" t="inlineStr">
         <is>
-          <t>SYSU-CD-256</t>
+          <t>LEVIR-CD-256</t>
         </is>
       </c>
       <c r="E104" s="2" t="n">
-        <v>80.77</v>
+        <v>91.56999999999999</v>
       </c>
       <c r="F104" s="2" t="n">
-        <v>84.27</v>
+        <v>92.33</v>
       </c>
       <c r="G104" s="2" t="n">
-        <v>91.91</v>
+        <v>99.18000000000001</v>
       </c>
       <c r="H104" s="2" t="n">
-        <v>82.48</v>
+        <v>91.95</v>
       </c>
       <c r="I104" s="2" t="n">
-        <v>70.19</v>
+        <v>85.09999999999999</v>
       </c>
       <c r="J104" s="2" t="n">
-        <v>77.23</v>
+        <v>91.52</v>
       </c>
       <c r="K104" s="2" t="n">
         <v>11.754</v>
@@ -6013,26 +6015,26 @@
       <c r="C105" t="inlineStr"/>
       <c r="D105" t="inlineStr">
         <is>
-          <t>WHU-CD-256</t>
+          <t>SYSU-CD-256</t>
         </is>
       </c>
       <c r="E105" s="2" t="n">
-        <v>93.62</v>
+        <v>80.77</v>
       </c>
       <c r="F105" s="2" t="n">
-        <v>96.09</v>
+        <v>84.27</v>
       </c>
       <c r="G105" s="2" t="n">
-        <v>99.59999999999999</v>
+        <v>91.91</v>
       </c>
       <c r="H105" s="2" t="n">
-        <v>94.84</v>
+        <v>82.48</v>
       </c>
       <c r="I105" s="2" t="n">
-        <v>90.18000000000001</v>
+        <v>70.19</v>
       </c>
       <c r="J105" s="2" t="n">
-        <v>94.63</v>
+        <v>77.23</v>
       </c>
       <c r="K105" s="2" t="n">
         <v>11.754</v>
@@ -6049,8 +6051,58 @@
         </is>
       </c>
     </row>
+    <row r="106">
+      <c r="A106" t="inlineStr">
+        <is>
+          <t>baseline</t>
+        </is>
+      </c>
+      <c r="B106" t="inlineStr">
+        <is>
+          <t>Run1</t>
+        </is>
+      </c>
+      <c r="C106" t="inlineStr"/>
+      <c r="D106" t="inlineStr">
+        <is>
+          <t>WHU-CD-256</t>
+        </is>
+      </c>
+      <c r="E106" s="2" t="n">
+        <v>93.62</v>
+      </c>
+      <c r="F106" s="2" t="n">
+        <v>96.09</v>
+      </c>
+      <c r="G106" s="2" t="n">
+        <v>99.59999999999999</v>
+      </c>
+      <c r="H106" s="2" t="n">
+        <v>94.84</v>
+      </c>
+      <c r="I106" s="2" t="n">
+        <v>90.18000000000001</v>
+      </c>
+      <c r="J106" s="2" t="n">
+        <v>94.63</v>
+      </c>
+      <c r="K106" s="2" t="n">
+        <v>11.754</v>
+      </c>
+      <c r="L106" s="2" t="n">
+        <v>20.661</v>
+      </c>
+      <c r="M106" s="2" t="n">
+        <v>26.3246</v>
+      </c>
+      <c r="N106" t="inlineStr">
+        <is>
+          <t>baseline</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:N105"/>
+  <autoFilter ref="A1:N106"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Support checkpoint continuation and strict deployment verification
</commit_message>
<xml_diff>
--- a/docs/experiment_metrics.xlsx
+++ b/docs/experiment_metrics.xlsx
@@ -10,7 +10,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="metrics" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'metrics'!$A$1:$N$106</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'metrics'!$A$1:$N$108</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -420,7 +420,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N106"/>
+  <dimension ref="A1:N108"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -4627,26 +4627,26 @@
       </c>
       <c r="D79" t="inlineStr">
         <is>
-          <t>SYSU-CD-256</t>
+          <t>LEVIR-CD-256</t>
         </is>
       </c>
       <c r="E79" s="2" t="n">
-        <v>78.67</v>
+        <v>90.55</v>
       </c>
       <c r="F79" s="2" t="n">
-        <v>85.08</v>
+        <v>92.03</v>
       </c>
       <c r="G79" s="2" t="n">
-        <v>91.72</v>
+        <v>99.12</v>
       </c>
       <c r="H79" s="2" t="n">
-        <v>81.75</v>
+        <v>91.28</v>
       </c>
       <c r="I79" s="2" t="n">
-        <v>69.13</v>
+        <v>83.95999999999999</v>
       </c>
       <c r="J79" s="2" t="n">
-        <v>76.40000000000001</v>
+        <v>90.81999999999999</v>
       </c>
       <c r="K79" s="2" t="n">
         <v>3.049509</v>
@@ -4674,7 +4674,7 @@
       </c>
       <c r="C80" t="inlineStr">
         <is>
-          <t>M2_CA_QKV</t>
+          <t>M1_HYPER_QKV</t>
         </is>
       </c>
       <c r="D80" t="inlineStr">
@@ -4683,22 +4683,22 @@
         </is>
       </c>
       <c r="E80" s="2" t="n">
-        <v>82.83</v>
+        <v>78.67</v>
       </c>
       <c r="F80" s="2" t="n">
-        <v>82.86</v>
+        <v>85.08</v>
       </c>
       <c r="G80" s="2" t="n">
-        <v>91.91</v>
+        <v>91.72</v>
       </c>
       <c r="H80" s="2" t="n">
-        <v>82.84999999999999</v>
+        <v>81.75</v>
       </c>
       <c r="I80" s="2" t="n">
-        <v>70.72</v>
+        <v>69.13</v>
       </c>
       <c r="J80" s="2" t="n">
-        <v>77.56</v>
+        <v>76.40000000000001</v>
       </c>
       <c r="K80" s="2" t="n">
         <v>3.049509</v>
@@ -4709,24 +4709,24 @@
       <c r="M80" s="2" t="n"/>
       <c r="N80" t="inlineStr">
         <is>
-          <t>casa_wdmf_str_qkv</t>
+          <t>casa_wdmf_str_hyperbolic</t>
         </is>
       </c>
     </row>
     <row r="81">
       <c r="A81" t="inlineStr">
         <is>
-          <t>CASAA</t>
+          <t>CASA-WDMF</t>
         </is>
       </c>
       <c r="B81" t="inlineStr">
         <is>
-          <t>Run1</t>
+          <t>Run2</t>
         </is>
       </c>
       <c r="C81" t="inlineStr">
         <is>
-          <t>A1_SAA</t>
+          <t>M2_CA_QKV</t>
         </is>
       </c>
       <c r="D81" t="inlineStr">
@@ -4735,52 +4735,50 @@
         </is>
       </c>
       <c r="E81" s="2" t="n">
-        <v>91.09</v>
+        <v>89.72</v>
       </c>
       <c r="F81" s="2" t="n">
-        <v>92.8</v>
+        <v>93.12</v>
       </c>
       <c r="G81" s="2" t="n">
-        <v>99.19</v>
+        <v>99.14</v>
       </c>
       <c r="H81" s="2" t="n">
-        <v>91.94</v>
+        <v>91.39</v>
       </c>
       <c r="I81" s="2" t="n">
-        <v>85.08</v>
+        <v>84.14</v>
       </c>
       <c r="J81" s="2" t="n">
-        <v>91.51000000000001</v>
+        <v>90.93000000000001</v>
       </c>
       <c r="K81" s="2" t="n">
-        <v>11.754</v>
+        <v>3.049509</v>
       </c>
       <c r="L81" s="2" t="n">
-        <v>20.661</v>
-      </c>
-      <c r="M81" s="2" t="n">
-        <v>26.3183</v>
-      </c>
+        <v>3.133176</v>
+      </c>
+      <c r="M81" s="2" t="n"/>
       <c r="N81" t="inlineStr">
         <is>
-          <t>saa</t>
+          <t>casa_wdmf_str_qkv</t>
         </is>
       </c>
     </row>
     <row r="82">
       <c r="A82" t="inlineStr">
         <is>
-          <t>CASAA</t>
+          <t>CASA-WDMF</t>
         </is>
       </c>
       <c r="B82" t="inlineStr">
         <is>
-          <t>Run1</t>
+          <t>Run2</t>
         </is>
       </c>
       <c r="C82" t="inlineStr">
         <is>
-          <t>A1_SAA</t>
+          <t>M2_CA_QKV</t>
         </is>
       </c>
       <c r="D82" t="inlineStr">
@@ -4789,35 +4787,33 @@
         </is>
       </c>
       <c r="E82" s="2" t="n">
-        <v>80.3</v>
+        <v>82.83</v>
       </c>
       <c r="F82" s="2" t="n">
-        <v>84.81</v>
+        <v>82.86</v>
       </c>
       <c r="G82" s="2" t="n">
-        <v>91.95999999999999</v>
+        <v>91.91</v>
       </c>
       <c r="H82" s="2" t="n">
-        <v>82.5</v>
+        <v>82.84999999999999</v>
       </c>
       <c r="I82" s="2" t="n">
-        <v>70.20999999999999</v>
+        <v>70.72</v>
       </c>
       <c r="J82" s="2" t="n">
-        <v>77.29000000000001</v>
+        <v>77.56</v>
       </c>
       <c r="K82" s="2" t="n">
-        <v>11.754</v>
+        <v>3.049509</v>
       </c>
       <c r="L82" s="2" t="n">
-        <v>20.661</v>
-      </c>
-      <c r="M82" s="2" t="n">
-        <v>26.3183</v>
-      </c>
+        <v>3.133176</v>
+      </c>
+      <c r="M82" s="2" t="n"/>
       <c r="N82" t="inlineStr">
         <is>
-          <t>saa</t>
+          <t>casa_wdmf_str_qkv</t>
         </is>
       </c>
     </row>
@@ -4834,7 +4830,7 @@
       </c>
       <c r="C83" t="inlineStr">
         <is>
-          <t>A2_CASAA</t>
+          <t>A1_SAA</t>
         </is>
       </c>
       <c r="D83" t="inlineStr">
@@ -4843,22 +4839,22 @@
         </is>
       </c>
       <c r="E83" s="2" t="n">
-        <v>90.98999999999999</v>
+        <v>91.09</v>
       </c>
       <c r="F83" s="2" t="n">
-        <v>92.75</v>
+        <v>92.8</v>
       </c>
       <c r="G83" s="2" t="n">
-        <v>99.18000000000001</v>
+        <v>99.19</v>
       </c>
       <c r="H83" s="2" t="n">
-        <v>91.86</v>
+        <v>91.94</v>
       </c>
       <c r="I83" s="2" t="n">
-        <v>84.94</v>
+        <v>85.08</v>
       </c>
       <c r="J83" s="2" t="n">
-        <v>91.43000000000001</v>
+        <v>91.51000000000001</v>
       </c>
       <c r="K83" s="2" t="n">
         <v>11.754</v>
@@ -4867,11 +4863,11 @@
         <v>20.661</v>
       </c>
       <c r="M83" s="2" t="n">
-        <v>26.2593</v>
+        <v>26.3183</v>
       </c>
       <c r="N83" t="inlineStr">
         <is>
-          <t>casaa</t>
+          <t>saa</t>
         </is>
       </c>
     </row>
@@ -4888,7 +4884,7 @@
       </c>
       <c r="C84" t="inlineStr">
         <is>
-          <t>A2_CASAA</t>
+          <t>A1_SAA</t>
         </is>
       </c>
       <c r="D84" t="inlineStr">
@@ -4897,22 +4893,22 @@
         </is>
       </c>
       <c r="E84" s="2" t="n">
-        <v>80.55</v>
+        <v>80.3</v>
       </c>
       <c r="F84" s="2" t="n">
-        <v>84.23</v>
+        <v>84.81</v>
       </c>
       <c r="G84" s="2" t="n">
-        <v>91.86</v>
+        <v>91.95999999999999</v>
       </c>
       <c r="H84" s="2" t="n">
-        <v>82.34999999999999</v>
+        <v>82.5</v>
       </c>
       <c r="I84" s="2" t="n">
-        <v>70</v>
+        <v>70.20999999999999</v>
       </c>
       <c r="J84" s="2" t="n">
-        <v>77.06</v>
+        <v>77.29000000000001</v>
       </c>
       <c r="K84" s="2" t="n">
         <v>11.754</v>
@@ -4921,11 +4917,11 @@
         <v>20.661</v>
       </c>
       <c r="M84" s="2" t="n">
-        <v>26.2593</v>
+        <v>26.3183</v>
       </c>
       <c r="N84" t="inlineStr">
         <is>
-          <t>casaa</t>
+          <t>saa</t>
         </is>
       </c>
     </row>
@@ -4937,12 +4933,12 @@
       </c>
       <c r="B85" t="inlineStr">
         <is>
-          <t>Run2</t>
+          <t>Run1</t>
         </is>
       </c>
       <c r="C85" t="inlineStr">
         <is>
-          <t>A1_SAA_FROZEN</t>
+          <t>A2_CASAA</t>
         </is>
       </c>
       <c r="D85" t="inlineStr">
@@ -4951,35 +4947,35 @@
         </is>
       </c>
       <c r="E85" s="2" t="n">
-        <v>91.38</v>
+        <v>90.98999999999999</v>
       </c>
       <c r="F85" s="2" t="n">
-        <v>92.3</v>
+        <v>92.75</v>
       </c>
       <c r="G85" s="2" t="n">
-        <v>99.17</v>
+        <v>99.18000000000001</v>
       </c>
       <c r="H85" s="2" t="n">
-        <v>91.84</v>
+        <v>91.86</v>
       </c>
       <c r="I85" s="2" t="n">
-        <v>84.91</v>
+        <v>84.94</v>
       </c>
       <c r="J85" s="2" t="n">
-        <v>91.40000000000001</v>
+        <v>91.43000000000001</v>
       </c>
       <c r="K85" s="2" t="n">
         <v>11.754</v>
       </c>
       <c r="L85" s="2" t="n">
-        <v>15.125</v>
+        <v>20.661</v>
       </c>
       <c r="M85" s="2" t="n">
-        <v>26.1484</v>
+        <v>26.2593</v>
       </c>
       <c r="N85" t="inlineStr">
         <is>
-          <t>saa</t>
+          <t>casaa</t>
         </is>
       </c>
     </row>
@@ -4991,12 +4987,12 @@
       </c>
       <c r="B86" t="inlineStr">
         <is>
-          <t>Run2</t>
+          <t>Run1</t>
         </is>
       </c>
       <c r="C86" t="inlineStr">
         <is>
-          <t>A1_SAA_FROZEN</t>
+          <t>A2_CASAA</t>
         </is>
       </c>
       <c r="D86" t="inlineStr">
@@ -5005,35 +5001,35 @@
         </is>
       </c>
       <c r="E86" s="2" t="n">
-        <v>78.40000000000001</v>
+        <v>80.55</v>
       </c>
       <c r="F86" s="2" t="n">
-        <v>86.03</v>
+        <v>84.23</v>
       </c>
       <c r="G86" s="2" t="n">
-        <v>91.90000000000001</v>
+        <v>91.86</v>
       </c>
       <c r="H86" s="2" t="n">
-        <v>82.04000000000001</v>
+        <v>82.34999999999999</v>
       </c>
       <c r="I86" s="2" t="n">
-        <v>69.55</v>
+        <v>70</v>
       </c>
       <c r="J86" s="2" t="n">
-        <v>76.83</v>
+        <v>77.06</v>
       </c>
       <c r="K86" s="2" t="n">
         <v>11.754</v>
       </c>
       <c r="L86" s="2" t="n">
-        <v>15.125</v>
+        <v>20.661</v>
       </c>
       <c r="M86" s="2" t="n">
-        <v>26.1484</v>
+        <v>26.2593</v>
       </c>
       <c r="N86" t="inlineStr">
         <is>
-          <t>saa</t>
+          <t>casaa</t>
         </is>
       </c>
     </row>
@@ -5050,7 +5046,7 @@
       </c>
       <c r="C87" t="inlineStr">
         <is>
-          <t>A3_ORACLE_FROZEN</t>
+          <t>A1_SAA_FROZEN</t>
         </is>
       </c>
       <c r="D87" t="inlineStr">
@@ -5059,22 +5055,22 @@
         </is>
       </c>
       <c r="E87" s="2" t="n">
-        <v>91.13</v>
+        <v>91.38</v>
       </c>
       <c r="F87" s="2" t="n">
-        <v>92.65000000000001</v>
+        <v>92.3</v>
       </c>
       <c r="G87" s="2" t="n">
-        <v>99.18000000000001</v>
+        <v>99.17</v>
       </c>
       <c r="H87" s="2" t="n">
-        <v>91.88</v>
+        <v>91.84</v>
       </c>
       <c r="I87" s="2" t="n">
-        <v>84.98</v>
+        <v>84.91</v>
       </c>
       <c r="J87" s="2" t="n">
-        <v>91.45</v>
+        <v>91.40000000000001</v>
       </c>
       <c r="K87" s="2" t="n">
         <v>11.754</v>
@@ -5083,11 +5079,11 @@
         <v>15.125</v>
       </c>
       <c r="M87" s="2" t="n">
-        <v>26.0894</v>
+        <v>26.1484</v>
       </c>
       <c r="N87" t="inlineStr">
         <is>
-          <t>casaa</t>
+          <t>saa</t>
         </is>
       </c>
     </row>
@@ -5104,7 +5100,7 @@
       </c>
       <c r="C88" t="inlineStr">
         <is>
-          <t>A3_ORACLE_FROZEN</t>
+          <t>A1_SAA_FROZEN</t>
         </is>
       </c>
       <c r="D88" t="inlineStr">
@@ -5113,22 +5109,22 @@
         </is>
       </c>
       <c r="E88" s="2" t="n">
+        <v>78.40000000000001</v>
+      </c>
+      <c r="F88" s="2" t="n">
+        <v>86.03</v>
+      </c>
+      <c r="G88" s="2" t="n">
+        <v>91.90000000000001</v>
+      </c>
+      <c r="H88" s="2" t="n">
         <v>82.04000000000001</v>
       </c>
-      <c r="F88" s="2" t="n">
-        <v>85.05</v>
-      </c>
-      <c r="G88" s="2" t="n">
-        <v>92.36</v>
-      </c>
-      <c r="H88" s="2" t="n">
-        <v>83.52</v>
-      </c>
       <c r="I88" s="2" t="n">
-        <v>71.7</v>
+        <v>69.55</v>
       </c>
       <c r="J88" s="2" t="n">
-        <v>78.55</v>
+        <v>76.83</v>
       </c>
       <c r="K88" s="2" t="n">
         <v>11.754</v>
@@ -5137,11 +5133,11 @@
         <v>15.125</v>
       </c>
       <c r="M88" s="2" t="n">
-        <v>26.0894</v>
+        <v>26.1484</v>
       </c>
       <c r="N88" t="inlineStr">
         <is>
-          <t>casaa</t>
+          <t>saa</t>
         </is>
       </c>
     </row>
@@ -5153,36 +5149,36 @@
       </c>
       <c r="B89" t="inlineStr">
         <is>
-          <t>Run3</t>
+          <t>Run2</t>
         </is>
       </c>
       <c r="C89" t="inlineStr">
         <is>
-          <t>A4_DETAIL_FROZEN</t>
+          <t>A3_ORACLE_FROZEN</t>
         </is>
       </c>
       <c r="D89" t="inlineStr">
         <is>
-          <t>SYSU-CD-256</t>
+          <t>LEVIR-CD-256</t>
         </is>
       </c>
       <c r="E89" s="2" t="n">
-        <v>79.68000000000001</v>
+        <v>91.13</v>
       </c>
       <c r="F89" s="2" t="n">
-        <v>84.28</v>
+        <v>92.65000000000001</v>
       </c>
       <c r="G89" s="2" t="n">
-        <v>91.7</v>
+        <v>99.18000000000001</v>
       </c>
       <c r="H89" s="2" t="n">
-        <v>81.92</v>
+        <v>91.88</v>
       </c>
       <c r="I89" s="2" t="n">
-        <v>69.37</v>
+        <v>84.98</v>
       </c>
       <c r="J89" s="2" t="n">
-        <v>76.54000000000001</v>
+        <v>91.45</v>
       </c>
       <c r="K89" s="2" t="n">
         <v>11.754</v>
@@ -5202,108 +5198,108 @@
     <row r="90">
       <c r="A90" t="inlineStr">
         <is>
-          <t>STR-Fusion</t>
+          <t>CASAA</t>
         </is>
       </c>
       <c r="B90" t="inlineStr">
         <is>
-          <t>Run2_TASS</t>
+          <t>Run2</t>
         </is>
       </c>
       <c r="C90" t="inlineStr">
         <is>
-          <t>C0_TOKEN</t>
+          <t>A3_ORACLE_FROZEN</t>
         </is>
       </c>
       <c r="D90" t="inlineStr">
         <is>
-          <t>CDD-CD-256</t>
+          <t>SYSU-CD-256</t>
         </is>
       </c>
       <c r="E90" s="2" t="n">
-        <v>93.13</v>
+        <v>82.04000000000001</v>
       </c>
       <c r="F90" s="2" t="n">
-        <v>95.16</v>
+        <v>85.05</v>
       </c>
       <c r="G90" s="2" t="n">
-        <v>98.56999999999999</v>
+        <v>92.36</v>
       </c>
       <c r="H90" s="2" t="n">
-        <v>94.13</v>
+        <v>83.52</v>
       </c>
       <c r="I90" s="2" t="n">
-        <v>88.91</v>
+        <v>71.7</v>
       </c>
       <c r="J90" s="2" t="n">
-        <v>93.31999999999999</v>
+        <v>78.55</v>
       </c>
       <c r="K90" s="2" t="n">
-        <v>2.596</v>
+        <v>11.754</v>
       </c>
       <c r="L90" s="2" t="n">
-        <v>0.62</v>
+        <v>15.125</v>
       </c>
       <c r="M90" s="2" t="n">
-        <v>2.2136</v>
+        <v>26.0894</v>
       </c>
       <c r="N90" t="inlineStr">
         <is>
-          <t>str_tass</t>
+          <t>casaa</t>
         </is>
       </c>
     </row>
     <row r="91">
       <c r="A91" t="inlineStr">
         <is>
-          <t>STR-Fusion</t>
+          <t>CASAA</t>
         </is>
       </c>
       <c r="B91" t="inlineStr">
         <is>
-          <t>Run2_TASS</t>
+          <t>Run3</t>
         </is>
       </c>
       <c r="C91" t="inlineStr">
         <is>
-          <t>C0_TOKEN</t>
+          <t>A4_DETAIL_FROZEN</t>
         </is>
       </c>
       <c r="D91" t="inlineStr">
         <is>
-          <t>LEVIR-CD-256</t>
+          <t>SYSU-CD-256</t>
         </is>
       </c>
       <c r="E91" s="2" t="n">
-        <v>86.37</v>
+        <v>79.68000000000001</v>
       </c>
       <c r="F91" s="2" t="n">
-        <v>89.25</v>
+        <v>84.28</v>
       </c>
       <c r="G91" s="2" t="n">
-        <v>98.78</v>
+        <v>91.7</v>
       </c>
       <c r="H91" s="2" t="n">
-        <v>87.79000000000001</v>
+        <v>81.92</v>
       </c>
       <c r="I91" s="2" t="n">
-        <v>78.23999999999999</v>
+        <v>69.37</v>
       </c>
       <c r="J91" s="2" t="n">
-        <v>87.14</v>
+        <v>76.54000000000001</v>
       </c>
       <c r="K91" s="2" t="n">
-        <v>2.596</v>
+        <v>11.754</v>
       </c>
       <c r="L91" s="2" t="n">
-        <v>0.62</v>
+        <v>15.125</v>
       </c>
       <c r="M91" s="2" t="n">
-        <v>2.2136</v>
+        <v>26.0894</v>
       </c>
       <c r="N91" t="inlineStr">
         <is>
-          <t>str_tass</t>
+          <t>casaa</t>
         </is>
       </c>
     </row>
@@ -5325,26 +5321,26 @@
       </c>
       <c r="D92" t="inlineStr">
         <is>
-          <t>SYSU-CD-256</t>
+          <t>CDD-CD-256</t>
         </is>
       </c>
       <c r="E92" s="2" t="n">
-        <v>79.93000000000001</v>
+        <v>93.13</v>
       </c>
       <c r="F92" s="2" t="n">
-        <v>84.5</v>
+        <v>95.16</v>
       </c>
       <c r="G92" s="2" t="n">
-        <v>91.81</v>
+        <v>98.56999999999999</v>
       </c>
       <c r="H92" s="2" t="n">
-        <v>82.15000000000001</v>
+        <v>94.13</v>
       </c>
       <c r="I92" s="2" t="n">
-        <v>69.70999999999999</v>
+        <v>88.91</v>
       </c>
       <c r="J92" s="2" t="n">
-        <v>76.84</v>
+        <v>93.31999999999999</v>
       </c>
       <c r="K92" s="2" t="n">
         <v>2.596</v>
@@ -5379,26 +5375,26 @@
       </c>
       <c r="D93" t="inlineStr">
         <is>
-          <t>WHU-CD-256</t>
+          <t>LEVIR-CD-256</t>
         </is>
       </c>
       <c r="E93" s="2" t="n">
-        <v>90.16</v>
+        <v>86.37</v>
       </c>
       <c r="F93" s="2" t="n">
-        <v>93.97</v>
+        <v>89.25</v>
       </c>
       <c r="G93" s="2" t="n">
-        <v>99.38</v>
+        <v>98.78</v>
       </c>
       <c r="H93" s="2" t="n">
-        <v>92.02</v>
+        <v>87.79000000000001</v>
       </c>
       <c r="I93" s="2" t="n">
-        <v>85.23</v>
+        <v>78.23999999999999</v>
       </c>
       <c r="J93" s="2" t="n">
-        <v>91.7</v>
+        <v>87.14</v>
       </c>
       <c r="K93" s="2" t="n">
         <v>2.596</v>
@@ -5428,40 +5424,40 @@
       </c>
       <c r="C94" t="inlineStr">
         <is>
-          <t>M1_TASS</t>
+          <t>C0_TOKEN</t>
         </is>
       </c>
       <c r="D94" t="inlineStr">
         <is>
-          <t>CDD-CD-256</t>
+          <t>SYSU-CD-256</t>
         </is>
       </c>
       <c r="E94" s="2" t="n">
-        <v>94.7</v>
+        <v>79.93000000000001</v>
       </c>
       <c r="F94" s="2" t="n">
-        <v>96.13</v>
+        <v>84.5</v>
       </c>
       <c r="G94" s="2" t="n">
-        <v>98.88</v>
+        <v>91.81</v>
       </c>
       <c r="H94" s="2" t="n">
-        <v>95.41</v>
+        <v>82.15000000000001</v>
       </c>
       <c r="I94" s="2" t="n">
-        <v>91.22</v>
+        <v>69.70999999999999</v>
       </c>
       <c r="J94" s="2" t="n">
-        <v>94.77</v>
+        <v>76.84</v>
       </c>
       <c r="K94" s="2" t="n">
-        <v>3.455</v>
+        <v>2.596</v>
       </c>
       <c r="L94" s="2" t="n">
-        <v>1.478</v>
+        <v>0.62</v>
       </c>
       <c r="M94" s="2" t="n">
-        <v>3.5459</v>
+        <v>2.2136</v>
       </c>
       <c r="N94" t="inlineStr">
         <is>
@@ -5482,40 +5478,40 @@
       </c>
       <c r="C95" t="inlineStr">
         <is>
-          <t>M1_TASS</t>
+          <t>C0_TOKEN</t>
         </is>
       </c>
       <c r="D95" t="inlineStr">
         <is>
-          <t>LEVIR-CD-256</t>
+          <t>WHU-CD-256</t>
         </is>
       </c>
       <c r="E95" s="2" t="n">
-        <v>88.42</v>
+        <v>90.16</v>
       </c>
       <c r="F95" s="2" t="n">
-        <v>91.97</v>
+        <v>93.97</v>
       </c>
       <c r="G95" s="2" t="n">
-        <v>99.02</v>
+        <v>99.38</v>
       </c>
       <c r="H95" s="2" t="n">
-        <v>90.16</v>
+        <v>92.02</v>
       </c>
       <c r="I95" s="2" t="n">
-        <v>82.08</v>
+        <v>85.23</v>
       </c>
       <c r="J95" s="2" t="n">
-        <v>89.64</v>
+        <v>91.7</v>
       </c>
       <c r="K95" s="2" t="n">
-        <v>3.455</v>
+        <v>2.596</v>
       </c>
       <c r="L95" s="2" t="n">
-        <v>1.478</v>
+        <v>0.62</v>
       </c>
       <c r="M95" s="2" t="n">
-        <v>3.5459</v>
+        <v>2.2136</v>
       </c>
       <c r="N95" t="inlineStr">
         <is>
@@ -5541,26 +5537,26 @@
       </c>
       <c r="D96" t="inlineStr">
         <is>
-          <t>SYSU-CD-256</t>
+          <t>CDD-CD-256</t>
         </is>
       </c>
       <c r="E96" s="2" t="n">
-        <v>78.73</v>
+        <v>94.7</v>
       </c>
       <c r="F96" s="2" t="n">
-        <v>84.98</v>
+        <v>96.13</v>
       </c>
       <c r="G96" s="2" t="n">
-        <v>91.7</v>
+        <v>98.88</v>
       </c>
       <c r="H96" s="2" t="n">
-        <v>81.73999999999999</v>
+        <v>95.41</v>
       </c>
       <c r="I96" s="2" t="n">
-        <v>69.11</v>
+        <v>91.22</v>
       </c>
       <c r="J96" s="2" t="n">
-        <v>76.38</v>
+        <v>94.77</v>
       </c>
       <c r="K96" s="2" t="n">
         <v>3.455</v>
@@ -5595,26 +5591,26 @@
       </c>
       <c r="D97" t="inlineStr">
         <is>
-          <t>WHU-CD-256</t>
+          <t>LEVIR-CD-256</t>
         </is>
       </c>
       <c r="E97" s="2" t="n">
-        <v>91.64</v>
+        <v>88.42</v>
       </c>
       <c r="F97" s="2" t="n">
-        <v>94.81999999999999</v>
+        <v>91.97</v>
       </c>
       <c r="G97" s="2" t="n">
-        <v>99.47</v>
+        <v>99.02</v>
       </c>
       <c r="H97" s="2" t="n">
-        <v>93.2</v>
+        <v>90.16</v>
       </c>
       <c r="I97" s="2" t="n">
-        <v>87.27</v>
+        <v>82.08</v>
       </c>
       <c r="J97" s="2" t="n">
-        <v>92.93000000000001</v>
+        <v>89.64</v>
       </c>
       <c r="K97" s="2" t="n">
         <v>3.455</v>
@@ -5634,17 +5630,17 @@
     <row r="98">
       <c r="A98" t="inlineStr">
         <is>
-          <t>UltraLight</t>
+          <t>STR-Fusion</t>
         </is>
       </c>
       <c r="B98" t="inlineStr">
         <is>
-          <t>Run4</t>
+          <t>Run2_TASS</t>
         </is>
       </c>
       <c r="C98" t="inlineStr">
         <is>
-          <t>R4_0_A0_FULL12_FROZEN</t>
+          <t>M1_TASS</t>
         </is>
       </c>
       <c r="D98" t="inlineStr">
@@ -5653,89 +5649,89 @@
         </is>
       </c>
       <c r="E98" s="2" t="n">
-        <v>82.42</v>
+        <v>78.73</v>
       </c>
       <c r="F98" s="2" t="n">
-        <v>83.87</v>
+        <v>84.98</v>
       </c>
       <c r="G98" s="2" t="n">
-        <v>92.12</v>
+        <v>91.7</v>
       </c>
       <c r="H98" s="2" t="n">
-        <v>83.14</v>
+        <v>81.73999999999999</v>
       </c>
       <c r="I98" s="2" t="n">
-        <v>71.14</v>
+        <v>69.11</v>
       </c>
       <c r="J98" s="2" t="n">
-        <v>77.98999999999999</v>
+        <v>76.38</v>
       </c>
       <c r="K98" s="2" t="n">
-        <v>11.754</v>
+        <v>3.455</v>
       </c>
       <c r="L98" s="2" t="n">
-        <v>15.125</v>
+        <v>1.478</v>
       </c>
       <c r="M98" s="2" t="n">
-        <v>26.3246</v>
+        <v>3.5459</v>
       </c>
       <c r="N98" t="inlineStr">
         <is>
-          <t>baseline</t>
+          <t>str_tass</t>
         </is>
       </c>
     </row>
     <row r="99">
       <c r="A99" t="inlineStr">
         <is>
-          <t>UltraLight</t>
+          <t>STR-Fusion</t>
         </is>
       </c>
       <c r="B99" t="inlineStr">
         <is>
-          <t>Run4</t>
+          <t>Run2_TASS</t>
         </is>
       </c>
       <c r="C99" t="inlineStr">
         <is>
-          <t>R4_1_VIT4_OLDHEAD</t>
+          <t>M1_TASS</t>
         </is>
       </c>
       <c r="D99" t="inlineStr">
         <is>
-          <t>SYSU-CD-256</t>
+          <t>WHU-CD-256</t>
         </is>
       </c>
       <c r="E99" s="2" t="n">
-        <v>82.15000000000001</v>
+        <v>91.64</v>
       </c>
       <c r="F99" s="2" t="n">
-        <v>83.40000000000001</v>
+        <v>94.81999999999999</v>
       </c>
       <c r="G99" s="2" t="n">
-        <v>91.94</v>
+        <v>99.47</v>
       </c>
       <c r="H99" s="2" t="n">
-        <v>82.77</v>
+        <v>93.2</v>
       </c>
       <c r="I99" s="2" t="n">
-        <v>70.61</v>
+        <v>87.27</v>
       </c>
       <c r="J99" s="2" t="n">
-        <v>77.51000000000001</v>
+        <v>92.93000000000001</v>
       </c>
       <c r="K99" s="2" t="n">
-        <v>8.195</v>
+        <v>3.455</v>
       </c>
       <c r="L99" s="2" t="n">
-        <v>15.125</v>
+        <v>1.478</v>
       </c>
       <c r="M99" s="2" t="n">
-        <v>24.1021</v>
+        <v>3.5459</v>
       </c>
       <c r="N99" t="inlineStr">
         <is>
-          <t>baseline</t>
+          <t>str_tass</t>
         </is>
       </c>
     </row>
@@ -5752,7 +5748,7 @@
       </c>
       <c r="C100" t="inlineStr">
         <is>
-          <t>R4_2_VIT4_LIGHTDETAIL</t>
+          <t>R4_0_A0_FULL12_FROZEN</t>
         </is>
       </c>
       <c r="D100" t="inlineStr">
@@ -5761,31 +5757,31 @@
         </is>
       </c>
       <c r="E100" s="2" t="n">
-        <v>79.94</v>
+        <v>82.42</v>
       </c>
       <c r="F100" s="2" t="n">
-        <v>84.79000000000001</v>
+        <v>83.87</v>
       </c>
       <c r="G100" s="2" t="n">
-        <v>91.89</v>
+        <v>92.12</v>
       </c>
       <c r="H100" s="2" t="n">
-        <v>82.3</v>
+        <v>83.14</v>
       </c>
       <c r="I100" s="2" t="n">
-        <v>69.92</v>
+        <v>71.14</v>
       </c>
       <c r="J100" s="2" t="n">
-        <v>77.04000000000001</v>
+        <v>77.98999999999999</v>
       </c>
       <c r="K100" s="2" t="n">
-        <v>5.492</v>
+        <v>11.754</v>
       </c>
       <c r="L100" s="2" t="n">
-        <v>3.515</v>
+        <v>15.125</v>
       </c>
       <c r="M100" s="2" t="n">
-        <v>10.7311</v>
+        <v>26.3246</v>
       </c>
       <c r="N100" t="inlineStr">
         <is>
@@ -5806,7 +5802,7 @@
       </c>
       <c r="C101" t="inlineStr">
         <is>
-          <t>R4_2b_VIT4_LIGHTDETAIL48</t>
+          <t>R4_1_VIT4_OLDHEAD</t>
         </is>
       </c>
       <c r="D101" t="inlineStr">
@@ -5815,31 +5811,31 @@
         </is>
       </c>
       <c r="E101" s="2" t="n">
-        <v>80.87</v>
+        <v>82.15000000000001</v>
       </c>
       <c r="F101" s="2" t="n">
-        <v>83.81</v>
+        <v>83.40000000000001</v>
       </c>
       <c r="G101" s="2" t="n">
-        <v>91.81</v>
+        <v>91.94</v>
       </c>
       <c r="H101" s="2" t="n">
-        <v>82.31999999999999</v>
+        <v>82.77</v>
       </c>
       <c r="I101" s="2" t="n">
-        <v>69.95</v>
+        <v>70.61</v>
       </c>
       <c r="J101" s="2" t="n">
-        <v>76.98999999999999</v>
+        <v>77.51000000000001</v>
       </c>
       <c r="K101" s="2" t="n">
-        <v>5.533</v>
+        <v>8.195</v>
       </c>
       <c r="L101" s="2" t="n">
-        <v>3.556</v>
+        <v>15.125</v>
       </c>
       <c r="M101" s="2" t="n">
-        <v>10.9824</v>
+        <v>24.1021</v>
       </c>
       <c r="N101" t="inlineStr">
         <is>
@@ -5860,7 +5856,7 @@
       </c>
       <c r="C102" t="inlineStr">
         <is>
-          <t>R4_2d_PSD_DETAIL</t>
+          <t>R4_2_VIT4_LIGHTDETAIL</t>
         </is>
       </c>
       <c r="D102" t="inlineStr">
@@ -5869,31 +5865,31 @@
         </is>
       </c>
       <c r="E102" s="2" t="n">
-        <v>79.78</v>
+        <v>79.94</v>
       </c>
       <c r="F102" s="2" t="n">
-        <v>84.39</v>
+        <v>84.79000000000001</v>
       </c>
       <c r="G102" s="2" t="n">
-        <v>91.75</v>
+        <v>91.89</v>
       </c>
       <c r="H102" s="2" t="n">
-        <v>82.02</v>
+        <v>82.3</v>
       </c>
       <c r="I102" s="2" t="n">
-        <v>69.52</v>
+        <v>69.92</v>
       </c>
       <c r="J102" s="2" t="n">
-        <v>76.68000000000001</v>
+        <v>77.04000000000001</v>
       </c>
       <c r="K102" s="2" t="n">
-        <v>5.491</v>
+        <v>5.492</v>
       </c>
       <c r="L102" s="2" t="n">
-        <v>3.514</v>
+        <v>3.515</v>
       </c>
       <c r="M102" s="2" t="n">
-        <v>11.5239</v>
+        <v>10.7311</v>
       </c>
       <c r="N102" t="inlineStr">
         <is>
@@ -5904,46 +5900,50 @@
     <row r="103">
       <c r="A103" t="inlineStr">
         <is>
-          <t>baseline</t>
+          <t>UltraLight</t>
         </is>
       </c>
       <c r="B103" t="inlineStr">
         <is>
-          <t>Run1</t>
-        </is>
-      </c>
-      <c r="C103" t="inlineStr"/>
+          <t>Run4</t>
+        </is>
+      </c>
+      <c r="C103" t="inlineStr">
+        <is>
+          <t>R4_2b_VIT4_LIGHTDETAIL48</t>
+        </is>
+      </c>
       <c r="D103" t="inlineStr">
         <is>
-          <t>CDD-CD-256</t>
+          <t>SYSU-CD-256</t>
         </is>
       </c>
       <c r="E103" s="2" t="n">
-        <v>97.72</v>
+        <v>80.87</v>
       </c>
       <c r="F103" s="2" t="n">
-        <v>97.78</v>
+        <v>83.81</v>
       </c>
       <c r="G103" s="2" t="n">
-        <v>99.44</v>
+        <v>91.81</v>
       </c>
       <c r="H103" s="2" t="n">
-        <v>97.75</v>
+        <v>82.31999999999999</v>
       </c>
       <c r="I103" s="2" t="n">
-        <v>95.59999999999999</v>
+        <v>69.95</v>
       </c>
       <c r="J103" s="2" t="n">
-        <v>97.43000000000001</v>
+        <v>76.98999999999999</v>
       </c>
       <c r="K103" s="2" t="n">
-        <v>11.754</v>
+        <v>5.533</v>
       </c>
       <c r="L103" s="2" t="n">
-        <v>20.661</v>
+        <v>3.556</v>
       </c>
       <c r="M103" s="2" t="n">
-        <v>26.3246</v>
+        <v>10.9824</v>
       </c>
       <c r="N103" t="inlineStr">
         <is>
@@ -5954,46 +5954,50 @@
     <row r="104">
       <c r="A104" t="inlineStr">
         <is>
-          <t>baseline</t>
+          <t>UltraLight</t>
         </is>
       </c>
       <c r="B104" t="inlineStr">
         <is>
-          <t>Run1</t>
-        </is>
-      </c>
-      <c r="C104" t="inlineStr"/>
+          <t>Run4</t>
+        </is>
+      </c>
+      <c r="C104" t="inlineStr">
+        <is>
+          <t>R4_2d_PSD_DETAIL</t>
+        </is>
+      </c>
       <c r="D104" t="inlineStr">
         <is>
-          <t>LEVIR-CD-256</t>
+          <t>SYSU-CD-256</t>
         </is>
       </c>
       <c r="E104" s="2" t="n">
-        <v>91.56999999999999</v>
+        <v>79.78</v>
       </c>
       <c r="F104" s="2" t="n">
-        <v>92.33</v>
+        <v>84.39</v>
       </c>
       <c r="G104" s="2" t="n">
-        <v>99.18000000000001</v>
+        <v>91.75</v>
       </c>
       <c r="H104" s="2" t="n">
-        <v>91.95</v>
+        <v>82.02</v>
       </c>
       <c r="I104" s="2" t="n">
-        <v>85.09999999999999</v>
+        <v>69.52</v>
       </c>
       <c r="J104" s="2" t="n">
-        <v>91.52</v>
+        <v>76.68000000000001</v>
       </c>
       <c r="K104" s="2" t="n">
-        <v>11.754</v>
+        <v>5.491</v>
       </c>
       <c r="L104" s="2" t="n">
-        <v>20.661</v>
+        <v>3.514</v>
       </c>
       <c r="M104" s="2" t="n">
-        <v>26.3246</v>
+        <v>11.5239</v>
       </c>
       <c r="N104" t="inlineStr">
         <is>
@@ -6015,26 +6019,26 @@
       <c r="C105" t="inlineStr"/>
       <c r="D105" t="inlineStr">
         <is>
-          <t>SYSU-CD-256</t>
+          <t>CDD-CD-256</t>
         </is>
       </c>
       <c r="E105" s="2" t="n">
-        <v>80.77</v>
+        <v>97.72</v>
       </c>
       <c r="F105" s="2" t="n">
-        <v>84.27</v>
+        <v>97.78</v>
       </c>
       <c r="G105" s="2" t="n">
-        <v>91.91</v>
+        <v>99.44</v>
       </c>
       <c r="H105" s="2" t="n">
-        <v>82.48</v>
+        <v>97.75</v>
       </c>
       <c r="I105" s="2" t="n">
-        <v>70.19</v>
+        <v>95.59999999999999</v>
       </c>
       <c r="J105" s="2" t="n">
-        <v>77.23</v>
+        <v>97.43000000000001</v>
       </c>
       <c r="K105" s="2" t="n">
         <v>11.754</v>
@@ -6065,26 +6069,26 @@
       <c r="C106" t="inlineStr"/>
       <c r="D106" t="inlineStr">
         <is>
-          <t>WHU-CD-256</t>
+          <t>LEVIR-CD-256</t>
         </is>
       </c>
       <c r="E106" s="2" t="n">
-        <v>93.62</v>
+        <v>91.56999999999999</v>
       </c>
       <c r="F106" s="2" t="n">
-        <v>96.09</v>
+        <v>92.33</v>
       </c>
       <c r="G106" s="2" t="n">
-        <v>99.59999999999999</v>
+        <v>99.18000000000001</v>
       </c>
       <c r="H106" s="2" t="n">
-        <v>94.84</v>
+        <v>91.95</v>
       </c>
       <c r="I106" s="2" t="n">
-        <v>90.18000000000001</v>
+        <v>85.09999999999999</v>
       </c>
       <c r="J106" s="2" t="n">
-        <v>94.63</v>
+        <v>91.52</v>
       </c>
       <c r="K106" s="2" t="n">
         <v>11.754</v>
@@ -6101,8 +6105,108 @@
         </is>
       </c>
     </row>
+    <row r="107">
+      <c r="A107" t="inlineStr">
+        <is>
+          <t>baseline</t>
+        </is>
+      </c>
+      <c r="B107" t="inlineStr">
+        <is>
+          <t>Run1</t>
+        </is>
+      </c>
+      <c r="C107" t="inlineStr"/>
+      <c r="D107" t="inlineStr">
+        <is>
+          <t>SYSU-CD-256</t>
+        </is>
+      </c>
+      <c r="E107" s="2" t="n">
+        <v>80.77</v>
+      </c>
+      <c r="F107" s="2" t="n">
+        <v>84.27</v>
+      </c>
+      <c r="G107" s="2" t="n">
+        <v>91.91</v>
+      </c>
+      <c r="H107" s="2" t="n">
+        <v>82.48</v>
+      </c>
+      <c r="I107" s="2" t="n">
+        <v>70.19</v>
+      </c>
+      <c r="J107" s="2" t="n">
+        <v>77.23</v>
+      </c>
+      <c r="K107" s="2" t="n">
+        <v>11.754</v>
+      </c>
+      <c r="L107" s="2" t="n">
+        <v>20.661</v>
+      </c>
+      <c r="M107" s="2" t="n">
+        <v>26.3246</v>
+      </c>
+      <c r="N107" t="inlineStr">
+        <is>
+          <t>baseline</t>
+        </is>
+      </c>
+    </row>
+    <row r="108">
+      <c r="A108" t="inlineStr">
+        <is>
+          <t>baseline</t>
+        </is>
+      </c>
+      <c r="B108" t="inlineStr">
+        <is>
+          <t>Run1</t>
+        </is>
+      </c>
+      <c r="C108" t="inlineStr"/>
+      <c r="D108" t="inlineStr">
+        <is>
+          <t>WHU-CD-256</t>
+        </is>
+      </c>
+      <c r="E108" s="2" t="n">
+        <v>93.62</v>
+      </c>
+      <c r="F108" s="2" t="n">
+        <v>96.09</v>
+      </c>
+      <c r="G108" s="2" t="n">
+        <v>99.59999999999999</v>
+      </c>
+      <c r="H108" s="2" t="n">
+        <v>94.84</v>
+      </c>
+      <c r="I108" s="2" t="n">
+        <v>90.18000000000001</v>
+      </c>
+      <c r="J108" s="2" t="n">
+        <v>94.63</v>
+      </c>
+      <c r="K108" s="2" t="n">
+        <v>11.754</v>
+      </c>
+      <c r="L108" s="2" t="n">
+        <v>20.661</v>
+      </c>
+      <c r="M108" s="2" t="n">
+        <v>26.3246</v>
+      </c>
+      <c r="N108" t="inlineStr">
+        <is>
+          <t>baseline</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:N106"/>
+  <autoFilter ref="A1:N108"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Record Run2 LEVIR control results
</commit_message>
<xml_diff>
--- a/docs/experiment_metrics.xlsx
+++ b/docs/experiment_metrics.xlsx
@@ -10,7 +10,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="metrics" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'metrics'!$A$1:$N$108</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'metrics'!$A$1:$N$109</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -420,7 +420,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N108"/>
+  <dimension ref="A1:N109"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -4575,26 +4575,26 @@
       </c>
       <c r="D78" t="inlineStr">
         <is>
-          <t>SYSU-CD-256</t>
+          <t>LEVIR-CD-256</t>
         </is>
       </c>
       <c r="E78" s="2" t="n">
-        <v>80.39</v>
+        <v>91.2</v>
       </c>
       <c r="F78" s="2" t="n">
-        <v>82.89</v>
+        <v>91.72</v>
       </c>
       <c r="G78" s="2" t="n">
+        <v>99.13</v>
+      </c>
+      <c r="H78" s="2" t="n">
         <v>91.45999999999999</v>
       </c>
-      <c r="H78" s="2" t="n">
-        <v>81.62</v>
-      </c>
       <c r="I78" s="2" t="n">
-        <v>68.95</v>
+        <v>84.26000000000001</v>
       </c>
       <c r="J78" s="2" t="n">
-        <v>76.06999999999999</v>
+        <v>91</v>
       </c>
       <c r="K78" s="2" t="n">
         <v>3.016737</v>
@@ -4622,42 +4622,42 @@
       </c>
       <c r="C79" t="inlineStr">
         <is>
-          <t>M1_HYPER_QKV</t>
+          <t>M0_CTRL</t>
         </is>
       </c>
       <c r="D79" t="inlineStr">
         <is>
-          <t>LEVIR-CD-256</t>
+          <t>SYSU-CD-256</t>
         </is>
       </c>
       <c r="E79" s="2" t="n">
-        <v>90.55</v>
+        <v>80.39</v>
       </c>
       <c r="F79" s="2" t="n">
-        <v>92.03</v>
+        <v>82.89</v>
       </c>
       <c r="G79" s="2" t="n">
-        <v>99.12</v>
+        <v>91.45999999999999</v>
       </c>
       <c r="H79" s="2" t="n">
-        <v>91.28</v>
+        <v>81.62</v>
       </c>
       <c r="I79" s="2" t="n">
-        <v>83.95999999999999</v>
+        <v>68.95</v>
       </c>
       <c r="J79" s="2" t="n">
-        <v>90.81999999999999</v>
+        <v>76.06999999999999</v>
       </c>
       <c r="K79" s="2" t="n">
-        <v>3.049509</v>
+        <v>3.016737</v>
       </c>
       <c r="L79" s="2" t="n">
-        <v>3.133176</v>
+        <v>3.100404</v>
       </c>
       <c r="M79" s="2" t="n"/>
       <c r="N79" t="inlineStr">
         <is>
-          <t>casa_wdmf_str_hyperbolic</t>
+          <t>casa_wdmf_str_none</t>
         </is>
       </c>
     </row>
@@ -4679,26 +4679,26 @@
       </c>
       <c r="D80" t="inlineStr">
         <is>
-          <t>SYSU-CD-256</t>
+          <t>LEVIR-CD-256</t>
         </is>
       </c>
       <c r="E80" s="2" t="n">
-        <v>78.67</v>
+        <v>90.55</v>
       </c>
       <c r="F80" s="2" t="n">
-        <v>85.08</v>
+        <v>92.03</v>
       </c>
       <c r="G80" s="2" t="n">
-        <v>91.72</v>
+        <v>99.12</v>
       </c>
       <c r="H80" s="2" t="n">
-        <v>81.75</v>
+        <v>91.28</v>
       </c>
       <c r="I80" s="2" t="n">
-        <v>69.13</v>
+        <v>83.95999999999999</v>
       </c>
       <c r="J80" s="2" t="n">
-        <v>76.40000000000001</v>
+        <v>90.81999999999999</v>
       </c>
       <c r="K80" s="2" t="n">
         <v>3.049509</v>
@@ -4726,31 +4726,31 @@
       </c>
       <c r="C81" t="inlineStr">
         <is>
-          <t>M2_CA_QKV</t>
+          <t>M1_HYPER_QKV</t>
         </is>
       </c>
       <c r="D81" t="inlineStr">
         <is>
-          <t>LEVIR-CD-256</t>
+          <t>SYSU-CD-256</t>
         </is>
       </c>
       <c r="E81" s="2" t="n">
-        <v>89.72</v>
+        <v>78.67</v>
       </c>
       <c r="F81" s="2" t="n">
-        <v>93.12</v>
+        <v>85.08</v>
       </c>
       <c r="G81" s="2" t="n">
-        <v>99.14</v>
+        <v>91.72</v>
       </c>
       <c r="H81" s="2" t="n">
-        <v>91.39</v>
+        <v>81.75</v>
       </c>
       <c r="I81" s="2" t="n">
-        <v>84.14</v>
+        <v>69.13</v>
       </c>
       <c r="J81" s="2" t="n">
-        <v>90.93000000000001</v>
+        <v>76.40000000000001</v>
       </c>
       <c r="K81" s="2" t="n">
         <v>3.049509</v>
@@ -4761,7 +4761,7 @@
       <c r="M81" s="2" t="n"/>
       <c r="N81" t="inlineStr">
         <is>
-          <t>casa_wdmf_str_qkv</t>
+          <t>casa_wdmf_str_hyperbolic</t>
         </is>
       </c>
     </row>
@@ -4783,26 +4783,26 @@
       </c>
       <c r="D82" t="inlineStr">
         <is>
-          <t>SYSU-CD-256</t>
+          <t>LEVIR-CD-256</t>
         </is>
       </c>
       <c r="E82" s="2" t="n">
-        <v>82.83</v>
+        <v>89.72</v>
       </c>
       <c r="F82" s="2" t="n">
-        <v>82.86</v>
+        <v>93.12</v>
       </c>
       <c r="G82" s="2" t="n">
-        <v>91.91</v>
+        <v>99.14</v>
       </c>
       <c r="H82" s="2" t="n">
-        <v>82.84999999999999</v>
+        <v>91.39</v>
       </c>
       <c r="I82" s="2" t="n">
-        <v>70.72</v>
+        <v>84.14</v>
       </c>
       <c r="J82" s="2" t="n">
-        <v>77.56</v>
+        <v>90.93000000000001</v>
       </c>
       <c r="K82" s="2" t="n">
         <v>3.049509</v>
@@ -4820,54 +4820,52 @@
     <row r="83">
       <c r="A83" t="inlineStr">
         <is>
-          <t>CASAA</t>
+          <t>CASA-WDMF</t>
         </is>
       </c>
       <c r="B83" t="inlineStr">
         <is>
-          <t>Run1</t>
+          <t>Run2</t>
         </is>
       </c>
       <c r="C83" t="inlineStr">
         <is>
-          <t>A1_SAA</t>
+          <t>M2_CA_QKV</t>
         </is>
       </c>
       <c r="D83" t="inlineStr">
         <is>
-          <t>LEVIR-CD-256</t>
+          <t>SYSU-CD-256</t>
         </is>
       </c>
       <c r="E83" s="2" t="n">
-        <v>91.09</v>
+        <v>82.83</v>
       </c>
       <c r="F83" s="2" t="n">
-        <v>92.8</v>
+        <v>82.86</v>
       </c>
       <c r="G83" s="2" t="n">
-        <v>99.19</v>
+        <v>91.91</v>
       </c>
       <c r="H83" s="2" t="n">
-        <v>91.94</v>
+        <v>82.84999999999999</v>
       </c>
       <c r="I83" s="2" t="n">
-        <v>85.08</v>
+        <v>70.72</v>
       </c>
       <c r="J83" s="2" t="n">
-        <v>91.51000000000001</v>
+        <v>77.56</v>
       </c>
       <c r="K83" s="2" t="n">
-        <v>11.754</v>
+        <v>3.049509</v>
       </c>
       <c r="L83" s="2" t="n">
-        <v>20.661</v>
-      </c>
-      <c r="M83" s="2" t="n">
-        <v>26.3183</v>
-      </c>
+        <v>3.133176</v>
+      </c>
+      <c r="M83" s="2" t="n"/>
       <c r="N83" t="inlineStr">
         <is>
-          <t>saa</t>
+          <t>casa_wdmf_str_qkv</t>
         </is>
       </c>
     </row>
@@ -4889,26 +4887,26 @@
       </c>
       <c r="D84" t="inlineStr">
         <is>
-          <t>SYSU-CD-256</t>
+          <t>LEVIR-CD-256</t>
         </is>
       </c>
       <c r="E84" s="2" t="n">
-        <v>80.3</v>
+        <v>91.09</v>
       </c>
       <c r="F84" s="2" t="n">
-        <v>84.81</v>
+        <v>92.8</v>
       </c>
       <c r="G84" s="2" t="n">
-        <v>91.95999999999999</v>
+        <v>99.19</v>
       </c>
       <c r="H84" s="2" t="n">
-        <v>82.5</v>
+        <v>91.94</v>
       </c>
       <c r="I84" s="2" t="n">
-        <v>70.20999999999999</v>
+        <v>85.08</v>
       </c>
       <c r="J84" s="2" t="n">
-        <v>77.29000000000001</v>
+        <v>91.51000000000001</v>
       </c>
       <c r="K84" s="2" t="n">
         <v>11.754</v>
@@ -4938,31 +4936,31 @@
       </c>
       <c r="C85" t="inlineStr">
         <is>
-          <t>A2_CASAA</t>
+          <t>A1_SAA</t>
         </is>
       </c>
       <c r="D85" t="inlineStr">
         <is>
-          <t>LEVIR-CD-256</t>
+          <t>SYSU-CD-256</t>
         </is>
       </c>
       <c r="E85" s="2" t="n">
-        <v>90.98999999999999</v>
+        <v>80.3</v>
       </c>
       <c r="F85" s="2" t="n">
-        <v>92.75</v>
+        <v>84.81</v>
       </c>
       <c r="G85" s="2" t="n">
-        <v>99.18000000000001</v>
+        <v>91.95999999999999</v>
       </c>
       <c r="H85" s="2" t="n">
-        <v>91.86</v>
+        <v>82.5</v>
       </c>
       <c r="I85" s="2" t="n">
-        <v>84.94</v>
+        <v>70.20999999999999</v>
       </c>
       <c r="J85" s="2" t="n">
-        <v>91.43000000000001</v>
+        <v>77.29000000000001</v>
       </c>
       <c r="K85" s="2" t="n">
         <v>11.754</v>
@@ -4971,11 +4969,11 @@
         <v>20.661</v>
       </c>
       <c r="M85" s="2" t="n">
-        <v>26.2593</v>
+        <v>26.3183</v>
       </c>
       <c r="N85" t="inlineStr">
         <is>
-          <t>casaa</t>
+          <t>saa</t>
         </is>
       </c>
     </row>
@@ -4997,26 +4995,26 @@
       </c>
       <c r="D86" t="inlineStr">
         <is>
-          <t>SYSU-CD-256</t>
+          <t>LEVIR-CD-256</t>
         </is>
       </c>
       <c r="E86" s="2" t="n">
-        <v>80.55</v>
+        <v>90.98999999999999</v>
       </c>
       <c r="F86" s="2" t="n">
-        <v>84.23</v>
+        <v>92.75</v>
       </c>
       <c r="G86" s="2" t="n">
+        <v>99.18000000000001</v>
+      </c>
+      <c r="H86" s="2" t="n">
         <v>91.86</v>
       </c>
-      <c r="H86" s="2" t="n">
-        <v>82.34999999999999</v>
-      </c>
       <c r="I86" s="2" t="n">
-        <v>70</v>
+        <v>84.94</v>
       </c>
       <c r="J86" s="2" t="n">
-        <v>77.06</v>
+        <v>91.43000000000001</v>
       </c>
       <c r="K86" s="2" t="n">
         <v>11.754</v>
@@ -5041,49 +5039,49 @@
       </c>
       <c r="B87" t="inlineStr">
         <is>
-          <t>Run2</t>
+          <t>Run1</t>
         </is>
       </c>
       <c r="C87" t="inlineStr">
         <is>
-          <t>A1_SAA_FROZEN</t>
+          <t>A2_CASAA</t>
         </is>
       </c>
       <c r="D87" t="inlineStr">
         <is>
-          <t>LEVIR-CD-256</t>
+          <t>SYSU-CD-256</t>
         </is>
       </c>
       <c r="E87" s="2" t="n">
-        <v>91.38</v>
+        <v>80.55</v>
       </c>
       <c r="F87" s="2" t="n">
-        <v>92.3</v>
+        <v>84.23</v>
       </c>
       <c r="G87" s="2" t="n">
-        <v>99.17</v>
+        <v>91.86</v>
       </c>
       <c r="H87" s="2" t="n">
-        <v>91.84</v>
+        <v>82.34999999999999</v>
       </c>
       <c r="I87" s="2" t="n">
-        <v>84.91</v>
+        <v>70</v>
       </c>
       <c r="J87" s="2" t="n">
-        <v>91.40000000000001</v>
+        <v>77.06</v>
       </c>
       <c r="K87" s="2" t="n">
         <v>11.754</v>
       </c>
       <c r="L87" s="2" t="n">
-        <v>15.125</v>
+        <v>20.661</v>
       </c>
       <c r="M87" s="2" t="n">
-        <v>26.1484</v>
+        <v>26.2593</v>
       </c>
       <c r="N87" t="inlineStr">
         <is>
-          <t>saa</t>
+          <t>casaa</t>
         </is>
       </c>
     </row>
@@ -5105,26 +5103,26 @@
       </c>
       <c r="D88" t="inlineStr">
         <is>
-          <t>SYSU-CD-256</t>
+          <t>LEVIR-CD-256</t>
         </is>
       </c>
       <c r="E88" s="2" t="n">
-        <v>78.40000000000001</v>
+        <v>91.38</v>
       </c>
       <c r="F88" s="2" t="n">
-        <v>86.03</v>
+        <v>92.3</v>
       </c>
       <c r="G88" s="2" t="n">
-        <v>91.90000000000001</v>
+        <v>99.17</v>
       </c>
       <c r="H88" s="2" t="n">
-        <v>82.04000000000001</v>
+        <v>91.84</v>
       </c>
       <c r="I88" s="2" t="n">
-        <v>69.55</v>
+        <v>84.91</v>
       </c>
       <c r="J88" s="2" t="n">
-        <v>76.83</v>
+        <v>91.40000000000001</v>
       </c>
       <c r="K88" s="2" t="n">
         <v>11.754</v>
@@ -5154,31 +5152,31 @@
       </c>
       <c r="C89" t="inlineStr">
         <is>
-          <t>A3_ORACLE_FROZEN</t>
+          <t>A1_SAA_FROZEN</t>
         </is>
       </c>
       <c r="D89" t="inlineStr">
         <is>
-          <t>LEVIR-CD-256</t>
+          <t>SYSU-CD-256</t>
         </is>
       </c>
       <c r="E89" s="2" t="n">
-        <v>91.13</v>
+        <v>78.40000000000001</v>
       </c>
       <c r="F89" s="2" t="n">
-        <v>92.65000000000001</v>
+        <v>86.03</v>
       </c>
       <c r="G89" s="2" t="n">
-        <v>99.18000000000001</v>
+        <v>91.90000000000001</v>
       </c>
       <c r="H89" s="2" t="n">
-        <v>91.88</v>
+        <v>82.04000000000001</v>
       </c>
       <c r="I89" s="2" t="n">
-        <v>84.98</v>
+        <v>69.55</v>
       </c>
       <c r="J89" s="2" t="n">
-        <v>91.45</v>
+        <v>76.83</v>
       </c>
       <c r="K89" s="2" t="n">
         <v>11.754</v>
@@ -5187,11 +5185,11 @@
         <v>15.125</v>
       </c>
       <c r="M89" s="2" t="n">
-        <v>26.0894</v>
+        <v>26.1484</v>
       </c>
       <c r="N89" t="inlineStr">
         <is>
-          <t>casaa</t>
+          <t>saa</t>
         </is>
       </c>
     </row>
@@ -5213,26 +5211,26 @@
       </c>
       <c r="D90" t="inlineStr">
         <is>
-          <t>SYSU-CD-256</t>
+          <t>LEVIR-CD-256</t>
         </is>
       </c>
       <c r="E90" s="2" t="n">
-        <v>82.04000000000001</v>
+        <v>91.13</v>
       </c>
       <c r="F90" s="2" t="n">
-        <v>85.05</v>
+        <v>92.65000000000001</v>
       </c>
       <c r="G90" s="2" t="n">
-        <v>92.36</v>
+        <v>99.18000000000001</v>
       </c>
       <c r="H90" s="2" t="n">
-        <v>83.52</v>
+        <v>91.88</v>
       </c>
       <c r="I90" s="2" t="n">
-        <v>71.7</v>
+        <v>84.98</v>
       </c>
       <c r="J90" s="2" t="n">
-        <v>78.55</v>
+        <v>91.45</v>
       </c>
       <c r="K90" s="2" t="n">
         <v>11.754</v>
@@ -5257,12 +5255,12 @@
       </c>
       <c r="B91" t="inlineStr">
         <is>
-          <t>Run3</t>
+          <t>Run2</t>
         </is>
       </c>
       <c r="C91" t="inlineStr">
         <is>
-          <t>A4_DETAIL_FROZEN</t>
+          <t>A3_ORACLE_FROZEN</t>
         </is>
       </c>
       <c r="D91" t="inlineStr">
@@ -5271,22 +5269,22 @@
         </is>
       </c>
       <c r="E91" s="2" t="n">
-        <v>79.68000000000001</v>
+        <v>82.04000000000001</v>
       </c>
       <c r="F91" s="2" t="n">
-        <v>84.28</v>
+        <v>85.05</v>
       </c>
       <c r="G91" s="2" t="n">
-        <v>91.7</v>
+        <v>92.36</v>
       </c>
       <c r="H91" s="2" t="n">
-        <v>81.92</v>
+        <v>83.52</v>
       </c>
       <c r="I91" s="2" t="n">
-        <v>69.37</v>
+        <v>71.7</v>
       </c>
       <c r="J91" s="2" t="n">
-        <v>76.54000000000001</v>
+        <v>78.55</v>
       </c>
       <c r="K91" s="2" t="n">
         <v>11.754</v>
@@ -5306,54 +5304,54 @@
     <row r="92">
       <c r="A92" t="inlineStr">
         <is>
-          <t>STR-Fusion</t>
+          <t>CASAA</t>
         </is>
       </c>
       <c r="B92" t="inlineStr">
         <is>
-          <t>Run2_TASS</t>
+          <t>Run3</t>
         </is>
       </c>
       <c r="C92" t="inlineStr">
         <is>
-          <t>C0_TOKEN</t>
+          <t>A4_DETAIL_FROZEN</t>
         </is>
       </c>
       <c r="D92" t="inlineStr">
         <is>
-          <t>CDD-CD-256</t>
+          <t>SYSU-CD-256</t>
         </is>
       </c>
       <c r="E92" s="2" t="n">
-        <v>93.13</v>
+        <v>79.68000000000001</v>
       </c>
       <c r="F92" s="2" t="n">
-        <v>95.16</v>
+        <v>84.28</v>
       </c>
       <c r="G92" s="2" t="n">
-        <v>98.56999999999999</v>
+        <v>91.7</v>
       </c>
       <c r="H92" s="2" t="n">
-        <v>94.13</v>
+        <v>81.92</v>
       </c>
       <c r="I92" s="2" t="n">
-        <v>88.91</v>
+        <v>69.37</v>
       </c>
       <c r="J92" s="2" t="n">
-        <v>93.31999999999999</v>
+        <v>76.54000000000001</v>
       </c>
       <c r="K92" s="2" t="n">
-        <v>2.596</v>
+        <v>11.754</v>
       </c>
       <c r="L92" s="2" t="n">
-        <v>0.62</v>
+        <v>15.125</v>
       </c>
       <c r="M92" s="2" t="n">
-        <v>2.2136</v>
+        <v>26.0894</v>
       </c>
       <c r="N92" t="inlineStr">
         <is>
-          <t>str_tass</t>
+          <t>casaa</t>
         </is>
       </c>
     </row>
@@ -5375,26 +5373,26 @@
       </c>
       <c r="D93" t="inlineStr">
         <is>
-          <t>LEVIR-CD-256</t>
+          <t>CDD-CD-256</t>
         </is>
       </c>
       <c r="E93" s="2" t="n">
-        <v>86.37</v>
+        <v>93.13</v>
       </c>
       <c r="F93" s="2" t="n">
-        <v>89.25</v>
+        <v>95.16</v>
       </c>
       <c r="G93" s="2" t="n">
-        <v>98.78</v>
+        <v>98.56999999999999</v>
       </c>
       <c r="H93" s="2" t="n">
-        <v>87.79000000000001</v>
+        <v>94.13</v>
       </c>
       <c r="I93" s="2" t="n">
-        <v>78.23999999999999</v>
+        <v>88.91</v>
       </c>
       <c r="J93" s="2" t="n">
-        <v>87.14</v>
+        <v>93.31999999999999</v>
       </c>
       <c r="K93" s="2" t="n">
         <v>2.596</v>
@@ -5429,26 +5427,26 @@
       </c>
       <c r="D94" t="inlineStr">
         <is>
-          <t>SYSU-CD-256</t>
+          <t>LEVIR-CD-256</t>
         </is>
       </c>
       <c r="E94" s="2" t="n">
-        <v>79.93000000000001</v>
+        <v>86.37</v>
       </c>
       <c r="F94" s="2" t="n">
-        <v>84.5</v>
+        <v>89.25</v>
       </c>
       <c r="G94" s="2" t="n">
-        <v>91.81</v>
+        <v>98.78</v>
       </c>
       <c r="H94" s="2" t="n">
-        <v>82.15000000000001</v>
+        <v>87.79000000000001</v>
       </c>
       <c r="I94" s="2" t="n">
-        <v>69.70999999999999</v>
+        <v>78.23999999999999</v>
       </c>
       <c r="J94" s="2" t="n">
-        <v>76.84</v>
+        <v>87.14</v>
       </c>
       <c r="K94" s="2" t="n">
         <v>2.596</v>
@@ -5483,26 +5481,26 @@
       </c>
       <c r="D95" t="inlineStr">
         <is>
-          <t>WHU-CD-256</t>
+          <t>SYSU-CD-256</t>
         </is>
       </c>
       <c r="E95" s="2" t="n">
-        <v>90.16</v>
+        <v>79.93000000000001</v>
       </c>
       <c r="F95" s="2" t="n">
-        <v>93.97</v>
+        <v>84.5</v>
       </c>
       <c r="G95" s="2" t="n">
-        <v>99.38</v>
+        <v>91.81</v>
       </c>
       <c r="H95" s="2" t="n">
-        <v>92.02</v>
+        <v>82.15000000000001</v>
       </c>
       <c r="I95" s="2" t="n">
-        <v>85.23</v>
+        <v>69.70999999999999</v>
       </c>
       <c r="J95" s="2" t="n">
-        <v>91.7</v>
+        <v>76.84</v>
       </c>
       <c r="K95" s="2" t="n">
         <v>2.596</v>
@@ -5532,40 +5530,40 @@
       </c>
       <c r="C96" t="inlineStr">
         <is>
-          <t>M1_TASS</t>
+          <t>C0_TOKEN</t>
         </is>
       </c>
       <c r="D96" t="inlineStr">
         <is>
-          <t>CDD-CD-256</t>
+          <t>WHU-CD-256</t>
         </is>
       </c>
       <c r="E96" s="2" t="n">
-        <v>94.7</v>
+        <v>90.16</v>
       </c>
       <c r="F96" s="2" t="n">
-        <v>96.13</v>
+        <v>93.97</v>
       </c>
       <c r="G96" s="2" t="n">
-        <v>98.88</v>
+        <v>99.38</v>
       </c>
       <c r="H96" s="2" t="n">
-        <v>95.41</v>
+        <v>92.02</v>
       </c>
       <c r="I96" s="2" t="n">
-        <v>91.22</v>
+        <v>85.23</v>
       </c>
       <c r="J96" s="2" t="n">
-        <v>94.77</v>
+        <v>91.7</v>
       </c>
       <c r="K96" s="2" t="n">
-        <v>3.455</v>
+        <v>2.596</v>
       </c>
       <c r="L96" s="2" t="n">
-        <v>1.478</v>
+        <v>0.62</v>
       </c>
       <c r="M96" s="2" t="n">
-        <v>3.5459</v>
+        <v>2.2136</v>
       </c>
       <c r="N96" t="inlineStr">
         <is>
@@ -5591,26 +5589,26 @@
       </c>
       <c r="D97" t="inlineStr">
         <is>
-          <t>LEVIR-CD-256</t>
+          <t>CDD-CD-256</t>
         </is>
       </c>
       <c r="E97" s="2" t="n">
-        <v>88.42</v>
+        <v>94.7</v>
       </c>
       <c r="F97" s="2" t="n">
-        <v>91.97</v>
+        <v>96.13</v>
       </c>
       <c r="G97" s="2" t="n">
-        <v>99.02</v>
+        <v>98.88</v>
       </c>
       <c r="H97" s="2" t="n">
-        <v>90.16</v>
+        <v>95.41</v>
       </c>
       <c r="I97" s="2" t="n">
-        <v>82.08</v>
+        <v>91.22</v>
       </c>
       <c r="J97" s="2" t="n">
-        <v>89.64</v>
+        <v>94.77</v>
       </c>
       <c r="K97" s="2" t="n">
         <v>3.455</v>
@@ -5645,26 +5643,26 @@
       </c>
       <c r="D98" t="inlineStr">
         <is>
-          <t>SYSU-CD-256</t>
+          <t>LEVIR-CD-256</t>
         </is>
       </c>
       <c r="E98" s="2" t="n">
-        <v>78.73</v>
+        <v>88.42</v>
       </c>
       <c r="F98" s="2" t="n">
-        <v>84.98</v>
+        <v>91.97</v>
       </c>
       <c r="G98" s="2" t="n">
-        <v>91.7</v>
+        <v>99.02</v>
       </c>
       <c r="H98" s="2" t="n">
-        <v>81.73999999999999</v>
+        <v>90.16</v>
       </c>
       <c r="I98" s="2" t="n">
-        <v>69.11</v>
+        <v>82.08</v>
       </c>
       <c r="J98" s="2" t="n">
-        <v>76.38</v>
+        <v>89.64</v>
       </c>
       <c r="K98" s="2" t="n">
         <v>3.455</v>
@@ -5699,26 +5697,26 @@
       </c>
       <c r="D99" t="inlineStr">
         <is>
-          <t>WHU-CD-256</t>
+          <t>SYSU-CD-256</t>
         </is>
       </c>
       <c r="E99" s="2" t="n">
-        <v>91.64</v>
+        <v>78.73</v>
       </c>
       <c r="F99" s="2" t="n">
-        <v>94.81999999999999</v>
+        <v>84.98</v>
       </c>
       <c r="G99" s="2" t="n">
-        <v>99.47</v>
+        <v>91.7</v>
       </c>
       <c r="H99" s="2" t="n">
-        <v>93.2</v>
+        <v>81.73999999999999</v>
       </c>
       <c r="I99" s="2" t="n">
-        <v>87.27</v>
+        <v>69.11</v>
       </c>
       <c r="J99" s="2" t="n">
-        <v>92.93000000000001</v>
+        <v>76.38</v>
       </c>
       <c r="K99" s="2" t="n">
         <v>3.455</v>
@@ -5738,54 +5736,54 @@
     <row r="100">
       <c r="A100" t="inlineStr">
         <is>
-          <t>UltraLight</t>
+          <t>STR-Fusion</t>
         </is>
       </c>
       <c r="B100" t="inlineStr">
         <is>
-          <t>Run4</t>
+          <t>Run2_TASS</t>
         </is>
       </c>
       <c r="C100" t="inlineStr">
         <is>
-          <t>R4_0_A0_FULL12_FROZEN</t>
+          <t>M1_TASS</t>
         </is>
       </c>
       <c r="D100" t="inlineStr">
         <is>
-          <t>SYSU-CD-256</t>
+          <t>WHU-CD-256</t>
         </is>
       </c>
       <c r="E100" s="2" t="n">
-        <v>82.42</v>
+        <v>91.64</v>
       </c>
       <c r="F100" s="2" t="n">
-        <v>83.87</v>
+        <v>94.81999999999999</v>
       </c>
       <c r="G100" s="2" t="n">
-        <v>92.12</v>
+        <v>99.47</v>
       </c>
       <c r="H100" s="2" t="n">
-        <v>83.14</v>
+        <v>93.2</v>
       </c>
       <c r="I100" s="2" t="n">
-        <v>71.14</v>
+        <v>87.27</v>
       </c>
       <c r="J100" s="2" t="n">
-        <v>77.98999999999999</v>
+        <v>92.93000000000001</v>
       </c>
       <c r="K100" s="2" t="n">
-        <v>11.754</v>
+        <v>3.455</v>
       </c>
       <c r="L100" s="2" t="n">
-        <v>15.125</v>
+        <v>1.478</v>
       </c>
       <c r="M100" s="2" t="n">
-        <v>26.3246</v>
+        <v>3.5459</v>
       </c>
       <c r="N100" t="inlineStr">
         <is>
-          <t>baseline</t>
+          <t>str_tass</t>
         </is>
       </c>
     </row>
@@ -5802,7 +5800,7 @@
       </c>
       <c r="C101" t="inlineStr">
         <is>
-          <t>R4_1_VIT4_OLDHEAD</t>
+          <t>R4_0_A0_FULL12_FROZEN</t>
         </is>
       </c>
       <c r="D101" t="inlineStr">
@@ -5811,31 +5809,31 @@
         </is>
       </c>
       <c r="E101" s="2" t="n">
-        <v>82.15000000000001</v>
+        <v>82.42</v>
       </c>
       <c r="F101" s="2" t="n">
-        <v>83.40000000000001</v>
+        <v>83.87</v>
       </c>
       <c r="G101" s="2" t="n">
-        <v>91.94</v>
+        <v>92.12</v>
       </c>
       <c r="H101" s="2" t="n">
-        <v>82.77</v>
+        <v>83.14</v>
       </c>
       <c r="I101" s="2" t="n">
-        <v>70.61</v>
+        <v>71.14</v>
       </c>
       <c r="J101" s="2" t="n">
-        <v>77.51000000000001</v>
+        <v>77.98999999999999</v>
       </c>
       <c r="K101" s="2" t="n">
-        <v>8.195</v>
+        <v>11.754</v>
       </c>
       <c r="L101" s="2" t="n">
         <v>15.125</v>
       </c>
       <c r="M101" s="2" t="n">
-        <v>24.1021</v>
+        <v>26.3246</v>
       </c>
       <c r="N101" t="inlineStr">
         <is>
@@ -5856,7 +5854,7 @@
       </c>
       <c r="C102" t="inlineStr">
         <is>
-          <t>R4_2_VIT4_LIGHTDETAIL</t>
+          <t>R4_1_VIT4_OLDHEAD</t>
         </is>
       </c>
       <c r="D102" t="inlineStr">
@@ -5865,31 +5863,31 @@
         </is>
       </c>
       <c r="E102" s="2" t="n">
-        <v>79.94</v>
+        <v>82.15000000000001</v>
       </c>
       <c r="F102" s="2" t="n">
-        <v>84.79000000000001</v>
+        <v>83.40000000000001</v>
       </c>
       <c r="G102" s="2" t="n">
-        <v>91.89</v>
+        <v>91.94</v>
       </c>
       <c r="H102" s="2" t="n">
-        <v>82.3</v>
+        <v>82.77</v>
       </c>
       <c r="I102" s="2" t="n">
-        <v>69.92</v>
+        <v>70.61</v>
       </c>
       <c r="J102" s="2" t="n">
-        <v>77.04000000000001</v>
+        <v>77.51000000000001</v>
       </c>
       <c r="K102" s="2" t="n">
-        <v>5.492</v>
+        <v>8.195</v>
       </c>
       <c r="L102" s="2" t="n">
-        <v>3.515</v>
+        <v>15.125</v>
       </c>
       <c r="M102" s="2" t="n">
-        <v>10.7311</v>
+        <v>24.1021</v>
       </c>
       <c r="N102" t="inlineStr">
         <is>
@@ -5910,7 +5908,7 @@
       </c>
       <c r="C103" t="inlineStr">
         <is>
-          <t>R4_2b_VIT4_LIGHTDETAIL48</t>
+          <t>R4_2_VIT4_LIGHTDETAIL</t>
         </is>
       </c>
       <c r="D103" t="inlineStr">
@@ -5919,31 +5917,31 @@
         </is>
       </c>
       <c r="E103" s="2" t="n">
-        <v>80.87</v>
+        <v>79.94</v>
       </c>
       <c r="F103" s="2" t="n">
-        <v>83.81</v>
+        <v>84.79000000000001</v>
       </c>
       <c r="G103" s="2" t="n">
-        <v>91.81</v>
+        <v>91.89</v>
       </c>
       <c r="H103" s="2" t="n">
-        <v>82.31999999999999</v>
+        <v>82.3</v>
       </c>
       <c r="I103" s="2" t="n">
-        <v>69.95</v>
+        <v>69.92</v>
       </c>
       <c r="J103" s="2" t="n">
-        <v>76.98999999999999</v>
+        <v>77.04000000000001</v>
       </c>
       <c r="K103" s="2" t="n">
-        <v>5.533</v>
+        <v>5.492</v>
       </c>
       <c r="L103" s="2" t="n">
-        <v>3.556</v>
+        <v>3.515</v>
       </c>
       <c r="M103" s="2" t="n">
-        <v>10.9824</v>
+        <v>10.7311</v>
       </c>
       <c r="N103" t="inlineStr">
         <is>
@@ -5964,7 +5962,7 @@
       </c>
       <c r="C104" t="inlineStr">
         <is>
-          <t>R4_2d_PSD_DETAIL</t>
+          <t>R4_2b_VIT4_LIGHTDETAIL48</t>
         </is>
       </c>
       <c r="D104" t="inlineStr">
@@ -5973,31 +5971,31 @@
         </is>
       </c>
       <c r="E104" s="2" t="n">
-        <v>79.78</v>
+        <v>80.87</v>
       </c>
       <c r="F104" s="2" t="n">
-        <v>84.39</v>
+        <v>83.81</v>
       </c>
       <c r="G104" s="2" t="n">
-        <v>91.75</v>
+        <v>91.81</v>
       </c>
       <c r="H104" s="2" t="n">
-        <v>82.02</v>
+        <v>82.31999999999999</v>
       </c>
       <c r="I104" s="2" t="n">
-        <v>69.52</v>
+        <v>69.95</v>
       </c>
       <c r="J104" s="2" t="n">
-        <v>76.68000000000001</v>
+        <v>76.98999999999999</v>
       </c>
       <c r="K104" s="2" t="n">
-        <v>5.491</v>
+        <v>5.533</v>
       </c>
       <c r="L104" s="2" t="n">
-        <v>3.514</v>
+        <v>3.556</v>
       </c>
       <c r="M104" s="2" t="n">
-        <v>11.5239</v>
+        <v>10.9824</v>
       </c>
       <c r="N104" t="inlineStr">
         <is>
@@ -6008,46 +6006,50 @@
     <row r="105">
       <c r="A105" t="inlineStr">
         <is>
-          <t>baseline</t>
+          <t>UltraLight</t>
         </is>
       </c>
       <c r="B105" t="inlineStr">
         <is>
-          <t>Run1</t>
-        </is>
-      </c>
-      <c r="C105" t="inlineStr"/>
+          <t>Run4</t>
+        </is>
+      </c>
+      <c r="C105" t="inlineStr">
+        <is>
+          <t>R4_2d_PSD_DETAIL</t>
+        </is>
+      </c>
       <c r="D105" t="inlineStr">
         <is>
-          <t>CDD-CD-256</t>
+          <t>SYSU-CD-256</t>
         </is>
       </c>
       <c r="E105" s="2" t="n">
-        <v>97.72</v>
+        <v>79.78</v>
       </c>
       <c r="F105" s="2" t="n">
-        <v>97.78</v>
+        <v>84.39</v>
       </c>
       <c r="G105" s="2" t="n">
-        <v>99.44</v>
+        <v>91.75</v>
       </c>
       <c r="H105" s="2" t="n">
-        <v>97.75</v>
+        <v>82.02</v>
       </c>
       <c r="I105" s="2" t="n">
-        <v>95.59999999999999</v>
+        <v>69.52</v>
       </c>
       <c r="J105" s="2" t="n">
-        <v>97.43000000000001</v>
+        <v>76.68000000000001</v>
       </c>
       <c r="K105" s="2" t="n">
-        <v>11.754</v>
+        <v>5.491</v>
       </c>
       <c r="L105" s="2" t="n">
-        <v>20.661</v>
+        <v>3.514</v>
       </c>
       <c r="M105" s="2" t="n">
-        <v>26.3246</v>
+        <v>11.5239</v>
       </c>
       <c r="N105" t="inlineStr">
         <is>
@@ -6069,26 +6071,26 @@
       <c r="C106" t="inlineStr"/>
       <c r="D106" t="inlineStr">
         <is>
-          <t>LEVIR-CD-256</t>
+          <t>CDD-CD-256</t>
         </is>
       </c>
       <c r="E106" s="2" t="n">
-        <v>91.56999999999999</v>
+        <v>97.72</v>
       </c>
       <c r="F106" s="2" t="n">
-        <v>92.33</v>
+        <v>97.78</v>
       </c>
       <c r="G106" s="2" t="n">
-        <v>99.18000000000001</v>
+        <v>99.44</v>
       </c>
       <c r="H106" s="2" t="n">
-        <v>91.95</v>
+        <v>97.75</v>
       </c>
       <c r="I106" s="2" t="n">
-        <v>85.09999999999999</v>
+        <v>95.59999999999999</v>
       </c>
       <c r="J106" s="2" t="n">
-        <v>91.52</v>
+        <v>97.43000000000001</v>
       </c>
       <c r="K106" s="2" t="n">
         <v>11.754</v>
@@ -6119,26 +6121,26 @@
       <c r="C107" t="inlineStr"/>
       <c r="D107" t="inlineStr">
         <is>
-          <t>SYSU-CD-256</t>
+          <t>LEVIR-CD-256</t>
         </is>
       </c>
       <c r="E107" s="2" t="n">
-        <v>80.77</v>
+        <v>91.56999999999999</v>
       </c>
       <c r="F107" s="2" t="n">
-        <v>84.27</v>
+        <v>92.33</v>
       </c>
       <c r="G107" s="2" t="n">
-        <v>91.91</v>
+        <v>99.18000000000001</v>
       </c>
       <c r="H107" s="2" t="n">
-        <v>82.48</v>
+        <v>91.95</v>
       </c>
       <c r="I107" s="2" t="n">
-        <v>70.19</v>
+        <v>85.09999999999999</v>
       </c>
       <c r="J107" s="2" t="n">
-        <v>77.23</v>
+        <v>91.52</v>
       </c>
       <c r="K107" s="2" t="n">
         <v>11.754</v>
@@ -6169,26 +6171,26 @@
       <c r="C108" t="inlineStr"/>
       <c r="D108" t="inlineStr">
         <is>
-          <t>WHU-CD-256</t>
+          <t>SYSU-CD-256</t>
         </is>
       </c>
       <c r="E108" s="2" t="n">
-        <v>93.62</v>
+        <v>80.77</v>
       </c>
       <c r="F108" s="2" t="n">
-        <v>96.09</v>
+        <v>84.27</v>
       </c>
       <c r="G108" s="2" t="n">
-        <v>99.59999999999999</v>
+        <v>91.91</v>
       </c>
       <c r="H108" s="2" t="n">
-        <v>94.84</v>
+        <v>82.48</v>
       </c>
       <c r="I108" s="2" t="n">
-        <v>90.18000000000001</v>
+        <v>70.19</v>
       </c>
       <c r="J108" s="2" t="n">
-        <v>94.63</v>
+        <v>77.23</v>
       </c>
       <c r="K108" s="2" t="n">
         <v>11.754</v>
@@ -6205,8 +6207,58 @@
         </is>
       </c>
     </row>
+    <row r="109">
+      <c r="A109" t="inlineStr">
+        <is>
+          <t>baseline</t>
+        </is>
+      </c>
+      <c r="B109" t="inlineStr">
+        <is>
+          <t>Run1</t>
+        </is>
+      </c>
+      <c r="C109" t="inlineStr"/>
+      <c r="D109" t="inlineStr">
+        <is>
+          <t>WHU-CD-256</t>
+        </is>
+      </c>
+      <c r="E109" s="2" t="n">
+        <v>93.62</v>
+      </c>
+      <c r="F109" s="2" t="n">
+        <v>96.09</v>
+      </c>
+      <c r="G109" s="2" t="n">
+        <v>99.59999999999999</v>
+      </c>
+      <c r="H109" s="2" t="n">
+        <v>94.84</v>
+      </c>
+      <c r="I109" s="2" t="n">
+        <v>90.18000000000001</v>
+      </c>
+      <c r="J109" s="2" t="n">
+        <v>94.63</v>
+      </c>
+      <c r="K109" s="2" t="n">
+        <v>11.754</v>
+      </c>
+      <c r="L109" s="2" t="n">
+        <v>20.661</v>
+      </c>
+      <c r="M109" s="2" t="n">
+        <v>26.3246</v>
+      </c>
+      <c r="N109" t="inlineStr">
+        <is>
+          <t>baseline</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:N108"/>
+  <autoFilter ref="A1:N109"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Separate Euclidean and hyperbolic change-context modules
</commit_message>
<xml_diff>
--- a/docs/experiment_metrics.xlsx
+++ b/docs/experiment_metrics.xlsx
@@ -10,7 +10,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="metrics" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'metrics'!$A$1:$N$109</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'metrics'!$A$1:$N$112</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -420,7 +420,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N109"/>
+  <dimension ref="A1:N112"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -4674,42 +4674,42 @@
       </c>
       <c r="C80" t="inlineStr">
         <is>
-          <t>M1_HYPER_QKV</t>
+          <t>M0_CTRL</t>
         </is>
       </c>
       <c r="D80" t="inlineStr">
         <is>
-          <t>LEVIR-CD-256</t>
+          <t>WHU-CD-256</t>
         </is>
       </c>
       <c r="E80" s="2" t="n">
-        <v>90.55</v>
+        <v>92.61</v>
       </c>
       <c r="F80" s="2" t="n">
-        <v>92.03</v>
+        <v>95.26000000000001</v>
       </c>
       <c r="G80" s="2" t="n">
-        <v>99.12</v>
+        <v>99.52</v>
       </c>
       <c r="H80" s="2" t="n">
-        <v>91.28</v>
+        <v>93.92</v>
       </c>
       <c r="I80" s="2" t="n">
-        <v>83.95999999999999</v>
+        <v>88.53</v>
       </c>
       <c r="J80" s="2" t="n">
-        <v>90.81999999999999</v>
+        <v>93.67</v>
       </c>
       <c r="K80" s="2" t="n">
-        <v>3.049509</v>
+        <v>3.016737</v>
       </c>
       <c r="L80" s="2" t="n">
-        <v>3.133176</v>
+        <v>3.100404</v>
       </c>
       <c r="M80" s="2" t="n"/>
       <c r="N80" t="inlineStr">
         <is>
-          <t>casa_wdmf_str_hyperbolic</t>
+          <t>casa_wdmf_str_none</t>
         </is>
       </c>
     </row>
@@ -4731,26 +4731,26 @@
       </c>
       <c r="D81" t="inlineStr">
         <is>
-          <t>SYSU-CD-256</t>
+          <t>LEVIR-CD-256</t>
         </is>
       </c>
       <c r="E81" s="2" t="n">
-        <v>78.67</v>
+        <v>90.55</v>
       </c>
       <c r="F81" s="2" t="n">
-        <v>85.08</v>
+        <v>92.03</v>
       </c>
       <c r="G81" s="2" t="n">
-        <v>91.72</v>
+        <v>99.12</v>
       </c>
       <c r="H81" s="2" t="n">
-        <v>81.75</v>
+        <v>91.28</v>
       </c>
       <c r="I81" s="2" t="n">
-        <v>69.13</v>
+        <v>83.95999999999999</v>
       </c>
       <c r="J81" s="2" t="n">
-        <v>76.40000000000001</v>
+        <v>90.81999999999999</v>
       </c>
       <c r="K81" s="2" t="n">
         <v>3.049509</v>
@@ -4778,31 +4778,31 @@
       </c>
       <c r="C82" t="inlineStr">
         <is>
-          <t>M2_CA_QKV</t>
+          <t>M1_HYPER_QKV</t>
         </is>
       </c>
       <c r="D82" t="inlineStr">
         <is>
-          <t>LEVIR-CD-256</t>
+          <t>SYSU-CD-256</t>
         </is>
       </c>
       <c r="E82" s="2" t="n">
-        <v>89.72</v>
+        <v>78.67</v>
       </c>
       <c r="F82" s="2" t="n">
-        <v>93.12</v>
+        <v>85.08</v>
       </c>
       <c r="G82" s="2" t="n">
-        <v>99.14</v>
+        <v>91.72</v>
       </c>
       <c r="H82" s="2" t="n">
-        <v>91.39</v>
+        <v>81.75</v>
       </c>
       <c r="I82" s="2" t="n">
-        <v>84.14</v>
+        <v>69.13</v>
       </c>
       <c r="J82" s="2" t="n">
-        <v>90.93000000000001</v>
+        <v>76.40000000000001</v>
       </c>
       <c r="K82" s="2" t="n">
         <v>3.049509</v>
@@ -4813,7 +4813,7 @@
       <c r="M82" s="2" t="n"/>
       <c r="N82" t="inlineStr">
         <is>
-          <t>casa_wdmf_str_qkv</t>
+          <t>casa_wdmf_str_hyperbolic</t>
         </is>
       </c>
     </row>
@@ -4830,31 +4830,31 @@
       </c>
       <c r="C83" t="inlineStr">
         <is>
-          <t>M2_CA_QKV</t>
+          <t>M1_HYPER_QKV</t>
         </is>
       </c>
       <c r="D83" t="inlineStr">
         <is>
-          <t>SYSU-CD-256</t>
+          <t>WHU-CD-256</t>
         </is>
       </c>
       <c r="E83" s="2" t="n">
-        <v>82.83</v>
+        <v>92.84999999999999</v>
       </c>
       <c r="F83" s="2" t="n">
-        <v>82.86</v>
+        <v>95.31999999999999</v>
       </c>
       <c r="G83" s="2" t="n">
-        <v>91.91</v>
+        <v>99.54000000000001</v>
       </c>
       <c r="H83" s="2" t="n">
-        <v>82.84999999999999</v>
+        <v>94.06999999999999</v>
       </c>
       <c r="I83" s="2" t="n">
-        <v>70.72</v>
+        <v>88.8</v>
       </c>
       <c r="J83" s="2" t="n">
-        <v>77.56</v>
+        <v>93.83</v>
       </c>
       <c r="K83" s="2" t="n">
         <v>3.049509</v>
@@ -4865,24 +4865,24 @@
       <c r="M83" s="2" t="n"/>
       <c r="N83" t="inlineStr">
         <is>
-          <t>casa_wdmf_str_qkv</t>
+          <t>casa_wdmf_str_hyperbolic</t>
         </is>
       </c>
     </row>
     <row r="84">
       <c r="A84" t="inlineStr">
         <is>
-          <t>CASAA</t>
+          <t>CASA-WDMF</t>
         </is>
       </c>
       <c r="B84" t="inlineStr">
         <is>
-          <t>Run1</t>
+          <t>Run2</t>
         </is>
       </c>
       <c r="C84" t="inlineStr">
         <is>
-          <t>A1_SAA</t>
+          <t>M2_CA_QKV</t>
         </is>
       </c>
       <c r="D84" t="inlineStr">
@@ -4891,52 +4891,50 @@
         </is>
       </c>
       <c r="E84" s="2" t="n">
-        <v>91.09</v>
+        <v>89.72</v>
       </c>
       <c r="F84" s="2" t="n">
-        <v>92.8</v>
+        <v>93.12</v>
       </c>
       <c r="G84" s="2" t="n">
-        <v>99.19</v>
+        <v>99.14</v>
       </c>
       <c r="H84" s="2" t="n">
-        <v>91.94</v>
+        <v>91.39</v>
       </c>
       <c r="I84" s="2" t="n">
-        <v>85.08</v>
+        <v>84.14</v>
       </c>
       <c r="J84" s="2" t="n">
-        <v>91.51000000000001</v>
+        <v>90.93000000000001</v>
       </c>
       <c r="K84" s="2" t="n">
-        <v>11.754</v>
+        <v>3.049509</v>
       </c>
       <c r="L84" s="2" t="n">
-        <v>20.661</v>
-      </c>
-      <c r="M84" s="2" t="n">
-        <v>26.3183</v>
-      </c>
+        <v>3.133176</v>
+      </c>
+      <c r="M84" s="2" t="n"/>
       <c r="N84" t="inlineStr">
         <is>
-          <t>saa</t>
+          <t>casa_wdmf_str_qkv</t>
         </is>
       </c>
     </row>
     <row r="85">
       <c r="A85" t="inlineStr">
         <is>
-          <t>CASAA</t>
+          <t>CASA-WDMF</t>
         </is>
       </c>
       <c r="B85" t="inlineStr">
         <is>
-          <t>Run1</t>
+          <t>Run2</t>
         </is>
       </c>
       <c r="C85" t="inlineStr">
         <is>
-          <t>A1_SAA</t>
+          <t>M2_CA_QKV</t>
         </is>
       </c>
       <c r="D85" t="inlineStr">
@@ -4945,89 +4943,85 @@
         </is>
       </c>
       <c r="E85" s="2" t="n">
-        <v>80.3</v>
+        <v>82.83</v>
       </c>
       <c r="F85" s="2" t="n">
-        <v>84.81</v>
+        <v>82.86</v>
       </c>
       <c r="G85" s="2" t="n">
-        <v>91.95999999999999</v>
+        <v>91.91</v>
       </c>
       <c r="H85" s="2" t="n">
-        <v>82.5</v>
+        <v>82.84999999999999</v>
       </c>
       <c r="I85" s="2" t="n">
-        <v>70.20999999999999</v>
+        <v>70.72</v>
       </c>
       <c r="J85" s="2" t="n">
-        <v>77.29000000000001</v>
+        <v>77.56</v>
       </c>
       <c r="K85" s="2" t="n">
-        <v>11.754</v>
+        <v>3.049509</v>
       </c>
       <c r="L85" s="2" t="n">
-        <v>20.661</v>
-      </c>
-      <c r="M85" s="2" t="n">
-        <v>26.3183</v>
-      </c>
+        <v>3.133176</v>
+      </c>
+      <c r="M85" s="2" t="n"/>
       <c r="N85" t="inlineStr">
         <is>
-          <t>saa</t>
+          <t>casa_wdmf_str_qkv</t>
         </is>
       </c>
     </row>
     <row r="86">
       <c r="A86" t="inlineStr">
         <is>
-          <t>CASAA</t>
+          <t>CASA-WDMF</t>
         </is>
       </c>
       <c r="B86" t="inlineStr">
         <is>
-          <t>Run1</t>
+          <t>Run2</t>
         </is>
       </c>
       <c r="C86" t="inlineStr">
         <is>
-          <t>A2_CASAA</t>
+          <t>M2_CA_QKV</t>
         </is>
       </c>
       <c r="D86" t="inlineStr">
         <is>
-          <t>LEVIR-CD-256</t>
+          <t>WHU-CD-256</t>
         </is>
       </c>
       <c r="E86" s="2" t="n">
-        <v>90.98999999999999</v>
+        <v>93.04000000000001</v>
       </c>
       <c r="F86" s="2" t="n">
-        <v>92.75</v>
+        <v>96.08</v>
       </c>
       <c r="G86" s="2" t="n">
-        <v>99.18000000000001</v>
+        <v>99.56999999999999</v>
       </c>
       <c r="H86" s="2" t="n">
-        <v>91.86</v>
+        <v>94.53</v>
       </c>
       <c r="I86" s="2" t="n">
-        <v>84.94</v>
+        <v>89.63</v>
       </c>
       <c r="J86" s="2" t="n">
-        <v>91.43000000000001</v>
+        <v>94.31</v>
       </c>
       <c r="K86" s="2" t="n">
-        <v>11.754</v>
+        <v>3.049509</v>
       </c>
       <c r="L86" s="2" t="n">
-        <v>20.661</v>
-      </c>
-      <c r="M86" s="2" t="n">
-        <v>26.2593</v>
-      </c>
+        <v>3.133176</v>
+      </c>
+      <c r="M86" s="2" t="n"/>
       <c r="N86" t="inlineStr">
         <is>
-          <t>casaa</t>
+          <t>casa_wdmf_str_qkv</t>
         </is>
       </c>
     </row>
@@ -5044,31 +5038,31 @@
       </c>
       <c r="C87" t="inlineStr">
         <is>
-          <t>A2_CASAA</t>
+          <t>A1_SAA</t>
         </is>
       </c>
       <c r="D87" t="inlineStr">
         <is>
-          <t>SYSU-CD-256</t>
+          <t>LEVIR-CD-256</t>
         </is>
       </c>
       <c r="E87" s="2" t="n">
-        <v>80.55</v>
+        <v>91.09</v>
       </c>
       <c r="F87" s="2" t="n">
-        <v>84.23</v>
+        <v>92.8</v>
       </c>
       <c r="G87" s="2" t="n">
-        <v>91.86</v>
+        <v>99.19</v>
       </c>
       <c r="H87" s="2" t="n">
-        <v>82.34999999999999</v>
+        <v>91.94</v>
       </c>
       <c r="I87" s="2" t="n">
-        <v>70</v>
+        <v>85.08</v>
       </c>
       <c r="J87" s="2" t="n">
-        <v>77.06</v>
+        <v>91.51000000000001</v>
       </c>
       <c r="K87" s="2" t="n">
         <v>11.754</v>
@@ -5077,11 +5071,11 @@
         <v>20.661</v>
       </c>
       <c r="M87" s="2" t="n">
-        <v>26.2593</v>
+        <v>26.3183</v>
       </c>
       <c r="N87" t="inlineStr">
         <is>
-          <t>casaa</t>
+          <t>saa</t>
         </is>
       </c>
     </row>
@@ -5093,45 +5087,45 @@
       </c>
       <c r="B88" t="inlineStr">
         <is>
-          <t>Run2</t>
+          <t>Run1</t>
         </is>
       </c>
       <c r="C88" t="inlineStr">
         <is>
-          <t>A1_SAA_FROZEN</t>
+          <t>A1_SAA</t>
         </is>
       </c>
       <c r="D88" t="inlineStr">
         <is>
-          <t>LEVIR-CD-256</t>
+          <t>SYSU-CD-256</t>
         </is>
       </c>
       <c r="E88" s="2" t="n">
-        <v>91.38</v>
+        <v>80.3</v>
       </c>
       <c r="F88" s="2" t="n">
-        <v>92.3</v>
+        <v>84.81</v>
       </c>
       <c r="G88" s="2" t="n">
-        <v>99.17</v>
+        <v>91.95999999999999</v>
       </c>
       <c r="H88" s="2" t="n">
-        <v>91.84</v>
+        <v>82.5</v>
       </c>
       <c r="I88" s="2" t="n">
-        <v>84.91</v>
+        <v>70.20999999999999</v>
       </c>
       <c r="J88" s="2" t="n">
-        <v>91.40000000000001</v>
+        <v>77.29000000000001</v>
       </c>
       <c r="K88" s="2" t="n">
         <v>11.754</v>
       </c>
       <c r="L88" s="2" t="n">
-        <v>15.125</v>
+        <v>20.661</v>
       </c>
       <c r="M88" s="2" t="n">
-        <v>26.1484</v>
+        <v>26.3183</v>
       </c>
       <c r="N88" t="inlineStr">
         <is>
@@ -5147,49 +5141,49 @@
       </c>
       <c r="B89" t="inlineStr">
         <is>
-          <t>Run2</t>
+          <t>Run1</t>
         </is>
       </c>
       <c r="C89" t="inlineStr">
         <is>
-          <t>A1_SAA_FROZEN</t>
+          <t>A2_CASAA</t>
         </is>
       </c>
       <c r="D89" t="inlineStr">
         <is>
-          <t>SYSU-CD-256</t>
+          <t>LEVIR-CD-256</t>
         </is>
       </c>
       <c r="E89" s="2" t="n">
-        <v>78.40000000000001</v>
+        <v>90.98999999999999</v>
       </c>
       <c r="F89" s="2" t="n">
-        <v>86.03</v>
+        <v>92.75</v>
       </c>
       <c r="G89" s="2" t="n">
-        <v>91.90000000000001</v>
+        <v>99.18000000000001</v>
       </c>
       <c r="H89" s="2" t="n">
-        <v>82.04000000000001</v>
+        <v>91.86</v>
       </c>
       <c r="I89" s="2" t="n">
-        <v>69.55</v>
+        <v>84.94</v>
       </c>
       <c r="J89" s="2" t="n">
-        <v>76.83</v>
+        <v>91.43000000000001</v>
       </c>
       <c r="K89" s="2" t="n">
         <v>11.754</v>
       </c>
       <c r="L89" s="2" t="n">
-        <v>15.125</v>
+        <v>20.661</v>
       </c>
       <c r="M89" s="2" t="n">
-        <v>26.1484</v>
+        <v>26.2593</v>
       </c>
       <c r="N89" t="inlineStr">
         <is>
-          <t>saa</t>
+          <t>casaa</t>
         </is>
       </c>
     </row>
@@ -5201,45 +5195,45 @@
       </c>
       <c r="B90" t="inlineStr">
         <is>
-          <t>Run2</t>
+          <t>Run1</t>
         </is>
       </c>
       <c r="C90" t="inlineStr">
         <is>
-          <t>A3_ORACLE_FROZEN</t>
+          <t>A2_CASAA</t>
         </is>
       </c>
       <c r="D90" t="inlineStr">
         <is>
-          <t>LEVIR-CD-256</t>
+          <t>SYSU-CD-256</t>
         </is>
       </c>
       <c r="E90" s="2" t="n">
-        <v>91.13</v>
+        <v>80.55</v>
       </c>
       <c r="F90" s="2" t="n">
-        <v>92.65000000000001</v>
+        <v>84.23</v>
       </c>
       <c r="G90" s="2" t="n">
-        <v>99.18000000000001</v>
+        <v>91.86</v>
       </c>
       <c r="H90" s="2" t="n">
-        <v>91.88</v>
+        <v>82.34999999999999</v>
       </c>
       <c r="I90" s="2" t="n">
-        <v>84.98</v>
+        <v>70</v>
       </c>
       <c r="J90" s="2" t="n">
-        <v>91.45</v>
+        <v>77.06</v>
       </c>
       <c r="K90" s="2" t="n">
         <v>11.754</v>
       </c>
       <c r="L90" s="2" t="n">
-        <v>15.125</v>
+        <v>20.661</v>
       </c>
       <c r="M90" s="2" t="n">
-        <v>26.0894</v>
+        <v>26.2593</v>
       </c>
       <c r="N90" t="inlineStr">
         <is>
@@ -5260,31 +5254,31 @@
       </c>
       <c r="C91" t="inlineStr">
         <is>
-          <t>A3_ORACLE_FROZEN</t>
+          <t>A1_SAA_FROZEN</t>
         </is>
       </c>
       <c r="D91" t="inlineStr">
         <is>
-          <t>SYSU-CD-256</t>
+          <t>LEVIR-CD-256</t>
         </is>
       </c>
       <c r="E91" s="2" t="n">
-        <v>82.04000000000001</v>
+        <v>91.38</v>
       </c>
       <c r="F91" s="2" t="n">
-        <v>85.05</v>
+        <v>92.3</v>
       </c>
       <c r="G91" s="2" t="n">
-        <v>92.36</v>
+        <v>99.17</v>
       </c>
       <c r="H91" s="2" t="n">
-        <v>83.52</v>
+        <v>91.84</v>
       </c>
       <c r="I91" s="2" t="n">
-        <v>71.7</v>
+        <v>84.91</v>
       </c>
       <c r="J91" s="2" t="n">
-        <v>78.55</v>
+        <v>91.40000000000001</v>
       </c>
       <c r="K91" s="2" t="n">
         <v>11.754</v>
@@ -5293,11 +5287,11 @@
         <v>15.125</v>
       </c>
       <c r="M91" s="2" t="n">
-        <v>26.0894</v>
+        <v>26.1484</v>
       </c>
       <c r="N91" t="inlineStr">
         <is>
-          <t>casaa</t>
+          <t>saa</t>
         </is>
       </c>
     </row>
@@ -5309,12 +5303,12 @@
       </c>
       <c r="B92" t="inlineStr">
         <is>
-          <t>Run3</t>
+          <t>Run2</t>
         </is>
       </c>
       <c r="C92" t="inlineStr">
         <is>
-          <t>A4_DETAIL_FROZEN</t>
+          <t>A1_SAA_FROZEN</t>
         </is>
       </c>
       <c r="D92" t="inlineStr">
@@ -5323,22 +5317,22 @@
         </is>
       </c>
       <c r="E92" s="2" t="n">
-        <v>79.68000000000001</v>
+        <v>78.40000000000001</v>
       </c>
       <c r="F92" s="2" t="n">
-        <v>84.28</v>
+        <v>86.03</v>
       </c>
       <c r="G92" s="2" t="n">
-        <v>91.7</v>
+        <v>91.90000000000001</v>
       </c>
       <c r="H92" s="2" t="n">
-        <v>81.92</v>
+        <v>82.04000000000001</v>
       </c>
       <c r="I92" s="2" t="n">
-        <v>69.37</v>
+        <v>69.55</v>
       </c>
       <c r="J92" s="2" t="n">
-        <v>76.54000000000001</v>
+        <v>76.83</v>
       </c>
       <c r="K92" s="2" t="n">
         <v>11.754</v>
@@ -5347,136 +5341,136 @@
         <v>15.125</v>
       </c>
       <c r="M92" s="2" t="n">
-        <v>26.0894</v>
+        <v>26.1484</v>
       </c>
       <c r="N92" t="inlineStr">
         <is>
-          <t>casaa</t>
+          <t>saa</t>
         </is>
       </c>
     </row>
     <row r="93">
       <c r="A93" t="inlineStr">
         <is>
-          <t>STR-Fusion</t>
+          <t>CASAA</t>
         </is>
       </c>
       <c r="B93" t="inlineStr">
         <is>
-          <t>Run2_TASS</t>
+          <t>Run2</t>
         </is>
       </c>
       <c r="C93" t="inlineStr">
         <is>
-          <t>C0_TOKEN</t>
+          <t>A3_ORACLE_FROZEN</t>
         </is>
       </c>
       <c r="D93" t="inlineStr">
         <is>
-          <t>CDD-CD-256</t>
+          <t>LEVIR-CD-256</t>
         </is>
       </c>
       <c r="E93" s="2" t="n">
-        <v>93.13</v>
+        <v>91.13</v>
       </c>
       <c r="F93" s="2" t="n">
-        <v>95.16</v>
+        <v>92.65000000000001</v>
       </c>
       <c r="G93" s="2" t="n">
-        <v>98.56999999999999</v>
+        <v>99.18000000000001</v>
       </c>
       <c r="H93" s="2" t="n">
-        <v>94.13</v>
+        <v>91.88</v>
       </c>
       <c r="I93" s="2" t="n">
-        <v>88.91</v>
+        <v>84.98</v>
       </c>
       <c r="J93" s="2" t="n">
-        <v>93.31999999999999</v>
+        <v>91.45</v>
       </c>
       <c r="K93" s="2" t="n">
-        <v>2.596</v>
+        <v>11.754</v>
       </c>
       <c r="L93" s="2" t="n">
-        <v>0.62</v>
+        <v>15.125</v>
       </c>
       <c r="M93" s="2" t="n">
-        <v>2.2136</v>
+        <v>26.0894</v>
       </c>
       <c r="N93" t="inlineStr">
         <is>
-          <t>str_tass</t>
+          <t>casaa</t>
         </is>
       </c>
     </row>
     <row r="94">
       <c r="A94" t="inlineStr">
         <is>
-          <t>STR-Fusion</t>
+          <t>CASAA</t>
         </is>
       </c>
       <c r="B94" t="inlineStr">
         <is>
-          <t>Run2_TASS</t>
+          <t>Run2</t>
         </is>
       </c>
       <c r="C94" t="inlineStr">
         <is>
-          <t>C0_TOKEN</t>
+          <t>A3_ORACLE_FROZEN</t>
         </is>
       </c>
       <c r="D94" t="inlineStr">
         <is>
-          <t>LEVIR-CD-256</t>
+          <t>SYSU-CD-256</t>
         </is>
       </c>
       <c r="E94" s="2" t="n">
-        <v>86.37</v>
+        <v>82.04000000000001</v>
       </c>
       <c r="F94" s="2" t="n">
-        <v>89.25</v>
+        <v>85.05</v>
       </c>
       <c r="G94" s="2" t="n">
-        <v>98.78</v>
+        <v>92.36</v>
       </c>
       <c r="H94" s="2" t="n">
-        <v>87.79000000000001</v>
+        <v>83.52</v>
       </c>
       <c r="I94" s="2" t="n">
-        <v>78.23999999999999</v>
+        <v>71.7</v>
       </c>
       <c r="J94" s="2" t="n">
-        <v>87.14</v>
+        <v>78.55</v>
       </c>
       <c r="K94" s="2" t="n">
-        <v>2.596</v>
+        <v>11.754</v>
       </c>
       <c r="L94" s="2" t="n">
-        <v>0.62</v>
+        <v>15.125</v>
       </c>
       <c r="M94" s="2" t="n">
-        <v>2.2136</v>
+        <v>26.0894</v>
       </c>
       <c r="N94" t="inlineStr">
         <is>
-          <t>str_tass</t>
+          <t>casaa</t>
         </is>
       </c>
     </row>
     <row r="95">
       <c r="A95" t="inlineStr">
         <is>
-          <t>STR-Fusion</t>
+          <t>CASAA</t>
         </is>
       </c>
       <c r="B95" t="inlineStr">
         <is>
-          <t>Run2_TASS</t>
+          <t>Run3</t>
         </is>
       </c>
       <c r="C95" t="inlineStr">
         <is>
-          <t>C0_TOKEN</t>
+          <t>A4_DETAIL_FROZEN</t>
         </is>
       </c>
       <c r="D95" t="inlineStr">
@@ -5485,35 +5479,35 @@
         </is>
       </c>
       <c r="E95" s="2" t="n">
-        <v>79.93000000000001</v>
+        <v>79.68000000000001</v>
       </c>
       <c r="F95" s="2" t="n">
-        <v>84.5</v>
+        <v>84.28</v>
       </c>
       <c r="G95" s="2" t="n">
-        <v>91.81</v>
+        <v>91.7</v>
       </c>
       <c r="H95" s="2" t="n">
-        <v>82.15000000000001</v>
+        <v>81.92</v>
       </c>
       <c r="I95" s="2" t="n">
-        <v>69.70999999999999</v>
+        <v>69.37</v>
       </c>
       <c r="J95" s="2" t="n">
-        <v>76.84</v>
+        <v>76.54000000000001</v>
       </c>
       <c r="K95" s="2" t="n">
-        <v>2.596</v>
+        <v>11.754</v>
       </c>
       <c r="L95" s="2" t="n">
-        <v>0.62</v>
+        <v>15.125</v>
       </c>
       <c r="M95" s="2" t="n">
-        <v>2.2136</v>
+        <v>26.0894</v>
       </c>
       <c r="N95" t="inlineStr">
         <is>
-          <t>str_tass</t>
+          <t>casaa</t>
         </is>
       </c>
     </row>
@@ -5535,26 +5529,26 @@
       </c>
       <c r="D96" t="inlineStr">
         <is>
-          <t>WHU-CD-256</t>
+          <t>CDD-CD-256</t>
         </is>
       </c>
       <c r="E96" s="2" t="n">
-        <v>90.16</v>
+        <v>93.13</v>
       </c>
       <c r="F96" s="2" t="n">
-        <v>93.97</v>
+        <v>95.16</v>
       </c>
       <c r="G96" s="2" t="n">
-        <v>99.38</v>
+        <v>98.56999999999999</v>
       </c>
       <c r="H96" s="2" t="n">
-        <v>92.02</v>
+        <v>94.13</v>
       </c>
       <c r="I96" s="2" t="n">
-        <v>85.23</v>
+        <v>88.91</v>
       </c>
       <c r="J96" s="2" t="n">
-        <v>91.7</v>
+        <v>93.31999999999999</v>
       </c>
       <c r="K96" s="2" t="n">
         <v>2.596</v>
@@ -5584,40 +5578,40 @@
       </c>
       <c r="C97" t="inlineStr">
         <is>
-          <t>M1_TASS</t>
+          <t>C0_TOKEN</t>
         </is>
       </c>
       <c r="D97" t="inlineStr">
         <is>
-          <t>CDD-CD-256</t>
+          <t>LEVIR-CD-256</t>
         </is>
       </c>
       <c r="E97" s="2" t="n">
-        <v>94.7</v>
+        <v>86.37</v>
       </c>
       <c r="F97" s="2" t="n">
-        <v>96.13</v>
+        <v>89.25</v>
       </c>
       <c r="G97" s="2" t="n">
-        <v>98.88</v>
+        <v>98.78</v>
       </c>
       <c r="H97" s="2" t="n">
-        <v>95.41</v>
+        <v>87.79000000000001</v>
       </c>
       <c r="I97" s="2" t="n">
-        <v>91.22</v>
+        <v>78.23999999999999</v>
       </c>
       <c r="J97" s="2" t="n">
-        <v>94.77</v>
+        <v>87.14</v>
       </c>
       <c r="K97" s="2" t="n">
-        <v>3.455</v>
+        <v>2.596</v>
       </c>
       <c r="L97" s="2" t="n">
-        <v>1.478</v>
+        <v>0.62</v>
       </c>
       <c r="M97" s="2" t="n">
-        <v>3.5459</v>
+        <v>2.2136</v>
       </c>
       <c r="N97" t="inlineStr">
         <is>
@@ -5638,40 +5632,40 @@
       </c>
       <c r="C98" t="inlineStr">
         <is>
-          <t>M1_TASS</t>
+          <t>C0_TOKEN</t>
         </is>
       </c>
       <c r="D98" t="inlineStr">
         <is>
-          <t>LEVIR-CD-256</t>
+          <t>SYSU-CD-256</t>
         </is>
       </c>
       <c r="E98" s="2" t="n">
-        <v>88.42</v>
+        <v>79.93000000000001</v>
       </c>
       <c r="F98" s="2" t="n">
-        <v>91.97</v>
+        <v>84.5</v>
       </c>
       <c r="G98" s="2" t="n">
-        <v>99.02</v>
+        <v>91.81</v>
       </c>
       <c r="H98" s="2" t="n">
-        <v>90.16</v>
+        <v>82.15000000000001</v>
       </c>
       <c r="I98" s="2" t="n">
-        <v>82.08</v>
+        <v>69.70999999999999</v>
       </c>
       <c r="J98" s="2" t="n">
-        <v>89.64</v>
+        <v>76.84</v>
       </c>
       <c r="K98" s="2" t="n">
-        <v>3.455</v>
+        <v>2.596</v>
       </c>
       <c r="L98" s="2" t="n">
-        <v>1.478</v>
+        <v>0.62</v>
       </c>
       <c r="M98" s="2" t="n">
-        <v>3.5459</v>
+        <v>2.2136</v>
       </c>
       <c r="N98" t="inlineStr">
         <is>
@@ -5692,40 +5686,40 @@
       </c>
       <c r="C99" t="inlineStr">
         <is>
-          <t>M1_TASS</t>
+          <t>C0_TOKEN</t>
         </is>
       </c>
       <c r="D99" t="inlineStr">
         <is>
-          <t>SYSU-CD-256</t>
+          <t>WHU-CD-256</t>
         </is>
       </c>
       <c r="E99" s="2" t="n">
-        <v>78.73</v>
+        <v>90.16</v>
       </c>
       <c r="F99" s="2" t="n">
-        <v>84.98</v>
+        <v>93.97</v>
       </c>
       <c r="G99" s="2" t="n">
+        <v>99.38</v>
+      </c>
+      <c r="H99" s="2" t="n">
+        <v>92.02</v>
+      </c>
+      <c r="I99" s="2" t="n">
+        <v>85.23</v>
+      </c>
+      <c r="J99" s="2" t="n">
         <v>91.7</v>
       </c>
-      <c r="H99" s="2" t="n">
-        <v>81.73999999999999</v>
-      </c>
-      <c r="I99" s="2" t="n">
-        <v>69.11</v>
-      </c>
-      <c r="J99" s="2" t="n">
-        <v>76.38</v>
-      </c>
       <c r="K99" s="2" t="n">
-        <v>3.455</v>
+        <v>2.596</v>
       </c>
       <c r="L99" s="2" t="n">
-        <v>1.478</v>
+        <v>0.62</v>
       </c>
       <c r="M99" s="2" t="n">
-        <v>3.5459</v>
+        <v>2.2136</v>
       </c>
       <c r="N99" t="inlineStr">
         <is>
@@ -5751,26 +5745,26 @@
       </c>
       <c r="D100" t="inlineStr">
         <is>
-          <t>WHU-CD-256</t>
+          <t>CDD-CD-256</t>
         </is>
       </c>
       <c r="E100" s="2" t="n">
-        <v>91.64</v>
+        <v>94.7</v>
       </c>
       <c r="F100" s="2" t="n">
-        <v>94.81999999999999</v>
+        <v>96.13</v>
       </c>
       <c r="G100" s="2" t="n">
-        <v>99.47</v>
+        <v>98.88</v>
       </c>
       <c r="H100" s="2" t="n">
-        <v>93.2</v>
+        <v>95.41</v>
       </c>
       <c r="I100" s="2" t="n">
-        <v>87.27</v>
+        <v>91.22</v>
       </c>
       <c r="J100" s="2" t="n">
-        <v>92.93000000000001</v>
+        <v>94.77</v>
       </c>
       <c r="K100" s="2" t="n">
         <v>3.455</v>
@@ -5790,71 +5784,71 @@
     <row r="101">
       <c r="A101" t="inlineStr">
         <is>
-          <t>UltraLight</t>
+          <t>STR-Fusion</t>
         </is>
       </c>
       <c r="B101" t="inlineStr">
         <is>
-          <t>Run4</t>
+          <t>Run2_TASS</t>
         </is>
       </c>
       <c r="C101" t="inlineStr">
         <is>
-          <t>R4_0_A0_FULL12_FROZEN</t>
+          <t>M1_TASS</t>
         </is>
       </c>
       <c r="D101" t="inlineStr">
         <is>
-          <t>SYSU-CD-256</t>
+          <t>LEVIR-CD-256</t>
         </is>
       </c>
       <c r="E101" s="2" t="n">
-        <v>82.42</v>
+        <v>88.42</v>
       </c>
       <c r="F101" s="2" t="n">
-        <v>83.87</v>
+        <v>91.97</v>
       </c>
       <c r="G101" s="2" t="n">
-        <v>92.12</v>
+        <v>99.02</v>
       </c>
       <c r="H101" s="2" t="n">
-        <v>83.14</v>
+        <v>90.16</v>
       </c>
       <c r="I101" s="2" t="n">
-        <v>71.14</v>
+        <v>82.08</v>
       </c>
       <c r="J101" s="2" t="n">
-        <v>77.98999999999999</v>
+        <v>89.64</v>
       </c>
       <c r="K101" s="2" t="n">
-        <v>11.754</v>
+        <v>3.455</v>
       </c>
       <c r="L101" s="2" t="n">
-        <v>15.125</v>
+        <v>1.478</v>
       </c>
       <c r="M101" s="2" t="n">
-        <v>26.3246</v>
+        <v>3.5459</v>
       </c>
       <c r="N101" t="inlineStr">
         <is>
-          <t>baseline</t>
+          <t>str_tass</t>
         </is>
       </c>
     </row>
     <row r="102">
       <c r="A102" t="inlineStr">
         <is>
-          <t>UltraLight</t>
+          <t>STR-Fusion</t>
         </is>
       </c>
       <c r="B102" t="inlineStr">
         <is>
-          <t>Run4</t>
+          <t>Run2_TASS</t>
         </is>
       </c>
       <c r="C102" t="inlineStr">
         <is>
-          <t>R4_1_VIT4_OLDHEAD</t>
+          <t>M1_TASS</t>
         </is>
       </c>
       <c r="D102" t="inlineStr">
@@ -5863,89 +5857,89 @@
         </is>
       </c>
       <c r="E102" s="2" t="n">
-        <v>82.15000000000001</v>
+        <v>78.73</v>
       </c>
       <c r="F102" s="2" t="n">
-        <v>83.40000000000001</v>
+        <v>84.98</v>
       </c>
       <c r="G102" s="2" t="n">
-        <v>91.94</v>
+        <v>91.7</v>
       </c>
       <c r="H102" s="2" t="n">
-        <v>82.77</v>
+        <v>81.73999999999999</v>
       </c>
       <c r="I102" s="2" t="n">
-        <v>70.61</v>
+        <v>69.11</v>
       </c>
       <c r="J102" s="2" t="n">
-        <v>77.51000000000001</v>
+        <v>76.38</v>
       </c>
       <c r="K102" s="2" t="n">
-        <v>8.195</v>
+        <v>3.455</v>
       </c>
       <c r="L102" s="2" t="n">
-        <v>15.125</v>
+        <v>1.478</v>
       </c>
       <c r="M102" s="2" t="n">
-        <v>24.1021</v>
+        <v>3.5459</v>
       </c>
       <c r="N102" t="inlineStr">
         <is>
-          <t>baseline</t>
+          <t>str_tass</t>
         </is>
       </c>
     </row>
     <row r="103">
       <c r="A103" t="inlineStr">
         <is>
-          <t>UltraLight</t>
+          <t>STR-Fusion</t>
         </is>
       </c>
       <c r="B103" t="inlineStr">
         <is>
-          <t>Run4</t>
+          <t>Run2_TASS</t>
         </is>
       </c>
       <c r="C103" t="inlineStr">
         <is>
-          <t>R4_2_VIT4_LIGHTDETAIL</t>
+          <t>M1_TASS</t>
         </is>
       </c>
       <c r="D103" t="inlineStr">
         <is>
-          <t>SYSU-CD-256</t>
+          <t>WHU-CD-256</t>
         </is>
       </c>
       <c r="E103" s="2" t="n">
-        <v>79.94</v>
+        <v>91.64</v>
       </c>
       <c r="F103" s="2" t="n">
-        <v>84.79000000000001</v>
+        <v>94.81999999999999</v>
       </c>
       <c r="G103" s="2" t="n">
-        <v>91.89</v>
+        <v>99.47</v>
       </c>
       <c r="H103" s="2" t="n">
-        <v>82.3</v>
+        <v>93.2</v>
       </c>
       <c r="I103" s="2" t="n">
-        <v>69.92</v>
+        <v>87.27</v>
       </c>
       <c r="J103" s="2" t="n">
-        <v>77.04000000000001</v>
+        <v>92.93000000000001</v>
       </c>
       <c r="K103" s="2" t="n">
-        <v>5.492</v>
+        <v>3.455</v>
       </c>
       <c r="L103" s="2" t="n">
-        <v>3.515</v>
+        <v>1.478</v>
       </c>
       <c r="M103" s="2" t="n">
-        <v>10.7311</v>
+        <v>3.5459</v>
       </c>
       <c r="N103" t="inlineStr">
         <is>
-          <t>baseline</t>
+          <t>str_tass</t>
         </is>
       </c>
     </row>
@@ -5962,7 +5956,7 @@
       </c>
       <c r="C104" t="inlineStr">
         <is>
-          <t>R4_2b_VIT4_LIGHTDETAIL48</t>
+          <t>R4_0_A0_FULL12_FROZEN</t>
         </is>
       </c>
       <c r="D104" t="inlineStr">
@@ -5971,31 +5965,31 @@
         </is>
       </c>
       <c r="E104" s="2" t="n">
-        <v>80.87</v>
+        <v>82.42</v>
       </c>
       <c r="F104" s="2" t="n">
-        <v>83.81</v>
+        <v>83.87</v>
       </c>
       <c r="G104" s="2" t="n">
-        <v>91.81</v>
+        <v>92.12</v>
       </c>
       <c r="H104" s="2" t="n">
-        <v>82.31999999999999</v>
+        <v>83.14</v>
       </c>
       <c r="I104" s="2" t="n">
-        <v>69.95</v>
+        <v>71.14</v>
       </c>
       <c r="J104" s="2" t="n">
-        <v>76.98999999999999</v>
+        <v>77.98999999999999</v>
       </c>
       <c r="K104" s="2" t="n">
-        <v>5.533</v>
+        <v>11.754</v>
       </c>
       <c r="L104" s="2" t="n">
-        <v>3.556</v>
+        <v>15.125</v>
       </c>
       <c r="M104" s="2" t="n">
-        <v>10.9824</v>
+        <v>26.3246</v>
       </c>
       <c r="N104" t="inlineStr">
         <is>
@@ -6016,7 +6010,7 @@
       </c>
       <c r="C105" t="inlineStr">
         <is>
-          <t>R4_2d_PSD_DETAIL</t>
+          <t>R4_1_VIT4_OLDHEAD</t>
         </is>
       </c>
       <c r="D105" t="inlineStr">
@@ -6025,31 +6019,31 @@
         </is>
       </c>
       <c r="E105" s="2" t="n">
-        <v>79.78</v>
+        <v>82.15000000000001</v>
       </c>
       <c r="F105" s="2" t="n">
-        <v>84.39</v>
+        <v>83.40000000000001</v>
       </c>
       <c r="G105" s="2" t="n">
-        <v>91.75</v>
+        <v>91.94</v>
       </c>
       <c r="H105" s="2" t="n">
-        <v>82.02</v>
+        <v>82.77</v>
       </c>
       <c r="I105" s="2" t="n">
-        <v>69.52</v>
+        <v>70.61</v>
       </c>
       <c r="J105" s="2" t="n">
-        <v>76.68000000000001</v>
+        <v>77.51000000000001</v>
       </c>
       <c r="K105" s="2" t="n">
-        <v>5.491</v>
+        <v>8.195</v>
       </c>
       <c r="L105" s="2" t="n">
-        <v>3.514</v>
+        <v>15.125</v>
       </c>
       <c r="M105" s="2" t="n">
-        <v>11.5239</v>
+        <v>24.1021</v>
       </c>
       <c r="N105" t="inlineStr">
         <is>
@@ -6060,46 +6054,50 @@
     <row r="106">
       <c r="A106" t="inlineStr">
         <is>
-          <t>baseline</t>
+          <t>UltraLight</t>
         </is>
       </c>
       <c r="B106" t="inlineStr">
         <is>
-          <t>Run1</t>
-        </is>
-      </c>
-      <c r="C106" t="inlineStr"/>
+          <t>Run4</t>
+        </is>
+      </c>
+      <c r="C106" t="inlineStr">
+        <is>
+          <t>R4_2_VIT4_LIGHTDETAIL</t>
+        </is>
+      </c>
       <c r="D106" t="inlineStr">
         <is>
-          <t>CDD-CD-256</t>
+          <t>SYSU-CD-256</t>
         </is>
       </c>
       <c r="E106" s="2" t="n">
-        <v>97.72</v>
+        <v>79.94</v>
       </c>
       <c r="F106" s="2" t="n">
-        <v>97.78</v>
+        <v>84.79000000000001</v>
       </c>
       <c r="G106" s="2" t="n">
-        <v>99.44</v>
+        <v>91.89</v>
       </c>
       <c r="H106" s="2" t="n">
-        <v>97.75</v>
+        <v>82.3</v>
       </c>
       <c r="I106" s="2" t="n">
-        <v>95.59999999999999</v>
+        <v>69.92</v>
       </c>
       <c r="J106" s="2" t="n">
-        <v>97.43000000000001</v>
+        <v>77.04000000000001</v>
       </c>
       <c r="K106" s="2" t="n">
-        <v>11.754</v>
+        <v>5.492</v>
       </c>
       <c r="L106" s="2" t="n">
-        <v>20.661</v>
+        <v>3.515</v>
       </c>
       <c r="M106" s="2" t="n">
-        <v>26.3246</v>
+        <v>10.7311</v>
       </c>
       <c r="N106" t="inlineStr">
         <is>
@@ -6110,46 +6108,50 @@
     <row r="107">
       <c r="A107" t="inlineStr">
         <is>
-          <t>baseline</t>
+          <t>UltraLight</t>
         </is>
       </c>
       <c r="B107" t="inlineStr">
         <is>
-          <t>Run1</t>
-        </is>
-      </c>
-      <c r="C107" t="inlineStr"/>
+          <t>Run4</t>
+        </is>
+      </c>
+      <c r="C107" t="inlineStr">
+        <is>
+          <t>R4_2b_VIT4_LIGHTDETAIL48</t>
+        </is>
+      </c>
       <c r="D107" t="inlineStr">
         <is>
-          <t>LEVIR-CD-256</t>
+          <t>SYSU-CD-256</t>
         </is>
       </c>
       <c r="E107" s="2" t="n">
-        <v>91.56999999999999</v>
+        <v>80.87</v>
       </c>
       <c r="F107" s="2" t="n">
-        <v>92.33</v>
+        <v>83.81</v>
       </c>
       <c r="G107" s="2" t="n">
-        <v>99.18000000000001</v>
+        <v>91.81</v>
       </c>
       <c r="H107" s="2" t="n">
-        <v>91.95</v>
+        <v>82.31999999999999</v>
       </c>
       <c r="I107" s="2" t="n">
-        <v>85.09999999999999</v>
+        <v>69.95</v>
       </c>
       <c r="J107" s="2" t="n">
-        <v>91.52</v>
+        <v>76.98999999999999</v>
       </c>
       <c r="K107" s="2" t="n">
-        <v>11.754</v>
+        <v>5.533</v>
       </c>
       <c r="L107" s="2" t="n">
-        <v>20.661</v>
+        <v>3.556</v>
       </c>
       <c r="M107" s="2" t="n">
-        <v>26.3246</v>
+        <v>10.9824</v>
       </c>
       <c r="N107" t="inlineStr">
         <is>
@@ -6160,46 +6162,50 @@
     <row r="108">
       <c r="A108" t="inlineStr">
         <is>
-          <t>baseline</t>
+          <t>UltraLight</t>
         </is>
       </c>
       <c r="B108" t="inlineStr">
         <is>
-          <t>Run1</t>
-        </is>
-      </c>
-      <c r="C108" t="inlineStr"/>
+          <t>Run4</t>
+        </is>
+      </c>
+      <c r="C108" t="inlineStr">
+        <is>
+          <t>R4_2d_PSD_DETAIL</t>
+        </is>
+      </c>
       <c r="D108" t="inlineStr">
         <is>
           <t>SYSU-CD-256</t>
         </is>
       </c>
       <c r="E108" s="2" t="n">
-        <v>80.77</v>
+        <v>79.78</v>
       </c>
       <c r="F108" s="2" t="n">
-        <v>84.27</v>
+        <v>84.39</v>
       </c>
       <c r="G108" s="2" t="n">
-        <v>91.91</v>
+        <v>91.75</v>
       </c>
       <c r="H108" s="2" t="n">
-        <v>82.48</v>
+        <v>82.02</v>
       </c>
       <c r="I108" s="2" t="n">
-        <v>70.19</v>
+        <v>69.52</v>
       </c>
       <c r="J108" s="2" t="n">
-        <v>77.23</v>
+        <v>76.68000000000001</v>
       </c>
       <c r="K108" s="2" t="n">
-        <v>11.754</v>
+        <v>5.491</v>
       </c>
       <c r="L108" s="2" t="n">
-        <v>20.661</v>
+        <v>3.514</v>
       </c>
       <c r="M108" s="2" t="n">
-        <v>26.3246</v>
+        <v>11.5239</v>
       </c>
       <c r="N108" t="inlineStr">
         <is>
@@ -6221,26 +6227,26 @@
       <c r="C109" t="inlineStr"/>
       <c r="D109" t="inlineStr">
         <is>
-          <t>WHU-CD-256</t>
+          <t>CDD-CD-256</t>
         </is>
       </c>
       <c r="E109" s="2" t="n">
-        <v>93.62</v>
+        <v>97.72</v>
       </c>
       <c r="F109" s="2" t="n">
-        <v>96.09</v>
+        <v>97.78</v>
       </c>
       <c r="G109" s="2" t="n">
-        <v>99.59999999999999</v>
+        <v>99.44</v>
       </c>
       <c r="H109" s="2" t="n">
-        <v>94.84</v>
+        <v>97.75</v>
       </c>
       <c r="I109" s="2" t="n">
-        <v>90.18000000000001</v>
+        <v>95.59999999999999</v>
       </c>
       <c r="J109" s="2" t="n">
-        <v>94.63</v>
+        <v>97.43000000000001</v>
       </c>
       <c r="K109" s="2" t="n">
         <v>11.754</v>
@@ -6257,8 +6263,158 @@
         </is>
       </c>
     </row>
+    <row r="110">
+      <c r="A110" t="inlineStr">
+        <is>
+          <t>baseline</t>
+        </is>
+      </c>
+      <c r="B110" t="inlineStr">
+        <is>
+          <t>Run1</t>
+        </is>
+      </c>
+      <c r="C110" t="inlineStr"/>
+      <c r="D110" t="inlineStr">
+        <is>
+          <t>LEVIR-CD-256</t>
+        </is>
+      </c>
+      <c r="E110" s="2" t="n">
+        <v>91.56999999999999</v>
+      </c>
+      <c r="F110" s="2" t="n">
+        <v>92.33</v>
+      </c>
+      <c r="G110" s="2" t="n">
+        <v>99.18000000000001</v>
+      </c>
+      <c r="H110" s="2" t="n">
+        <v>91.95</v>
+      </c>
+      <c r="I110" s="2" t="n">
+        <v>85.09999999999999</v>
+      </c>
+      <c r="J110" s="2" t="n">
+        <v>91.52</v>
+      </c>
+      <c r="K110" s="2" t="n">
+        <v>11.754</v>
+      </c>
+      <c r="L110" s="2" t="n">
+        <v>20.661</v>
+      </c>
+      <c r="M110" s="2" t="n">
+        <v>26.3246</v>
+      </c>
+      <c r="N110" t="inlineStr">
+        <is>
+          <t>baseline</t>
+        </is>
+      </c>
+    </row>
+    <row r="111">
+      <c r="A111" t="inlineStr">
+        <is>
+          <t>baseline</t>
+        </is>
+      </c>
+      <c r="B111" t="inlineStr">
+        <is>
+          <t>Run1</t>
+        </is>
+      </c>
+      <c r="C111" t="inlineStr"/>
+      <c r="D111" t="inlineStr">
+        <is>
+          <t>SYSU-CD-256</t>
+        </is>
+      </c>
+      <c r="E111" s="2" t="n">
+        <v>80.77</v>
+      </c>
+      <c r="F111" s="2" t="n">
+        <v>84.27</v>
+      </c>
+      <c r="G111" s="2" t="n">
+        <v>91.91</v>
+      </c>
+      <c r="H111" s="2" t="n">
+        <v>82.48</v>
+      </c>
+      <c r="I111" s="2" t="n">
+        <v>70.19</v>
+      </c>
+      <c r="J111" s="2" t="n">
+        <v>77.23</v>
+      </c>
+      <c r="K111" s="2" t="n">
+        <v>11.754</v>
+      </c>
+      <c r="L111" s="2" t="n">
+        <v>20.661</v>
+      </c>
+      <c r="M111" s="2" t="n">
+        <v>26.3246</v>
+      </c>
+      <c r="N111" t="inlineStr">
+        <is>
+          <t>baseline</t>
+        </is>
+      </c>
+    </row>
+    <row r="112">
+      <c r="A112" t="inlineStr">
+        <is>
+          <t>baseline</t>
+        </is>
+      </c>
+      <c r="B112" t="inlineStr">
+        <is>
+          <t>Run1</t>
+        </is>
+      </c>
+      <c r="C112" t="inlineStr"/>
+      <c r="D112" t="inlineStr">
+        <is>
+          <t>WHU-CD-256</t>
+        </is>
+      </c>
+      <c r="E112" s="2" t="n">
+        <v>93.62</v>
+      </c>
+      <c r="F112" s="2" t="n">
+        <v>96.09</v>
+      </c>
+      <c r="G112" s="2" t="n">
+        <v>99.59999999999999</v>
+      </c>
+      <c r="H112" s="2" t="n">
+        <v>94.84</v>
+      </c>
+      <c r="I112" s="2" t="n">
+        <v>90.18000000000001</v>
+      </c>
+      <c r="J112" s="2" t="n">
+        <v>94.63</v>
+      </c>
+      <c r="K112" s="2" t="n">
+        <v>11.754</v>
+      </c>
+      <c r="L112" s="2" t="n">
+        <v>20.661</v>
+      </c>
+      <c r="M112" s="2" t="n">
+        <v>26.3246</v>
+      </c>
+      <c r="N112" t="inlineStr">
+        <is>
+          <t>baseline</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:N109"/>
+  <autoFilter ref="A1:N112"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Record CASA Run3 LEVIR and SYSU control results
</commit_message>
<xml_diff>
--- a/docs/experiment_metrics.xlsx
+++ b/docs/experiment_metrics.xlsx
@@ -10,7 +10,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="metrics" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'metrics'!$A$1:$N$112</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'metrics'!$A$1:$N$116</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -420,7 +420,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N112"/>
+  <dimension ref="A1:N116"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -5514,216 +5514,208 @@
     <row r="96">
       <c r="A96" t="inlineStr">
         <is>
-          <t>STR-Fusion</t>
+          <t>CASA</t>
         </is>
       </c>
       <c r="B96" t="inlineStr">
         <is>
-          <t>Run2_TASS</t>
+          <t>Run3</t>
         </is>
       </c>
       <c r="C96" t="inlineStr">
         <is>
-          <t>C0_TOKEN</t>
+          <t>M0_CTRL</t>
         </is>
       </c>
       <c r="D96" t="inlineStr">
         <is>
-          <t>CDD-CD-256</t>
+          <t>LEVIR-CD-256</t>
         </is>
       </c>
       <c r="E96" s="2" t="n">
-        <v>93.13</v>
+        <v>90.41</v>
       </c>
       <c r="F96" s="2" t="n">
-        <v>95.16</v>
+        <v>91.83</v>
       </c>
       <c r="G96" s="2" t="n">
-        <v>98.56999999999999</v>
+        <v>99.09999999999999</v>
       </c>
       <c r="H96" s="2" t="n">
-        <v>94.13</v>
+        <v>91.11</v>
       </c>
       <c r="I96" s="2" t="n">
-        <v>88.91</v>
+        <v>83.67</v>
       </c>
       <c r="J96" s="2" t="n">
-        <v>93.31999999999999</v>
+        <v>90.64</v>
       </c>
       <c r="K96" s="2" t="n">
-        <v>2.596</v>
+        <v>3.016737</v>
       </c>
       <c r="L96" s="2" t="n">
-        <v>0.62</v>
-      </c>
-      <c r="M96" s="2" t="n">
-        <v>2.2136</v>
-      </c>
+        <v>3.100404</v>
+      </c>
+      <c r="M96" s="2" t="n"/>
       <c r="N96" t="inlineStr">
         <is>
-          <t>str_tass</t>
+          <t>casa_none</t>
         </is>
       </c>
     </row>
     <row r="97">
       <c r="A97" t="inlineStr">
         <is>
-          <t>STR-Fusion</t>
+          <t>CASA</t>
         </is>
       </c>
       <c r="B97" t="inlineStr">
         <is>
-          <t>Run2_TASS</t>
+          <t>Run3</t>
         </is>
       </c>
       <c r="C97" t="inlineStr">
         <is>
-          <t>C0_TOKEN</t>
+          <t>M0_CTRL</t>
         </is>
       </c>
       <c r="D97" t="inlineStr">
         <is>
-          <t>LEVIR-CD-256</t>
+          <t>SYSU-CD-256</t>
         </is>
       </c>
       <c r="E97" s="2" t="n">
-        <v>86.37</v>
+        <v>79.81</v>
       </c>
       <c r="F97" s="2" t="n">
-        <v>89.25</v>
+        <v>83.84999999999999</v>
       </c>
       <c r="G97" s="2" t="n">
-        <v>98.78</v>
+        <v>91.61</v>
       </c>
       <c r="H97" s="2" t="n">
-        <v>87.79000000000001</v>
+        <v>81.78</v>
       </c>
       <c r="I97" s="2" t="n">
-        <v>78.23999999999999</v>
+        <v>69.18000000000001</v>
       </c>
       <c r="J97" s="2" t="n">
-        <v>87.14</v>
+        <v>76.34</v>
       </c>
       <c r="K97" s="2" t="n">
-        <v>2.596</v>
+        <v>3.016737</v>
       </c>
       <c r="L97" s="2" t="n">
-        <v>0.62</v>
-      </c>
-      <c r="M97" s="2" t="n">
-        <v>2.2136</v>
-      </c>
+        <v>3.100404</v>
+      </c>
+      <c r="M97" s="2" t="n"/>
       <c r="N97" t="inlineStr">
         <is>
-          <t>str_tass</t>
+          <t>casa_none</t>
         </is>
       </c>
     </row>
     <row r="98">
       <c r="A98" t="inlineStr">
         <is>
-          <t>STR-Fusion</t>
+          <t>CASA</t>
         </is>
       </c>
       <c r="B98" t="inlineStr">
         <is>
-          <t>Run2_TASS</t>
+          <t>Run3</t>
         </is>
       </c>
       <c r="C98" t="inlineStr">
         <is>
-          <t>C0_TOKEN</t>
+          <t>M1_HYPER_QKV</t>
         </is>
       </c>
       <c r="D98" t="inlineStr">
         <is>
-          <t>SYSU-CD-256</t>
+          <t>LEVIR-CD-256</t>
         </is>
       </c>
       <c r="E98" s="2" t="n">
-        <v>79.93000000000001</v>
+        <v>90.61</v>
       </c>
       <c r="F98" s="2" t="n">
-        <v>84.5</v>
+        <v>92.37</v>
       </c>
       <c r="G98" s="2" t="n">
-        <v>91.81</v>
+        <v>99.14</v>
       </c>
       <c r="H98" s="2" t="n">
-        <v>82.15000000000001</v>
+        <v>91.48</v>
       </c>
       <c r="I98" s="2" t="n">
-        <v>69.70999999999999</v>
+        <v>84.3</v>
       </c>
       <c r="J98" s="2" t="n">
-        <v>76.84</v>
+        <v>91.03</v>
       </c>
       <c r="K98" s="2" t="n">
-        <v>2.596</v>
+        <v>3.050665</v>
       </c>
       <c r="L98" s="2" t="n">
-        <v>0.62</v>
-      </c>
-      <c r="M98" s="2" t="n">
-        <v>2.2136</v>
-      </c>
+        <v>3.134332</v>
+      </c>
+      <c r="M98" s="2" t="n"/>
       <c r="N98" t="inlineStr">
         <is>
-          <t>str_tass</t>
+          <t>casa_hyperbolic</t>
         </is>
       </c>
     </row>
     <row r="99">
       <c r="A99" t="inlineStr">
         <is>
-          <t>STR-Fusion</t>
+          <t>CASA</t>
         </is>
       </c>
       <c r="B99" t="inlineStr">
         <is>
-          <t>Run2_TASS</t>
+          <t>Run3</t>
         </is>
       </c>
       <c r="C99" t="inlineStr">
         <is>
-          <t>C0_TOKEN</t>
+          <t>M2_CA_QKV</t>
         </is>
       </c>
       <c r="D99" t="inlineStr">
         <is>
-          <t>WHU-CD-256</t>
+          <t>LEVIR-CD-256</t>
         </is>
       </c>
       <c r="E99" s="2" t="n">
-        <v>90.16</v>
+        <v>90.58</v>
       </c>
       <c r="F99" s="2" t="n">
-        <v>93.97</v>
+        <v>91.77</v>
       </c>
       <c r="G99" s="2" t="n">
-        <v>99.38</v>
+        <v>99.11</v>
       </c>
       <c r="H99" s="2" t="n">
-        <v>92.02</v>
+        <v>91.17</v>
       </c>
       <c r="I99" s="2" t="n">
-        <v>85.23</v>
+        <v>83.77</v>
       </c>
       <c r="J99" s="2" t="n">
-        <v>91.7</v>
+        <v>90.7</v>
       </c>
       <c r="K99" s="2" t="n">
-        <v>2.596</v>
+        <v>3.059369</v>
       </c>
       <c r="L99" s="2" t="n">
-        <v>0.62</v>
-      </c>
-      <c r="M99" s="2" t="n">
-        <v>2.2136</v>
-      </c>
+        <v>3.143036</v>
+      </c>
+      <c r="M99" s="2" t="n"/>
       <c r="N99" t="inlineStr">
         <is>
-          <t>str_tass</t>
+          <t>casa_qkv</t>
         </is>
       </c>
     </row>
@@ -5740,7 +5732,7 @@
       </c>
       <c r="C100" t="inlineStr">
         <is>
-          <t>M1_TASS</t>
+          <t>C0_TOKEN</t>
         </is>
       </c>
       <c r="D100" t="inlineStr">
@@ -5749,31 +5741,31 @@
         </is>
       </c>
       <c r="E100" s="2" t="n">
-        <v>94.7</v>
+        <v>93.13</v>
       </c>
       <c r="F100" s="2" t="n">
-        <v>96.13</v>
+        <v>95.16</v>
       </c>
       <c r="G100" s="2" t="n">
-        <v>98.88</v>
+        <v>98.56999999999999</v>
       </c>
       <c r="H100" s="2" t="n">
-        <v>95.41</v>
+        <v>94.13</v>
       </c>
       <c r="I100" s="2" t="n">
-        <v>91.22</v>
+        <v>88.91</v>
       </c>
       <c r="J100" s="2" t="n">
-        <v>94.77</v>
+        <v>93.31999999999999</v>
       </c>
       <c r="K100" s="2" t="n">
-        <v>3.455</v>
+        <v>2.596</v>
       </c>
       <c r="L100" s="2" t="n">
-        <v>1.478</v>
+        <v>0.62</v>
       </c>
       <c r="M100" s="2" t="n">
-        <v>3.5459</v>
+        <v>2.2136</v>
       </c>
       <c r="N100" t="inlineStr">
         <is>
@@ -5794,7 +5786,7 @@
       </c>
       <c r="C101" t="inlineStr">
         <is>
-          <t>M1_TASS</t>
+          <t>C0_TOKEN</t>
         </is>
       </c>
       <c r="D101" t="inlineStr">
@@ -5803,31 +5795,31 @@
         </is>
       </c>
       <c r="E101" s="2" t="n">
-        <v>88.42</v>
+        <v>86.37</v>
       </c>
       <c r="F101" s="2" t="n">
-        <v>91.97</v>
+        <v>89.25</v>
       </c>
       <c r="G101" s="2" t="n">
-        <v>99.02</v>
+        <v>98.78</v>
       </c>
       <c r="H101" s="2" t="n">
-        <v>90.16</v>
+        <v>87.79000000000001</v>
       </c>
       <c r="I101" s="2" t="n">
-        <v>82.08</v>
+        <v>78.23999999999999</v>
       </c>
       <c r="J101" s="2" t="n">
-        <v>89.64</v>
+        <v>87.14</v>
       </c>
       <c r="K101" s="2" t="n">
-        <v>3.455</v>
+        <v>2.596</v>
       </c>
       <c r="L101" s="2" t="n">
-        <v>1.478</v>
+        <v>0.62</v>
       </c>
       <c r="M101" s="2" t="n">
-        <v>3.5459</v>
+        <v>2.2136</v>
       </c>
       <c r="N101" t="inlineStr">
         <is>
@@ -5848,7 +5840,7 @@
       </c>
       <c r="C102" t="inlineStr">
         <is>
-          <t>M1_TASS</t>
+          <t>C0_TOKEN</t>
         </is>
       </c>
       <c r="D102" t="inlineStr">
@@ -5857,31 +5849,31 @@
         </is>
       </c>
       <c r="E102" s="2" t="n">
-        <v>78.73</v>
+        <v>79.93000000000001</v>
       </c>
       <c r="F102" s="2" t="n">
-        <v>84.98</v>
+        <v>84.5</v>
       </c>
       <c r="G102" s="2" t="n">
-        <v>91.7</v>
+        <v>91.81</v>
       </c>
       <c r="H102" s="2" t="n">
-        <v>81.73999999999999</v>
+        <v>82.15000000000001</v>
       </c>
       <c r="I102" s="2" t="n">
-        <v>69.11</v>
+        <v>69.70999999999999</v>
       </c>
       <c r="J102" s="2" t="n">
-        <v>76.38</v>
+        <v>76.84</v>
       </c>
       <c r="K102" s="2" t="n">
-        <v>3.455</v>
+        <v>2.596</v>
       </c>
       <c r="L102" s="2" t="n">
-        <v>1.478</v>
+        <v>0.62</v>
       </c>
       <c r="M102" s="2" t="n">
-        <v>3.5459</v>
+        <v>2.2136</v>
       </c>
       <c r="N102" t="inlineStr">
         <is>
@@ -5902,7 +5894,7 @@
       </c>
       <c r="C103" t="inlineStr">
         <is>
-          <t>M1_TASS</t>
+          <t>C0_TOKEN</t>
         </is>
       </c>
       <c r="D103" t="inlineStr">
@@ -5911,31 +5903,31 @@
         </is>
       </c>
       <c r="E103" s="2" t="n">
-        <v>91.64</v>
+        <v>90.16</v>
       </c>
       <c r="F103" s="2" t="n">
-        <v>94.81999999999999</v>
+        <v>93.97</v>
       </c>
       <c r="G103" s="2" t="n">
-        <v>99.47</v>
+        <v>99.38</v>
       </c>
       <c r="H103" s="2" t="n">
-        <v>93.2</v>
+        <v>92.02</v>
       </c>
       <c r="I103" s="2" t="n">
-        <v>87.27</v>
+        <v>85.23</v>
       </c>
       <c r="J103" s="2" t="n">
-        <v>92.93000000000001</v>
+        <v>91.7</v>
       </c>
       <c r="K103" s="2" t="n">
-        <v>3.455</v>
+        <v>2.596</v>
       </c>
       <c r="L103" s="2" t="n">
-        <v>1.478</v>
+        <v>0.62</v>
       </c>
       <c r="M103" s="2" t="n">
-        <v>3.5459</v>
+        <v>2.2136</v>
       </c>
       <c r="N103" t="inlineStr">
         <is>
@@ -5946,125 +5938,125 @@
     <row r="104">
       <c r="A104" t="inlineStr">
         <is>
-          <t>UltraLight</t>
+          <t>STR-Fusion</t>
         </is>
       </c>
       <c r="B104" t="inlineStr">
         <is>
-          <t>Run4</t>
+          <t>Run2_TASS</t>
         </is>
       </c>
       <c r="C104" t="inlineStr">
         <is>
-          <t>R4_0_A0_FULL12_FROZEN</t>
+          <t>M1_TASS</t>
         </is>
       </c>
       <c r="D104" t="inlineStr">
         <is>
-          <t>SYSU-CD-256</t>
+          <t>CDD-CD-256</t>
         </is>
       </c>
       <c r="E104" s="2" t="n">
-        <v>82.42</v>
+        <v>94.7</v>
       </c>
       <c r="F104" s="2" t="n">
-        <v>83.87</v>
+        <v>96.13</v>
       </c>
       <c r="G104" s="2" t="n">
-        <v>92.12</v>
+        <v>98.88</v>
       </c>
       <c r="H104" s="2" t="n">
-        <v>83.14</v>
+        <v>95.41</v>
       </c>
       <c r="I104" s="2" t="n">
-        <v>71.14</v>
+        <v>91.22</v>
       </c>
       <c r="J104" s="2" t="n">
-        <v>77.98999999999999</v>
+        <v>94.77</v>
       </c>
       <c r="K104" s="2" t="n">
-        <v>11.754</v>
+        <v>3.455</v>
       </c>
       <c r="L104" s="2" t="n">
-        <v>15.125</v>
+        <v>1.478</v>
       </c>
       <c r="M104" s="2" t="n">
-        <v>26.3246</v>
+        <v>3.5459</v>
       </c>
       <c r="N104" t="inlineStr">
         <is>
-          <t>baseline</t>
+          <t>str_tass</t>
         </is>
       </c>
     </row>
     <row r="105">
       <c r="A105" t="inlineStr">
         <is>
-          <t>UltraLight</t>
+          <t>STR-Fusion</t>
         </is>
       </c>
       <c r="B105" t="inlineStr">
         <is>
-          <t>Run4</t>
+          <t>Run2_TASS</t>
         </is>
       </c>
       <c r="C105" t="inlineStr">
         <is>
-          <t>R4_1_VIT4_OLDHEAD</t>
+          <t>M1_TASS</t>
         </is>
       </c>
       <c r="D105" t="inlineStr">
         <is>
-          <t>SYSU-CD-256</t>
+          <t>LEVIR-CD-256</t>
         </is>
       </c>
       <c r="E105" s="2" t="n">
-        <v>82.15000000000001</v>
+        <v>88.42</v>
       </c>
       <c r="F105" s="2" t="n">
-        <v>83.40000000000001</v>
+        <v>91.97</v>
       </c>
       <c r="G105" s="2" t="n">
-        <v>91.94</v>
+        <v>99.02</v>
       </c>
       <c r="H105" s="2" t="n">
-        <v>82.77</v>
+        <v>90.16</v>
       </c>
       <c r="I105" s="2" t="n">
-        <v>70.61</v>
+        <v>82.08</v>
       </c>
       <c r="J105" s="2" t="n">
-        <v>77.51000000000001</v>
+        <v>89.64</v>
       </c>
       <c r="K105" s="2" t="n">
-        <v>8.195</v>
+        <v>3.455</v>
       </c>
       <c r="L105" s="2" t="n">
-        <v>15.125</v>
+        <v>1.478</v>
       </c>
       <c r="M105" s="2" t="n">
-        <v>24.1021</v>
+        <v>3.5459</v>
       </c>
       <c r="N105" t="inlineStr">
         <is>
-          <t>baseline</t>
+          <t>str_tass</t>
         </is>
       </c>
     </row>
     <row r="106">
       <c r="A106" t="inlineStr">
         <is>
-          <t>UltraLight</t>
+          <t>STR-Fusion</t>
         </is>
       </c>
       <c r="B106" t="inlineStr">
         <is>
-          <t>Run4</t>
+          <t>Run2_TASS</t>
         </is>
       </c>
       <c r="C106" t="inlineStr">
         <is>
-          <t>R4_2_VIT4_LIGHTDETAIL</t>
+          <t>M1_TASS</t>
         </is>
       </c>
       <c r="D106" t="inlineStr">
@@ -6073,89 +6065,89 @@
         </is>
       </c>
       <c r="E106" s="2" t="n">
-        <v>79.94</v>
+        <v>78.73</v>
       </c>
       <c r="F106" s="2" t="n">
-        <v>84.79000000000001</v>
+        <v>84.98</v>
       </c>
       <c r="G106" s="2" t="n">
-        <v>91.89</v>
+        <v>91.7</v>
       </c>
       <c r="H106" s="2" t="n">
-        <v>82.3</v>
+        <v>81.73999999999999</v>
       </c>
       <c r="I106" s="2" t="n">
-        <v>69.92</v>
+        <v>69.11</v>
       </c>
       <c r="J106" s="2" t="n">
-        <v>77.04000000000001</v>
+        <v>76.38</v>
       </c>
       <c r="K106" s="2" t="n">
-        <v>5.492</v>
+        <v>3.455</v>
       </c>
       <c r="L106" s="2" t="n">
-        <v>3.515</v>
+        <v>1.478</v>
       </c>
       <c r="M106" s="2" t="n">
-        <v>10.7311</v>
+        <v>3.5459</v>
       </c>
       <c r="N106" t="inlineStr">
         <is>
-          <t>baseline</t>
+          <t>str_tass</t>
         </is>
       </c>
     </row>
     <row r="107">
       <c r="A107" t="inlineStr">
         <is>
-          <t>UltraLight</t>
+          <t>STR-Fusion</t>
         </is>
       </c>
       <c r="B107" t="inlineStr">
         <is>
-          <t>Run4</t>
+          <t>Run2_TASS</t>
         </is>
       </c>
       <c r="C107" t="inlineStr">
         <is>
-          <t>R4_2b_VIT4_LIGHTDETAIL48</t>
+          <t>M1_TASS</t>
         </is>
       </c>
       <c r="D107" t="inlineStr">
         <is>
-          <t>SYSU-CD-256</t>
+          <t>WHU-CD-256</t>
         </is>
       </c>
       <c r="E107" s="2" t="n">
-        <v>80.87</v>
+        <v>91.64</v>
       </c>
       <c r="F107" s="2" t="n">
-        <v>83.81</v>
+        <v>94.81999999999999</v>
       </c>
       <c r="G107" s="2" t="n">
-        <v>91.81</v>
+        <v>99.47</v>
       </c>
       <c r="H107" s="2" t="n">
-        <v>82.31999999999999</v>
+        <v>93.2</v>
       </c>
       <c r="I107" s="2" t="n">
-        <v>69.95</v>
+        <v>87.27</v>
       </c>
       <c r="J107" s="2" t="n">
-        <v>76.98999999999999</v>
+        <v>92.93000000000001</v>
       </c>
       <c r="K107" s="2" t="n">
-        <v>5.533</v>
+        <v>3.455</v>
       </c>
       <c r="L107" s="2" t="n">
-        <v>3.556</v>
+        <v>1.478</v>
       </c>
       <c r="M107" s="2" t="n">
-        <v>10.9824</v>
+        <v>3.5459</v>
       </c>
       <c r="N107" t="inlineStr">
         <is>
-          <t>baseline</t>
+          <t>str_tass</t>
         </is>
       </c>
     </row>
@@ -6172,7 +6164,7 @@
       </c>
       <c r="C108" t="inlineStr">
         <is>
-          <t>R4_2d_PSD_DETAIL</t>
+          <t>R4_0_A0_FULL12_FROZEN</t>
         </is>
       </c>
       <c r="D108" t="inlineStr">
@@ -6181,31 +6173,31 @@
         </is>
       </c>
       <c r="E108" s="2" t="n">
-        <v>79.78</v>
+        <v>82.42</v>
       </c>
       <c r="F108" s="2" t="n">
-        <v>84.39</v>
+        <v>83.87</v>
       </c>
       <c r="G108" s="2" t="n">
-        <v>91.75</v>
+        <v>92.12</v>
       </c>
       <c r="H108" s="2" t="n">
-        <v>82.02</v>
+        <v>83.14</v>
       </c>
       <c r="I108" s="2" t="n">
-        <v>69.52</v>
+        <v>71.14</v>
       </c>
       <c r="J108" s="2" t="n">
-        <v>76.68000000000001</v>
+        <v>77.98999999999999</v>
       </c>
       <c r="K108" s="2" t="n">
-        <v>5.491</v>
+        <v>11.754</v>
       </c>
       <c r="L108" s="2" t="n">
-        <v>3.514</v>
+        <v>15.125</v>
       </c>
       <c r="M108" s="2" t="n">
-        <v>11.5239</v>
+        <v>26.3246</v>
       </c>
       <c r="N108" t="inlineStr">
         <is>
@@ -6216,46 +6208,50 @@
     <row r="109">
       <c r="A109" t="inlineStr">
         <is>
-          <t>baseline</t>
+          <t>UltraLight</t>
         </is>
       </c>
       <c r="B109" t="inlineStr">
         <is>
-          <t>Run1</t>
-        </is>
-      </c>
-      <c r="C109" t="inlineStr"/>
+          <t>Run4</t>
+        </is>
+      </c>
+      <c r="C109" t="inlineStr">
+        <is>
+          <t>R4_1_VIT4_OLDHEAD</t>
+        </is>
+      </c>
       <c r="D109" t="inlineStr">
         <is>
-          <t>CDD-CD-256</t>
+          <t>SYSU-CD-256</t>
         </is>
       </c>
       <c r="E109" s="2" t="n">
-        <v>97.72</v>
+        <v>82.15000000000001</v>
       </c>
       <c r="F109" s="2" t="n">
-        <v>97.78</v>
+        <v>83.40000000000001</v>
       </c>
       <c r="G109" s="2" t="n">
-        <v>99.44</v>
+        <v>91.94</v>
       </c>
       <c r="H109" s="2" t="n">
-        <v>97.75</v>
+        <v>82.77</v>
       </c>
       <c r="I109" s="2" t="n">
-        <v>95.59999999999999</v>
+        <v>70.61</v>
       </c>
       <c r="J109" s="2" t="n">
-        <v>97.43000000000001</v>
+        <v>77.51000000000001</v>
       </c>
       <c r="K109" s="2" t="n">
-        <v>11.754</v>
+        <v>8.195</v>
       </c>
       <c r="L109" s="2" t="n">
-        <v>20.661</v>
+        <v>15.125</v>
       </c>
       <c r="M109" s="2" t="n">
-        <v>26.3246</v>
+        <v>24.1021</v>
       </c>
       <c r="N109" t="inlineStr">
         <is>
@@ -6266,46 +6262,50 @@
     <row r="110">
       <c r="A110" t="inlineStr">
         <is>
-          <t>baseline</t>
+          <t>UltraLight</t>
         </is>
       </c>
       <c r="B110" t="inlineStr">
         <is>
-          <t>Run1</t>
-        </is>
-      </c>
-      <c r="C110" t="inlineStr"/>
+          <t>Run4</t>
+        </is>
+      </c>
+      <c r="C110" t="inlineStr">
+        <is>
+          <t>R4_2_VIT4_LIGHTDETAIL</t>
+        </is>
+      </c>
       <c r="D110" t="inlineStr">
         <is>
-          <t>LEVIR-CD-256</t>
+          <t>SYSU-CD-256</t>
         </is>
       </c>
       <c r="E110" s="2" t="n">
-        <v>91.56999999999999</v>
+        <v>79.94</v>
       </c>
       <c r="F110" s="2" t="n">
-        <v>92.33</v>
+        <v>84.79000000000001</v>
       </c>
       <c r="G110" s="2" t="n">
-        <v>99.18000000000001</v>
+        <v>91.89</v>
       </c>
       <c r="H110" s="2" t="n">
-        <v>91.95</v>
+        <v>82.3</v>
       </c>
       <c r="I110" s="2" t="n">
-        <v>85.09999999999999</v>
+        <v>69.92</v>
       </c>
       <c r="J110" s="2" t="n">
-        <v>91.52</v>
+        <v>77.04000000000001</v>
       </c>
       <c r="K110" s="2" t="n">
-        <v>11.754</v>
+        <v>5.492</v>
       </c>
       <c r="L110" s="2" t="n">
-        <v>20.661</v>
+        <v>3.515</v>
       </c>
       <c r="M110" s="2" t="n">
-        <v>26.3246</v>
+        <v>10.7311</v>
       </c>
       <c r="N110" t="inlineStr">
         <is>
@@ -6316,46 +6316,50 @@
     <row r="111">
       <c r="A111" t="inlineStr">
         <is>
-          <t>baseline</t>
+          <t>UltraLight</t>
         </is>
       </c>
       <c r="B111" t="inlineStr">
         <is>
-          <t>Run1</t>
-        </is>
-      </c>
-      <c r="C111" t="inlineStr"/>
+          <t>Run4</t>
+        </is>
+      </c>
+      <c r="C111" t="inlineStr">
+        <is>
+          <t>R4_2b_VIT4_LIGHTDETAIL48</t>
+        </is>
+      </c>
       <c r="D111" t="inlineStr">
         <is>
           <t>SYSU-CD-256</t>
         </is>
       </c>
       <c r="E111" s="2" t="n">
-        <v>80.77</v>
+        <v>80.87</v>
       </c>
       <c r="F111" s="2" t="n">
-        <v>84.27</v>
+        <v>83.81</v>
       </c>
       <c r="G111" s="2" t="n">
-        <v>91.91</v>
+        <v>91.81</v>
       </c>
       <c r="H111" s="2" t="n">
-        <v>82.48</v>
+        <v>82.31999999999999</v>
       </c>
       <c r="I111" s="2" t="n">
-        <v>70.19</v>
+        <v>69.95</v>
       </c>
       <c r="J111" s="2" t="n">
-        <v>77.23</v>
+        <v>76.98999999999999</v>
       </c>
       <c r="K111" s="2" t="n">
-        <v>11.754</v>
+        <v>5.533</v>
       </c>
       <c r="L111" s="2" t="n">
-        <v>20.661</v>
+        <v>3.556</v>
       </c>
       <c r="M111" s="2" t="n">
-        <v>26.3246</v>
+        <v>10.9824</v>
       </c>
       <c r="N111" t="inlineStr">
         <is>
@@ -6366,55 +6370,259 @@
     <row r="112">
       <c r="A112" t="inlineStr">
         <is>
+          <t>UltraLight</t>
+        </is>
+      </c>
+      <c r="B112" t="inlineStr">
+        <is>
+          <t>Run4</t>
+        </is>
+      </c>
+      <c r="C112" t="inlineStr">
+        <is>
+          <t>R4_2d_PSD_DETAIL</t>
+        </is>
+      </c>
+      <c r="D112" t="inlineStr">
+        <is>
+          <t>SYSU-CD-256</t>
+        </is>
+      </c>
+      <c r="E112" s="2" t="n">
+        <v>79.78</v>
+      </c>
+      <c r="F112" s="2" t="n">
+        <v>84.39</v>
+      </c>
+      <c r="G112" s="2" t="n">
+        <v>91.75</v>
+      </c>
+      <c r="H112" s="2" t="n">
+        <v>82.02</v>
+      </c>
+      <c r="I112" s="2" t="n">
+        <v>69.52</v>
+      </c>
+      <c r="J112" s="2" t="n">
+        <v>76.68000000000001</v>
+      </c>
+      <c r="K112" s="2" t="n">
+        <v>5.491</v>
+      </c>
+      <c r="L112" s="2" t="n">
+        <v>3.514</v>
+      </c>
+      <c r="M112" s="2" t="n">
+        <v>11.5239</v>
+      </c>
+      <c r="N112" t="inlineStr">
+        <is>
           <t>baseline</t>
         </is>
       </c>
-      <c r="B112" t="inlineStr">
+    </row>
+    <row r="113">
+      <c r="A113" t="inlineStr">
+        <is>
+          <t>baseline</t>
+        </is>
+      </c>
+      <c r="B113" t="inlineStr">
         <is>
           <t>Run1</t>
         </is>
       </c>
-      <c r="C112" t="inlineStr"/>
-      <c r="D112" t="inlineStr">
+      <c r="C113" t="inlineStr"/>
+      <c r="D113" t="inlineStr">
+        <is>
+          <t>CDD-CD-256</t>
+        </is>
+      </c>
+      <c r="E113" s="2" t="n">
+        <v>97.72</v>
+      </c>
+      <c r="F113" s="2" t="n">
+        <v>97.78</v>
+      </c>
+      <c r="G113" s="2" t="n">
+        <v>99.44</v>
+      </c>
+      <c r="H113" s="2" t="n">
+        <v>97.75</v>
+      </c>
+      <c r="I113" s="2" t="n">
+        <v>95.59999999999999</v>
+      </c>
+      <c r="J113" s="2" t="n">
+        <v>97.43000000000001</v>
+      </c>
+      <c r="K113" s="2" t="n">
+        <v>11.754</v>
+      </c>
+      <c r="L113" s="2" t="n">
+        <v>20.661</v>
+      </c>
+      <c r="M113" s="2" t="n">
+        <v>26.3246</v>
+      </c>
+      <c r="N113" t="inlineStr">
+        <is>
+          <t>baseline</t>
+        </is>
+      </c>
+    </row>
+    <row r="114">
+      <c r="A114" t="inlineStr">
+        <is>
+          <t>baseline</t>
+        </is>
+      </c>
+      <c r="B114" t="inlineStr">
+        <is>
+          <t>Run1</t>
+        </is>
+      </c>
+      <c r="C114" t="inlineStr"/>
+      <c r="D114" t="inlineStr">
+        <is>
+          <t>LEVIR-CD-256</t>
+        </is>
+      </c>
+      <c r="E114" s="2" t="n">
+        <v>91.56999999999999</v>
+      </c>
+      <c r="F114" s="2" t="n">
+        <v>92.33</v>
+      </c>
+      <c r="G114" s="2" t="n">
+        <v>99.18000000000001</v>
+      </c>
+      <c r="H114" s="2" t="n">
+        <v>91.95</v>
+      </c>
+      <c r="I114" s="2" t="n">
+        <v>85.09999999999999</v>
+      </c>
+      <c r="J114" s="2" t="n">
+        <v>91.52</v>
+      </c>
+      <c r="K114" s="2" t="n">
+        <v>11.754</v>
+      </c>
+      <c r="L114" s="2" t="n">
+        <v>20.661</v>
+      </c>
+      <c r="M114" s="2" t="n">
+        <v>26.3246</v>
+      </c>
+      <c r="N114" t="inlineStr">
+        <is>
+          <t>baseline</t>
+        </is>
+      </c>
+    </row>
+    <row r="115">
+      <c r="A115" t="inlineStr">
+        <is>
+          <t>baseline</t>
+        </is>
+      </c>
+      <c r="B115" t="inlineStr">
+        <is>
+          <t>Run1</t>
+        </is>
+      </c>
+      <c r="C115" t="inlineStr"/>
+      <c r="D115" t="inlineStr">
+        <is>
+          <t>SYSU-CD-256</t>
+        </is>
+      </c>
+      <c r="E115" s="2" t="n">
+        <v>80.77</v>
+      </c>
+      <c r="F115" s="2" t="n">
+        <v>84.27</v>
+      </c>
+      <c r="G115" s="2" t="n">
+        <v>91.91</v>
+      </c>
+      <c r="H115" s="2" t="n">
+        <v>82.48</v>
+      </c>
+      <c r="I115" s="2" t="n">
+        <v>70.19</v>
+      </c>
+      <c r="J115" s="2" t="n">
+        <v>77.23</v>
+      </c>
+      <c r="K115" s="2" t="n">
+        <v>11.754</v>
+      </c>
+      <c r="L115" s="2" t="n">
+        <v>20.661</v>
+      </c>
+      <c r="M115" s="2" t="n">
+        <v>26.3246</v>
+      </c>
+      <c r="N115" t="inlineStr">
+        <is>
+          <t>baseline</t>
+        </is>
+      </c>
+    </row>
+    <row r="116">
+      <c r="A116" t="inlineStr">
+        <is>
+          <t>baseline</t>
+        </is>
+      </c>
+      <c r="B116" t="inlineStr">
+        <is>
+          <t>Run1</t>
+        </is>
+      </c>
+      <c r="C116" t="inlineStr"/>
+      <c r="D116" t="inlineStr">
         <is>
           <t>WHU-CD-256</t>
         </is>
       </c>
-      <c r="E112" s="2" t="n">
+      <c r="E116" s="2" t="n">
         <v>93.62</v>
       </c>
-      <c r="F112" s="2" t="n">
+      <c r="F116" s="2" t="n">
         <v>96.09</v>
       </c>
-      <c r="G112" s="2" t="n">
+      <c r="G116" s="2" t="n">
         <v>99.59999999999999</v>
       </c>
-      <c r="H112" s="2" t="n">
+      <c r="H116" s="2" t="n">
         <v>94.84</v>
       </c>
-      <c r="I112" s="2" t="n">
+      <c r="I116" s="2" t="n">
         <v>90.18000000000001</v>
       </c>
-      <c r="J112" s="2" t="n">
+      <c r="J116" s="2" t="n">
         <v>94.63</v>
       </c>
-      <c r="K112" s="2" t="n">
+      <c r="K116" s="2" t="n">
         <v>11.754</v>
       </c>
-      <c r="L112" s="2" t="n">
+      <c r="L116" s="2" t="n">
         <v>20.661</v>
       </c>
-      <c r="M112" s="2" t="n">
+      <c r="M116" s="2" t="n">
         <v>26.3246</v>
       </c>
-      <c r="N112" t="inlineStr">
+      <c r="N116" t="inlineStr">
         <is>
           <t>baseline</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:N112"/>
+  <autoFilter ref="A1:N116"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Record CASA Run3 SYSU hyperbolic results
</commit_message>
<xml_diff>
--- a/docs/experiment_metrics.xlsx
+++ b/docs/experiment_metrics.xlsx
@@ -10,7 +10,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="metrics" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'metrics'!$A$1:$N$116</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'metrics'!$A$1:$N$117</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -420,7 +420,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N116"/>
+  <dimension ref="A1:N117"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -5680,96 +5680,94 @@
       </c>
       <c r="C99" t="inlineStr">
         <is>
-          <t>M2_CA_QKV</t>
+          <t>M1_HYPER_QKV</t>
         </is>
       </c>
       <c r="D99" t="inlineStr">
         <is>
-          <t>LEVIR-CD-256</t>
+          <t>SYSU-CD-256</t>
         </is>
       </c>
       <c r="E99" s="2" t="n">
-        <v>90.58</v>
+        <v>77.55</v>
       </c>
       <c r="F99" s="2" t="n">
-        <v>91.77</v>
+        <v>85.81</v>
       </c>
       <c r="G99" s="2" t="n">
-        <v>99.11</v>
+        <v>91.68000000000001</v>
       </c>
       <c r="H99" s="2" t="n">
-        <v>91.17</v>
+        <v>81.47</v>
       </c>
       <c r="I99" s="2" t="n">
-        <v>83.77</v>
+        <v>68.73</v>
       </c>
       <c r="J99" s="2" t="n">
-        <v>90.7</v>
+        <v>76.12</v>
       </c>
       <c r="K99" s="2" t="n">
-        <v>3.059369</v>
+        <v>3.050665</v>
       </c>
       <c r="L99" s="2" t="n">
-        <v>3.143036</v>
+        <v>3.134332</v>
       </c>
       <c r="M99" s="2" t="n"/>
       <c r="N99" t="inlineStr">
         <is>
-          <t>casa_qkv</t>
+          <t>casa_hyperbolic</t>
         </is>
       </c>
     </row>
     <row r="100">
       <c r="A100" t="inlineStr">
         <is>
-          <t>STR-Fusion</t>
+          <t>CASA</t>
         </is>
       </c>
       <c r="B100" t="inlineStr">
         <is>
-          <t>Run2_TASS</t>
+          <t>Run3</t>
         </is>
       </c>
       <c r="C100" t="inlineStr">
         <is>
-          <t>C0_TOKEN</t>
+          <t>M2_CA_QKV</t>
         </is>
       </c>
       <c r="D100" t="inlineStr">
         <is>
-          <t>CDD-CD-256</t>
+          <t>LEVIR-CD-256</t>
         </is>
       </c>
       <c r="E100" s="2" t="n">
-        <v>93.13</v>
+        <v>90.58</v>
       </c>
       <c r="F100" s="2" t="n">
-        <v>95.16</v>
+        <v>91.77</v>
       </c>
       <c r="G100" s="2" t="n">
-        <v>98.56999999999999</v>
+        <v>99.11</v>
       </c>
       <c r="H100" s="2" t="n">
-        <v>94.13</v>
+        <v>91.17</v>
       </c>
       <c r="I100" s="2" t="n">
-        <v>88.91</v>
+        <v>83.77</v>
       </c>
       <c r="J100" s="2" t="n">
-        <v>93.31999999999999</v>
+        <v>90.7</v>
       </c>
       <c r="K100" s="2" t="n">
-        <v>2.596</v>
+        <v>3.059369</v>
       </c>
       <c r="L100" s="2" t="n">
-        <v>0.62</v>
-      </c>
-      <c r="M100" s="2" t="n">
-        <v>2.2136</v>
-      </c>
+        <v>3.143036</v>
+      </c>
+      <c r="M100" s="2" t="n"/>
       <c r="N100" t="inlineStr">
         <is>
-          <t>str_tass</t>
+          <t>casa_qkv</t>
         </is>
       </c>
     </row>
@@ -5791,26 +5789,26 @@
       </c>
       <c r="D101" t="inlineStr">
         <is>
-          <t>LEVIR-CD-256</t>
+          <t>CDD-CD-256</t>
         </is>
       </c>
       <c r="E101" s="2" t="n">
-        <v>86.37</v>
+        <v>93.13</v>
       </c>
       <c r="F101" s="2" t="n">
-        <v>89.25</v>
+        <v>95.16</v>
       </c>
       <c r="G101" s="2" t="n">
-        <v>98.78</v>
+        <v>98.56999999999999</v>
       </c>
       <c r="H101" s="2" t="n">
-        <v>87.79000000000001</v>
+        <v>94.13</v>
       </c>
       <c r="I101" s="2" t="n">
-        <v>78.23999999999999</v>
+        <v>88.91</v>
       </c>
       <c r="J101" s="2" t="n">
-        <v>87.14</v>
+        <v>93.31999999999999</v>
       </c>
       <c r="K101" s="2" t="n">
         <v>2.596</v>
@@ -5845,26 +5843,26 @@
       </c>
       <c r="D102" t="inlineStr">
         <is>
-          <t>SYSU-CD-256</t>
+          <t>LEVIR-CD-256</t>
         </is>
       </c>
       <c r="E102" s="2" t="n">
-        <v>79.93000000000001</v>
+        <v>86.37</v>
       </c>
       <c r="F102" s="2" t="n">
-        <v>84.5</v>
+        <v>89.25</v>
       </c>
       <c r="G102" s="2" t="n">
-        <v>91.81</v>
+        <v>98.78</v>
       </c>
       <c r="H102" s="2" t="n">
-        <v>82.15000000000001</v>
+        <v>87.79000000000001</v>
       </c>
       <c r="I102" s="2" t="n">
-        <v>69.70999999999999</v>
+        <v>78.23999999999999</v>
       </c>
       <c r="J102" s="2" t="n">
-        <v>76.84</v>
+        <v>87.14</v>
       </c>
       <c r="K102" s="2" t="n">
         <v>2.596</v>
@@ -5899,26 +5897,26 @@
       </c>
       <c r="D103" t="inlineStr">
         <is>
-          <t>WHU-CD-256</t>
+          <t>SYSU-CD-256</t>
         </is>
       </c>
       <c r="E103" s="2" t="n">
-        <v>90.16</v>
+        <v>79.93000000000001</v>
       </c>
       <c r="F103" s="2" t="n">
-        <v>93.97</v>
+        <v>84.5</v>
       </c>
       <c r="G103" s="2" t="n">
-        <v>99.38</v>
+        <v>91.81</v>
       </c>
       <c r="H103" s="2" t="n">
-        <v>92.02</v>
+        <v>82.15000000000001</v>
       </c>
       <c r="I103" s="2" t="n">
-        <v>85.23</v>
+        <v>69.70999999999999</v>
       </c>
       <c r="J103" s="2" t="n">
-        <v>91.7</v>
+        <v>76.84</v>
       </c>
       <c r="K103" s="2" t="n">
         <v>2.596</v>
@@ -5948,40 +5946,40 @@
       </c>
       <c r="C104" t="inlineStr">
         <is>
-          <t>M1_TASS</t>
+          <t>C0_TOKEN</t>
         </is>
       </c>
       <c r="D104" t="inlineStr">
         <is>
-          <t>CDD-CD-256</t>
+          <t>WHU-CD-256</t>
         </is>
       </c>
       <c r="E104" s="2" t="n">
-        <v>94.7</v>
+        <v>90.16</v>
       </c>
       <c r="F104" s="2" t="n">
-        <v>96.13</v>
+        <v>93.97</v>
       </c>
       <c r="G104" s="2" t="n">
-        <v>98.88</v>
+        <v>99.38</v>
       </c>
       <c r="H104" s="2" t="n">
-        <v>95.41</v>
+        <v>92.02</v>
       </c>
       <c r="I104" s="2" t="n">
-        <v>91.22</v>
+        <v>85.23</v>
       </c>
       <c r="J104" s="2" t="n">
-        <v>94.77</v>
+        <v>91.7</v>
       </c>
       <c r="K104" s="2" t="n">
-        <v>3.455</v>
+        <v>2.596</v>
       </c>
       <c r="L104" s="2" t="n">
-        <v>1.478</v>
+        <v>0.62</v>
       </c>
       <c r="M104" s="2" t="n">
-        <v>3.5459</v>
+        <v>2.2136</v>
       </c>
       <c r="N104" t="inlineStr">
         <is>
@@ -6007,26 +6005,26 @@
       </c>
       <c r="D105" t="inlineStr">
         <is>
-          <t>LEVIR-CD-256</t>
+          <t>CDD-CD-256</t>
         </is>
       </c>
       <c r="E105" s="2" t="n">
-        <v>88.42</v>
+        <v>94.7</v>
       </c>
       <c r="F105" s="2" t="n">
-        <v>91.97</v>
+        <v>96.13</v>
       </c>
       <c r="G105" s="2" t="n">
-        <v>99.02</v>
+        <v>98.88</v>
       </c>
       <c r="H105" s="2" t="n">
-        <v>90.16</v>
+        <v>95.41</v>
       </c>
       <c r="I105" s="2" t="n">
-        <v>82.08</v>
+        <v>91.22</v>
       </c>
       <c r="J105" s="2" t="n">
-        <v>89.64</v>
+        <v>94.77</v>
       </c>
       <c r="K105" s="2" t="n">
         <v>3.455</v>
@@ -6061,26 +6059,26 @@
       </c>
       <c r="D106" t="inlineStr">
         <is>
-          <t>SYSU-CD-256</t>
+          <t>LEVIR-CD-256</t>
         </is>
       </c>
       <c r="E106" s="2" t="n">
-        <v>78.73</v>
+        <v>88.42</v>
       </c>
       <c r="F106" s="2" t="n">
-        <v>84.98</v>
+        <v>91.97</v>
       </c>
       <c r="G106" s="2" t="n">
-        <v>91.7</v>
+        <v>99.02</v>
       </c>
       <c r="H106" s="2" t="n">
-        <v>81.73999999999999</v>
+        <v>90.16</v>
       </c>
       <c r="I106" s="2" t="n">
-        <v>69.11</v>
+        <v>82.08</v>
       </c>
       <c r="J106" s="2" t="n">
-        <v>76.38</v>
+        <v>89.64</v>
       </c>
       <c r="K106" s="2" t="n">
         <v>3.455</v>
@@ -6115,26 +6113,26 @@
       </c>
       <c r="D107" t="inlineStr">
         <is>
-          <t>WHU-CD-256</t>
+          <t>SYSU-CD-256</t>
         </is>
       </c>
       <c r="E107" s="2" t="n">
-        <v>91.64</v>
+        <v>78.73</v>
       </c>
       <c r="F107" s="2" t="n">
-        <v>94.81999999999999</v>
+        <v>84.98</v>
       </c>
       <c r="G107" s="2" t="n">
-        <v>99.47</v>
+        <v>91.7</v>
       </c>
       <c r="H107" s="2" t="n">
-        <v>93.2</v>
+        <v>81.73999999999999</v>
       </c>
       <c r="I107" s="2" t="n">
-        <v>87.27</v>
+        <v>69.11</v>
       </c>
       <c r="J107" s="2" t="n">
-        <v>92.93000000000001</v>
+        <v>76.38</v>
       </c>
       <c r="K107" s="2" t="n">
         <v>3.455</v>
@@ -6154,54 +6152,54 @@
     <row r="108">
       <c r="A108" t="inlineStr">
         <is>
-          <t>UltraLight</t>
+          <t>STR-Fusion</t>
         </is>
       </c>
       <c r="B108" t="inlineStr">
         <is>
-          <t>Run4</t>
+          <t>Run2_TASS</t>
         </is>
       </c>
       <c r="C108" t="inlineStr">
         <is>
-          <t>R4_0_A0_FULL12_FROZEN</t>
+          <t>M1_TASS</t>
         </is>
       </c>
       <c r="D108" t="inlineStr">
         <is>
-          <t>SYSU-CD-256</t>
+          <t>WHU-CD-256</t>
         </is>
       </c>
       <c r="E108" s="2" t="n">
-        <v>82.42</v>
+        <v>91.64</v>
       </c>
       <c r="F108" s="2" t="n">
-        <v>83.87</v>
+        <v>94.81999999999999</v>
       </c>
       <c r="G108" s="2" t="n">
-        <v>92.12</v>
+        <v>99.47</v>
       </c>
       <c r="H108" s="2" t="n">
-        <v>83.14</v>
+        <v>93.2</v>
       </c>
       <c r="I108" s="2" t="n">
-        <v>71.14</v>
+        <v>87.27</v>
       </c>
       <c r="J108" s="2" t="n">
-        <v>77.98999999999999</v>
+        <v>92.93000000000001</v>
       </c>
       <c r="K108" s="2" t="n">
-        <v>11.754</v>
+        <v>3.455</v>
       </c>
       <c r="L108" s="2" t="n">
-        <v>15.125</v>
+        <v>1.478</v>
       </c>
       <c r="M108" s="2" t="n">
-        <v>26.3246</v>
+        <v>3.5459</v>
       </c>
       <c r="N108" t="inlineStr">
         <is>
-          <t>baseline</t>
+          <t>str_tass</t>
         </is>
       </c>
     </row>
@@ -6218,7 +6216,7 @@
       </c>
       <c r="C109" t="inlineStr">
         <is>
-          <t>R4_1_VIT4_OLDHEAD</t>
+          <t>R4_0_A0_FULL12_FROZEN</t>
         </is>
       </c>
       <c r="D109" t="inlineStr">
@@ -6227,31 +6225,31 @@
         </is>
       </c>
       <c r="E109" s="2" t="n">
-        <v>82.15000000000001</v>
+        <v>82.42</v>
       </c>
       <c r="F109" s="2" t="n">
-        <v>83.40000000000001</v>
+        <v>83.87</v>
       </c>
       <c r="G109" s="2" t="n">
-        <v>91.94</v>
+        <v>92.12</v>
       </c>
       <c r="H109" s="2" t="n">
-        <v>82.77</v>
+        <v>83.14</v>
       </c>
       <c r="I109" s="2" t="n">
-        <v>70.61</v>
+        <v>71.14</v>
       </c>
       <c r="J109" s="2" t="n">
-        <v>77.51000000000001</v>
+        <v>77.98999999999999</v>
       </c>
       <c r="K109" s="2" t="n">
-        <v>8.195</v>
+        <v>11.754</v>
       </c>
       <c r="L109" s="2" t="n">
         <v>15.125</v>
       </c>
       <c r="M109" s="2" t="n">
-        <v>24.1021</v>
+        <v>26.3246</v>
       </c>
       <c r="N109" t="inlineStr">
         <is>
@@ -6272,7 +6270,7 @@
       </c>
       <c r="C110" t="inlineStr">
         <is>
-          <t>R4_2_VIT4_LIGHTDETAIL</t>
+          <t>R4_1_VIT4_OLDHEAD</t>
         </is>
       </c>
       <c r="D110" t="inlineStr">
@@ -6281,31 +6279,31 @@
         </is>
       </c>
       <c r="E110" s="2" t="n">
-        <v>79.94</v>
+        <v>82.15000000000001</v>
       </c>
       <c r="F110" s="2" t="n">
-        <v>84.79000000000001</v>
+        <v>83.40000000000001</v>
       </c>
       <c r="G110" s="2" t="n">
-        <v>91.89</v>
+        <v>91.94</v>
       </c>
       <c r="H110" s="2" t="n">
-        <v>82.3</v>
+        <v>82.77</v>
       </c>
       <c r="I110" s="2" t="n">
-        <v>69.92</v>
+        <v>70.61</v>
       </c>
       <c r="J110" s="2" t="n">
-        <v>77.04000000000001</v>
+        <v>77.51000000000001</v>
       </c>
       <c r="K110" s="2" t="n">
-        <v>5.492</v>
+        <v>8.195</v>
       </c>
       <c r="L110" s="2" t="n">
-        <v>3.515</v>
+        <v>15.125</v>
       </c>
       <c r="M110" s="2" t="n">
-        <v>10.7311</v>
+        <v>24.1021</v>
       </c>
       <c r="N110" t="inlineStr">
         <is>
@@ -6326,7 +6324,7 @@
       </c>
       <c r="C111" t="inlineStr">
         <is>
-          <t>R4_2b_VIT4_LIGHTDETAIL48</t>
+          <t>R4_2_VIT4_LIGHTDETAIL</t>
         </is>
       </c>
       <c r="D111" t="inlineStr">
@@ -6335,31 +6333,31 @@
         </is>
       </c>
       <c r="E111" s="2" t="n">
-        <v>80.87</v>
+        <v>79.94</v>
       </c>
       <c r="F111" s="2" t="n">
-        <v>83.81</v>
+        <v>84.79000000000001</v>
       </c>
       <c r="G111" s="2" t="n">
-        <v>91.81</v>
+        <v>91.89</v>
       </c>
       <c r="H111" s="2" t="n">
-        <v>82.31999999999999</v>
+        <v>82.3</v>
       </c>
       <c r="I111" s="2" t="n">
-        <v>69.95</v>
+        <v>69.92</v>
       </c>
       <c r="J111" s="2" t="n">
-        <v>76.98999999999999</v>
+        <v>77.04000000000001</v>
       </c>
       <c r="K111" s="2" t="n">
-        <v>5.533</v>
+        <v>5.492</v>
       </c>
       <c r="L111" s="2" t="n">
-        <v>3.556</v>
+        <v>3.515</v>
       </c>
       <c r="M111" s="2" t="n">
-        <v>10.9824</v>
+        <v>10.7311</v>
       </c>
       <c r="N111" t="inlineStr">
         <is>
@@ -6380,7 +6378,7 @@
       </c>
       <c r="C112" t="inlineStr">
         <is>
-          <t>R4_2d_PSD_DETAIL</t>
+          <t>R4_2b_VIT4_LIGHTDETAIL48</t>
         </is>
       </c>
       <c r="D112" t="inlineStr">
@@ -6389,31 +6387,31 @@
         </is>
       </c>
       <c r="E112" s="2" t="n">
-        <v>79.78</v>
+        <v>80.87</v>
       </c>
       <c r="F112" s="2" t="n">
-        <v>84.39</v>
+        <v>83.81</v>
       </c>
       <c r="G112" s="2" t="n">
-        <v>91.75</v>
+        <v>91.81</v>
       </c>
       <c r="H112" s="2" t="n">
-        <v>82.02</v>
+        <v>82.31999999999999</v>
       </c>
       <c r="I112" s="2" t="n">
-        <v>69.52</v>
+        <v>69.95</v>
       </c>
       <c r="J112" s="2" t="n">
-        <v>76.68000000000001</v>
+        <v>76.98999999999999</v>
       </c>
       <c r="K112" s="2" t="n">
-        <v>5.491</v>
+        <v>5.533</v>
       </c>
       <c r="L112" s="2" t="n">
-        <v>3.514</v>
+        <v>3.556</v>
       </c>
       <c r="M112" s="2" t="n">
-        <v>11.5239</v>
+        <v>10.9824</v>
       </c>
       <c r="N112" t="inlineStr">
         <is>
@@ -6424,46 +6422,50 @@
     <row r="113">
       <c r="A113" t="inlineStr">
         <is>
-          <t>baseline</t>
+          <t>UltraLight</t>
         </is>
       </c>
       <c r="B113" t="inlineStr">
         <is>
-          <t>Run1</t>
-        </is>
-      </c>
-      <c r="C113" t="inlineStr"/>
+          <t>Run4</t>
+        </is>
+      </c>
+      <c r="C113" t="inlineStr">
+        <is>
+          <t>R4_2d_PSD_DETAIL</t>
+        </is>
+      </c>
       <c r="D113" t="inlineStr">
         <is>
-          <t>CDD-CD-256</t>
+          <t>SYSU-CD-256</t>
         </is>
       </c>
       <c r="E113" s="2" t="n">
-        <v>97.72</v>
+        <v>79.78</v>
       </c>
       <c r="F113" s="2" t="n">
-        <v>97.78</v>
+        <v>84.39</v>
       </c>
       <c r="G113" s="2" t="n">
-        <v>99.44</v>
+        <v>91.75</v>
       </c>
       <c r="H113" s="2" t="n">
-        <v>97.75</v>
+        <v>82.02</v>
       </c>
       <c r="I113" s="2" t="n">
-        <v>95.59999999999999</v>
+        <v>69.52</v>
       </c>
       <c r="J113" s="2" t="n">
-        <v>97.43000000000001</v>
+        <v>76.68000000000001</v>
       </c>
       <c r="K113" s="2" t="n">
-        <v>11.754</v>
+        <v>5.491</v>
       </c>
       <c r="L113" s="2" t="n">
-        <v>20.661</v>
+        <v>3.514</v>
       </c>
       <c r="M113" s="2" t="n">
-        <v>26.3246</v>
+        <v>11.5239</v>
       </c>
       <c r="N113" t="inlineStr">
         <is>
@@ -6485,26 +6487,26 @@
       <c r="C114" t="inlineStr"/>
       <c r="D114" t="inlineStr">
         <is>
-          <t>LEVIR-CD-256</t>
+          <t>CDD-CD-256</t>
         </is>
       </c>
       <c r="E114" s="2" t="n">
-        <v>91.56999999999999</v>
+        <v>97.72</v>
       </c>
       <c r="F114" s="2" t="n">
-        <v>92.33</v>
+        <v>97.78</v>
       </c>
       <c r="G114" s="2" t="n">
-        <v>99.18000000000001</v>
+        <v>99.44</v>
       </c>
       <c r="H114" s="2" t="n">
-        <v>91.95</v>
+        <v>97.75</v>
       </c>
       <c r="I114" s="2" t="n">
-        <v>85.09999999999999</v>
+        <v>95.59999999999999</v>
       </c>
       <c r="J114" s="2" t="n">
-        <v>91.52</v>
+        <v>97.43000000000001</v>
       </c>
       <c r="K114" s="2" t="n">
         <v>11.754</v>
@@ -6535,26 +6537,26 @@
       <c r="C115" t="inlineStr"/>
       <c r="D115" t="inlineStr">
         <is>
-          <t>SYSU-CD-256</t>
+          <t>LEVIR-CD-256</t>
         </is>
       </c>
       <c r="E115" s="2" t="n">
-        <v>80.77</v>
+        <v>91.56999999999999</v>
       </c>
       <c r="F115" s="2" t="n">
-        <v>84.27</v>
+        <v>92.33</v>
       </c>
       <c r="G115" s="2" t="n">
-        <v>91.91</v>
+        <v>99.18000000000001</v>
       </c>
       <c r="H115" s="2" t="n">
-        <v>82.48</v>
+        <v>91.95</v>
       </c>
       <c r="I115" s="2" t="n">
-        <v>70.19</v>
+        <v>85.09999999999999</v>
       </c>
       <c r="J115" s="2" t="n">
-        <v>77.23</v>
+        <v>91.52</v>
       </c>
       <c r="K115" s="2" t="n">
         <v>11.754</v>
@@ -6585,26 +6587,26 @@
       <c r="C116" t="inlineStr"/>
       <c r="D116" t="inlineStr">
         <is>
-          <t>WHU-CD-256</t>
+          <t>SYSU-CD-256</t>
         </is>
       </c>
       <c r="E116" s="2" t="n">
-        <v>93.62</v>
+        <v>80.77</v>
       </c>
       <c r="F116" s="2" t="n">
-        <v>96.09</v>
+        <v>84.27</v>
       </c>
       <c r="G116" s="2" t="n">
-        <v>99.59999999999999</v>
+        <v>91.91</v>
       </c>
       <c r="H116" s="2" t="n">
-        <v>94.84</v>
+        <v>82.48</v>
       </c>
       <c r="I116" s="2" t="n">
-        <v>90.18000000000001</v>
+        <v>70.19</v>
       </c>
       <c r="J116" s="2" t="n">
-        <v>94.63</v>
+        <v>77.23</v>
       </c>
       <c r="K116" s="2" t="n">
         <v>11.754</v>
@@ -6621,8 +6623,58 @@
         </is>
       </c>
     </row>
+    <row r="117">
+      <c r="A117" t="inlineStr">
+        <is>
+          <t>baseline</t>
+        </is>
+      </c>
+      <c r="B117" t="inlineStr">
+        <is>
+          <t>Run1</t>
+        </is>
+      </c>
+      <c r="C117" t="inlineStr"/>
+      <c r="D117" t="inlineStr">
+        <is>
+          <t>WHU-CD-256</t>
+        </is>
+      </c>
+      <c r="E117" s="2" t="n">
+        <v>93.62</v>
+      </c>
+      <c r="F117" s="2" t="n">
+        <v>96.09</v>
+      </c>
+      <c r="G117" s="2" t="n">
+        <v>99.59999999999999</v>
+      </c>
+      <c r="H117" s="2" t="n">
+        <v>94.84</v>
+      </c>
+      <c r="I117" s="2" t="n">
+        <v>90.18000000000001</v>
+      </c>
+      <c r="J117" s="2" t="n">
+        <v>94.63</v>
+      </c>
+      <c r="K117" s="2" t="n">
+        <v>11.754</v>
+      </c>
+      <c r="L117" s="2" t="n">
+        <v>20.661</v>
+      </c>
+      <c r="M117" s="2" t="n">
+        <v>26.3246</v>
+      </c>
+      <c r="N117" t="inlineStr">
+        <is>
+          <t>baseline</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:N116"/>
+  <autoFilter ref="A1:N117"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Record complete CASA Run3 benchmark results
</commit_message>
<xml_diff>
--- a/docs/experiment_metrics.xlsx
+++ b/docs/experiment_metrics.xlsx
@@ -10,7 +10,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="metrics" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'metrics'!$A$1:$N$117</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'metrics'!$A$1:$N$124</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -420,7 +420,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N117"/>
+  <dimension ref="A1:N124"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -5529,26 +5529,26 @@
       </c>
       <c r="D96" t="inlineStr">
         <is>
-          <t>LEVIR-CD-256</t>
+          <t>CDD-CD-256</t>
         </is>
       </c>
       <c r="E96" s="2" t="n">
-        <v>90.41</v>
+        <v>97.43000000000001</v>
       </c>
       <c r="F96" s="2" t="n">
-        <v>91.83</v>
+        <v>97.47</v>
       </c>
       <c r="G96" s="2" t="n">
-        <v>99.09999999999999</v>
+        <v>99.37</v>
       </c>
       <c r="H96" s="2" t="n">
-        <v>91.11</v>
+        <v>97.45</v>
       </c>
       <c r="I96" s="2" t="n">
-        <v>83.67</v>
+        <v>95.02</v>
       </c>
       <c r="J96" s="2" t="n">
-        <v>90.64</v>
+        <v>97.09</v>
       </c>
       <c r="K96" s="2" t="n">
         <v>3.016737</v>
@@ -5581,26 +5581,26 @@
       </c>
       <c r="D97" t="inlineStr">
         <is>
-          <t>SYSU-CD-256</t>
+          <t>LEVIR-CD-256</t>
         </is>
       </c>
       <c r="E97" s="2" t="n">
-        <v>79.81</v>
+        <v>90.41</v>
       </c>
       <c r="F97" s="2" t="n">
-        <v>83.84999999999999</v>
+        <v>91.83</v>
       </c>
       <c r="G97" s="2" t="n">
-        <v>91.61</v>
+        <v>99.09999999999999</v>
       </c>
       <c r="H97" s="2" t="n">
-        <v>81.78</v>
+        <v>91.11</v>
       </c>
       <c r="I97" s="2" t="n">
-        <v>69.18000000000001</v>
+        <v>83.67</v>
       </c>
       <c r="J97" s="2" t="n">
-        <v>76.34</v>
+        <v>90.64</v>
       </c>
       <c r="K97" s="2" t="n">
         <v>3.016737</v>
@@ -5628,42 +5628,42 @@
       </c>
       <c r="C98" t="inlineStr">
         <is>
-          <t>M1_HYPER_QKV</t>
+          <t>M0_CTRL</t>
         </is>
       </c>
       <c r="D98" t="inlineStr">
         <is>
-          <t>LEVIR-CD-256</t>
+          <t>SYSU-CD-256</t>
         </is>
       </c>
       <c r="E98" s="2" t="n">
-        <v>90.61</v>
+        <v>79.81</v>
       </c>
       <c r="F98" s="2" t="n">
-        <v>92.37</v>
+        <v>83.84999999999999</v>
       </c>
       <c r="G98" s="2" t="n">
-        <v>99.14</v>
+        <v>91.61</v>
       </c>
       <c r="H98" s="2" t="n">
-        <v>91.48</v>
+        <v>81.78</v>
       </c>
       <c r="I98" s="2" t="n">
-        <v>84.3</v>
+        <v>69.18000000000001</v>
       </c>
       <c r="J98" s="2" t="n">
-        <v>91.03</v>
+        <v>76.34</v>
       </c>
       <c r="K98" s="2" t="n">
-        <v>3.050665</v>
+        <v>3.016737</v>
       </c>
       <c r="L98" s="2" t="n">
-        <v>3.134332</v>
+        <v>3.100404</v>
       </c>
       <c r="M98" s="2" t="n"/>
       <c r="N98" t="inlineStr">
         <is>
-          <t>casa_hyperbolic</t>
+          <t>casa_none</t>
         </is>
       </c>
     </row>
@@ -5680,42 +5680,42 @@
       </c>
       <c r="C99" t="inlineStr">
         <is>
-          <t>M1_HYPER_QKV</t>
+          <t>M0_CTRL</t>
         </is>
       </c>
       <c r="D99" t="inlineStr">
         <is>
-          <t>SYSU-CD-256</t>
+          <t>WHU-CD-256</t>
         </is>
       </c>
       <c r="E99" s="2" t="n">
-        <v>77.55</v>
+        <v>93.2</v>
       </c>
       <c r="F99" s="2" t="n">
-        <v>85.81</v>
+        <v>94.70999999999999</v>
       </c>
       <c r="G99" s="2" t="n">
-        <v>91.68000000000001</v>
+        <v>99.52</v>
       </c>
       <c r="H99" s="2" t="n">
-        <v>81.47</v>
+        <v>93.95</v>
       </c>
       <c r="I99" s="2" t="n">
-        <v>68.73</v>
+        <v>88.59</v>
       </c>
       <c r="J99" s="2" t="n">
-        <v>76.12</v>
+        <v>93.7</v>
       </c>
       <c r="K99" s="2" t="n">
-        <v>3.050665</v>
+        <v>3.016737</v>
       </c>
       <c r="L99" s="2" t="n">
-        <v>3.134332</v>
+        <v>3.100404</v>
       </c>
       <c r="M99" s="2" t="n"/>
       <c r="N99" t="inlineStr">
         <is>
-          <t>casa_hyperbolic</t>
+          <t>casa_none</t>
         </is>
       </c>
     </row>
@@ -5732,420 +5732,406 @@
       </c>
       <c r="C100" t="inlineStr">
         <is>
-          <t>M2_CA_QKV</t>
+          <t>M1_HYPER_QKV</t>
         </is>
       </c>
       <c r="D100" t="inlineStr">
         <is>
-          <t>LEVIR-CD-256</t>
+          <t>CDD-CD-256</t>
         </is>
       </c>
       <c r="E100" s="2" t="n">
-        <v>90.58</v>
+        <v>97.48</v>
       </c>
       <c r="F100" s="2" t="n">
-        <v>91.77</v>
+        <v>97.45</v>
       </c>
       <c r="G100" s="2" t="n">
-        <v>99.11</v>
+        <v>99.37</v>
       </c>
       <c r="H100" s="2" t="n">
-        <v>91.17</v>
+        <v>97.47</v>
       </c>
       <c r="I100" s="2" t="n">
-        <v>83.77</v>
+        <v>95.06</v>
       </c>
       <c r="J100" s="2" t="n">
-        <v>90.7</v>
+        <v>97.11</v>
       </c>
       <c r="K100" s="2" t="n">
-        <v>3.059369</v>
+        <v>3.050665</v>
       </c>
       <c r="L100" s="2" t="n">
-        <v>3.143036</v>
+        <v>3.134332</v>
       </c>
       <c r="M100" s="2" t="n"/>
       <c r="N100" t="inlineStr">
         <is>
-          <t>casa_qkv</t>
+          <t>casa_hyperbolic</t>
         </is>
       </c>
     </row>
     <row r="101">
       <c r="A101" t="inlineStr">
         <is>
-          <t>STR-Fusion</t>
+          <t>CASA</t>
         </is>
       </c>
       <c r="B101" t="inlineStr">
         <is>
-          <t>Run2_TASS</t>
+          <t>Run3</t>
         </is>
       </c>
       <c r="C101" t="inlineStr">
         <is>
-          <t>C0_TOKEN</t>
+          <t>M1_HYPER_QKV</t>
         </is>
       </c>
       <c r="D101" t="inlineStr">
         <is>
-          <t>CDD-CD-256</t>
+          <t>LEVIR-CD-256</t>
         </is>
       </c>
       <c r="E101" s="2" t="n">
-        <v>93.13</v>
+        <v>90.61</v>
       </c>
       <c r="F101" s="2" t="n">
-        <v>95.16</v>
+        <v>92.37</v>
       </c>
       <c r="G101" s="2" t="n">
-        <v>98.56999999999999</v>
+        <v>99.14</v>
       </c>
       <c r="H101" s="2" t="n">
-        <v>94.13</v>
+        <v>91.48</v>
       </c>
       <c r="I101" s="2" t="n">
-        <v>88.91</v>
+        <v>84.3</v>
       </c>
       <c r="J101" s="2" t="n">
-        <v>93.31999999999999</v>
+        <v>91.03</v>
       </c>
       <c r="K101" s="2" t="n">
-        <v>2.596</v>
+        <v>3.050665</v>
       </c>
       <c r="L101" s="2" t="n">
-        <v>0.62</v>
-      </c>
-      <c r="M101" s="2" t="n">
-        <v>2.2136</v>
-      </c>
+        <v>3.134332</v>
+      </c>
+      <c r="M101" s="2" t="n"/>
       <c r="N101" t="inlineStr">
         <is>
-          <t>str_tass</t>
+          <t>casa_hyperbolic</t>
         </is>
       </c>
     </row>
     <row r="102">
       <c r="A102" t="inlineStr">
         <is>
-          <t>STR-Fusion</t>
+          <t>CASA</t>
         </is>
       </c>
       <c r="B102" t="inlineStr">
         <is>
-          <t>Run2_TASS</t>
+          <t>Run3</t>
         </is>
       </c>
       <c r="C102" t="inlineStr">
         <is>
-          <t>C0_TOKEN</t>
+          <t>M1_HYPER_QKV</t>
         </is>
       </c>
       <c r="D102" t="inlineStr">
         <is>
-          <t>LEVIR-CD-256</t>
+          <t>SYSU-CD-256</t>
         </is>
       </c>
       <c r="E102" s="2" t="n">
-        <v>86.37</v>
+        <v>77.55</v>
       </c>
       <c r="F102" s="2" t="n">
-        <v>89.25</v>
+        <v>85.81</v>
       </c>
       <c r="G102" s="2" t="n">
-        <v>98.78</v>
+        <v>91.68000000000001</v>
       </c>
       <c r="H102" s="2" t="n">
-        <v>87.79000000000001</v>
+        <v>81.47</v>
       </c>
       <c r="I102" s="2" t="n">
-        <v>78.23999999999999</v>
+        <v>68.73</v>
       </c>
       <c r="J102" s="2" t="n">
-        <v>87.14</v>
+        <v>76.12</v>
       </c>
       <c r="K102" s="2" t="n">
-        <v>2.596</v>
+        <v>3.050665</v>
       </c>
       <c r="L102" s="2" t="n">
-        <v>0.62</v>
-      </c>
-      <c r="M102" s="2" t="n">
-        <v>2.2136</v>
-      </c>
+        <v>3.134332</v>
+      </c>
+      <c r="M102" s="2" t="n"/>
       <c r="N102" t="inlineStr">
         <is>
-          <t>str_tass</t>
+          <t>casa_hyperbolic</t>
         </is>
       </c>
     </row>
     <row r="103">
       <c r="A103" t="inlineStr">
         <is>
-          <t>STR-Fusion</t>
+          <t>CASA</t>
         </is>
       </c>
       <c r="B103" t="inlineStr">
         <is>
-          <t>Run2_TASS</t>
+          <t>Run3</t>
         </is>
       </c>
       <c r="C103" t="inlineStr">
         <is>
-          <t>C0_TOKEN</t>
+          <t>M1_HYPER_QKV</t>
         </is>
       </c>
       <c r="D103" t="inlineStr">
         <is>
-          <t>SYSU-CD-256</t>
+          <t>WHU-CD-256</t>
         </is>
       </c>
       <c r="E103" s="2" t="n">
-        <v>79.93000000000001</v>
+        <v>92.5</v>
       </c>
       <c r="F103" s="2" t="n">
-        <v>84.5</v>
+        <v>96.20999999999999</v>
       </c>
       <c r="G103" s="2" t="n">
-        <v>91.81</v>
+        <v>99.56</v>
       </c>
       <c r="H103" s="2" t="n">
-        <v>82.15000000000001</v>
+        <v>94.31999999999999</v>
       </c>
       <c r="I103" s="2" t="n">
-        <v>69.70999999999999</v>
+        <v>89.25</v>
       </c>
       <c r="J103" s="2" t="n">
-        <v>76.84</v>
+        <v>94.09</v>
       </c>
       <c r="K103" s="2" t="n">
-        <v>2.596</v>
+        <v>3.050665</v>
       </c>
       <c r="L103" s="2" t="n">
-        <v>0.62</v>
-      </c>
-      <c r="M103" s="2" t="n">
-        <v>2.2136</v>
-      </c>
+        <v>3.134332</v>
+      </c>
+      <c r="M103" s="2" t="n"/>
       <c r="N103" t="inlineStr">
         <is>
-          <t>str_tass</t>
+          <t>casa_hyperbolic</t>
         </is>
       </c>
     </row>
     <row r="104">
       <c r="A104" t="inlineStr">
         <is>
-          <t>STR-Fusion</t>
+          <t>CASA</t>
         </is>
       </c>
       <c r="B104" t="inlineStr">
         <is>
-          <t>Run2_TASS</t>
+          <t>Run3</t>
         </is>
       </c>
       <c r="C104" t="inlineStr">
         <is>
-          <t>C0_TOKEN</t>
+          <t>M2_CA_QKV</t>
         </is>
       </c>
       <c r="D104" t="inlineStr">
         <is>
-          <t>WHU-CD-256</t>
+          <t>CDD-CD-256</t>
         </is>
       </c>
       <c r="E104" s="2" t="n">
-        <v>90.16</v>
+        <v>97.51000000000001</v>
       </c>
       <c r="F104" s="2" t="n">
-        <v>93.97</v>
+        <v>97.45</v>
       </c>
       <c r="G104" s="2" t="n">
         <v>99.38</v>
       </c>
       <c r="H104" s="2" t="n">
-        <v>92.02</v>
+        <v>97.48</v>
       </c>
       <c r="I104" s="2" t="n">
-        <v>85.23</v>
+        <v>95.09</v>
       </c>
       <c r="J104" s="2" t="n">
-        <v>91.7</v>
+        <v>97.13</v>
       </c>
       <c r="K104" s="2" t="n">
-        <v>2.596</v>
+        <v>3.059369</v>
       </c>
       <c r="L104" s="2" t="n">
-        <v>0.62</v>
-      </c>
-      <c r="M104" s="2" t="n">
-        <v>2.2136</v>
-      </c>
+        <v>3.143036</v>
+      </c>
+      <c r="M104" s="2" t="n"/>
       <c r="N104" t="inlineStr">
         <is>
-          <t>str_tass</t>
+          <t>casa_qkv</t>
         </is>
       </c>
     </row>
     <row r="105">
       <c r="A105" t="inlineStr">
         <is>
-          <t>STR-Fusion</t>
+          <t>CASA</t>
         </is>
       </c>
       <c r="B105" t="inlineStr">
         <is>
-          <t>Run2_TASS</t>
+          <t>Run3</t>
         </is>
       </c>
       <c r="C105" t="inlineStr">
         <is>
-          <t>M1_TASS</t>
+          <t>M2_CA_QKV</t>
         </is>
       </c>
       <c r="D105" t="inlineStr">
         <is>
-          <t>CDD-CD-256</t>
+          <t>LEVIR-CD-256</t>
         </is>
       </c>
       <c r="E105" s="2" t="n">
-        <v>94.7</v>
+        <v>90.58</v>
       </c>
       <c r="F105" s="2" t="n">
-        <v>96.13</v>
+        <v>91.77</v>
       </c>
       <c r="G105" s="2" t="n">
-        <v>98.88</v>
+        <v>99.11</v>
       </c>
       <c r="H105" s="2" t="n">
-        <v>95.41</v>
+        <v>91.17</v>
       </c>
       <c r="I105" s="2" t="n">
-        <v>91.22</v>
+        <v>83.77</v>
       </c>
       <c r="J105" s="2" t="n">
-        <v>94.77</v>
+        <v>90.7</v>
       </c>
       <c r="K105" s="2" t="n">
-        <v>3.455</v>
+        <v>3.059369</v>
       </c>
       <c r="L105" s="2" t="n">
-        <v>1.478</v>
-      </c>
-      <c r="M105" s="2" t="n">
-        <v>3.5459</v>
-      </c>
+        <v>3.143036</v>
+      </c>
+      <c r="M105" s="2" t="n"/>
       <c r="N105" t="inlineStr">
         <is>
-          <t>str_tass</t>
+          <t>casa_qkv</t>
         </is>
       </c>
     </row>
     <row r="106">
       <c r="A106" t="inlineStr">
         <is>
-          <t>STR-Fusion</t>
+          <t>CASA</t>
         </is>
       </c>
       <c r="B106" t="inlineStr">
         <is>
-          <t>Run2_TASS</t>
+          <t>Run3</t>
         </is>
       </c>
       <c r="C106" t="inlineStr">
         <is>
-          <t>M1_TASS</t>
+          <t>M2_CA_QKV</t>
         </is>
       </c>
       <c r="D106" t="inlineStr">
         <is>
-          <t>LEVIR-CD-256</t>
+          <t>SYSU-CD-256</t>
         </is>
       </c>
       <c r="E106" s="2" t="n">
-        <v>88.42</v>
+        <v>76.7</v>
       </c>
       <c r="F106" s="2" t="n">
-        <v>91.97</v>
+        <v>85.81999999999999</v>
       </c>
       <c r="G106" s="2" t="n">
-        <v>99.02</v>
+        <v>91.52</v>
       </c>
       <c r="H106" s="2" t="n">
-        <v>90.16</v>
+        <v>81.01000000000001</v>
       </c>
       <c r="I106" s="2" t="n">
-        <v>82.08</v>
+        <v>68.06999999999999</v>
       </c>
       <c r="J106" s="2" t="n">
-        <v>89.64</v>
+        <v>75.56999999999999</v>
       </c>
       <c r="K106" s="2" t="n">
-        <v>3.455</v>
+        <v>3.059369</v>
       </c>
       <c r="L106" s="2" t="n">
-        <v>1.478</v>
-      </c>
-      <c r="M106" s="2" t="n">
-        <v>3.5459</v>
-      </c>
+        <v>3.143036</v>
+      </c>
+      <c r="M106" s="2" t="n"/>
       <c r="N106" t="inlineStr">
         <is>
-          <t>str_tass</t>
+          <t>casa_qkv</t>
         </is>
       </c>
     </row>
     <row r="107">
       <c r="A107" t="inlineStr">
         <is>
-          <t>STR-Fusion</t>
+          <t>CASA</t>
         </is>
       </c>
       <c r="B107" t="inlineStr">
         <is>
-          <t>Run2_TASS</t>
+          <t>Run3</t>
         </is>
       </c>
       <c r="C107" t="inlineStr">
         <is>
-          <t>M1_TASS</t>
+          <t>M2_CA_QKV</t>
         </is>
       </c>
       <c r="D107" t="inlineStr">
         <is>
-          <t>SYSU-CD-256</t>
+          <t>WHU-CD-256</t>
         </is>
       </c>
       <c r="E107" s="2" t="n">
-        <v>78.73</v>
+        <v>92.61</v>
       </c>
       <c r="F107" s="2" t="n">
-        <v>84.98</v>
+        <v>95.31</v>
       </c>
       <c r="G107" s="2" t="n">
-        <v>91.7</v>
+        <v>99.53</v>
       </c>
       <c r="H107" s="2" t="n">
-        <v>81.73999999999999</v>
+        <v>93.94</v>
       </c>
       <c r="I107" s="2" t="n">
-        <v>69.11</v>
+        <v>88.58</v>
       </c>
       <c r="J107" s="2" t="n">
-        <v>76.38</v>
+        <v>93.69</v>
       </c>
       <c r="K107" s="2" t="n">
-        <v>3.455</v>
+        <v>3.059369</v>
       </c>
       <c r="L107" s="2" t="n">
-        <v>1.478</v>
-      </c>
-      <c r="M107" s="2" t="n">
-        <v>3.5459</v>
-      </c>
+        <v>3.143036</v>
+      </c>
+      <c r="M107" s="2" t="n"/>
       <c r="N107" t="inlineStr">
         <is>
-          <t>str_tass</t>
+          <t>casa_qkv</t>
         </is>
       </c>
     </row>
@@ -6162,40 +6148,40 @@
       </c>
       <c r="C108" t="inlineStr">
         <is>
-          <t>M1_TASS</t>
+          <t>C0_TOKEN</t>
         </is>
       </c>
       <c r="D108" t="inlineStr">
         <is>
-          <t>WHU-CD-256</t>
+          <t>CDD-CD-256</t>
         </is>
       </c>
       <c r="E108" s="2" t="n">
-        <v>91.64</v>
+        <v>93.13</v>
       </c>
       <c r="F108" s="2" t="n">
-        <v>94.81999999999999</v>
+        <v>95.16</v>
       </c>
       <c r="G108" s="2" t="n">
-        <v>99.47</v>
+        <v>98.56999999999999</v>
       </c>
       <c r="H108" s="2" t="n">
-        <v>93.2</v>
+        <v>94.13</v>
       </c>
       <c r="I108" s="2" t="n">
-        <v>87.27</v>
+        <v>88.91</v>
       </c>
       <c r="J108" s="2" t="n">
-        <v>92.93000000000001</v>
+        <v>93.31999999999999</v>
       </c>
       <c r="K108" s="2" t="n">
-        <v>3.455</v>
+        <v>2.596</v>
       </c>
       <c r="L108" s="2" t="n">
-        <v>1.478</v>
+        <v>0.62</v>
       </c>
       <c r="M108" s="2" t="n">
-        <v>3.5459</v>
+        <v>2.2136</v>
       </c>
       <c r="N108" t="inlineStr">
         <is>
@@ -6206,71 +6192,71 @@
     <row r="109">
       <c r="A109" t="inlineStr">
         <is>
-          <t>UltraLight</t>
+          <t>STR-Fusion</t>
         </is>
       </c>
       <c r="B109" t="inlineStr">
         <is>
-          <t>Run4</t>
+          <t>Run2_TASS</t>
         </is>
       </c>
       <c r="C109" t="inlineStr">
         <is>
-          <t>R4_0_A0_FULL12_FROZEN</t>
+          <t>C0_TOKEN</t>
         </is>
       </c>
       <c r="D109" t="inlineStr">
         <is>
-          <t>SYSU-CD-256</t>
+          <t>LEVIR-CD-256</t>
         </is>
       </c>
       <c r="E109" s="2" t="n">
-        <v>82.42</v>
+        <v>86.37</v>
       </c>
       <c r="F109" s="2" t="n">
-        <v>83.87</v>
+        <v>89.25</v>
       </c>
       <c r="G109" s="2" t="n">
-        <v>92.12</v>
+        <v>98.78</v>
       </c>
       <c r="H109" s="2" t="n">
-        <v>83.14</v>
+        <v>87.79000000000001</v>
       </c>
       <c r="I109" s="2" t="n">
-        <v>71.14</v>
+        <v>78.23999999999999</v>
       </c>
       <c r="J109" s="2" t="n">
-        <v>77.98999999999999</v>
+        <v>87.14</v>
       </c>
       <c r="K109" s="2" t="n">
-        <v>11.754</v>
+        <v>2.596</v>
       </c>
       <c r="L109" s="2" t="n">
-        <v>15.125</v>
+        <v>0.62</v>
       </c>
       <c r="M109" s="2" t="n">
-        <v>26.3246</v>
+        <v>2.2136</v>
       </c>
       <c r="N109" t="inlineStr">
         <is>
-          <t>baseline</t>
+          <t>str_tass</t>
         </is>
       </c>
     </row>
     <row r="110">
       <c r="A110" t="inlineStr">
         <is>
-          <t>UltraLight</t>
+          <t>STR-Fusion</t>
         </is>
       </c>
       <c r="B110" t="inlineStr">
         <is>
-          <t>Run4</t>
+          <t>Run2_TASS</t>
         </is>
       </c>
       <c r="C110" t="inlineStr">
         <is>
-          <t>R4_1_VIT4_OLDHEAD</t>
+          <t>C0_TOKEN</t>
         </is>
       </c>
       <c r="D110" t="inlineStr">
@@ -6279,340 +6265,352 @@
         </is>
       </c>
       <c r="E110" s="2" t="n">
+        <v>79.93000000000001</v>
+      </c>
+      <c r="F110" s="2" t="n">
+        <v>84.5</v>
+      </c>
+      <c r="G110" s="2" t="n">
+        <v>91.81</v>
+      </c>
+      <c r="H110" s="2" t="n">
         <v>82.15000000000001</v>
       </c>
-      <c r="F110" s="2" t="n">
-        <v>83.40000000000001</v>
-      </c>
-      <c r="G110" s="2" t="n">
-        <v>91.94</v>
-      </c>
-      <c r="H110" s="2" t="n">
-        <v>82.77</v>
-      </c>
       <c r="I110" s="2" t="n">
-        <v>70.61</v>
+        <v>69.70999999999999</v>
       </c>
       <c r="J110" s="2" t="n">
-        <v>77.51000000000001</v>
+        <v>76.84</v>
       </c>
       <c r="K110" s="2" t="n">
-        <v>8.195</v>
+        <v>2.596</v>
       </c>
       <c r="L110" s="2" t="n">
-        <v>15.125</v>
+        <v>0.62</v>
       </c>
       <c r="M110" s="2" t="n">
-        <v>24.1021</v>
+        <v>2.2136</v>
       </c>
       <c r="N110" t="inlineStr">
         <is>
-          <t>baseline</t>
+          <t>str_tass</t>
         </is>
       </c>
     </row>
     <row r="111">
       <c r="A111" t="inlineStr">
         <is>
-          <t>UltraLight</t>
+          <t>STR-Fusion</t>
         </is>
       </c>
       <c r="B111" t="inlineStr">
         <is>
-          <t>Run4</t>
+          <t>Run2_TASS</t>
         </is>
       </c>
       <c r="C111" t="inlineStr">
         <is>
-          <t>R4_2_VIT4_LIGHTDETAIL</t>
+          <t>C0_TOKEN</t>
         </is>
       </c>
       <c r="D111" t="inlineStr">
         <is>
-          <t>SYSU-CD-256</t>
+          <t>WHU-CD-256</t>
         </is>
       </c>
       <c r="E111" s="2" t="n">
-        <v>79.94</v>
+        <v>90.16</v>
       </c>
       <c r="F111" s="2" t="n">
-        <v>84.79000000000001</v>
+        <v>93.97</v>
       </c>
       <c r="G111" s="2" t="n">
-        <v>91.89</v>
+        <v>99.38</v>
       </c>
       <c r="H111" s="2" t="n">
-        <v>82.3</v>
+        <v>92.02</v>
       </c>
       <c r="I111" s="2" t="n">
-        <v>69.92</v>
+        <v>85.23</v>
       </c>
       <c r="J111" s="2" t="n">
-        <v>77.04000000000001</v>
+        <v>91.7</v>
       </c>
       <c r="K111" s="2" t="n">
-        <v>5.492</v>
+        <v>2.596</v>
       </c>
       <c r="L111" s="2" t="n">
-        <v>3.515</v>
+        <v>0.62</v>
       </c>
       <c r="M111" s="2" t="n">
-        <v>10.7311</v>
+        <v>2.2136</v>
       </c>
       <c r="N111" t="inlineStr">
         <is>
-          <t>baseline</t>
+          <t>str_tass</t>
         </is>
       </c>
     </row>
     <row r="112">
       <c r="A112" t="inlineStr">
         <is>
-          <t>UltraLight</t>
+          <t>STR-Fusion</t>
         </is>
       </c>
       <c r="B112" t="inlineStr">
         <is>
-          <t>Run4</t>
+          <t>Run2_TASS</t>
         </is>
       </c>
       <c r="C112" t="inlineStr">
         <is>
-          <t>R4_2b_VIT4_LIGHTDETAIL48</t>
+          <t>M1_TASS</t>
         </is>
       </c>
       <c r="D112" t="inlineStr">
         <is>
-          <t>SYSU-CD-256</t>
+          <t>CDD-CD-256</t>
         </is>
       </c>
       <c r="E112" s="2" t="n">
-        <v>80.87</v>
+        <v>94.7</v>
       </c>
       <c r="F112" s="2" t="n">
-        <v>83.81</v>
+        <v>96.13</v>
       </c>
       <c r="G112" s="2" t="n">
-        <v>91.81</v>
+        <v>98.88</v>
       </c>
       <c r="H112" s="2" t="n">
-        <v>82.31999999999999</v>
+        <v>95.41</v>
       </c>
       <c r="I112" s="2" t="n">
-        <v>69.95</v>
+        <v>91.22</v>
       </c>
       <c r="J112" s="2" t="n">
-        <v>76.98999999999999</v>
+        <v>94.77</v>
       </c>
       <c r="K112" s="2" t="n">
-        <v>5.533</v>
+        <v>3.455</v>
       </c>
       <c r="L112" s="2" t="n">
-        <v>3.556</v>
+        <v>1.478</v>
       </c>
       <c r="M112" s="2" t="n">
-        <v>10.9824</v>
+        <v>3.5459</v>
       </c>
       <c r="N112" t="inlineStr">
         <is>
-          <t>baseline</t>
+          <t>str_tass</t>
         </is>
       </c>
     </row>
     <row r="113">
       <c r="A113" t="inlineStr">
         <is>
-          <t>UltraLight</t>
+          <t>STR-Fusion</t>
         </is>
       </c>
       <c r="B113" t="inlineStr">
         <is>
-          <t>Run4</t>
+          <t>Run2_TASS</t>
         </is>
       </c>
       <c r="C113" t="inlineStr">
         <is>
-          <t>R4_2d_PSD_DETAIL</t>
+          <t>M1_TASS</t>
         </is>
       </c>
       <c r="D113" t="inlineStr">
         <is>
-          <t>SYSU-CD-256</t>
+          <t>LEVIR-CD-256</t>
         </is>
       </c>
       <c r="E113" s="2" t="n">
-        <v>79.78</v>
+        <v>88.42</v>
       </c>
       <c r="F113" s="2" t="n">
-        <v>84.39</v>
+        <v>91.97</v>
       </c>
       <c r="G113" s="2" t="n">
-        <v>91.75</v>
+        <v>99.02</v>
       </c>
       <c r="H113" s="2" t="n">
-        <v>82.02</v>
+        <v>90.16</v>
       </c>
       <c r="I113" s="2" t="n">
-        <v>69.52</v>
+        <v>82.08</v>
       </c>
       <c r="J113" s="2" t="n">
-        <v>76.68000000000001</v>
+        <v>89.64</v>
       </c>
       <c r="K113" s="2" t="n">
-        <v>5.491</v>
+        <v>3.455</v>
       </c>
       <c r="L113" s="2" t="n">
-        <v>3.514</v>
+        <v>1.478</v>
       </c>
       <c r="M113" s="2" t="n">
-        <v>11.5239</v>
+        <v>3.5459</v>
       </c>
       <c r="N113" t="inlineStr">
         <is>
-          <t>baseline</t>
+          <t>str_tass</t>
         </is>
       </c>
     </row>
     <row r="114">
       <c r="A114" t="inlineStr">
         <is>
-          <t>baseline</t>
+          <t>STR-Fusion</t>
         </is>
       </c>
       <c r="B114" t="inlineStr">
         <is>
-          <t>Run1</t>
-        </is>
-      </c>
-      <c r="C114" t="inlineStr"/>
+          <t>Run2_TASS</t>
+        </is>
+      </c>
+      <c r="C114" t="inlineStr">
+        <is>
+          <t>M1_TASS</t>
+        </is>
+      </c>
       <c r="D114" t="inlineStr">
         <is>
-          <t>CDD-CD-256</t>
+          <t>SYSU-CD-256</t>
         </is>
       </c>
       <c r="E114" s="2" t="n">
-        <v>97.72</v>
+        <v>78.73</v>
       </c>
       <c r="F114" s="2" t="n">
-        <v>97.78</v>
+        <v>84.98</v>
       </c>
       <c r="G114" s="2" t="n">
-        <v>99.44</v>
+        <v>91.7</v>
       </c>
       <c r="H114" s="2" t="n">
-        <v>97.75</v>
+        <v>81.73999999999999</v>
       </c>
       <c r="I114" s="2" t="n">
-        <v>95.59999999999999</v>
+        <v>69.11</v>
       </c>
       <c r="J114" s="2" t="n">
-        <v>97.43000000000001</v>
+        <v>76.38</v>
       </c>
       <c r="K114" s="2" t="n">
-        <v>11.754</v>
+        <v>3.455</v>
       </c>
       <c r="L114" s="2" t="n">
-        <v>20.661</v>
+        <v>1.478</v>
       </c>
       <c r="M114" s="2" t="n">
-        <v>26.3246</v>
+        <v>3.5459</v>
       </c>
       <c r="N114" t="inlineStr">
         <is>
-          <t>baseline</t>
+          <t>str_tass</t>
         </is>
       </c>
     </row>
     <row r="115">
       <c r="A115" t="inlineStr">
         <is>
-          <t>baseline</t>
+          <t>STR-Fusion</t>
         </is>
       </c>
       <c r="B115" t="inlineStr">
         <is>
-          <t>Run1</t>
-        </is>
-      </c>
-      <c r="C115" t="inlineStr"/>
+          <t>Run2_TASS</t>
+        </is>
+      </c>
+      <c r="C115" t="inlineStr">
+        <is>
+          <t>M1_TASS</t>
+        </is>
+      </c>
       <c r="D115" t="inlineStr">
         <is>
-          <t>LEVIR-CD-256</t>
+          <t>WHU-CD-256</t>
         </is>
       </c>
       <c r="E115" s="2" t="n">
-        <v>91.56999999999999</v>
+        <v>91.64</v>
       </c>
       <c r="F115" s="2" t="n">
-        <v>92.33</v>
+        <v>94.81999999999999</v>
       </c>
       <c r="G115" s="2" t="n">
-        <v>99.18000000000001</v>
+        <v>99.47</v>
       </c>
       <c r="H115" s="2" t="n">
-        <v>91.95</v>
+        <v>93.2</v>
       </c>
       <c r="I115" s="2" t="n">
-        <v>85.09999999999999</v>
+        <v>87.27</v>
       </c>
       <c r="J115" s="2" t="n">
-        <v>91.52</v>
+        <v>92.93000000000001</v>
       </c>
       <c r="K115" s="2" t="n">
-        <v>11.754</v>
+        <v>3.455</v>
       </c>
       <c r="L115" s="2" t="n">
-        <v>20.661</v>
+        <v>1.478</v>
       </c>
       <c r="M115" s="2" t="n">
-        <v>26.3246</v>
+        <v>3.5459</v>
       </c>
       <c r="N115" t="inlineStr">
         <is>
-          <t>baseline</t>
+          <t>str_tass</t>
         </is>
       </c>
     </row>
     <row r="116">
       <c r="A116" t="inlineStr">
         <is>
-          <t>baseline</t>
+          <t>UltraLight</t>
         </is>
       </c>
       <c r="B116" t="inlineStr">
         <is>
-          <t>Run1</t>
-        </is>
-      </c>
-      <c r="C116" t="inlineStr"/>
+          <t>Run4</t>
+        </is>
+      </c>
+      <c r="C116" t="inlineStr">
+        <is>
+          <t>R4_0_A0_FULL12_FROZEN</t>
+        </is>
+      </c>
       <c r="D116" t="inlineStr">
         <is>
           <t>SYSU-CD-256</t>
         </is>
       </c>
       <c r="E116" s="2" t="n">
-        <v>80.77</v>
+        <v>82.42</v>
       </c>
       <c r="F116" s="2" t="n">
-        <v>84.27</v>
+        <v>83.87</v>
       </c>
       <c r="G116" s="2" t="n">
-        <v>91.91</v>
+        <v>92.12</v>
       </c>
       <c r="H116" s="2" t="n">
-        <v>82.48</v>
+        <v>83.14</v>
       </c>
       <c r="I116" s="2" t="n">
-        <v>70.19</v>
+        <v>71.14</v>
       </c>
       <c r="J116" s="2" t="n">
-        <v>77.23</v>
+        <v>77.98999999999999</v>
       </c>
       <c r="K116" s="2" t="n">
         <v>11.754</v>
       </c>
       <c r="L116" s="2" t="n">
-        <v>20.661</v>
+        <v>15.125</v>
       </c>
       <c r="M116" s="2" t="n">
         <v>26.3246</v>
@@ -6626,55 +6624,421 @@
     <row r="117">
       <c r="A117" t="inlineStr">
         <is>
+          <t>UltraLight</t>
+        </is>
+      </c>
+      <c r="B117" t="inlineStr">
+        <is>
+          <t>Run4</t>
+        </is>
+      </c>
+      <c r="C117" t="inlineStr">
+        <is>
+          <t>R4_1_VIT4_OLDHEAD</t>
+        </is>
+      </c>
+      <c r="D117" t="inlineStr">
+        <is>
+          <t>SYSU-CD-256</t>
+        </is>
+      </c>
+      <c r="E117" s="2" t="n">
+        <v>82.15000000000001</v>
+      </c>
+      <c r="F117" s="2" t="n">
+        <v>83.40000000000001</v>
+      </c>
+      <c r="G117" s="2" t="n">
+        <v>91.94</v>
+      </c>
+      <c r="H117" s="2" t="n">
+        <v>82.77</v>
+      </c>
+      <c r="I117" s="2" t="n">
+        <v>70.61</v>
+      </c>
+      <c r="J117" s="2" t="n">
+        <v>77.51000000000001</v>
+      </c>
+      <c r="K117" s="2" t="n">
+        <v>8.195</v>
+      </c>
+      <c r="L117" s="2" t="n">
+        <v>15.125</v>
+      </c>
+      <c r="M117" s="2" t="n">
+        <v>24.1021</v>
+      </c>
+      <c r="N117" t="inlineStr">
+        <is>
           <t>baseline</t>
         </is>
       </c>
-      <c r="B117" t="inlineStr">
+    </row>
+    <row r="118">
+      <c r="A118" t="inlineStr">
+        <is>
+          <t>UltraLight</t>
+        </is>
+      </c>
+      <c r="B118" t="inlineStr">
+        <is>
+          <t>Run4</t>
+        </is>
+      </c>
+      <c r="C118" t="inlineStr">
+        <is>
+          <t>R4_2_VIT4_LIGHTDETAIL</t>
+        </is>
+      </c>
+      <c r="D118" t="inlineStr">
+        <is>
+          <t>SYSU-CD-256</t>
+        </is>
+      </c>
+      <c r="E118" s="2" t="n">
+        <v>79.94</v>
+      </c>
+      <c r="F118" s="2" t="n">
+        <v>84.79000000000001</v>
+      </c>
+      <c r="G118" s="2" t="n">
+        <v>91.89</v>
+      </c>
+      <c r="H118" s="2" t="n">
+        <v>82.3</v>
+      </c>
+      <c r="I118" s="2" t="n">
+        <v>69.92</v>
+      </c>
+      <c r="J118" s="2" t="n">
+        <v>77.04000000000001</v>
+      </c>
+      <c r="K118" s="2" t="n">
+        <v>5.492</v>
+      </c>
+      <c r="L118" s="2" t="n">
+        <v>3.515</v>
+      </c>
+      <c r="M118" s="2" t="n">
+        <v>10.7311</v>
+      </c>
+      <c r="N118" t="inlineStr">
+        <is>
+          <t>baseline</t>
+        </is>
+      </c>
+    </row>
+    <row r="119">
+      <c r="A119" t="inlineStr">
+        <is>
+          <t>UltraLight</t>
+        </is>
+      </c>
+      <c r="B119" t="inlineStr">
+        <is>
+          <t>Run4</t>
+        </is>
+      </c>
+      <c r="C119" t="inlineStr">
+        <is>
+          <t>R4_2b_VIT4_LIGHTDETAIL48</t>
+        </is>
+      </c>
+      <c r="D119" t="inlineStr">
+        <is>
+          <t>SYSU-CD-256</t>
+        </is>
+      </c>
+      <c r="E119" s="2" t="n">
+        <v>80.87</v>
+      </c>
+      <c r="F119" s="2" t="n">
+        <v>83.81</v>
+      </c>
+      <c r="G119" s="2" t="n">
+        <v>91.81</v>
+      </c>
+      <c r="H119" s="2" t="n">
+        <v>82.31999999999999</v>
+      </c>
+      <c r="I119" s="2" t="n">
+        <v>69.95</v>
+      </c>
+      <c r="J119" s="2" t="n">
+        <v>76.98999999999999</v>
+      </c>
+      <c r="K119" s="2" t="n">
+        <v>5.533</v>
+      </c>
+      <c r="L119" s="2" t="n">
+        <v>3.556</v>
+      </c>
+      <c r="M119" s="2" t="n">
+        <v>10.9824</v>
+      </c>
+      <c r="N119" t="inlineStr">
+        <is>
+          <t>baseline</t>
+        </is>
+      </c>
+    </row>
+    <row r="120">
+      <c r="A120" t="inlineStr">
+        <is>
+          <t>UltraLight</t>
+        </is>
+      </c>
+      <c r="B120" t="inlineStr">
+        <is>
+          <t>Run4</t>
+        </is>
+      </c>
+      <c r="C120" t="inlineStr">
+        <is>
+          <t>R4_2d_PSD_DETAIL</t>
+        </is>
+      </c>
+      <c r="D120" t="inlineStr">
+        <is>
+          <t>SYSU-CD-256</t>
+        </is>
+      </c>
+      <c r="E120" s="2" t="n">
+        <v>79.78</v>
+      </c>
+      <c r="F120" s="2" t="n">
+        <v>84.39</v>
+      </c>
+      <c r="G120" s="2" t="n">
+        <v>91.75</v>
+      </c>
+      <c r="H120" s="2" t="n">
+        <v>82.02</v>
+      </c>
+      <c r="I120" s="2" t="n">
+        <v>69.52</v>
+      </c>
+      <c r="J120" s="2" t="n">
+        <v>76.68000000000001</v>
+      </c>
+      <c r="K120" s="2" t="n">
+        <v>5.491</v>
+      </c>
+      <c r="L120" s="2" t="n">
+        <v>3.514</v>
+      </c>
+      <c r="M120" s="2" t="n">
+        <v>11.5239</v>
+      </c>
+      <c r="N120" t="inlineStr">
+        <is>
+          <t>baseline</t>
+        </is>
+      </c>
+    </row>
+    <row r="121">
+      <c r="A121" t="inlineStr">
+        <is>
+          <t>baseline</t>
+        </is>
+      </c>
+      <c r="B121" t="inlineStr">
         <is>
           <t>Run1</t>
         </is>
       </c>
-      <c r="C117" t="inlineStr"/>
-      <c r="D117" t="inlineStr">
+      <c r="C121" t="inlineStr"/>
+      <c r="D121" t="inlineStr">
+        <is>
+          <t>CDD-CD-256</t>
+        </is>
+      </c>
+      <c r="E121" s="2" t="n">
+        <v>97.72</v>
+      </c>
+      <c r="F121" s="2" t="n">
+        <v>97.78</v>
+      </c>
+      <c r="G121" s="2" t="n">
+        <v>99.44</v>
+      </c>
+      <c r="H121" s="2" t="n">
+        <v>97.75</v>
+      </c>
+      <c r="I121" s="2" t="n">
+        <v>95.59999999999999</v>
+      </c>
+      <c r="J121" s="2" t="n">
+        <v>97.43000000000001</v>
+      </c>
+      <c r="K121" s="2" t="n">
+        <v>11.754</v>
+      </c>
+      <c r="L121" s="2" t="n">
+        <v>20.661</v>
+      </c>
+      <c r="M121" s="2" t="n">
+        <v>26.3246</v>
+      </c>
+      <c r="N121" t="inlineStr">
+        <is>
+          <t>baseline</t>
+        </is>
+      </c>
+    </row>
+    <row r="122">
+      <c r="A122" t="inlineStr">
+        <is>
+          <t>baseline</t>
+        </is>
+      </c>
+      <c r="B122" t="inlineStr">
+        <is>
+          <t>Run1</t>
+        </is>
+      </c>
+      <c r="C122" t="inlineStr"/>
+      <c r="D122" t="inlineStr">
+        <is>
+          <t>LEVIR-CD-256</t>
+        </is>
+      </c>
+      <c r="E122" s="2" t="n">
+        <v>91.56999999999999</v>
+      </c>
+      <c r="F122" s="2" t="n">
+        <v>92.33</v>
+      </c>
+      <c r="G122" s="2" t="n">
+        <v>99.18000000000001</v>
+      </c>
+      <c r="H122" s="2" t="n">
+        <v>91.95</v>
+      </c>
+      <c r="I122" s="2" t="n">
+        <v>85.09999999999999</v>
+      </c>
+      <c r="J122" s="2" t="n">
+        <v>91.52</v>
+      </c>
+      <c r="K122" s="2" t="n">
+        <v>11.754</v>
+      </c>
+      <c r="L122" s="2" t="n">
+        <v>20.661</v>
+      </c>
+      <c r="M122" s="2" t="n">
+        <v>26.3246</v>
+      </c>
+      <c r="N122" t="inlineStr">
+        <is>
+          <t>baseline</t>
+        </is>
+      </c>
+    </row>
+    <row r="123">
+      <c r="A123" t="inlineStr">
+        <is>
+          <t>baseline</t>
+        </is>
+      </c>
+      <c r="B123" t="inlineStr">
+        <is>
+          <t>Run1</t>
+        </is>
+      </c>
+      <c r="C123" t="inlineStr"/>
+      <c r="D123" t="inlineStr">
+        <is>
+          <t>SYSU-CD-256</t>
+        </is>
+      </c>
+      <c r="E123" s="2" t="n">
+        <v>80.77</v>
+      </c>
+      <c r="F123" s="2" t="n">
+        <v>84.27</v>
+      </c>
+      <c r="G123" s="2" t="n">
+        <v>91.91</v>
+      </c>
+      <c r="H123" s="2" t="n">
+        <v>82.48</v>
+      </c>
+      <c r="I123" s="2" t="n">
+        <v>70.19</v>
+      </c>
+      <c r="J123" s="2" t="n">
+        <v>77.23</v>
+      </c>
+      <c r="K123" s="2" t="n">
+        <v>11.754</v>
+      </c>
+      <c r="L123" s="2" t="n">
+        <v>20.661</v>
+      </c>
+      <c r="M123" s="2" t="n">
+        <v>26.3246</v>
+      </c>
+      <c r="N123" t="inlineStr">
+        <is>
+          <t>baseline</t>
+        </is>
+      </c>
+    </row>
+    <row r="124">
+      <c r="A124" t="inlineStr">
+        <is>
+          <t>baseline</t>
+        </is>
+      </c>
+      <c r="B124" t="inlineStr">
+        <is>
+          <t>Run1</t>
+        </is>
+      </c>
+      <c r="C124" t="inlineStr"/>
+      <c r="D124" t="inlineStr">
         <is>
           <t>WHU-CD-256</t>
         </is>
       </c>
-      <c r="E117" s="2" t="n">
+      <c r="E124" s="2" t="n">
         <v>93.62</v>
       </c>
-      <c r="F117" s="2" t="n">
+      <c r="F124" s="2" t="n">
         <v>96.09</v>
       </c>
-      <c r="G117" s="2" t="n">
+      <c r="G124" s="2" t="n">
         <v>99.59999999999999</v>
       </c>
-      <c r="H117" s="2" t="n">
+      <c r="H124" s="2" t="n">
         <v>94.84</v>
       </c>
-      <c r="I117" s="2" t="n">
+      <c r="I124" s="2" t="n">
         <v>90.18000000000001</v>
       </c>
-      <c r="J117" s="2" t="n">
+      <c r="J124" s="2" t="n">
         <v>94.63</v>
       </c>
-      <c r="K117" s="2" t="n">
+      <c r="K124" s="2" t="n">
         <v>11.754</v>
       </c>
-      <c r="L117" s="2" t="n">
+      <c r="L124" s="2" t="n">
         <v>20.661</v>
       </c>
-      <c r="M117" s="2" t="n">
+      <c r="M124" s="2" t="n">
         <v>26.3246</v>
       </c>
-      <c r="N117" t="inlineStr">
+      <c r="N124" t="inlineStr">
         <is>
           <t>baseline</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:N117"/>
+  <autoFilter ref="A1:N124"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Collect all CASA Run5 results and update experiment records
</commit_message>
<xml_diff>
--- a/docs/experiment_metrics.xlsx
+++ b/docs/experiment_metrics.xlsx
@@ -10,7 +10,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="metrics" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'metrics'!$A$1:$N$124</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'metrics'!$A$1:$N$136</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -420,7 +420,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N124"/>
+  <dimension ref="A1:N136"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -6138,17 +6138,17 @@
     <row r="108">
       <c r="A108" t="inlineStr">
         <is>
-          <t>STR-Fusion</t>
+          <t>CASA</t>
         </is>
       </c>
       <c r="B108" t="inlineStr">
         <is>
-          <t>Run2_TASS</t>
+          <t>Run5</t>
         </is>
       </c>
       <c r="C108" t="inlineStr">
         <is>
-          <t>C0_TOKEN</t>
+          <t>M0_CTRL</t>
         </is>
       </c>
       <c r="D108" t="inlineStr">
@@ -6157,52 +6157,50 @@
         </is>
       </c>
       <c r="E108" s="2" t="n">
-        <v>93.13</v>
+        <v>97.41</v>
       </c>
       <c r="F108" s="2" t="n">
-        <v>95.16</v>
+        <v>97.43000000000001</v>
       </c>
       <c r="G108" s="2" t="n">
-        <v>98.56999999999999</v>
+        <v>99.36</v>
       </c>
       <c r="H108" s="2" t="n">
-        <v>94.13</v>
+        <v>97.42</v>
       </c>
       <c r="I108" s="2" t="n">
-        <v>88.91</v>
+        <v>94.98</v>
       </c>
       <c r="J108" s="2" t="n">
-        <v>93.31999999999999</v>
+        <v>97.06</v>
       </c>
       <c r="K108" s="2" t="n">
-        <v>2.596</v>
+        <v>3.016737</v>
       </c>
       <c r="L108" s="2" t="n">
-        <v>0.62</v>
-      </c>
-      <c r="M108" s="2" t="n">
-        <v>2.2136</v>
-      </c>
+        <v>3.100404</v>
+      </c>
+      <c r="M108" s="2" t="n"/>
       <c r="N108" t="inlineStr">
         <is>
-          <t>str_tass</t>
+          <t>casa_none</t>
         </is>
       </c>
     </row>
     <row r="109">
       <c r="A109" t="inlineStr">
         <is>
-          <t>STR-Fusion</t>
+          <t>CASA</t>
         </is>
       </c>
       <c r="B109" t="inlineStr">
         <is>
-          <t>Run2_TASS</t>
+          <t>Run5</t>
         </is>
       </c>
       <c r="C109" t="inlineStr">
         <is>
-          <t>C0_TOKEN</t>
+          <t>M0_CTRL</t>
         </is>
       </c>
       <c r="D109" t="inlineStr">
@@ -6211,52 +6209,50 @@
         </is>
       </c>
       <c r="E109" s="2" t="n">
-        <v>86.37</v>
+        <v>90.29000000000001</v>
       </c>
       <c r="F109" s="2" t="n">
-        <v>89.25</v>
+        <v>92.58</v>
       </c>
       <c r="G109" s="2" t="n">
-        <v>98.78</v>
+        <v>99.14</v>
       </c>
       <c r="H109" s="2" t="n">
-        <v>87.79000000000001</v>
+        <v>91.42</v>
       </c>
       <c r="I109" s="2" t="n">
-        <v>78.23999999999999</v>
+        <v>84.19</v>
       </c>
       <c r="J109" s="2" t="n">
-        <v>87.14</v>
+        <v>90.95999999999999</v>
       </c>
       <c r="K109" s="2" t="n">
-        <v>2.596</v>
+        <v>3.016737</v>
       </c>
       <c r="L109" s="2" t="n">
-        <v>0.62</v>
-      </c>
-      <c r="M109" s="2" t="n">
-        <v>2.2136</v>
-      </c>
+        <v>3.100404</v>
+      </c>
+      <c r="M109" s="2" t="n"/>
       <c r="N109" t="inlineStr">
         <is>
-          <t>str_tass</t>
+          <t>casa_none</t>
         </is>
       </c>
     </row>
     <row r="110">
       <c r="A110" t="inlineStr">
         <is>
-          <t>STR-Fusion</t>
+          <t>CASA</t>
         </is>
       </c>
       <c r="B110" t="inlineStr">
         <is>
-          <t>Run2_TASS</t>
+          <t>Run5</t>
         </is>
       </c>
       <c r="C110" t="inlineStr">
         <is>
-          <t>C0_TOKEN</t>
+          <t>M0_CTRL</t>
         </is>
       </c>
       <c r="D110" t="inlineStr">
@@ -6265,52 +6261,50 @@
         </is>
       </c>
       <c r="E110" s="2" t="n">
-        <v>79.93000000000001</v>
+        <v>80.38</v>
       </c>
       <c r="F110" s="2" t="n">
-        <v>84.5</v>
+        <v>85.22</v>
       </c>
       <c r="G110" s="2" t="n">
-        <v>91.81</v>
+        <v>92.09</v>
       </c>
       <c r="H110" s="2" t="n">
-        <v>82.15000000000001</v>
+        <v>82.73</v>
       </c>
       <c r="I110" s="2" t="n">
-        <v>69.70999999999999</v>
+        <v>70.55</v>
       </c>
       <c r="J110" s="2" t="n">
-        <v>76.84</v>
+        <v>77.59999999999999</v>
       </c>
       <c r="K110" s="2" t="n">
-        <v>2.596</v>
+        <v>3.016737</v>
       </c>
       <c r="L110" s="2" t="n">
-        <v>0.62</v>
-      </c>
-      <c r="M110" s="2" t="n">
-        <v>2.2136</v>
-      </c>
+        <v>3.100404</v>
+      </c>
+      <c r="M110" s="2" t="n"/>
       <c r="N110" t="inlineStr">
         <is>
-          <t>str_tass</t>
+          <t>casa_none</t>
         </is>
       </c>
     </row>
     <row r="111">
       <c r="A111" t="inlineStr">
         <is>
-          <t>STR-Fusion</t>
+          <t>CASA</t>
         </is>
       </c>
       <c r="B111" t="inlineStr">
         <is>
-          <t>Run2_TASS</t>
+          <t>Run5</t>
         </is>
       </c>
       <c r="C111" t="inlineStr">
         <is>
-          <t>C0_TOKEN</t>
+          <t>M0_CTRL</t>
         </is>
       </c>
       <c r="D111" t="inlineStr">
@@ -6319,52 +6313,50 @@
         </is>
       </c>
       <c r="E111" s="2" t="n">
-        <v>90.16</v>
+        <v>92.87</v>
       </c>
       <c r="F111" s="2" t="n">
-        <v>93.97</v>
+        <v>96.04000000000001</v>
       </c>
       <c r="G111" s="2" t="n">
-        <v>99.38</v>
+        <v>99.56999999999999</v>
       </c>
       <c r="H111" s="2" t="n">
-        <v>92.02</v>
+        <v>94.43000000000001</v>
       </c>
       <c r="I111" s="2" t="n">
-        <v>85.23</v>
+        <v>89.44</v>
       </c>
       <c r="J111" s="2" t="n">
-        <v>91.7</v>
+        <v>94.2</v>
       </c>
       <c r="K111" s="2" t="n">
-        <v>2.596</v>
+        <v>3.016737</v>
       </c>
       <c r="L111" s="2" t="n">
-        <v>0.62</v>
-      </c>
-      <c r="M111" s="2" t="n">
-        <v>2.2136</v>
-      </c>
+        <v>3.100404</v>
+      </c>
+      <c r="M111" s="2" t="n"/>
       <c r="N111" t="inlineStr">
         <is>
-          <t>str_tass</t>
+          <t>casa_none</t>
         </is>
       </c>
     </row>
     <row r="112">
       <c r="A112" t="inlineStr">
         <is>
-          <t>STR-Fusion</t>
+          <t>CASA</t>
         </is>
       </c>
       <c r="B112" t="inlineStr">
         <is>
-          <t>Run2_TASS</t>
+          <t>Run5</t>
         </is>
       </c>
       <c r="C112" t="inlineStr">
         <is>
-          <t>M1_TASS</t>
+          <t>M1_HYPER_QKV</t>
         </is>
       </c>
       <c r="D112" t="inlineStr">
@@ -6373,52 +6365,50 @@
         </is>
       </c>
       <c r="E112" s="2" t="n">
-        <v>94.7</v>
+        <v>97.52</v>
       </c>
       <c r="F112" s="2" t="n">
-        <v>96.13</v>
+        <v>97.42</v>
       </c>
       <c r="G112" s="2" t="n">
-        <v>98.88</v>
+        <v>99.38</v>
       </c>
       <c r="H112" s="2" t="n">
-        <v>95.41</v>
+        <v>97.47</v>
       </c>
       <c r="I112" s="2" t="n">
-        <v>91.22</v>
+        <v>95.06999999999999</v>
       </c>
       <c r="J112" s="2" t="n">
-        <v>94.77</v>
+        <v>97.11</v>
       </c>
       <c r="K112" s="2" t="n">
-        <v>3.455</v>
+        <v>3.060525</v>
       </c>
       <c r="L112" s="2" t="n">
-        <v>1.478</v>
-      </c>
-      <c r="M112" s="2" t="n">
-        <v>3.5459</v>
-      </c>
+        <v>3.144192</v>
+      </c>
+      <c r="M112" s="2" t="n"/>
       <c r="N112" t="inlineStr">
         <is>
-          <t>str_tass</t>
+          <t>casa_hyperbolic</t>
         </is>
       </c>
     </row>
     <row r="113">
       <c r="A113" t="inlineStr">
         <is>
-          <t>STR-Fusion</t>
+          <t>CASA</t>
         </is>
       </c>
       <c r="B113" t="inlineStr">
         <is>
-          <t>Run2_TASS</t>
+          <t>Run5</t>
         </is>
       </c>
       <c r="C113" t="inlineStr">
         <is>
-          <t>M1_TASS</t>
+          <t>M1_HYPER_QKV</t>
         </is>
       </c>
       <c r="D113" t="inlineStr">
@@ -6427,52 +6417,50 @@
         </is>
       </c>
       <c r="E113" s="2" t="n">
-        <v>88.42</v>
+        <v>90.48</v>
       </c>
       <c r="F113" s="2" t="n">
-        <v>91.97</v>
+        <v>92.91</v>
       </c>
       <c r="G113" s="2" t="n">
-        <v>99.02</v>
+        <v>99.16</v>
       </c>
       <c r="H113" s="2" t="n">
-        <v>90.16</v>
+        <v>91.68000000000001</v>
       </c>
       <c r="I113" s="2" t="n">
-        <v>82.08</v>
+        <v>84.64</v>
       </c>
       <c r="J113" s="2" t="n">
-        <v>89.64</v>
+        <v>91.23999999999999</v>
       </c>
       <c r="K113" s="2" t="n">
-        <v>3.455</v>
+        <v>3.060525</v>
       </c>
       <c r="L113" s="2" t="n">
-        <v>1.478</v>
-      </c>
-      <c r="M113" s="2" t="n">
-        <v>3.5459</v>
-      </c>
+        <v>3.144192</v>
+      </c>
+      <c r="M113" s="2" t="n"/>
       <c r="N113" t="inlineStr">
         <is>
-          <t>str_tass</t>
+          <t>casa_hyperbolic</t>
         </is>
       </c>
     </row>
     <row r="114">
       <c r="A114" t="inlineStr">
         <is>
-          <t>STR-Fusion</t>
+          <t>CASA</t>
         </is>
       </c>
       <c r="B114" t="inlineStr">
         <is>
-          <t>Run2_TASS</t>
+          <t>Run5</t>
         </is>
       </c>
       <c r="C114" t="inlineStr">
         <is>
-          <t>M1_TASS</t>
+          <t>M1_HYPER_QKV</t>
         </is>
       </c>
       <c r="D114" t="inlineStr">
@@ -6481,52 +6469,50 @@
         </is>
       </c>
       <c r="E114" s="2" t="n">
-        <v>78.73</v>
+        <v>83.2</v>
       </c>
       <c r="F114" s="2" t="n">
-        <v>84.98</v>
+        <v>80.95</v>
       </c>
       <c r="G114" s="2" t="n">
-        <v>91.7</v>
+        <v>91.42</v>
       </c>
       <c r="H114" s="2" t="n">
-        <v>81.73999999999999</v>
+        <v>82.06</v>
       </c>
       <c r="I114" s="2" t="n">
-        <v>69.11</v>
+        <v>69.58</v>
       </c>
       <c r="J114" s="2" t="n">
-        <v>76.38</v>
+        <v>76.42</v>
       </c>
       <c r="K114" s="2" t="n">
-        <v>3.455</v>
+        <v>3.060525</v>
       </c>
       <c r="L114" s="2" t="n">
-        <v>1.478</v>
-      </c>
-      <c r="M114" s="2" t="n">
-        <v>3.5459</v>
-      </c>
+        <v>3.144192</v>
+      </c>
+      <c r="M114" s="2" t="n"/>
       <c r="N114" t="inlineStr">
         <is>
-          <t>str_tass</t>
+          <t>casa_hyperbolic</t>
         </is>
       </c>
     </row>
     <row r="115">
       <c r="A115" t="inlineStr">
         <is>
-          <t>STR-Fusion</t>
+          <t>CASA</t>
         </is>
       </c>
       <c r="B115" t="inlineStr">
         <is>
-          <t>Run2_TASS</t>
+          <t>Run5</t>
         </is>
       </c>
       <c r="C115" t="inlineStr">
         <is>
-          <t>M1_TASS</t>
+          <t>M1_HYPER_QKV</t>
         </is>
       </c>
       <c r="D115" t="inlineStr">
@@ -6535,160 +6521,154 @@
         </is>
       </c>
       <c r="E115" s="2" t="n">
-        <v>91.64</v>
+        <v>92.36</v>
       </c>
       <c r="F115" s="2" t="n">
-        <v>94.81999999999999</v>
+        <v>95.44</v>
       </c>
       <c r="G115" s="2" t="n">
-        <v>99.47</v>
+        <v>99.52</v>
       </c>
       <c r="H115" s="2" t="n">
-        <v>93.2</v>
+        <v>93.88</v>
       </c>
       <c r="I115" s="2" t="n">
-        <v>87.27</v>
+        <v>88.45999999999999</v>
       </c>
       <c r="J115" s="2" t="n">
-        <v>92.93000000000001</v>
+        <v>93.63</v>
       </c>
       <c r="K115" s="2" t="n">
-        <v>3.455</v>
+        <v>3.060525</v>
       </c>
       <c r="L115" s="2" t="n">
-        <v>1.478</v>
-      </c>
-      <c r="M115" s="2" t="n">
-        <v>3.5459</v>
-      </c>
+        <v>3.144192</v>
+      </c>
+      <c r="M115" s="2" t="n"/>
       <c r="N115" t="inlineStr">
         <is>
-          <t>str_tass</t>
+          <t>casa_hyperbolic</t>
         </is>
       </c>
     </row>
     <row r="116">
       <c r="A116" t="inlineStr">
         <is>
-          <t>UltraLight</t>
+          <t>CASA</t>
         </is>
       </c>
       <c r="B116" t="inlineStr">
         <is>
-          <t>Run4</t>
+          <t>Run5</t>
         </is>
       </c>
       <c r="C116" t="inlineStr">
         <is>
-          <t>R4_0_A0_FULL12_FROZEN</t>
+          <t>M2_CA_QKV</t>
         </is>
       </c>
       <c r="D116" t="inlineStr">
         <is>
-          <t>SYSU-CD-256</t>
+          <t>CDD-CD-256</t>
         </is>
       </c>
       <c r="E116" s="2" t="n">
-        <v>82.42</v>
+        <v>97.43000000000001</v>
       </c>
       <c r="F116" s="2" t="n">
-        <v>83.87</v>
+        <v>97.51000000000001</v>
       </c>
       <c r="G116" s="2" t="n">
-        <v>92.12</v>
+        <v>99.38</v>
       </c>
       <c r="H116" s="2" t="n">
-        <v>83.14</v>
+        <v>97.47</v>
       </c>
       <c r="I116" s="2" t="n">
-        <v>71.14</v>
+        <v>95.06</v>
       </c>
       <c r="J116" s="2" t="n">
-        <v>77.98999999999999</v>
+        <v>97.11</v>
       </c>
       <c r="K116" s="2" t="n">
-        <v>11.754</v>
+        <v>3.077293</v>
       </c>
       <c r="L116" s="2" t="n">
-        <v>15.125</v>
-      </c>
-      <c r="M116" s="2" t="n">
-        <v>26.3246</v>
-      </c>
+        <v>3.16096</v>
+      </c>
+      <c r="M116" s="2" t="n"/>
       <c r="N116" t="inlineStr">
         <is>
-          <t>baseline</t>
+          <t>casa_qkv</t>
         </is>
       </c>
     </row>
     <row r="117">
       <c r="A117" t="inlineStr">
         <is>
-          <t>UltraLight</t>
+          <t>CASA</t>
         </is>
       </c>
       <c r="B117" t="inlineStr">
         <is>
-          <t>Run4</t>
+          <t>Run5</t>
         </is>
       </c>
       <c r="C117" t="inlineStr">
         <is>
-          <t>R4_1_VIT4_OLDHEAD</t>
+          <t>M2_CA_QKV</t>
         </is>
       </c>
       <c r="D117" t="inlineStr">
         <is>
-          <t>SYSU-CD-256</t>
+          <t>LEVIR-CD-256</t>
         </is>
       </c>
       <c r="E117" s="2" t="n">
-        <v>82.15000000000001</v>
+        <v>90.45</v>
       </c>
       <c r="F117" s="2" t="n">
-        <v>83.40000000000001</v>
+        <v>92.68000000000001</v>
       </c>
       <c r="G117" s="2" t="n">
-        <v>91.94</v>
+        <v>99.15000000000001</v>
       </c>
       <c r="H117" s="2" t="n">
-        <v>82.77</v>
+        <v>91.55</v>
       </c>
       <c r="I117" s="2" t="n">
-        <v>70.61</v>
+        <v>84.42</v>
       </c>
       <c r="J117" s="2" t="n">
-        <v>77.51000000000001</v>
+        <v>91.11</v>
       </c>
       <c r="K117" s="2" t="n">
-        <v>8.195</v>
+        <v>3.077293</v>
       </c>
       <c r="L117" s="2" t="n">
-        <v>15.125</v>
-      </c>
-      <c r="M117" s="2" t="n">
-        <v>24.1021</v>
-      </c>
+        <v>3.16096</v>
+      </c>
+      <c r="M117" s="2" t="n"/>
       <c r="N117" t="inlineStr">
         <is>
-          <t>baseline</t>
+          <t>casa_qkv</t>
         </is>
       </c>
     </row>
     <row r="118">
       <c r="A118" t="inlineStr">
         <is>
-          <t>UltraLight</t>
+          <t>CASA</t>
         </is>
       </c>
       <c r="B118" t="inlineStr">
         <is>
-          <t>Run4</t>
+          <t>Run5</t>
         </is>
       </c>
       <c r="C118" t="inlineStr">
         <is>
-          <t>R4_2_VIT4_LIGHTDETAIL</t>
+          <t>M2_CA_QKV</t>
         </is>
       </c>
       <c r="D118" t="inlineStr">
@@ -6697,348 +6677,992 @@
         </is>
       </c>
       <c r="E118" s="2" t="n">
-        <v>79.94</v>
+        <v>78.5</v>
       </c>
       <c r="F118" s="2" t="n">
-        <v>84.79000000000001</v>
+        <v>86.2</v>
       </c>
       <c r="G118" s="2" t="n">
-        <v>91.89</v>
+        <v>91.97</v>
       </c>
       <c r="H118" s="2" t="n">
-        <v>82.3</v>
+        <v>82.17</v>
       </c>
       <c r="I118" s="2" t="n">
-        <v>69.92</v>
+        <v>69.73999999999999</v>
       </c>
       <c r="J118" s="2" t="n">
-        <v>77.04000000000001</v>
+        <v>77</v>
       </c>
       <c r="K118" s="2" t="n">
-        <v>5.492</v>
+        <v>3.077293</v>
       </c>
       <c r="L118" s="2" t="n">
-        <v>3.515</v>
-      </c>
-      <c r="M118" s="2" t="n">
-        <v>10.7311</v>
-      </c>
+        <v>3.16096</v>
+      </c>
+      <c r="M118" s="2" t="n"/>
       <c r="N118" t="inlineStr">
         <is>
-          <t>baseline</t>
+          <t>casa_qkv</t>
         </is>
       </c>
     </row>
     <row r="119">
       <c r="A119" t="inlineStr">
         <is>
-          <t>UltraLight</t>
+          <t>CASA</t>
         </is>
       </c>
       <c r="B119" t="inlineStr">
         <is>
-          <t>Run4</t>
+          <t>Run5</t>
         </is>
       </c>
       <c r="C119" t="inlineStr">
         <is>
-          <t>R4_2b_VIT4_LIGHTDETAIL48</t>
+          <t>M2_CA_QKV</t>
         </is>
       </c>
       <c r="D119" t="inlineStr">
         <is>
-          <t>SYSU-CD-256</t>
+          <t>WHU-CD-256</t>
         </is>
       </c>
       <c r="E119" s="2" t="n">
-        <v>80.87</v>
+        <v>91.88</v>
       </c>
       <c r="F119" s="2" t="n">
-        <v>83.81</v>
+        <v>94.98999999999999</v>
       </c>
       <c r="G119" s="2" t="n">
-        <v>91.81</v>
+        <v>99.48999999999999</v>
       </c>
       <c r="H119" s="2" t="n">
-        <v>82.31999999999999</v>
+        <v>93.41</v>
       </c>
       <c r="I119" s="2" t="n">
-        <v>69.95</v>
+        <v>87.63</v>
       </c>
       <c r="J119" s="2" t="n">
-        <v>76.98999999999999</v>
+        <v>93.14</v>
       </c>
       <c r="K119" s="2" t="n">
-        <v>5.533</v>
+        <v>3.077293</v>
       </c>
       <c r="L119" s="2" t="n">
-        <v>3.556</v>
-      </c>
-      <c r="M119" s="2" t="n">
-        <v>10.9824</v>
-      </c>
+        <v>3.16096</v>
+      </c>
+      <c r="M119" s="2" t="n"/>
       <c r="N119" t="inlineStr">
         <is>
-          <t>baseline</t>
+          <t>casa_qkv</t>
         </is>
       </c>
     </row>
     <row r="120">
       <c r="A120" t="inlineStr">
         <is>
-          <t>UltraLight</t>
+          <t>STR-Fusion</t>
         </is>
       </c>
       <c r="B120" t="inlineStr">
         <is>
-          <t>Run4</t>
+          <t>Run2_TASS</t>
         </is>
       </c>
       <c r="C120" t="inlineStr">
         <is>
-          <t>R4_2d_PSD_DETAIL</t>
+          <t>C0_TOKEN</t>
         </is>
       </c>
       <c r="D120" t="inlineStr">
         <is>
-          <t>SYSU-CD-256</t>
+          <t>CDD-CD-256</t>
         </is>
       </c>
       <c r="E120" s="2" t="n">
-        <v>79.78</v>
+        <v>93.13</v>
       </c>
       <c r="F120" s="2" t="n">
-        <v>84.39</v>
+        <v>95.16</v>
       </c>
       <c r="G120" s="2" t="n">
-        <v>91.75</v>
+        <v>98.56999999999999</v>
       </c>
       <c r="H120" s="2" t="n">
-        <v>82.02</v>
+        <v>94.13</v>
       </c>
       <c r="I120" s="2" t="n">
-        <v>69.52</v>
+        <v>88.91</v>
       </c>
       <c r="J120" s="2" t="n">
-        <v>76.68000000000001</v>
+        <v>93.31999999999999</v>
       </c>
       <c r="K120" s="2" t="n">
-        <v>5.491</v>
+        <v>2.596</v>
       </c>
       <c r="L120" s="2" t="n">
-        <v>3.514</v>
+        <v>0.62</v>
       </c>
       <c r="M120" s="2" t="n">
-        <v>11.5239</v>
+        <v>2.2136</v>
       </c>
       <c r="N120" t="inlineStr">
         <is>
-          <t>baseline</t>
+          <t>str_tass</t>
         </is>
       </c>
     </row>
     <row r="121">
       <c r="A121" t="inlineStr">
         <is>
-          <t>baseline</t>
+          <t>STR-Fusion</t>
         </is>
       </c>
       <c r="B121" t="inlineStr">
         <is>
-          <t>Run1</t>
-        </is>
-      </c>
-      <c r="C121" t="inlineStr"/>
+          <t>Run2_TASS</t>
+        </is>
+      </c>
+      <c r="C121" t="inlineStr">
+        <is>
+          <t>C0_TOKEN</t>
+        </is>
+      </c>
       <c r="D121" t="inlineStr">
         <is>
-          <t>CDD-CD-256</t>
+          <t>LEVIR-CD-256</t>
         </is>
       </c>
       <c r="E121" s="2" t="n">
-        <v>97.72</v>
+        <v>86.37</v>
       </c>
       <c r="F121" s="2" t="n">
-        <v>97.78</v>
+        <v>89.25</v>
       </c>
       <c r="G121" s="2" t="n">
-        <v>99.44</v>
+        <v>98.78</v>
       </c>
       <c r="H121" s="2" t="n">
-        <v>97.75</v>
+        <v>87.79000000000001</v>
       </c>
       <c r="I121" s="2" t="n">
-        <v>95.59999999999999</v>
+        <v>78.23999999999999</v>
       </c>
       <c r="J121" s="2" t="n">
-        <v>97.43000000000001</v>
+        <v>87.14</v>
       </c>
       <c r="K121" s="2" t="n">
-        <v>11.754</v>
+        <v>2.596</v>
       </c>
       <c r="L121" s="2" t="n">
-        <v>20.661</v>
+        <v>0.62</v>
       </c>
       <c r="M121" s="2" t="n">
-        <v>26.3246</v>
+        <v>2.2136</v>
       </c>
       <c r="N121" t="inlineStr">
         <is>
-          <t>baseline</t>
+          <t>str_tass</t>
         </is>
       </c>
     </row>
     <row r="122">
       <c r="A122" t="inlineStr">
         <is>
-          <t>baseline</t>
+          <t>STR-Fusion</t>
         </is>
       </c>
       <c r="B122" t="inlineStr">
         <is>
-          <t>Run1</t>
-        </is>
-      </c>
-      <c r="C122" t="inlineStr"/>
+          <t>Run2_TASS</t>
+        </is>
+      </c>
+      <c r="C122" t="inlineStr">
+        <is>
+          <t>C0_TOKEN</t>
+        </is>
+      </c>
       <c r="D122" t="inlineStr">
         <is>
-          <t>LEVIR-CD-256</t>
+          <t>SYSU-CD-256</t>
         </is>
       </c>
       <c r="E122" s="2" t="n">
-        <v>91.56999999999999</v>
+        <v>79.93000000000001</v>
       </c>
       <c r="F122" s="2" t="n">
-        <v>92.33</v>
+        <v>84.5</v>
       </c>
       <c r="G122" s="2" t="n">
-        <v>99.18000000000001</v>
+        <v>91.81</v>
       </c>
       <c r="H122" s="2" t="n">
-        <v>91.95</v>
+        <v>82.15000000000001</v>
       </c>
       <c r="I122" s="2" t="n">
-        <v>85.09999999999999</v>
+        <v>69.70999999999999</v>
       </c>
       <c r="J122" s="2" t="n">
-        <v>91.52</v>
+        <v>76.84</v>
       </c>
       <c r="K122" s="2" t="n">
-        <v>11.754</v>
+        <v>2.596</v>
       </c>
       <c r="L122" s="2" t="n">
-        <v>20.661</v>
+        <v>0.62</v>
       </c>
       <c r="M122" s="2" t="n">
-        <v>26.3246</v>
+        <v>2.2136</v>
       </c>
       <c r="N122" t="inlineStr">
         <is>
-          <t>baseline</t>
+          <t>str_tass</t>
         </is>
       </c>
     </row>
     <row r="123">
       <c r="A123" t="inlineStr">
         <is>
-          <t>baseline</t>
+          <t>STR-Fusion</t>
         </is>
       </c>
       <c r="B123" t="inlineStr">
         <is>
-          <t>Run1</t>
-        </is>
-      </c>
-      <c r="C123" t="inlineStr"/>
+          <t>Run2_TASS</t>
+        </is>
+      </c>
+      <c r="C123" t="inlineStr">
+        <is>
+          <t>C0_TOKEN</t>
+        </is>
+      </c>
       <c r="D123" t="inlineStr">
         <is>
-          <t>SYSU-CD-256</t>
+          <t>WHU-CD-256</t>
         </is>
       </c>
       <c r="E123" s="2" t="n">
-        <v>80.77</v>
+        <v>90.16</v>
       </c>
       <c r="F123" s="2" t="n">
-        <v>84.27</v>
+        <v>93.97</v>
       </c>
       <c r="G123" s="2" t="n">
-        <v>91.91</v>
+        <v>99.38</v>
       </c>
       <c r="H123" s="2" t="n">
-        <v>82.48</v>
+        <v>92.02</v>
       </c>
       <c r="I123" s="2" t="n">
-        <v>70.19</v>
+        <v>85.23</v>
       </c>
       <c r="J123" s="2" t="n">
-        <v>77.23</v>
+        <v>91.7</v>
       </c>
       <c r="K123" s="2" t="n">
-        <v>11.754</v>
+        <v>2.596</v>
       </c>
       <c r="L123" s="2" t="n">
-        <v>20.661</v>
+        <v>0.62</v>
       </c>
       <c r="M123" s="2" t="n">
-        <v>26.3246</v>
+        <v>2.2136</v>
       </c>
       <c r="N123" t="inlineStr">
         <is>
-          <t>baseline</t>
+          <t>str_tass</t>
         </is>
       </c>
     </row>
     <row r="124">
       <c r="A124" t="inlineStr">
         <is>
+          <t>STR-Fusion</t>
+        </is>
+      </c>
+      <c r="B124" t="inlineStr">
+        <is>
+          <t>Run2_TASS</t>
+        </is>
+      </c>
+      <c r="C124" t="inlineStr">
+        <is>
+          <t>M1_TASS</t>
+        </is>
+      </c>
+      <c r="D124" t="inlineStr">
+        <is>
+          <t>CDD-CD-256</t>
+        </is>
+      </c>
+      <c r="E124" s="2" t="n">
+        <v>94.7</v>
+      </c>
+      <c r="F124" s="2" t="n">
+        <v>96.13</v>
+      </c>
+      <c r="G124" s="2" t="n">
+        <v>98.88</v>
+      </c>
+      <c r="H124" s="2" t="n">
+        <v>95.41</v>
+      </c>
+      <c r="I124" s="2" t="n">
+        <v>91.22</v>
+      </c>
+      <c r="J124" s="2" t="n">
+        <v>94.77</v>
+      </c>
+      <c r="K124" s="2" t="n">
+        <v>3.455</v>
+      </c>
+      <c r="L124" s="2" t="n">
+        <v>1.478</v>
+      </c>
+      <c r="M124" s="2" t="n">
+        <v>3.5459</v>
+      </c>
+      <c r="N124" t="inlineStr">
+        <is>
+          <t>str_tass</t>
+        </is>
+      </c>
+    </row>
+    <row r="125">
+      <c r="A125" t="inlineStr">
+        <is>
+          <t>STR-Fusion</t>
+        </is>
+      </c>
+      <c r="B125" t="inlineStr">
+        <is>
+          <t>Run2_TASS</t>
+        </is>
+      </c>
+      <c r="C125" t="inlineStr">
+        <is>
+          <t>M1_TASS</t>
+        </is>
+      </c>
+      <c r="D125" t="inlineStr">
+        <is>
+          <t>LEVIR-CD-256</t>
+        </is>
+      </c>
+      <c r="E125" s="2" t="n">
+        <v>88.42</v>
+      </c>
+      <c r="F125" s="2" t="n">
+        <v>91.97</v>
+      </c>
+      <c r="G125" s="2" t="n">
+        <v>99.02</v>
+      </c>
+      <c r="H125" s="2" t="n">
+        <v>90.16</v>
+      </c>
+      <c r="I125" s="2" t="n">
+        <v>82.08</v>
+      </c>
+      <c r="J125" s="2" t="n">
+        <v>89.64</v>
+      </c>
+      <c r="K125" s="2" t="n">
+        <v>3.455</v>
+      </c>
+      <c r="L125" s="2" t="n">
+        <v>1.478</v>
+      </c>
+      <c r="M125" s="2" t="n">
+        <v>3.5459</v>
+      </c>
+      <c r="N125" t="inlineStr">
+        <is>
+          <t>str_tass</t>
+        </is>
+      </c>
+    </row>
+    <row r="126">
+      <c r="A126" t="inlineStr">
+        <is>
+          <t>STR-Fusion</t>
+        </is>
+      </c>
+      <c r="B126" t="inlineStr">
+        <is>
+          <t>Run2_TASS</t>
+        </is>
+      </c>
+      <c r="C126" t="inlineStr">
+        <is>
+          <t>M1_TASS</t>
+        </is>
+      </c>
+      <c r="D126" t="inlineStr">
+        <is>
+          <t>SYSU-CD-256</t>
+        </is>
+      </c>
+      <c r="E126" s="2" t="n">
+        <v>78.73</v>
+      </c>
+      <c r="F126" s="2" t="n">
+        <v>84.98</v>
+      </c>
+      <c r="G126" s="2" t="n">
+        <v>91.7</v>
+      </c>
+      <c r="H126" s="2" t="n">
+        <v>81.73999999999999</v>
+      </c>
+      <c r="I126" s="2" t="n">
+        <v>69.11</v>
+      </c>
+      <c r="J126" s="2" t="n">
+        <v>76.38</v>
+      </c>
+      <c r="K126" s="2" t="n">
+        <v>3.455</v>
+      </c>
+      <c r="L126" s="2" t="n">
+        <v>1.478</v>
+      </c>
+      <c r="M126" s="2" t="n">
+        <v>3.5459</v>
+      </c>
+      <c r="N126" t="inlineStr">
+        <is>
+          <t>str_tass</t>
+        </is>
+      </c>
+    </row>
+    <row r="127">
+      <c r="A127" t="inlineStr">
+        <is>
+          <t>STR-Fusion</t>
+        </is>
+      </c>
+      <c r="B127" t="inlineStr">
+        <is>
+          <t>Run2_TASS</t>
+        </is>
+      </c>
+      <c r="C127" t="inlineStr">
+        <is>
+          <t>M1_TASS</t>
+        </is>
+      </c>
+      <c r="D127" t="inlineStr">
+        <is>
+          <t>WHU-CD-256</t>
+        </is>
+      </c>
+      <c r="E127" s="2" t="n">
+        <v>91.64</v>
+      </c>
+      <c r="F127" s="2" t="n">
+        <v>94.81999999999999</v>
+      </c>
+      <c r="G127" s="2" t="n">
+        <v>99.47</v>
+      </c>
+      <c r="H127" s="2" t="n">
+        <v>93.2</v>
+      </c>
+      <c r="I127" s="2" t="n">
+        <v>87.27</v>
+      </c>
+      <c r="J127" s="2" t="n">
+        <v>92.93000000000001</v>
+      </c>
+      <c r="K127" s="2" t="n">
+        <v>3.455</v>
+      </c>
+      <c r="L127" s="2" t="n">
+        <v>1.478</v>
+      </c>
+      <c r="M127" s="2" t="n">
+        <v>3.5459</v>
+      </c>
+      <c r="N127" t="inlineStr">
+        <is>
+          <t>str_tass</t>
+        </is>
+      </c>
+    </row>
+    <row r="128">
+      <c r="A128" t="inlineStr">
+        <is>
+          <t>UltraLight</t>
+        </is>
+      </c>
+      <c r="B128" t="inlineStr">
+        <is>
+          <t>Run4</t>
+        </is>
+      </c>
+      <c r="C128" t="inlineStr">
+        <is>
+          <t>R4_0_A0_FULL12_FROZEN</t>
+        </is>
+      </c>
+      <c r="D128" t="inlineStr">
+        <is>
+          <t>SYSU-CD-256</t>
+        </is>
+      </c>
+      <c r="E128" s="2" t="n">
+        <v>82.42</v>
+      </c>
+      <c r="F128" s="2" t="n">
+        <v>83.87</v>
+      </c>
+      <c r="G128" s="2" t="n">
+        <v>92.12</v>
+      </c>
+      <c r="H128" s="2" t="n">
+        <v>83.14</v>
+      </c>
+      <c r="I128" s="2" t="n">
+        <v>71.14</v>
+      </c>
+      <c r="J128" s="2" t="n">
+        <v>77.98999999999999</v>
+      </c>
+      <c r="K128" s="2" t="n">
+        <v>11.754</v>
+      </c>
+      <c r="L128" s="2" t="n">
+        <v>15.125</v>
+      </c>
+      <c r="M128" s="2" t="n">
+        <v>26.3246</v>
+      </c>
+      <c r="N128" t="inlineStr">
+        <is>
           <t>baseline</t>
         </is>
       </c>
-      <c r="B124" t="inlineStr">
+    </row>
+    <row r="129">
+      <c r="A129" t="inlineStr">
+        <is>
+          <t>UltraLight</t>
+        </is>
+      </c>
+      <c r="B129" t="inlineStr">
+        <is>
+          <t>Run4</t>
+        </is>
+      </c>
+      <c r="C129" t="inlineStr">
+        <is>
+          <t>R4_1_VIT4_OLDHEAD</t>
+        </is>
+      </c>
+      <c r="D129" t="inlineStr">
+        <is>
+          <t>SYSU-CD-256</t>
+        </is>
+      </c>
+      <c r="E129" s="2" t="n">
+        <v>82.15000000000001</v>
+      </c>
+      <c r="F129" s="2" t="n">
+        <v>83.40000000000001</v>
+      </c>
+      <c r="G129" s="2" t="n">
+        <v>91.94</v>
+      </c>
+      <c r="H129" s="2" t="n">
+        <v>82.77</v>
+      </c>
+      <c r="I129" s="2" t="n">
+        <v>70.61</v>
+      </c>
+      <c r="J129" s="2" t="n">
+        <v>77.51000000000001</v>
+      </c>
+      <c r="K129" s="2" t="n">
+        <v>8.195</v>
+      </c>
+      <c r="L129" s="2" t="n">
+        <v>15.125</v>
+      </c>
+      <c r="M129" s="2" t="n">
+        <v>24.1021</v>
+      </c>
+      <c r="N129" t="inlineStr">
+        <is>
+          <t>baseline</t>
+        </is>
+      </c>
+    </row>
+    <row r="130">
+      <c r="A130" t="inlineStr">
+        <is>
+          <t>UltraLight</t>
+        </is>
+      </c>
+      <c r="B130" t="inlineStr">
+        <is>
+          <t>Run4</t>
+        </is>
+      </c>
+      <c r="C130" t="inlineStr">
+        <is>
+          <t>R4_2_VIT4_LIGHTDETAIL</t>
+        </is>
+      </c>
+      <c r="D130" t="inlineStr">
+        <is>
+          <t>SYSU-CD-256</t>
+        </is>
+      </c>
+      <c r="E130" s="2" t="n">
+        <v>79.94</v>
+      </c>
+      <c r="F130" s="2" t="n">
+        <v>84.79000000000001</v>
+      </c>
+      <c r="G130" s="2" t="n">
+        <v>91.89</v>
+      </c>
+      <c r="H130" s="2" t="n">
+        <v>82.3</v>
+      </c>
+      <c r="I130" s="2" t="n">
+        <v>69.92</v>
+      </c>
+      <c r="J130" s="2" t="n">
+        <v>77.04000000000001</v>
+      </c>
+      <c r="K130" s="2" t="n">
+        <v>5.492</v>
+      </c>
+      <c r="L130" s="2" t="n">
+        <v>3.515</v>
+      </c>
+      <c r="M130" s="2" t="n">
+        <v>10.7311</v>
+      </c>
+      <c r="N130" t="inlineStr">
+        <is>
+          <t>baseline</t>
+        </is>
+      </c>
+    </row>
+    <row r="131">
+      <c r="A131" t="inlineStr">
+        <is>
+          <t>UltraLight</t>
+        </is>
+      </c>
+      <c r="B131" t="inlineStr">
+        <is>
+          <t>Run4</t>
+        </is>
+      </c>
+      <c r="C131" t="inlineStr">
+        <is>
+          <t>R4_2b_VIT4_LIGHTDETAIL48</t>
+        </is>
+      </c>
+      <c r="D131" t="inlineStr">
+        <is>
+          <t>SYSU-CD-256</t>
+        </is>
+      </c>
+      <c r="E131" s="2" t="n">
+        <v>80.87</v>
+      </c>
+      <c r="F131" s="2" t="n">
+        <v>83.81</v>
+      </c>
+      <c r="G131" s="2" t="n">
+        <v>91.81</v>
+      </c>
+      <c r="H131" s="2" t="n">
+        <v>82.31999999999999</v>
+      </c>
+      <c r="I131" s="2" t="n">
+        <v>69.95</v>
+      </c>
+      <c r="J131" s="2" t="n">
+        <v>76.98999999999999</v>
+      </c>
+      <c r="K131" s="2" t="n">
+        <v>5.533</v>
+      </c>
+      <c r="L131" s="2" t="n">
+        <v>3.556</v>
+      </c>
+      <c r="M131" s="2" t="n">
+        <v>10.9824</v>
+      </c>
+      <c r="N131" t="inlineStr">
+        <is>
+          <t>baseline</t>
+        </is>
+      </c>
+    </row>
+    <row r="132">
+      <c r="A132" t="inlineStr">
+        <is>
+          <t>UltraLight</t>
+        </is>
+      </c>
+      <c r="B132" t="inlineStr">
+        <is>
+          <t>Run4</t>
+        </is>
+      </c>
+      <c r="C132" t="inlineStr">
+        <is>
+          <t>R4_2d_PSD_DETAIL</t>
+        </is>
+      </c>
+      <c r="D132" t="inlineStr">
+        <is>
+          <t>SYSU-CD-256</t>
+        </is>
+      </c>
+      <c r="E132" s="2" t="n">
+        <v>79.78</v>
+      </c>
+      <c r="F132" s="2" t="n">
+        <v>84.39</v>
+      </c>
+      <c r="G132" s="2" t="n">
+        <v>91.75</v>
+      </c>
+      <c r="H132" s="2" t="n">
+        <v>82.02</v>
+      </c>
+      <c r="I132" s="2" t="n">
+        <v>69.52</v>
+      </c>
+      <c r="J132" s="2" t="n">
+        <v>76.68000000000001</v>
+      </c>
+      <c r="K132" s="2" t="n">
+        <v>5.491</v>
+      </c>
+      <c r="L132" s="2" t="n">
+        <v>3.514</v>
+      </c>
+      <c r="M132" s="2" t="n">
+        <v>11.5239</v>
+      </c>
+      <c r="N132" t="inlineStr">
+        <is>
+          <t>baseline</t>
+        </is>
+      </c>
+    </row>
+    <row r="133">
+      <c r="A133" t="inlineStr">
+        <is>
+          <t>baseline</t>
+        </is>
+      </c>
+      <c r="B133" t="inlineStr">
         <is>
           <t>Run1</t>
         </is>
       </c>
-      <c r="C124" t="inlineStr"/>
-      <c r="D124" t="inlineStr">
+      <c r="C133" t="inlineStr"/>
+      <c r="D133" t="inlineStr">
+        <is>
+          <t>CDD-CD-256</t>
+        </is>
+      </c>
+      <c r="E133" s="2" t="n">
+        <v>97.72</v>
+      </c>
+      <c r="F133" s="2" t="n">
+        <v>97.78</v>
+      </c>
+      <c r="G133" s="2" t="n">
+        <v>99.44</v>
+      </c>
+      <c r="H133" s="2" t="n">
+        <v>97.75</v>
+      </c>
+      <c r="I133" s="2" t="n">
+        <v>95.59999999999999</v>
+      </c>
+      <c r="J133" s="2" t="n">
+        <v>97.43000000000001</v>
+      </c>
+      <c r="K133" s="2" t="n">
+        <v>11.754</v>
+      </c>
+      <c r="L133" s="2" t="n">
+        <v>20.661</v>
+      </c>
+      <c r="M133" s="2" t="n">
+        <v>26.3246</v>
+      </c>
+      <c r="N133" t="inlineStr">
+        <is>
+          <t>baseline</t>
+        </is>
+      </c>
+    </row>
+    <row r="134">
+      <c r="A134" t="inlineStr">
+        <is>
+          <t>baseline</t>
+        </is>
+      </c>
+      <c r="B134" t="inlineStr">
+        <is>
+          <t>Run1</t>
+        </is>
+      </c>
+      <c r="C134" t="inlineStr"/>
+      <c r="D134" t="inlineStr">
+        <is>
+          <t>LEVIR-CD-256</t>
+        </is>
+      </c>
+      <c r="E134" s="2" t="n">
+        <v>91.56999999999999</v>
+      </c>
+      <c r="F134" s="2" t="n">
+        <v>92.33</v>
+      </c>
+      <c r="G134" s="2" t="n">
+        <v>99.18000000000001</v>
+      </c>
+      <c r="H134" s="2" t="n">
+        <v>91.95</v>
+      </c>
+      <c r="I134" s="2" t="n">
+        <v>85.09999999999999</v>
+      </c>
+      <c r="J134" s="2" t="n">
+        <v>91.52</v>
+      </c>
+      <c r="K134" s="2" t="n">
+        <v>11.754</v>
+      </c>
+      <c r="L134" s="2" t="n">
+        <v>20.661</v>
+      </c>
+      <c r="M134" s="2" t="n">
+        <v>26.3246</v>
+      </c>
+      <c r="N134" t="inlineStr">
+        <is>
+          <t>baseline</t>
+        </is>
+      </c>
+    </row>
+    <row r="135">
+      <c r="A135" t="inlineStr">
+        <is>
+          <t>baseline</t>
+        </is>
+      </c>
+      <c r="B135" t="inlineStr">
+        <is>
+          <t>Run1</t>
+        </is>
+      </c>
+      <c r="C135" t="inlineStr"/>
+      <c r="D135" t="inlineStr">
+        <is>
+          <t>SYSU-CD-256</t>
+        </is>
+      </c>
+      <c r="E135" s="2" t="n">
+        <v>80.77</v>
+      </c>
+      <c r="F135" s="2" t="n">
+        <v>84.27</v>
+      </c>
+      <c r="G135" s="2" t="n">
+        <v>91.91</v>
+      </c>
+      <c r="H135" s="2" t="n">
+        <v>82.48</v>
+      </c>
+      <c r="I135" s="2" t="n">
+        <v>70.19</v>
+      </c>
+      <c r="J135" s="2" t="n">
+        <v>77.23</v>
+      </c>
+      <c r="K135" s="2" t="n">
+        <v>11.754</v>
+      </c>
+      <c r="L135" s="2" t="n">
+        <v>20.661</v>
+      </c>
+      <c r="M135" s="2" t="n">
+        <v>26.3246</v>
+      </c>
+      <c r="N135" t="inlineStr">
+        <is>
+          <t>baseline</t>
+        </is>
+      </c>
+    </row>
+    <row r="136">
+      <c r="A136" t="inlineStr">
+        <is>
+          <t>baseline</t>
+        </is>
+      </c>
+      <c r="B136" t="inlineStr">
+        <is>
+          <t>Run1</t>
+        </is>
+      </c>
+      <c r="C136" t="inlineStr"/>
+      <c r="D136" t="inlineStr">
         <is>
           <t>WHU-CD-256</t>
         </is>
       </c>
-      <c r="E124" s="2" t="n">
+      <c r="E136" s="2" t="n">
         <v>93.62</v>
       </c>
-      <c r="F124" s="2" t="n">
+      <c r="F136" s="2" t="n">
         <v>96.09</v>
       </c>
-      <c r="G124" s="2" t="n">
+      <c r="G136" s="2" t="n">
         <v>99.59999999999999</v>
       </c>
-      <c r="H124" s="2" t="n">
+      <c r="H136" s="2" t="n">
         <v>94.84</v>
       </c>
-      <c r="I124" s="2" t="n">
+      <c r="I136" s="2" t="n">
         <v>90.18000000000001</v>
       </c>
-      <c r="J124" s="2" t="n">
+      <c r="J136" s="2" t="n">
         <v>94.63</v>
       </c>
-      <c r="K124" s="2" t="n">
+      <c r="K136" s="2" t="n">
         <v>11.754</v>
       </c>
-      <c r="L124" s="2" t="n">
+      <c r="L136" s="2" t="n">
         <v>20.661</v>
       </c>
-      <c r="M124" s="2" t="n">
+      <c r="M136" s="2" t="n">
         <v>26.3246</v>
       </c>
-      <c r="N124" t="inlineStr">
+      <c r="N136" t="inlineStr">
         <is>
           <t>baseline</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:N124"/>
+  <autoFilter ref="A1:N136"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Record all twelve Run6 test results and source snapshots
</commit_message>
<xml_diff>
--- a/docs/experiment_metrics.xlsx
+++ b/docs/experiment_metrics.xlsx
@@ -10,7 +10,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="metrics" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'metrics'!$A$1:$N$136</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'metrics'!$A$1:$N$148</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -420,7 +420,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N136"/>
+  <dimension ref="A1:N148"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -6762,17 +6762,17 @@
     <row r="120">
       <c r="A120" t="inlineStr">
         <is>
-          <t>STR-Fusion</t>
+          <t>CASA</t>
         </is>
       </c>
       <c r="B120" t="inlineStr">
         <is>
-          <t>Run2_TASS</t>
+          <t>Run6</t>
         </is>
       </c>
       <c r="C120" t="inlineStr">
         <is>
-          <t>C0_TOKEN</t>
+          <t>M0_CTRL</t>
         </is>
       </c>
       <c r="D120" t="inlineStr">
@@ -6781,52 +6781,50 @@
         </is>
       </c>
       <c r="E120" s="2" t="n">
-        <v>93.13</v>
+        <v>97.5</v>
       </c>
       <c r="F120" s="2" t="n">
-        <v>95.16</v>
+        <v>97.34999999999999</v>
       </c>
       <c r="G120" s="2" t="n">
-        <v>98.56999999999999</v>
+        <v>99.36</v>
       </c>
       <c r="H120" s="2" t="n">
-        <v>94.13</v>
+        <v>97.43000000000001</v>
       </c>
       <c r="I120" s="2" t="n">
-        <v>88.91</v>
+        <v>94.98999999999999</v>
       </c>
       <c r="J120" s="2" t="n">
-        <v>93.31999999999999</v>
+        <v>97.06999999999999</v>
       </c>
       <c r="K120" s="2" t="n">
-        <v>2.596</v>
+        <v>3.016737</v>
       </c>
       <c r="L120" s="2" t="n">
-        <v>0.62</v>
-      </c>
-      <c r="M120" s="2" t="n">
-        <v>2.2136</v>
-      </c>
+        <v>3.100404</v>
+      </c>
+      <c r="M120" s="2" t="n"/>
       <c r="N120" t="inlineStr">
         <is>
-          <t>str_tass</t>
+          <t>casa_none</t>
         </is>
       </c>
     </row>
     <row r="121">
       <c r="A121" t="inlineStr">
         <is>
-          <t>STR-Fusion</t>
+          <t>CASA</t>
         </is>
       </c>
       <c r="B121" t="inlineStr">
         <is>
-          <t>Run2_TASS</t>
+          <t>Run6</t>
         </is>
       </c>
       <c r="C121" t="inlineStr">
         <is>
-          <t>C0_TOKEN</t>
+          <t>M0_CTRL</t>
         </is>
       </c>
       <c r="D121" t="inlineStr">
@@ -6835,52 +6833,50 @@
         </is>
       </c>
       <c r="E121" s="2" t="n">
-        <v>86.37</v>
+        <v>90.69</v>
       </c>
       <c r="F121" s="2" t="n">
-        <v>89.25</v>
+        <v>92.43000000000001</v>
       </c>
       <c r="G121" s="2" t="n">
-        <v>98.78</v>
+        <v>99.15000000000001</v>
       </c>
       <c r="H121" s="2" t="n">
-        <v>87.79000000000001</v>
+        <v>91.55</v>
       </c>
       <c r="I121" s="2" t="n">
-        <v>78.23999999999999</v>
+        <v>84.42</v>
       </c>
       <c r="J121" s="2" t="n">
-        <v>87.14</v>
+        <v>91.09999999999999</v>
       </c>
       <c r="K121" s="2" t="n">
-        <v>2.596</v>
+        <v>3.016737</v>
       </c>
       <c r="L121" s="2" t="n">
-        <v>0.62</v>
-      </c>
-      <c r="M121" s="2" t="n">
-        <v>2.2136</v>
-      </c>
+        <v>3.100404</v>
+      </c>
+      <c r="M121" s="2" t="n"/>
       <c r="N121" t="inlineStr">
         <is>
-          <t>str_tass</t>
+          <t>casa_none</t>
         </is>
       </c>
     </row>
     <row r="122">
       <c r="A122" t="inlineStr">
         <is>
-          <t>STR-Fusion</t>
+          <t>CASA</t>
         </is>
       </c>
       <c r="B122" t="inlineStr">
         <is>
-          <t>Run2_TASS</t>
+          <t>Run6</t>
         </is>
       </c>
       <c r="C122" t="inlineStr">
         <is>
-          <t>C0_TOKEN</t>
+          <t>M0_CTRL</t>
         </is>
       </c>
       <c r="D122" t="inlineStr">
@@ -6889,52 +6885,50 @@
         </is>
       </c>
       <c r="E122" s="2" t="n">
-        <v>79.93000000000001</v>
+        <v>82.58</v>
       </c>
       <c r="F122" s="2" t="n">
-        <v>84.5</v>
+        <v>82.25</v>
       </c>
       <c r="G122" s="2" t="n">
-        <v>91.81</v>
+        <v>91.69</v>
       </c>
       <c r="H122" s="2" t="n">
-        <v>82.15000000000001</v>
+        <v>82.42</v>
       </c>
       <c r="I122" s="2" t="n">
-        <v>69.70999999999999</v>
+        <v>70.09</v>
       </c>
       <c r="J122" s="2" t="n">
-        <v>76.84</v>
+        <v>76.98</v>
       </c>
       <c r="K122" s="2" t="n">
-        <v>2.596</v>
+        <v>3.016737</v>
       </c>
       <c r="L122" s="2" t="n">
-        <v>0.62</v>
-      </c>
-      <c r="M122" s="2" t="n">
-        <v>2.2136</v>
-      </c>
+        <v>3.100404</v>
+      </c>
+      <c r="M122" s="2" t="n"/>
       <c r="N122" t="inlineStr">
         <is>
-          <t>str_tass</t>
+          <t>casa_none</t>
         </is>
       </c>
     </row>
     <row r="123">
       <c r="A123" t="inlineStr">
         <is>
-          <t>STR-Fusion</t>
+          <t>CASA</t>
         </is>
       </c>
       <c r="B123" t="inlineStr">
         <is>
-          <t>Run2_TASS</t>
+          <t>Run6</t>
         </is>
       </c>
       <c r="C123" t="inlineStr">
         <is>
-          <t>C0_TOKEN</t>
+          <t>M0_CTRL</t>
         </is>
       </c>
       <c r="D123" t="inlineStr">
@@ -6943,52 +6937,50 @@
         </is>
       </c>
       <c r="E123" s="2" t="n">
-        <v>90.16</v>
+        <v>92.31</v>
       </c>
       <c r="F123" s="2" t="n">
-        <v>93.97</v>
+        <v>94.59999999999999</v>
       </c>
       <c r="G123" s="2" t="n">
-        <v>99.38</v>
+        <v>99.48999999999999</v>
       </c>
       <c r="H123" s="2" t="n">
-        <v>92.02</v>
+        <v>93.44</v>
       </c>
       <c r="I123" s="2" t="n">
-        <v>85.23</v>
+        <v>87.69</v>
       </c>
       <c r="J123" s="2" t="n">
-        <v>91.7</v>
+        <v>93.17</v>
       </c>
       <c r="K123" s="2" t="n">
-        <v>2.596</v>
+        <v>3.016737</v>
       </c>
       <c r="L123" s="2" t="n">
-        <v>0.62</v>
-      </c>
-      <c r="M123" s="2" t="n">
-        <v>2.2136</v>
-      </c>
+        <v>3.100404</v>
+      </c>
+      <c r="M123" s="2" t="n"/>
       <c r="N123" t="inlineStr">
         <is>
-          <t>str_tass</t>
+          <t>casa_none</t>
         </is>
       </c>
     </row>
     <row r="124">
       <c r="A124" t="inlineStr">
         <is>
-          <t>STR-Fusion</t>
+          <t>CASA</t>
         </is>
       </c>
       <c r="B124" t="inlineStr">
         <is>
-          <t>Run2_TASS</t>
+          <t>Run6</t>
         </is>
       </c>
       <c r="C124" t="inlineStr">
         <is>
-          <t>M1_TASS</t>
+          <t>M1_HYPER_QKV</t>
         </is>
       </c>
       <c r="D124" t="inlineStr">
@@ -6997,52 +6989,50 @@
         </is>
       </c>
       <c r="E124" s="2" t="n">
-        <v>94.7</v>
+        <v>97.53</v>
       </c>
       <c r="F124" s="2" t="n">
-        <v>96.13</v>
+        <v>97.38</v>
       </c>
       <c r="G124" s="2" t="n">
-        <v>98.88</v>
+        <v>99.37</v>
       </c>
       <c r="H124" s="2" t="n">
-        <v>95.41</v>
+        <v>97.45</v>
       </c>
       <c r="I124" s="2" t="n">
-        <v>91.22</v>
+        <v>95.03</v>
       </c>
       <c r="J124" s="2" t="n">
-        <v>94.77</v>
+        <v>97.09</v>
       </c>
       <c r="K124" s="2" t="n">
-        <v>3.455</v>
+        <v>3.050665</v>
       </c>
       <c r="L124" s="2" t="n">
-        <v>1.478</v>
-      </c>
-      <c r="M124" s="2" t="n">
-        <v>3.5459</v>
-      </c>
+        <v>3.134332</v>
+      </c>
+      <c r="M124" s="2" t="n"/>
       <c r="N124" t="inlineStr">
         <is>
-          <t>str_tass</t>
+          <t>casa_hyperbolic</t>
         </is>
       </c>
     </row>
     <row r="125">
       <c r="A125" t="inlineStr">
         <is>
-          <t>STR-Fusion</t>
+          <t>CASA</t>
         </is>
       </c>
       <c r="B125" t="inlineStr">
         <is>
-          <t>Run2_TASS</t>
+          <t>Run6</t>
         </is>
       </c>
       <c r="C125" t="inlineStr">
         <is>
-          <t>M1_TASS</t>
+          <t>M1_HYPER_QKV</t>
         </is>
       </c>
       <c r="D125" t="inlineStr">
@@ -7051,52 +7041,50 @@
         </is>
       </c>
       <c r="E125" s="2" t="n">
-        <v>88.42</v>
+        <v>90.34999999999999</v>
       </c>
       <c r="F125" s="2" t="n">
-        <v>91.97</v>
+        <v>91.77</v>
       </c>
       <c r="G125" s="2" t="n">
-        <v>99.02</v>
+        <v>99.09999999999999</v>
       </c>
       <c r="H125" s="2" t="n">
-        <v>90.16</v>
+        <v>91.05</v>
       </c>
       <c r="I125" s="2" t="n">
-        <v>82.08</v>
+        <v>83.56999999999999</v>
       </c>
       <c r="J125" s="2" t="n">
-        <v>89.64</v>
+        <v>90.58</v>
       </c>
       <c r="K125" s="2" t="n">
-        <v>3.455</v>
+        <v>3.050665</v>
       </c>
       <c r="L125" s="2" t="n">
-        <v>1.478</v>
-      </c>
-      <c r="M125" s="2" t="n">
-        <v>3.5459</v>
-      </c>
+        <v>3.134332</v>
+      </c>
+      <c r="M125" s="2" t="n"/>
       <c r="N125" t="inlineStr">
         <is>
-          <t>str_tass</t>
+          <t>casa_hyperbolic</t>
         </is>
       </c>
     </row>
     <row r="126">
       <c r="A126" t="inlineStr">
         <is>
-          <t>STR-Fusion</t>
+          <t>CASA</t>
         </is>
       </c>
       <c r="B126" t="inlineStr">
         <is>
-          <t>Run2_TASS</t>
+          <t>Run6</t>
         </is>
       </c>
       <c r="C126" t="inlineStr">
         <is>
-          <t>M1_TASS</t>
+          <t>M1_HYPER_QKV</t>
         </is>
       </c>
       <c r="D126" t="inlineStr">
@@ -7105,52 +7093,50 @@
         </is>
       </c>
       <c r="E126" s="2" t="n">
-        <v>78.73</v>
+        <v>76.31999999999999</v>
       </c>
       <c r="F126" s="2" t="n">
-        <v>84.98</v>
+        <v>85.91</v>
       </c>
       <c r="G126" s="2" t="n">
-        <v>91.7</v>
+        <v>91.45999999999999</v>
       </c>
       <c r="H126" s="2" t="n">
-        <v>81.73999999999999</v>
+        <v>80.83</v>
       </c>
       <c r="I126" s="2" t="n">
-        <v>69.11</v>
+        <v>67.83</v>
       </c>
       <c r="J126" s="2" t="n">
-        <v>76.38</v>
+        <v>75.37</v>
       </c>
       <c r="K126" s="2" t="n">
-        <v>3.455</v>
+        <v>3.050665</v>
       </c>
       <c r="L126" s="2" t="n">
-        <v>1.478</v>
-      </c>
-      <c r="M126" s="2" t="n">
-        <v>3.5459</v>
-      </c>
+        <v>3.134332</v>
+      </c>
+      <c r="M126" s="2" t="n"/>
       <c r="N126" t="inlineStr">
         <is>
-          <t>str_tass</t>
+          <t>casa_hyperbolic</t>
         </is>
       </c>
     </row>
     <row r="127">
       <c r="A127" t="inlineStr">
         <is>
-          <t>STR-Fusion</t>
+          <t>CASA</t>
         </is>
       </c>
       <c r="B127" t="inlineStr">
         <is>
-          <t>Run2_TASS</t>
+          <t>Run6</t>
         </is>
       </c>
       <c r="C127" t="inlineStr">
         <is>
-          <t>M1_TASS</t>
+          <t>M1_HYPER_QKV</t>
         </is>
       </c>
       <c r="D127" t="inlineStr">
@@ -7159,160 +7145,154 @@
         </is>
       </c>
       <c r="E127" s="2" t="n">
-        <v>91.64</v>
+        <v>93.55</v>
       </c>
       <c r="F127" s="2" t="n">
-        <v>94.81999999999999</v>
+        <v>95.95</v>
       </c>
       <c r="G127" s="2" t="n">
-        <v>99.47</v>
+        <v>99.59</v>
       </c>
       <c r="H127" s="2" t="n">
-        <v>93.2</v>
+        <v>94.73</v>
       </c>
       <c r="I127" s="2" t="n">
-        <v>87.27</v>
+        <v>89.98999999999999</v>
       </c>
       <c r="J127" s="2" t="n">
-        <v>92.93000000000001</v>
+        <v>94.52</v>
       </c>
       <c r="K127" s="2" t="n">
-        <v>3.455</v>
+        <v>3.050665</v>
       </c>
       <c r="L127" s="2" t="n">
-        <v>1.478</v>
-      </c>
-      <c r="M127" s="2" t="n">
-        <v>3.5459</v>
-      </c>
+        <v>3.134332</v>
+      </c>
+      <c r="M127" s="2" t="n"/>
       <c r="N127" t="inlineStr">
         <is>
-          <t>str_tass</t>
+          <t>casa_hyperbolic</t>
         </is>
       </c>
     </row>
     <row r="128">
       <c r="A128" t="inlineStr">
         <is>
-          <t>UltraLight</t>
+          <t>CASA</t>
         </is>
       </c>
       <c r="B128" t="inlineStr">
         <is>
-          <t>Run4</t>
+          <t>Run6</t>
         </is>
       </c>
       <c r="C128" t="inlineStr">
         <is>
-          <t>R4_0_A0_FULL12_FROZEN</t>
+          <t>M2_CA_QKV</t>
         </is>
       </c>
       <c r="D128" t="inlineStr">
         <is>
-          <t>SYSU-CD-256</t>
+          <t>CDD-CD-256</t>
         </is>
       </c>
       <c r="E128" s="2" t="n">
-        <v>82.42</v>
+        <v>97.45</v>
       </c>
       <c r="F128" s="2" t="n">
-        <v>83.87</v>
+        <v>97.48999999999999</v>
       </c>
       <c r="G128" s="2" t="n">
-        <v>92.12</v>
+        <v>99.38</v>
       </c>
       <c r="H128" s="2" t="n">
-        <v>83.14</v>
+        <v>97.47</v>
       </c>
       <c r="I128" s="2" t="n">
-        <v>71.14</v>
+        <v>95.06999999999999</v>
       </c>
       <c r="J128" s="2" t="n">
-        <v>77.98999999999999</v>
+        <v>97.12</v>
       </c>
       <c r="K128" s="2" t="n">
-        <v>11.754</v>
+        <v>3.067561</v>
       </c>
       <c r="L128" s="2" t="n">
-        <v>15.125</v>
-      </c>
-      <c r="M128" s="2" t="n">
-        <v>26.3246</v>
-      </c>
+        <v>3.151228</v>
+      </c>
+      <c r="M128" s="2" t="n"/>
       <c r="N128" t="inlineStr">
         <is>
-          <t>baseline</t>
+          <t>casa_qkv</t>
         </is>
       </c>
     </row>
     <row r="129">
       <c r="A129" t="inlineStr">
         <is>
-          <t>UltraLight</t>
+          <t>CASA</t>
         </is>
       </c>
       <c r="B129" t="inlineStr">
         <is>
-          <t>Run4</t>
+          <t>Run6</t>
         </is>
       </c>
       <c r="C129" t="inlineStr">
         <is>
-          <t>R4_1_VIT4_OLDHEAD</t>
+          <t>M2_CA_QKV</t>
         </is>
       </c>
       <c r="D129" t="inlineStr">
         <is>
-          <t>SYSU-CD-256</t>
+          <t>LEVIR-CD-256</t>
         </is>
       </c>
       <c r="E129" s="2" t="n">
-        <v>82.15000000000001</v>
+        <v>90.67</v>
       </c>
       <c r="F129" s="2" t="n">
-        <v>83.40000000000001</v>
+        <v>92.58</v>
       </c>
       <c r="G129" s="2" t="n">
-        <v>91.94</v>
+        <v>99.15000000000001</v>
       </c>
       <c r="H129" s="2" t="n">
-        <v>82.77</v>
+        <v>91.62</v>
       </c>
       <c r="I129" s="2" t="n">
-        <v>70.61</v>
+        <v>84.53</v>
       </c>
       <c r="J129" s="2" t="n">
-        <v>77.51000000000001</v>
+        <v>91.17</v>
       </c>
       <c r="K129" s="2" t="n">
-        <v>8.195</v>
+        <v>3.067561</v>
       </c>
       <c r="L129" s="2" t="n">
-        <v>15.125</v>
-      </c>
-      <c r="M129" s="2" t="n">
-        <v>24.1021</v>
-      </c>
+        <v>3.151228</v>
+      </c>
+      <c r="M129" s="2" t="n"/>
       <c r="N129" t="inlineStr">
         <is>
-          <t>baseline</t>
+          <t>casa_qkv</t>
         </is>
       </c>
     </row>
     <row r="130">
       <c r="A130" t="inlineStr">
         <is>
-          <t>UltraLight</t>
+          <t>CASA</t>
         </is>
       </c>
       <c r="B130" t="inlineStr">
         <is>
-          <t>Run4</t>
+          <t>Run6</t>
         </is>
       </c>
       <c r="C130" t="inlineStr">
         <is>
-          <t>R4_2_VIT4_LIGHTDETAIL</t>
+          <t>M2_CA_QKV</t>
         </is>
       </c>
       <c r="D130" t="inlineStr">
@@ -7321,348 +7301,992 @@
         </is>
       </c>
       <c r="E130" s="2" t="n">
-        <v>79.94</v>
+        <v>77.90000000000001</v>
       </c>
       <c r="F130" s="2" t="n">
-        <v>84.79000000000001</v>
+        <v>87.42</v>
       </c>
       <c r="G130" s="2" t="n">
-        <v>91.89</v>
+        <v>92.15000000000001</v>
       </c>
       <c r="H130" s="2" t="n">
-        <v>82.3</v>
+        <v>82.39</v>
       </c>
       <c r="I130" s="2" t="n">
-        <v>69.92</v>
+        <v>70.05</v>
       </c>
       <c r="J130" s="2" t="n">
-        <v>77.04000000000001</v>
+        <v>77.36</v>
       </c>
       <c r="K130" s="2" t="n">
-        <v>5.492</v>
+        <v>3.067561</v>
       </c>
       <c r="L130" s="2" t="n">
-        <v>3.515</v>
-      </c>
-      <c r="M130" s="2" t="n">
-        <v>10.7311</v>
-      </c>
+        <v>3.151228</v>
+      </c>
+      <c r="M130" s="2" t="n"/>
       <c r="N130" t="inlineStr">
         <is>
-          <t>baseline</t>
+          <t>casa_qkv</t>
         </is>
       </c>
     </row>
     <row r="131">
       <c r="A131" t="inlineStr">
         <is>
-          <t>UltraLight</t>
+          <t>CASA</t>
         </is>
       </c>
       <c r="B131" t="inlineStr">
         <is>
-          <t>Run4</t>
+          <t>Run6</t>
         </is>
       </c>
       <c r="C131" t="inlineStr">
         <is>
-          <t>R4_2b_VIT4_LIGHTDETAIL48</t>
+          <t>M2_CA_QKV</t>
         </is>
       </c>
       <c r="D131" t="inlineStr">
         <is>
-          <t>SYSU-CD-256</t>
+          <t>WHU-CD-256</t>
         </is>
       </c>
       <c r="E131" s="2" t="n">
-        <v>80.87</v>
+        <v>92.61</v>
       </c>
       <c r="F131" s="2" t="n">
-        <v>83.81</v>
+        <v>95.77</v>
       </c>
       <c r="G131" s="2" t="n">
-        <v>91.81</v>
+        <v>99.54000000000001</v>
       </c>
       <c r="H131" s="2" t="n">
-        <v>82.31999999999999</v>
+        <v>94.16</v>
       </c>
       <c r="I131" s="2" t="n">
-        <v>69.95</v>
+        <v>88.97</v>
       </c>
       <c r="J131" s="2" t="n">
-        <v>76.98999999999999</v>
+        <v>93.93000000000001</v>
       </c>
       <c r="K131" s="2" t="n">
-        <v>5.533</v>
+        <v>3.067561</v>
       </c>
       <c r="L131" s="2" t="n">
-        <v>3.556</v>
-      </c>
-      <c r="M131" s="2" t="n">
-        <v>10.9824</v>
-      </c>
+        <v>3.151228</v>
+      </c>
+      <c r="M131" s="2" t="n"/>
       <c r="N131" t="inlineStr">
         <is>
-          <t>baseline</t>
+          <t>casa_qkv</t>
         </is>
       </c>
     </row>
     <row r="132">
       <c r="A132" t="inlineStr">
         <is>
-          <t>UltraLight</t>
+          <t>STR-Fusion</t>
         </is>
       </c>
       <c r="B132" t="inlineStr">
         <is>
-          <t>Run4</t>
+          <t>Run2_TASS</t>
         </is>
       </c>
       <c r="C132" t="inlineStr">
         <is>
-          <t>R4_2d_PSD_DETAIL</t>
+          <t>C0_TOKEN</t>
         </is>
       </c>
       <c r="D132" t="inlineStr">
         <is>
-          <t>SYSU-CD-256</t>
+          <t>CDD-CD-256</t>
         </is>
       </c>
       <c r="E132" s="2" t="n">
-        <v>79.78</v>
+        <v>93.13</v>
       </c>
       <c r="F132" s="2" t="n">
-        <v>84.39</v>
+        <v>95.16</v>
       </c>
       <c r="G132" s="2" t="n">
-        <v>91.75</v>
+        <v>98.56999999999999</v>
       </c>
       <c r="H132" s="2" t="n">
-        <v>82.02</v>
+        <v>94.13</v>
       </c>
       <c r="I132" s="2" t="n">
-        <v>69.52</v>
+        <v>88.91</v>
       </c>
       <c r="J132" s="2" t="n">
-        <v>76.68000000000001</v>
+        <v>93.31999999999999</v>
       </c>
       <c r="K132" s="2" t="n">
-        <v>5.491</v>
+        <v>2.596</v>
       </c>
       <c r="L132" s="2" t="n">
-        <v>3.514</v>
+        <v>0.62</v>
       </c>
       <c r="M132" s="2" t="n">
-        <v>11.5239</v>
+        <v>2.2136</v>
       </c>
       <c r="N132" t="inlineStr">
         <is>
-          <t>baseline</t>
+          <t>str_tass</t>
         </is>
       </c>
     </row>
     <row r="133">
       <c r="A133" t="inlineStr">
         <is>
-          <t>baseline</t>
+          <t>STR-Fusion</t>
         </is>
       </c>
       <c r="B133" t="inlineStr">
         <is>
-          <t>Run1</t>
-        </is>
-      </c>
-      <c r="C133" t="inlineStr"/>
+          <t>Run2_TASS</t>
+        </is>
+      </c>
+      <c r="C133" t="inlineStr">
+        <is>
+          <t>C0_TOKEN</t>
+        </is>
+      </c>
       <c r="D133" t="inlineStr">
         <is>
-          <t>CDD-CD-256</t>
+          <t>LEVIR-CD-256</t>
         </is>
       </c>
       <c r="E133" s="2" t="n">
-        <v>97.72</v>
+        <v>86.37</v>
       </c>
       <c r="F133" s="2" t="n">
-        <v>97.78</v>
+        <v>89.25</v>
       </c>
       <c r="G133" s="2" t="n">
-        <v>99.44</v>
+        <v>98.78</v>
       </c>
       <c r="H133" s="2" t="n">
-        <v>97.75</v>
+        <v>87.79000000000001</v>
       </c>
       <c r="I133" s="2" t="n">
-        <v>95.59999999999999</v>
+        <v>78.23999999999999</v>
       </c>
       <c r="J133" s="2" t="n">
-        <v>97.43000000000001</v>
+        <v>87.14</v>
       </c>
       <c r="K133" s="2" t="n">
-        <v>11.754</v>
+        <v>2.596</v>
       </c>
       <c r="L133" s="2" t="n">
-        <v>20.661</v>
+        <v>0.62</v>
       </c>
       <c r="M133" s="2" t="n">
-        <v>26.3246</v>
+        <v>2.2136</v>
       </c>
       <c r="N133" t="inlineStr">
         <is>
-          <t>baseline</t>
+          <t>str_tass</t>
         </is>
       </c>
     </row>
     <row r="134">
       <c r="A134" t="inlineStr">
         <is>
-          <t>baseline</t>
+          <t>STR-Fusion</t>
         </is>
       </c>
       <c r="B134" t="inlineStr">
         <is>
-          <t>Run1</t>
-        </is>
-      </c>
-      <c r="C134" t="inlineStr"/>
+          <t>Run2_TASS</t>
+        </is>
+      </c>
+      <c r="C134" t="inlineStr">
+        <is>
+          <t>C0_TOKEN</t>
+        </is>
+      </c>
       <c r="D134" t="inlineStr">
         <is>
-          <t>LEVIR-CD-256</t>
+          <t>SYSU-CD-256</t>
         </is>
       </c>
       <c r="E134" s="2" t="n">
-        <v>91.56999999999999</v>
+        <v>79.93000000000001</v>
       </c>
       <c r="F134" s="2" t="n">
-        <v>92.33</v>
+        <v>84.5</v>
       </c>
       <c r="G134" s="2" t="n">
-        <v>99.18000000000001</v>
+        <v>91.81</v>
       </c>
       <c r="H134" s="2" t="n">
-        <v>91.95</v>
+        <v>82.15000000000001</v>
       </c>
       <c r="I134" s="2" t="n">
-        <v>85.09999999999999</v>
+        <v>69.70999999999999</v>
       </c>
       <c r="J134" s="2" t="n">
-        <v>91.52</v>
+        <v>76.84</v>
       </c>
       <c r="K134" s="2" t="n">
-        <v>11.754</v>
+        <v>2.596</v>
       </c>
       <c r="L134" s="2" t="n">
-        <v>20.661</v>
+        <v>0.62</v>
       </c>
       <c r="M134" s="2" t="n">
-        <v>26.3246</v>
+        <v>2.2136</v>
       </c>
       <c r="N134" t="inlineStr">
         <is>
-          <t>baseline</t>
+          <t>str_tass</t>
         </is>
       </c>
     </row>
     <row r="135">
       <c r="A135" t="inlineStr">
         <is>
-          <t>baseline</t>
+          <t>STR-Fusion</t>
         </is>
       </c>
       <c r="B135" t="inlineStr">
         <is>
-          <t>Run1</t>
-        </is>
-      </c>
-      <c r="C135" t="inlineStr"/>
+          <t>Run2_TASS</t>
+        </is>
+      </c>
+      <c r="C135" t="inlineStr">
+        <is>
+          <t>C0_TOKEN</t>
+        </is>
+      </c>
       <c r="D135" t="inlineStr">
         <is>
-          <t>SYSU-CD-256</t>
+          <t>WHU-CD-256</t>
         </is>
       </c>
       <c r="E135" s="2" t="n">
-        <v>80.77</v>
+        <v>90.16</v>
       </c>
       <c r="F135" s="2" t="n">
-        <v>84.27</v>
+        <v>93.97</v>
       </c>
       <c r="G135" s="2" t="n">
-        <v>91.91</v>
+        <v>99.38</v>
       </c>
       <c r="H135" s="2" t="n">
-        <v>82.48</v>
+        <v>92.02</v>
       </c>
       <c r="I135" s="2" t="n">
-        <v>70.19</v>
+        <v>85.23</v>
       </c>
       <c r="J135" s="2" t="n">
-        <v>77.23</v>
+        <v>91.7</v>
       </c>
       <c r="K135" s="2" t="n">
-        <v>11.754</v>
+        <v>2.596</v>
       </c>
       <c r="L135" s="2" t="n">
-        <v>20.661</v>
+        <v>0.62</v>
       </c>
       <c r="M135" s="2" t="n">
-        <v>26.3246</v>
+        <v>2.2136</v>
       </c>
       <c r="N135" t="inlineStr">
         <is>
-          <t>baseline</t>
+          <t>str_tass</t>
         </is>
       </c>
     </row>
     <row r="136">
       <c r="A136" t="inlineStr">
         <is>
+          <t>STR-Fusion</t>
+        </is>
+      </c>
+      <c r="B136" t="inlineStr">
+        <is>
+          <t>Run2_TASS</t>
+        </is>
+      </c>
+      <c r="C136" t="inlineStr">
+        <is>
+          <t>M1_TASS</t>
+        </is>
+      </c>
+      <c r="D136" t="inlineStr">
+        <is>
+          <t>CDD-CD-256</t>
+        </is>
+      </c>
+      <c r="E136" s="2" t="n">
+        <v>94.7</v>
+      </c>
+      <c r="F136" s="2" t="n">
+        <v>96.13</v>
+      </c>
+      <c r="G136" s="2" t="n">
+        <v>98.88</v>
+      </c>
+      <c r="H136" s="2" t="n">
+        <v>95.41</v>
+      </c>
+      <c r="I136" s="2" t="n">
+        <v>91.22</v>
+      </c>
+      <c r="J136" s="2" t="n">
+        <v>94.77</v>
+      </c>
+      <c r="K136" s="2" t="n">
+        <v>3.455</v>
+      </c>
+      <c r="L136" s="2" t="n">
+        <v>1.478</v>
+      </c>
+      <c r="M136" s="2" t="n">
+        <v>3.5459</v>
+      </c>
+      <c r="N136" t="inlineStr">
+        <is>
+          <t>str_tass</t>
+        </is>
+      </c>
+    </row>
+    <row r="137">
+      <c r="A137" t="inlineStr">
+        <is>
+          <t>STR-Fusion</t>
+        </is>
+      </c>
+      <c r="B137" t="inlineStr">
+        <is>
+          <t>Run2_TASS</t>
+        </is>
+      </c>
+      <c r="C137" t="inlineStr">
+        <is>
+          <t>M1_TASS</t>
+        </is>
+      </c>
+      <c r="D137" t="inlineStr">
+        <is>
+          <t>LEVIR-CD-256</t>
+        </is>
+      </c>
+      <c r="E137" s="2" t="n">
+        <v>88.42</v>
+      </c>
+      <c r="F137" s="2" t="n">
+        <v>91.97</v>
+      </c>
+      <c r="G137" s="2" t="n">
+        <v>99.02</v>
+      </c>
+      <c r="H137" s="2" t="n">
+        <v>90.16</v>
+      </c>
+      <c r="I137" s="2" t="n">
+        <v>82.08</v>
+      </c>
+      <c r="J137" s="2" t="n">
+        <v>89.64</v>
+      </c>
+      <c r="K137" s="2" t="n">
+        <v>3.455</v>
+      </c>
+      <c r="L137" s="2" t="n">
+        <v>1.478</v>
+      </c>
+      <c r="M137" s="2" t="n">
+        <v>3.5459</v>
+      </c>
+      <c r="N137" t="inlineStr">
+        <is>
+          <t>str_tass</t>
+        </is>
+      </c>
+    </row>
+    <row r="138">
+      <c r="A138" t="inlineStr">
+        <is>
+          <t>STR-Fusion</t>
+        </is>
+      </c>
+      <c r="B138" t="inlineStr">
+        <is>
+          <t>Run2_TASS</t>
+        </is>
+      </c>
+      <c r="C138" t="inlineStr">
+        <is>
+          <t>M1_TASS</t>
+        </is>
+      </c>
+      <c r="D138" t="inlineStr">
+        <is>
+          <t>SYSU-CD-256</t>
+        </is>
+      </c>
+      <c r="E138" s="2" t="n">
+        <v>78.73</v>
+      </c>
+      <c r="F138" s="2" t="n">
+        <v>84.98</v>
+      </c>
+      <c r="G138" s="2" t="n">
+        <v>91.7</v>
+      </c>
+      <c r="H138" s="2" t="n">
+        <v>81.73999999999999</v>
+      </c>
+      <c r="I138" s="2" t="n">
+        <v>69.11</v>
+      </c>
+      <c r="J138" s="2" t="n">
+        <v>76.38</v>
+      </c>
+      <c r="K138" s="2" t="n">
+        <v>3.455</v>
+      </c>
+      <c r="L138" s="2" t="n">
+        <v>1.478</v>
+      </c>
+      <c r="M138" s="2" t="n">
+        <v>3.5459</v>
+      </c>
+      <c r="N138" t="inlineStr">
+        <is>
+          <t>str_tass</t>
+        </is>
+      </c>
+    </row>
+    <row r="139">
+      <c r="A139" t="inlineStr">
+        <is>
+          <t>STR-Fusion</t>
+        </is>
+      </c>
+      <c r="B139" t="inlineStr">
+        <is>
+          <t>Run2_TASS</t>
+        </is>
+      </c>
+      <c r="C139" t="inlineStr">
+        <is>
+          <t>M1_TASS</t>
+        </is>
+      </c>
+      <c r="D139" t="inlineStr">
+        <is>
+          <t>WHU-CD-256</t>
+        </is>
+      </c>
+      <c r="E139" s="2" t="n">
+        <v>91.64</v>
+      </c>
+      <c r="F139" s="2" t="n">
+        <v>94.81999999999999</v>
+      </c>
+      <c r="G139" s="2" t="n">
+        <v>99.47</v>
+      </c>
+      <c r="H139" s="2" t="n">
+        <v>93.2</v>
+      </c>
+      <c r="I139" s="2" t="n">
+        <v>87.27</v>
+      </c>
+      <c r="J139" s="2" t="n">
+        <v>92.93000000000001</v>
+      </c>
+      <c r="K139" s="2" t="n">
+        <v>3.455</v>
+      </c>
+      <c r="L139" s="2" t="n">
+        <v>1.478</v>
+      </c>
+      <c r="M139" s="2" t="n">
+        <v>3.5459</v>
+      </c>
+      <c r="N139" t="inlineStr">
+        <is>
+          <t>str_tass</t>
+        </is>
+      </c>
+    </row>
+    <row r="140">
+      <c r="A140" t="inlineStr">
+        <is>
+          <t>UltraLight</t>
+        </is>
+      </c>
+      <c r="B140" t="inlineStr">
+        <is>
+          <t>Run4</t>
+        </is>
+      </c>
+      <c r="C140" t="inlineStr">
+        <is>
+          <t>R4_0_A0_FULL12_FROZEN</t>
+        </is>
+      </c>
+      <c r="D140" t="inlineStr">
+        <is>
+          <t>SYSU-CD-256</t>
+        </is>
+      </c>
+      <c r="E140" s="2" t="n">
+        <v>82.42</v>
+      </c>
+      <c r="F140" s="2" t="n">
+        <v>83.87</v>
+      </c>
+      <c r="G140" s="2" t="n">
+        <v>92.12</v>
+      </c>
+      <c r="H140" s="2" t="n">
+        <v>83.14</v>
+      </c>
+      <c r="I140" s="2" t="n">
+        <v>71.14</v>
+      </c>
+      <c r="J140" s="2" t="n">
+        <v>77.98999999999999</v>
+      </c>
+      <c r="K140" s="2" t="n">
+        <v>11.754</v>
+      </c>
+      <c r="L140" s="2" t="n">
+        <v>15.125</v>
+      </c>
+      <c r="M140" s="2" t="n">
+        <v>26.3246</v>
+      </c>
+      <c r="N140" t="inlineStr">
+        <is>
           <t>baseline</t>
         </is>
       </c>
-      <c r="B136" t="inlineStr">
+    </row>
+    <row r="141">
+      <c r="A141" t="inlineStr">
+        <is>
+          <t>UltraLight</t>
+        </is>
+      </c>
+      <c r="B141" t="inlineStr">
+        <is>
+          <t>Run4</t>
+        </is>
+      </c>
+      <c r="C141" t="inlineStr">
+        <is>
+          <t>R4_1_VIT4_OLDHEAD</t>
+        </is>
+      </c>
+      <c r="D141" t="inlineStr">
+        <is>
+          <t>SYSU-CD-256</t>
+        </is>
+      </c>
+      <c r="E141" s="2" t="n">
+        <v>82.15000000000001</v>
+      </c>
+      <c r="F141" s="2" t="n">
+        <v>83.40000000000001</v>
+      </c>
+      <c r="G141" s="2" t="n">
+        <v>91.94</v>
+      </c>
+      <c r="H141" s="2" t="n">
+        <v>82.77</v>
+      </c>
+      <c r="I141" s="2" t="n">
+        <v>70.61</v>
+      </c>
+      <c r="J141" s="2" t="n">
+        <v>77.51000000000001</v>
+      </c>
+      <c r="K141" s="2" t="n">
+        <v>8.195</v>
+      </c>
+      <c r="L141" s="2" t="n">
+        <v>15.125</v>
+      </c>
+      <c r="M141" s="2" t="n">
+        <v>24.1021</v>
+      </c>
+      <c r="N141" t="inlineStr">
+        <is>
+          <t>baseline</t>
+        </is>
+      </c>
+    </row>
+    <row r="142">
+      <c r="A142" t="inlineStr">
+        <is>
+          <t>UltraLight</t>
+        </is>
+      </c>
+      <c r="B142" t="inlineStr">
+        <is>
+          <t>Run4</t>
+        </is>
+      </c>
+      <c r="C142" t="inlineStr">
+        <is>
+          <t>R4_2_VIT4_LIGHTDETAIL</t>
+        </is>
+      </c>
+      <c r="D142" t="inlineStr">
+        <is>
+          <t>SYSU-CD-256</t>
+        </is>
+      </c>
+      <c r="E142" s="2" t="n">
+        <v>79.94</v>
+      </c>
+      <c r="F142" s="2" t="n">
+        <v>84.79000000000001</v>
+      </c>
+      <c r="G142" s="2" t="n">
+        <v>91.89</v>
+      </c>
+      <c r="H142" s="2" t="n">
+        <v>82.3</v>
+      </c>
+      <c r="I142" s="2" t="n">
+        <v>69.92</v>
+      </c>
+      <c r="J142" s="2" t="n">
+        <v>77.04000000000001</v>
+      </c>
+      <c r="K142" s="2" t="n">
+        <v>5.492</v>
+      </c>
+      <c r="L142" s="2" t="n">
+        <v>3.515</v>
+      </c>
+      <c r="M142" s="2" t="n">
+        <v>10.7311</v>
+      </c>
+      <c r="N142" t="inlineStr">
+        <is>
+          <t>baseline</t>
+        </is>
+      </c>
+    </row>
+    <row r="143">
+      <c r="A143" t="inlineStr">
+        <is>
+          <t>UltraLight</t>
+        </is>
+      </c>
+      <c r="B143" t="inlineStr">
+        <is>
+          <t>Run4</t>
+        </is>
+      </c>
+      <c r="C143" t="inlineStr">
+        <is>
+          <t>R4_2b_VIT4_LIGHTDETAIL48</t>
+        </is>
+      </c>
+      <c r="D143" t="inlineStr">
+        <is>
+          <t>SYSU-CD-256</t>
+        </is>
+      </c>
+      <c r="E143" s="2" t="n">
+        <v>80.87</v>
+      </c>
+      <c r="F143" s="2" t="n">
+        <v>83.81</v>
+      </c>
+      <c r="G143" s="2" t="n">
+        <v>91.81</v>
+      </c>
+      <c r="H143" s="2" t="n">
+        <v>82.31999999999999</v>
+      </c>
+      <c r="I143" s="2" t="n">
+        <v>69.95</v>
+      </c>
+      <c r="J143" s="2" t="n">
+        <v>76.98999999999999</v>
+      </c>
+      <c r="K143" s="2" t="n">
+        <v>5.533</v>
+      </c>
+      <c r="L143" s="2" t="n">
+        <v>3.556</v>
+      </c>
+      <c r="M143" s="2" t="n">
+        <v>10.9824</v>
+      </c>
+      <c r="N143" t="inlineStr">
+        <is>
+          <t>baseline</t>
+        </is>
+      </c>
+    </row>
+    <row r="144">
+      <c r="A144" t="inlineStr">
+        <is>
+          <t>UltraLight</t>
+        </is>
+      </c>
+      <c r="B144" t="inlineStr">
+        <is>
+          <t>Run4</t>
+        </is>
+      </c>
+      <c r="C144" t="inlineStr">
+        <is>
+          <t>R4_2d_PSD_DETAIL</t>
+        </is>
+      </c>
+      <c r="D144" t="inlineStr">
+        <is>
+          <t>SYSU-CD-256</t>
+        </is>
+      </c>
+      <c r="E144" s="2" t="n">
+        <v>79.78</v>
+      </c>
+      <c r="F144" s="2" t="n">
+        <v>84.39</v>
+      </c>
+      <c r="G144" s="2" t="n">
+        <v>91.75</v>
+      </c>
+      <c r="H144" s="2" t="n">
+        <v>82.02</v>
+      </c>
+      <c r="I144" s="2" t="n">
+        <v>69.52</v>
+      </c>
+      <c r="J144" s="2" t="n">
+        <v>76.68000000000001</v>
+      </c>
+      <c r="K144" s="2" t="n">
+        <v>5.491</v>
+      </c>
+      <c r="L144" s="2" t="n">
+        <v>3.514</v>
+      </c>
+      <c r="M144" s="2" t="n">
+        <v>11.5239</v>
+      </c>
+      <c r="N144" t="inlineStr">
+        <is>
+          <t>baseline</t>
+        </is>
+      </c>
+    </row>
+    <row r="145">
+      <c r="A145" t="inlineStr">
+        <is>
+          <t>baseline</t>
+        </is>
+      </c>
+      <c r="B145" t="inlineStr">
         <is>
           <t>Run1</t>
         </is>
       </c>
-      <c r="C136" t="inlineStr"/>
-      <c r="D136" t="inlineStr">
+      <c r="C145" t="inlineStr"/>
+      <c r="D145" t="inlineStr">
+        <is>
+          <t>CDD-CD-256</t>
+        </is>
+      </c>
+      <c r="E145" s="2" t="n">
+        <v>97.72</v>
+      </c>
+      <c r="F145" s="2" t="n">
+        <v>97.78</v>
+      </c>
+      <c r="G145" s="2" t="n">
+        <v>99.44</v>
+      </c>
+      <c r="H145" s="2" t="n">
+        <v>97.75</v>
+      </c>
+      <c r="I145" s="2" t="n">
+        <v>95.59999999999999</v>
+      </c>
+      <c r="J145" s="2" t="n">
+        <v>97.43000000000001</v>
+      </c>
+      <c r="K145" s="2" t="n">
+        <v>11.754</v>
+      </c>
+      <c r="L145" s="2" t="n">
+        <v>20.661</v>
+      </c>
+      <c r="M145" s="2" t="n">
+        <v>26.3246</v>
+      </c>
+      <c r="N145" t="inlineStr">
+        <is>
+          <t>baseline</t>
+        </is>
+      </c>
+    </row>
+    <row r="146">
+      <c r="A146" t="inlineStr">
+        <is>
+          <t>baseline</t>
+        </is>
+      </c>
+      <c r="B146" t="inlineStr">
+        <is>
+          <t>Run1</t>
+        </is>
+      </c>
+      <c r="C146" t="inlineStr"/>
+      <c r="D146" t="inlineStr">
+        <is>
+          <t>LEVIR-CD-256</t>
+        </is>
+      </c>
+      <c r="E146" s="2" t="n">
+        <v>91.56999999999999</v>
+      </c>
+      <c r="F146" s="2" t="n">
+        <v>92.33</v>
+      </c>
+      <c r="G146" s="2" t="n">
+        <v>99.18000000000001</v>
+      </c>
+      <c r="H146" s="2" t="n">
+        <v>91.95</v>
+      </c>
+      <c r="I146" s="2" t="n">
+        <v>85.09999999999999</v>
+      </c>
+      <c r="J146" s="2" t="n">
+        <v>91.52</v>
+      </c>
+      <c r="K146" s="2" t="n">
+        <v>11.754</v>
+      </c>
+      <c r="L146" s="2" t="n">
+        <v>20.661</v>
+      </c>
+      <c r="M146" s="2" t="n">
+        <v>26.3246</v>
+      </c>
+      <c r="N146" t="inlineStr">
+        <is>
+          <t>baseline</t>
+        </is>
+      </c>
+    </row>
+    <row r="147">
+      <c r="A147" t="inlineStr">
+        <is>
+          <t>baseline</t>
+        </is>
+      </c>
+      <c r="B147" t="inlineStr">
+        <is>
+          <t>Run1</t>
+        </is>
+      </c>
+      <c r="C147" t="inlineStr"/>
+      <c r="D147" t="inlineStr">
+        <is>
+          <t>SYSU-CD-256</t>
+        </is>
+      </c>
+      <c r="E147" s="2" t="n">
+        <v>80.77</v>
+      </c>
+      <c r="F147" s="2" t="n">
+        <v>84.27</v>
+      </c>
+      <c r="G147" s="2" t="n">
+        <v>91.91</v>
+      </c>
+      <c r="H147" s="2" t="n">
+        <v>82.48</v>
+      </c>
+      <c r="I147" s="2" t="n">
+        <v>70.19</v>
+      </c>
+      <c r="J147" s="2" t="n">
+        <v>77.23</v>
+      </c>
+      <c r="K147" s="2" t="n">
+        <v>11.754</v>
+      </c>
+      <c r="L147" s="2" t="n">
+        <v>20.661</v>
+      </c>
+      <c r="M147" s="2" t="n">
+        <v>26.3246</v>
+      </c>
+      <c r="N147" t="inlineStr">
+        <is>
+          <t>baseline</t>
+        </is>
+      </c>
+    </row>
+    <row r="148">
+      <c r="A148" t="inlineStr">
+        <is>
+          <t>baseline</t>
+        </is>
+      </c>
+      <c r="B148" t="inlineStr">
+        <is>
+          <t>Run1</t>
+        </is>
+      </c>
+      <c r="C148" t="inlineStr"/>
+      <c r="D148" t="inlineStr">
         <is>
           <t>WHU-CD-256</t>
         </is>
       </c>
-      <c r="E136" s="2" t="n">
+      <c r="E148" s="2" t="n">
         <v>93.62</v>
       </c>
-      <c r="F136" s="2" t="n">
+      <c r="F148" s="2" t="n">
         <v>96.09</v>
       </c>
-      <c r="G136" s="2" t="n">
+      <c r="G148" s="2" t="n">
         <v>99.59999999999999</v>
       </c>
-      <c r="H136" s="2" t="n">
+      <c r="H148" s="2" t="n">
         <v>94.84</v>
       </c>
-      <c r="I136" s="2" t="n">
+      <c r="I148" s="2" t="n">
         <v>90.18000000000001</v>
       </c>
-      <c r="J136" s="2" t="n">
+      <c r="J148" s="2" t="n">
         <v>94.63</v>
       </c>
-      <c r="K136" s="2" t="n">
+      <c r="K148" s="2" t="n">
         <v>11.754</v>
       </c>
-      <c r="L136" s="2" t="n">
+      <c r="L148" s="2" t="n">
         <v>20.661</v>
       </c>
-      <c r="M136" s="2" t="n">
+      <c r="M148" s="2" t="n">
         <v>26.3246</v>
       </c>
-      <c r="N136" t="inlineStr">
+      <c r="N148" t="inlineStr">
         <is>
           <t>baseline</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:N136"/>
+  <autoFilter ref="A1:N148"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Record complete Run7 results and metric snapshots
</commit_message>
<xml_diff>
--- a/docs/experiment_metrics.xlsx
+++ b/docs/experiment_metrics.xlsx
@@ -10,7 +10,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="metrics" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'metrics'!$A$1:$N$148</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'metrics'!$A$1:$N$160</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -420,7 +420,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N148"/>
+  <dimension ref="A1:N160"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -7386,17 +7386,17 @@
     <row r="132">
       <c r="A132" t="inlineStr">
         <is>
-          <t>STR-Fusion</t>
+          <t>CASA</t>
         </is>
       </c>
       <c r="B132" t="inlineStr">
         <is>
-          <t>Run2_TASS</t>
+          <t>Run7</t>
         </is>
       </c>
       <c r="C132" t="inlineStr">
         <is>
-          <t>C0_TOKEN</t>
+          <t>M0_CTRL</t>
         </is>
       </c>
       <c r="D132" t="inlineStr">
@@ -7405,52 +7405,50 @@
         </is>
       </c>
       <c r="E132" s="2" t="n">
-        <v>93.13</v>
+        <v>97.31999999999999</v>
       </c>
       <c r="F132" s="2" t="n">
-        <v>95.16</v>
+        <v>97.54000000000001</v>
       </c>
       <c r="G132" s="2" t="n">
-        <v>98.56999999999999</v>
+        <v>99.37</v>
       </c>
       <c r="H132" s="2" t="n">
-        <v>94.13</v>
+        <v>97.43000000000001</v>
       </c>
       <c r="I132" s="2" t="n">
-        <v>88.91</v>
+        <v>94.98999999999999</v>
       </c>
       <c r="J132" s="2" t="n">
-        <v>93.31999999999999</v>
+        <v>97.06999999999999</v>
       </c>
       <c r="K132" s="2" t="n">
-        <v>2.596</v>
+        <v>3.016737</v>
       </c>
       <c r="L132" s="2" t="n">
-        <v>0.62</v>
-      </c>
-      <c r="M132" s="2" t="n">
-        <v>2.2136</v>
-      </c>
+        <v>3.100404</v>
+      </c>
+      <c r="M132" s="2" t="n"/>
       <c r="N132" t="inlineStr">
         <is>
-          <t>str_tass</t>
+          <t>casa_none</t>
         </is>
       </c>
     </row>
     <row r="133">
       <c r="A133" t="inlineStr">
         <is>
-          <t>STR-Fusion</t>
+          <t>CASA</t>
         </is>
       </c>
       <c r="B133" t="inlineStr">
         <is>
-          <t>Run2_TASS</t>
+          <t>Run7</t>
         </is>
       </c>
       <c r="C133" t="inlineStr">
         <is>
-          <t>C0_TOKEN</t>
+          <t>M0_CTRL</t>
         </is>
       </c>
       <c r="D133" t="inlineStr">
@@ -7459,52 +7457,50 @@
         </is>
       </c>
       <c r="E133" s="2" t="n">
-        <v>86.37</v>
+        <v>89.79000000000001</v>
       </c>
       <c r="F133" s="2" t="n">
-        <v>89.25</v>
+        <v>92.27</v>
       </c>
       <c r="G133" s="2" t="n">
-        <v>98.78</v>
+        <v>99.09999999999999</v>
       </c>
       <c r="H133" s="2" t="n">
-        <v>87.79000000000001</v>
+        <v>91.01000000000001</v>
       </c>
       <c r="I133" s="2" t="n">
-        <v>78.23999999999999</v>
+        <v>83.51000000000001</v>
       </c>
       <c r="J133" s="2" t="n">
-        <v>87.14</v>
+        <v>90.54000000000001</v>
       </c>
       <c r="K133" s="2" t="n">
-        <v>2.596</v>
+        <v>3.016737</v>
       </c>
       <c r="L133" s="2" t="n">
-        <v>0.62</v>
-      </c>
-      <c r="M133" s="2" t="n">
-        <v>2.2136</v>
-      </c>
+        <v>3.100404</v>
+      </c>
+      <c r="M133" s="2" t="n"/>
       <c r="N133" t="inlineStr">
         <is>
-          <t>str_tass</t>
+          <t>casa_none</t>
         </is>
       </c>
     </row>
     <row r="134">
       <c r="A134" t="inlineStr">
         <is>
-          <t>STR-Fusion</t>
+          <t>CASA</t>
         </is>
       </c>
       <c r="B134" t="inlineStr">
         <is>
-          <t>Run2_TASS</t>
+          <t>Run7</t>
         </is>
       </c>
       <c r="C134" t="inlineStr">
         <is>
-          <t>C0_TOKEN</t>
+          <t>M0_CTRL</t>
         </is>
       </c>
       <c r="D134" t="inlineStr">
@@ -7513,52 +7509,50 @@
         </is>
       </c>
       <c r="E134" s="2" t="n">
-        <v>79.93000000000001</v>
+        <v>79.92</v>
       </c>
       <c r="F134" s="2" t="n">
-        <v>84.5</v>
+        <v>84.81</v>
       </c>
       <c r="G134" s="2" t="n">
-        <v>91.81</v>
+        <v>91.89</v>
       </c>
       <c r="H134" s="2" t="n">
-        <v>82.15000000000001</v>
+        <v>82.29000000000001</v>
       </c>
       <c r="I134" s="2" t="n">
-        <v>69.70999999999999</v>
+        <v>69.91</v>
       </c>
       <c r="J134" s="2" t="n">
-        <v>76.84</v>
+        <v>77.04000000000001</v>
       </c>
       <c r="K134" s="2" t="n">
-        <v>2.596</v>
+        <v>3.016737</v>
       </c>
       <c r="L134" s="2" t="n">
-        <v>0.62</v>
-      </c>
-      <c r="M134" s="2" t="n">
-        <v>2.2136</v>
-      </c>
+        <v>3.100404</v>
+      </c>
+      <c r="M134" s="2" t="n"/>
       <c r="N134" t="inlineStr">
         <is>
-          <t>str_tass</t>
+          <t>casa_none</t>
         </is>
       </c>
     </row>
     <row r="135">
       <c r="A135" t="inlineStr">
         <is>
-          <t>STR-Fusion</t>
+          <t>CASA</t>
         </is>
       </c>
       <c r="B135" t="inlineStr">
         <is>
-          <t>Run2_TASS</t>
+          <t>Run7</t>
         </is>
       </c>
       <c r="C135" t="inlineStr">
         <is>
-          <t>C0_TOKEN</t>
+          <t>M0_CTRL</t>
         </is>
       </c>
       <c r="D135" t="inlineStr">
@@ -7567,52 +7561,50 @@
         </is>
       </c>
       <c r="E135" s="2" t="n">
-        <v>90.16</v>
+        <v>92.78</v>
       </c>
       <c r="F135" s="2" t="n">
-        <v>93.97</v>
+        <v>95.23</v>
       </c>
       <c r="G135" s="2" t="n">
-        <v>99.38</v>
+        <v>99.53</v>
       </c>
       <c r="H135" s="2" t="n">
-        <v>92.02</v>
+        <v>93.98999999999999</v>
       </c>
       <c r="I135" s="2" t="n">
-        <v>85.23</v>
+        <v>88.66</v>
       </c>
       <c r="J135" s="2" t="n">
-        <v>91.7</v>
+        <v>93.75</v>
       </c>
       <c r="K135" s="2" t="n">
-        <v>2.596</v>
+        <v>3.016737</v>
       </c>
       <c r="L135" s="2" t="n">
-        <v>0.62</v>
-      </c>
-      <c r="M135" s="2" t="n">
-        <v>2.2136</v>
-      </c>
+        <v>3.100404</v>
+      </c>
+      <c r="M135" s="2" t="n"/>
       <c r="N135" t="inlineStr">
         <is>
-          <t>str_tass</t>
+          <t>casa_none</t>
         </is>
       </c>
     </row>
     <row r="136">
       <c r="A136" t="inlineStr">
         <is>
-          <t>STR-Fusion</t>
+          <t>CASA</t>
         </is>
       </c>
       <c r="B136" t="inlineStr">
         <is>
-          <t>Run2_TASS</t>
+          <t>Run7</t>
         </is>
       </c>
       <c r="C136" t="inlineStr">
         <is>
-          <t>M1_TASS</t>
+          <t>M1_HYPER_QKV</t>
         </is>
       </c>
       <c r="D136" t="inlineStr">
@@ -7621,52 +7613,50 @@
         </is>
       </c>
       <c r="E136" s="2" t="n">
-        <v>94.7</v>
+        <v>97.48999999999999</v>
       </c>
       <c r="F136" s="2" t="n">
-        <v>96.13</v>
+        <v>97.45</v>
       </c>
       <c r="G136" s="2" t="n">
-        <v>98.88</v>
+        <v>99.37</v>
       </c>
       <c r="H136" s="2" t="n">
-        <v>95.41</v>
+        <v>97.47</v>
       </c>
       <c r="I136" s="2" t="n">
-        <v>91.22</v>
+        <v>95.06</v>
       </c>
       <c r="J136" s="2" t="n">
-        <v>94.77</v>
+        <v>97.11</v>
       </c>
       <c r="K136" s="2" t="n">
-        <v>3.455</v>
+        <v>3.050665</v>
       </c>
       <c r="L136" s="2" t="n">
-        <v>1.478</v>
-      </c>
-      <c r="M136" s="2" t="n">
-        <v>3.5459</v>
-      </c>
+        <v>3.134332</v>
+      </c>
+      <c r="M136" s="2" t="n"/>
       <c r="N136" t="inlineStr">
         <is>
-          <t>str_tass</t>
+          <t>casa_hyperbolic</t>
         </is>
       </c>
     </row>
     <row r="137">
       <c r="A137" t="inlineStr">
         <is>
-          <t>STR-Fusion</t>
+          <t>CASA</t>
         </is>
       </c>
       <c r="B137" t="inlineStr">
         <is>
-          <t>Run2_TASS</t>
+          <t>Run7</t>
         </is>
       </c>
       <c r="C137" t="inlineStr">
         <is>
-          <t>M1_TASS</t>
+          <t>M1_HYPER_QKV</t>
         </is>
       </c>
       <c r="D137" t="inlineStr">
@@ -7675,52 +7665,50 @@
         </is>
       </c>
       <c r="E137" s="2" t="n">
-        <v>88.42</v>
+        <v>89.73999999999999</v>
       </c>
       <c r="F137" s="2" t="n">
-        <v>91.97</v>
+        <v>93.42</v>
       </c>
       <c r="G137" s="2" t="n">
-        <v>99.02</v>
+        <v>99.16</v>
       </c>
       <c r="H137" s="2" t="n">
-        <v>90.16</v>
+        <v>91.54000000000001</v>
       </c>
       <c r="I137" s="2" t="n">
-        <v>82.08</v>
+        <v>84.40000000000001</v>
       </c>
       <c r="J137" s="2" t="n">
-        <v>89.64</v>
+        <v>91.09999999999999</v>
       </c>
       <c r="K137" s="2" t="n">
-        <v>3.455</v>
+        <v>3.050665</v>
       </c>
       <c r="L137" s="2" t="n">
-        <v>1.478</v>
-      </c>
-      <c r="M137" s="2" t="n">
-        <v>3.5459</v>
-      </c>
+        <v>3.134332</v>
+      </c>
+      <c r="M137" s="2" t="n"/>
       <c r="N137" t="inlineStr">
         <is>
-          <t>str_tass</t>
+          <t>casa_hyperbolic</t>
         </is>
       </c>
     </row>
     <row r="138">
       <c r="A138" t="inlineStr">
         <is>
-          <t>STR-Fusion</t>
+          <t>CASA</t>
         </is>
       </c>
       <c r="B138" t="inlineStr">
         <is>
-          <t>Run2_TASS</t>
+          <t>Run7</t>
         </is>
       </c>
       <c r="C138" t="inlineStr">
         <is>
-          <t>M1_TASS</t>
+          <t>M1_HYPER_QKV</t>
         </is>
       </c>
       <c r="D138" t="inlineStr">
@@ -7729,52 +7717,50 @@
         </is>
       </c>
       <c r="E138" s="2" t="n">
-        <v>78.73</v>
+        <v>77.78</v>
       </c>
       <c r="F138" s="2" t="n">
-        <v>84.98</v>
+        <v>84.04000000000001</v>
       </c>
       <c r="G138" s="2" t="n">
-        <v>91.7</v>
+        <v>91.28</v>
       </c>
       <c r="H138" s="2" t="n">
-        <v>81.73999999999999</v>
+        <v>80.79000000000001</v>
       </c>
       <c r="I138" s="2" t="n">
-        <v>69.11</v>
+        <v>67.77</v>
       </c>
       <c r="J138" s="2" t="n">
-        <v>76.38</v>
+        <v>75.16</v>
       </c>
       <c r="K138" s="2" t="n">
-        <v>3.455</v>
+        <v>3.050665</v>
       </c>
       <c r="L138" s="2" t="n">
-        <v>1.478</v>
-      </c>
-      <c r="M138" s="2" t="n">
-        <v>3.5459</v>
-      </c>
+        <v>3.134332</v>
+      </c>
+      <c r="M138" s="2" t="n"/>
       <c r="N138" t="inlineStr">
         <is>
-          <t>str_tass</t>
+          <t>casa_hyperbolic</t>
         </is>
       </c>
     </row>
     <row r="139">
       <c r="A139" t="inlineStr">
         <is>
-          <t>STR-Fusion</t>
+          <t>CASA</t>
         </is>
       </c>
       <c r="B139" t="inlineStr">
         <is>
-          <t>Run2_TASS</t>
+          <t>Run7</t>
         </is>
       </c>
       <c r="C139" t="inlineStr">
         <is>
-          <t>M1_TASS</t>
+          <t>M1_HYPER_QKV</t>
         </is>
       </c>
       <c r="D139" t="inlineStr">
@@ -7783,160 +7769,154 @@
         </is>
       </c>
       <c r="E139" s="2" t="n">
-        <v>91.64</v>
+        <v>93.05</v>
       </c>
       <c r="F139" s="2" t="n">
-        <v>94.81999999999999</v>
+        <v>96.14</v>
       </c>
       <c r="G139" s="2" t="n">
-        <v>99.47</v>
+        <v>99.58</v>
       </c>
       <c r="H139" s="2" t="n">
-        <v>93.2</v>
+        <v>94.56999999999999</v>
       </c>
       <c r="I139" s="2" t="n">
-        <v>87.27</v>
+        <v>89.7</v>
       </c>
       <c r="J139" s="2" t="n">
-        <v>92.93000000000001</v>
+        <v>94.34999999999999</v>
       </c>
       <c r="K139" s="2" t="n">
-        <v>3.455</v>
+        <v>3.050665</v>
       </c>
       <c r="L139" s="2" t="n">
-        <v>1.478</v>
-      </c>
-      <c r="M139" s="2" t="n">
-        <v>3.5459</v>
-      </c>
+        <v>3.134332</v>
+      </c>
+      <c r="M139" s="2" t="n"/>
       <c r="N139" t="inlineStr">
         <is>
-          <t>str_tass</t>
+          <t>casa_hyperbolic</t>
         </is>
       </c>
     </row>
     <row r="140">
       <c r="A140" t="inlineStr">
         <is>
-          <t>UltraLight</t>
+          <t>CASA</t>
         </is>
       </c>
       <c r="B140" t="inlineStr">
         <is>
-          <t>Run4</t>
+          <t>Run7</t>
         </is>
       </c>
       <c r="C140" t="inlineStr">
         <is>
-          <t>R4_0_A0_FULL12_FROZEN</t>
+          <t>M2_CA_QKV</t>
         </is>
       </c>
       <c r="D140" t="inlineStr">
         <is>
-          <t>SYSU-CD-256</t>
+          <t>CDD-CD-256</t>
         </is>
       </c>
       <c r="E140" s="2" t="n">
-        <v>82.42</v>
+        <v>97.41</v>
       </c>
       <c r="F140" s="2" t="n">
-        <v>83.87</v>
+        <v>97.53</v>
       </c>
       <c r="G140" s="2" t="n">
-        <v>92.12</v>
+        <v>99.38</v>
       </c>
       <c r="H140" s="2" t="n">
-        <v>83.14</v>
+        <v>97.47</v>
       </c>
       <c r="I140" s="2" t="n">
-        <v>71.14</v>
+        <v>95.06</v>
       </c>
       <c r="J140" s="2" t="n">
-        <v>77.98999999999999</v>
+        <v>97.11</v>
       </c>
       <c r="K140" s="2" t="n">
-        <v>11.754</v>
+        <v>3.067561</v>
       </c>
       <c r="L140" s="2" t="n">
-        <v>15.125</v>
-      </c>
-      <c r="M140" s="2" t="n">
-        <v>26.3246</v>
-      </c>
+        <v>3.151228</v>
+      </c>
+      <c r="M140" s="2" t="n"/>
       <c r="N140" t="inlineStr">
         <is>
-          <t>baseline</t>
+          <t>casa_qkv</t>
         </is>
       </c>
     </row>
     <row r="141">
       <c r="A141" t="inlineStr">
         <is>
-          <t>UltraLight</t>
+          <t>CASA</t>
         </is>
       </c>
       <c r="B141" t="inlineStr">
         <is>
-          <t>Run4</t>
+          <t>Run7</t>
         </is>
       </c>
       <c r="C141" t="inlineStr">
         <is>
-          <t>R4_1_VIT4_OLDHEAD</t>
+          <t>M2_CA_QKV</t>
         </is>
       </c>
       <c r="D141" t="inlineStr">
         <is>
-          <t>SYSU-CD-256</t>
+          <t>LEVIR-CD-256</t>
         </is>
       </c>
       <c r="E141" s="2" t="n">
-        <v>82.15000000000001</v>
+        <v>90.68000000000001</v>
       </c>
       <c r="F141" s="2" t="n">
-        <v>83.40000000000001</v>
+        <v>91.98</v>
       </c>
       <c r="G141" s="2" t="n">
-        <v>91.94</v>
+        <v>99.12</v>
       </c>
       <c r="H141" s="2" t="n">
-        <v>82.77</v>
+        <v>91.33</v>
       </c>
       <c r="I141" s="2" t="n">
-        <v>70.61</v>
+        <v>84.04000000000001</v>
       </c>
       <c r="J141" s="2" t="n">
-        <v>77.51000000000001</v>
+        <v>90.87</v>
       </c>
       <c r="K141" s="2" t="n">
-        <v>8.195</v>
+        <v>3.067561</v>
       </c>
       <c r="L141" s="2" t="n">
-        <v>15.125</v>
-      </c>
-      <c r="M141" s="2" t="n">
-        <v>24.1021</v>
-      </c>
+        <v>3.151228</v>
+      </c>
+      <c r="M141" s="2" t="n"/>
       <c r="N141" t="inlineStr">
         <is>
-          <t>baseline</t>
+          <t>casa_qkv</t>
         </is>
       </c>
     </row>
     <row r="142">
       <c r="A142" t="inlineStr">
         <is>
-          <t>UltraLight</t>
+          <t>CASA</t>
         </is>
       </c>
       <c r="B142" t="inlineStr">
         <is>
-          <t>Run4</t>
+          <t>Run7</t>
         </is>
       </c>
       <c r="C142" t="inlineStr">
         <is>
-          <t>R4_2_VIT4_LIGHTDETAIL</t>
+          <t>M2_CA_QKV</t>
         </is>
       </c>
       <c r="D142" t="inlineStr">
@@ -7945,348 +7925,992 @@
         </is>
       </c>
       <c r="E142" s="2" t="n">
-        <v>79.94</v>
+        <v>77.18000000000001</v>
       </c>
       <c r="F142" s="2" t="n">
-        <v>84.79000000000001</v>
+        <v>85.53</v>
       </c>
       <c r="G142" s="2" t="n">
-        <v>91.89</v>
+        <v>91.54000000000001</v>
       </c>
       <c r="H142" s="2" t="n">
-        <v>82.3</v>
+        <v>81.14</v>
       </c>
       <c r="I142" s="2" t="n">
-        <v>69.92</v>
+        <v>68.27</v>
       </c>
       <c r="J142" s="2" t="n">
-        <v>77.04000000000001</v>
+        <v>75.70999999999999</v>
       </c>
       <c r="K142" s="2" t="n">
-        <v>5.492</v>
+        <v>3.067561</v>
       </c>
       <c r="L142" s="2" t="n">
-        <v>3.515</v>
-      </c>
-      <c r="M142" s="2" t="n">
-        <v>10.7311</v>
-      </c>
+        <v>3.151228</v>
+      </c>
+      <c r="M142" s="2" t="n"/>
       <c r="N142" t="inlineStr">
         <is>
-          <t>baseline</t>
+          <t>casa_qkv</t>
         </is>
       </c>
     </row>
     <row r="143">
       <c r="A143" t="inlineStr">
         <is>
-          <t>UltraLight</t>
+          <t>CASA</t>
         </is>
       </c>
       <c r="B143" t="inlineStr">
         <is>
-          <t>Run4</t>
+          <t>Run7</t>
         </is>
       </c>
       <c r="C143" t="inlineStr">
         <is>
-          <t>R4_2b_VIT4_LIGHTDETAIL48</t>
+          <t>M2_CA_QKV</t>
         </is>
       </c>
       <c r="D143" t="inlineStr">
         <is>
-          <t>SYSU-CD-256</t>
+          <t>WHU-CD-256</t>
         </is>
       </c>
       <c r="E143" s="2" t="n">
-        <v>80.87</v>
+        <v>92.63</v>
       </c>
       <c r="F143" s="2" t="n">
-        <v>83.81</v>
+        <v>96.55</v>
       </c>
       <c r="G143" s="2" t="n">
-        <v>91.81</v>
+        <v>99.58</v>
       </c>
       <c r="H143" s="2" t="n">
-        <v>82.31999999999999</v>
+        <v>94.55</v>
       </c>
       <c r="I143" s="2" t="n">
-        <v>69.95</v>
+        <v>89.67</v>
       </c>
       <c r="J143" s="2" t="n">
-        <v>76.98999999999999</v>
+        <v>94.33</v>
       </c>
       <c r="K143" s="2" t="n">
-        <v>5.533</v>
+        <v>3.067561</v>
       </c>
       <c r="L143" s="2" t="n">
-        <v>3.556</v>
-      </c>
-      <c r="M143" s="2" t="n">
-        <v>10.9824</v>
-      </c>
+        <v>3.151228</v>
+      </c>
+      <c r="M143" s="2" t="n"/>
       <c r="N143" t="inlineStr">
         <is>
-          <t>baseline</t>
+          <t>casa_qkv</t>
         </is>
       </c>
     </row>
     <row r="144">
       <c r="A144" t="inlineStr">
         <is>
-          <t>UltraLight</t>
+          <t>STR-Fusion</t>
         </is>
       </c>
       <c r="B144" t="inlineStr">
         <is>
-          <t>Run4</t>
+          <t>Run2_TASS</t>
         </is>
       </c>
       <c r="C144" t="inlineStr">
         <is>
-          <t>R4_2d_PSD_DETAIL</t>
+          <t>C0_TOKEN</t>
         </is>
       </c>
       <c r="D144" t="inlineStr">
         <is>
-          <t>SYSU-CD-256</t>
+          <t>CDD-CD-256</t>
         </is>
       </c>
       <c r="E144" s="2" t="n">
-        <v>79.78</v>
+        <v>93.13</v>
       </c>
       <c r="F144" s="2" t="n">
-        <v>84.39</v>
+        <v>95.16</v>
       </c>
       <c r="G144" s="2" t="n">
-        <v>91.75</v>
+        <v>98.56999999999999</v>
       </c>
       <c r="H144" s="2" t="n">
-        <v>82.02</v>
+        <v>94.13</v>
       </c>
       <c r="I144" s="2" t="n">
-        <v>69.52</v>
+        <v>88.91</v>
       </c>
       <c r="J144" s="2" t="n">
-        <v>76.68000000000001</v>
+        <v>93.31999999999999</v>
       </c>
       <c r="K144" s="2" t="n">
-        <v>5.491</v>
+        <v>2.596</v>
       </c>
       <c r="L144" s="2" t="n">
-        <v>3.514</v>
+        <v>0.62</v>
       </c>
       <c r="M144" s="2" t="n">
-        <v>11.5239</v>
+        <v>2.2136</v>
       </c>
       <c r="N144" t="inlineStr">
         <is>
-          <t>baseline</t>
+          <t>str_tass</t>
         </is>
       </c>
     </row>
     <row r="145">
       <c r="A145" t="inlineStr">
         <is>
-          <t>baseline</t>
+          <t>STR-Fusion</t>
         </is>
       </c>
       <c r="B145" t="inlineStr">
         <is>
-          <t>Run1</t>
-        </is>
-      </c>
-      <c r="C145" t="inlineStr"/>
+          <t>Run2_TASS</t>
+        </is>
+      </c>
+      <c r="C145" t="inlineStr">
+        <is>
+          <t>C0_TOKEN</t>
+        </is>
+      </c>
       <c r="D145" t="inlineStr">
         <is>
-          <t>CDD-CD-256</t>
+          <t>LEVIR-CD-256</t>
         </is>
       </c>
       <c r="E145" s="2" t="n">
-        <v>97.72</v>
+        <v>86.37</v>
       </c>
       <c r="F145" s="2" t="n">
-        <v>97.78</v>
+        <v>89.25</v>
       </c>
       <c r="G145" s="2" t="n">
-        <v>99.44</v>
+        <v>98.78</v>
       </c>
       <c r="H145" s="2" t="n">
-        <v>97.75</v>
+        <v>87.79000000000001</v>
       </c>
       <c r="I145" s="2" t="n">
-        <v>95.59999999999999</v>
+        <v>78.23999999999999</v>
       </c>
       <c r="J145" s="2" t="n">
-        <v>97.43000000000001</v>
+        <v>87.14</v>
       </c>
       <c r="K145" s="2" t="n">
-        <v>11.754</v>
+        <v>2.596</v>
       </c>
       <c r="L145" s="2" t="n">
-        <v>20.661</v>
+        <v>0.62</v>
       </c>
       <c r="M145" s="2" t="n">
-        <v>26.3246</v>
+        <v>2.2136</v>
       </c>
       <c r="N145" t="inlineStr">
         <is>
-          <t>baseline</t>
+          <t>str_tass</t>
         </is>
       </c>
     </row>
     <row r="146">
       <c r="A146" t="inlineStr">
         <is>
-          <t>baseline</t>
+          <t>STR-Fusion</t>
         </is>
       </c>
       <c r="B146" t="inlineStr">
         <is>
-          <t>Run1</t>
-        </is>
-      </c>
-      <c r="C146" t="inlineStr"/>
+          <t>Run2_TASS</t>
+        </is>
+      </c>
+      <c r="C146" t="inlineStr">
+        <is>
+          <t>C0_TOKEN</t>
+        </is>
+      </c>
       <c r="D146" t="inlineStr">
         <is>
-          <t>LEVIR-CD-256</t>
+          <t>SYSU-CD-256</t>
         </is>
       </c>
       <c r="E146" s="2" t="n">
-        <v>91.56999999999999</v>
+        <v>79.93000000000001</v>
       </c>
       <c r="F146" s="2" t="n">
-        <v>92.33</v>
+        <v>84.5</v>
       </c>
       <c r="G146" s="2" t="n">
-        <v>99.18000000000001</v>
+        <v>91.81</v>
       </c>
       <c r="H146" s="2" t="n">
-        <v>91.95</v>
+        <v>82.15000000000001</v>
       </c>
       <c r="I146" s="2" t="n">
-        <v>85.09999999999999</v>
+        <v>69.70999999999999</v>
       </c>
       <c r="J146" s="2" t="n">
-        <v>91.52</v>
+        <v>76.84</v>
       </c>
       <c r="K146" s="2" t="n">
-        <v>11.754</v>
+        <v>2.596</v>
       </c>
       <c r="L146" s="2" t="n">
-        <v>20.661</v>
+        <v>0.62</v>
       </c>
       <c r="M146" s="2" t="n">
-        <v>26.3246</v>
+        <v>2.2136</v>
       </c>
       <c r="N146" t="inlineStr">
         <is>
-          <t>baseline</t>
+          <t>str_tass</t>
         </is>
       </c>
     </row>
     <row r="147">
       <c r="A147" t="inlineStr">
         <is>
-          <t>baseline</t>
+          <t>STR-Fusion</t>
         </is>
       </c>
       <c r="B147" t="inlineStr">
         <is>
-          <t>Run1</t>
-        </is>
-      </c>
-      <c r="C147" t="inlineStr"/>
+          <t>Run2_TASS</t>
+        </is>
+      </c>
+      <c r="C147" t="inlineStr">
+        <is>
+          <t>C0_TOKEN</t>
+        </is>
+      </c>
       <c r="D147" t="inlineStr">
         <is>
-          <t>SYSU-CD-256</t>
+          <t>WHU-CD-256</t>
         </is>
       </c>
       <c r="E147" s="2" t="n">
-        <v>80.77</v>
+        <v>90.16</v>
       </c>
       <c r="F147" s="2" t="n">
-        <v>84.27</v>
+        <v>93.97</v>
       </c>
       <c r="G147" s="2" t="n">
-        <v>91.91</v>
+        <v>99.38</v>
       </c>
       <c r="H147" s="2" t="n">
-        <v>82.48</v>
+        <v>92.02</v>
       </c>
       <c r="I147" s="2" t="n">
-        <v>70.19</v>
+        <v>85.23</v>
       </c>
       <c r="J147" s="2" t="n">
-        <v>77.23</v>
+        <v>91.7</v>
       </c>
       <c r="K147" s="2" t="n">
-        <v>11.754</v>
+        <v>2.596</v>
       </c>
       <c r="L147" s="2" t="n">
-        <v>20.661</v>
+        <v>0.62</v>
       </c>
       <c r="M147" s="2" t="n">
-        <v>26.3246</v>
+        <v>2.2136</v>
       </c>
       <c r="N147" t="inlineStr">
         <is>
-          <t>baseline</t>
+          <t>str_tass</t>
         </is>
       </c>
     </row>
     <row r="148">
       <c r="A148" t="inlineStr">
         <is>
+          <t>STR-Fusion</t>
+        </is>
+      </c>
+      <c r="B148" t="inlineStr">
+        <is>
+          <t>Run2_TASS</t>
+        </is>
+      </c>
+      <c r="C148" t="inlineStr">
+        <is>
+          <t>M1_TASS</t>
+        </is>
+      </c>
+      <c r="D148" t="inlineStr">
+        <is>
+          <t>CDD-CD-256</t>
+        </is>
+      </c>
+      <c r="E148" s="2" t="n">
+        <v>94.7</v>
+      </c>
+      <c r="F148" s="2" t="n">
+        <v>96.13</v>
+      </c>
+      <c r="G148" s="2" t="n">
+        <v>98.88</v>
+      </c>
+      <c r="H148" s="2" t="n">
+        <v>95.41</v>
+      </c>
+      <c r="I148" s="2" t="n">
+        <v>91.22</v>
+      </c>
+      <c r="J148" s="2" t="n">
+        <v>94.77</v>
+      </c>
+      <c r="K148" s="2" t="n">
+        <v>3.455</v>
+      </c>
+      <c r="L148" s="2" t="n">
+        <v>1.478</v>
+      </c>
+      <c r="M148" s="2" t="n">
+        <v>3.5459</v>
+      </c>
+      <c r="N148" t="inlineStr">
+        <is>
+          <t>str_tass</t>
+        </is>
+      </c>
+    </row>
+    <row r="149">
+      <c r="A149" t="inlineStr">
+        <is>
+          <t>STR-Fusion</t>
+        </is>
+      </c>
+      <c r="B149" t="inlineStr">
+        <is>
+          <t>Run2_TASS</t>
+        </is>
+      </c>
+      <c r="C149" t="inlineStr">
+        <is>
+          <t>M1_TASS</t>
+        </is>
+      </c>
+      <c r="D149" t="inlineStr">
+        <is>
+          <t>LEVIR-CD-256</t>
+        </is>
+      </c>
+      <c r="E149" s="2" t="n">
+        <v>88.42</v>
+      </c>
+      <c r="F149" s="2" t="n">
+        <v>91.97</v>
+      </c>
+      <c r="G149" s="2" t="n">
+        <v>99.02</v>
+      </c>
+      <c r="H149" s="2" t="n">
+        <v>90.16</v>
+      </c>
+      <c r="I149" s="2" t="n">
+        <v>82.08</v>
+      </c>
+      <c r="J149" s="2" t="n">
+        <v>89.64</v>
+      </c>
+      <c r="K149" s="2" t="n">
+        <v>3.455</v>
+      </c>
+      <c r="L149" s="2" t="n">
+        <v>1.478</v>
+      </c>
+      <c r="M149" s="2" t="n">
+        <v>3.5459</v>
+      </c>
+      <c r="N149" t="inlineStr">
+        <is>
+          <t>str_tass</t>
+        </is>
+      </c>
+    </row>
+    <row r="150">
+      <c r="A150" t="inlineStr">
+        <is>
+          <t>STR-Fusion</t>
+        </is>
+      </c>
+      <c r="B150" t="inlineStr">
+        <is>
+          <t>Run2_TASS</t>
+        </is>
+      </c>
+      <c r="C150" t="inlineStr">
+        <is>
+          <t>M1_TASS</t>
+        </is>
+      </c>
+      <c r="D150" t="inlineStr">
+        <is>
+          <t>SYSU-CD-256</t>
+        </is>
+      </c>
+      <c r="E150" s="2" t="n">
+        <v>78.73</v>
+      </c>
+      <c r="F150" s="2" t="n">
+        <v>84.98</v>
+      </c>
+      <c r="G150" s="2" t="n">
+        <v>91.7</v>
+      </c>
+      <c r="H150" s="2" t="n">
+        <v>81.73999999999999</v>
+      </c>
+      <c r="I150" s="2" t="n">
+        <v>69.11</v>
+      </c>
+      <c r="J150" s="2" t="n">
+        <v>76.38</v>
+      </c>
+      <c r="K150" s="2" t="n">
+        <v>3.455</v>
+      </c>
+      <c r="L150" s="2" t="n">
+        <v>1.478</v>
+      </c>
+      <c r="M150" s="2" t="n">
+        <v>3.5459</v>
+      </c>
+      <c r="N150" t="inlineStr">
+        <is>
+          <t>str_tass</t>
+        </is>
+      </c>
+    </row>
+    <row r="151">
+      <c r="A151" t="inlineStr">
+        <is>
+          <t>STR-Fusion</t>
+        </is>
+      </c>
+      <c r="B151" t="inlineStr">
+        <is>
+          <t>Run2_TASS</t>
+        </is>
+      </c>
+      <c r="C151" t="inlineStr">
+        <is>
+          <t>M1_TASS</t>
+        </is>
+      </c>
+      <c r="D151" t="inlineStr">
+        <is>
+          <t>WHU-CD-256</t>
+        </is>
+      </c>
+      <c r="E151" s="2" t="n">
+        <v>91.64</v>
+      </c>
+      <c r="F151" s="2" t="n">
+        <v>94.81999999999999</v>
+      </c>
+      <c r="G151" s="2" t="n">
+        <v>99.47</v>
+      </c>
+      <c r="H151" s="2" t="n">
+        <v>93.2</v>
+      </c>
+      <c r="I151" s="2" t="n">
+        <v>87.27</v>
+      </c>
+      <c r="J151" s="2" t="n">
+        <v>92.93000000000001</v>
+      </c>
+      <c r="K151" s="2" t="n">
+        <v>3.455</v>
+      </c>
+      <c r="L151" s="2" t="n">
+        <v>1.478</v>
+      </c>
+      <c r="M151" s="2" t="n">
+        <v>3.5459</v>
+      </c>
+      <c r="N151" t="inlineStr">
+        <is>
+          <t>str_tass</t>
+        </is>
+      </c>
+    </row>
+    <row r="152">
+      <c r="A152" t="inlineStr">
+        <is>
+          <t>UltraLight</t>
+        </is>
+      </c>
+      <c r="B152" t="inlineStr">
+        <is>
+          <t>Run4</t>
+        </is>
+      </c>
+      <c r="C152" t="inlineStr">
+        <is>
+          <t>R4_0_A0_FULL12_FROZEN</t>
+        </is>
+      </c>
+      <c r="D152" t="inlineStr">
+        <is>
+          <t>SYSU-CD-256</t>
+        </is>
+      </c>
+      <c r="E152" s="2" t="n">
+        <v>82.42</v>
+      </c>
+      <c r="F152" s="2" t="n">
+        <v>83.87</v>
+      </c>
+      <c r="G152" s="2" t="n">
+        <v>92.12</v>
+      </c>
+      <c r="H152" s="2" t="n">
+        <v>83.14</v>
+      </c>
+      <c r="I152" s="2" t="n">
+        <v>71.14</v>
+      </c>
+      <c r="J152" s="2" t="n">
+        <v>77.98999999999999</v>
+      </c>
+      <c r="K152" s="2" t="n">
+        <v>11.754</v>
+      </c>
+      <c r="L152" s="2" t="n">
+        <v>15.125</v>
+      </c>
+      <c r="M152" s="2" t="n">
+        <v>26.3246</v>
+      </c>
+      <c r="N152" t="inlineStr">
+        <is>
           <t>baseline</t>
         </is>
       </c>
-      <c r="B148" t="inlineStr">
+    </row>
+    <row r="153">
+      <c r="A153" t="inlineStr">
+        <is>
+          <t>UltraLight</t>
+        </is>
+      </c>
+      <c r="B153" t="inlineStr">
+        <is>
+          <t>Run4</t>
+        </is>
+      </c>
+      <c r="C153" t="inlineStr">
+        <is>
+          <t>R4_1_VIT4_OLDHEAD</t>
+        </is>
+      </c>
+      <c r="D153" t="inlineStr">
+        <is>
+          <t>SYSU-CD-256</t>
+        </is>
+      </c>
+      <c r="E153" s="2" t="n">
+        <v>82.15000000000001</v>
+      </c>
+      <c r="F153" s="2" t="n">
+        <v>83.40000000000001</v>
+      </c>
+      <c r="G153" s="2" t="n">
+        <v>91.94</v>
+      </c>
+      <c r="H153" s="2" t="n">
+        <v>82.77</v>
+      </c>
+      <c r="I153" s="2" t="n">
+        <v>70.61</v>
+      </c>
+      <c r="J153" s="2" t="n">
+        <v>77.51000000000001</v>
+      </c>
+      <c r="K153" s="2" t="n">
+        <v>8.195</v>
+      </c>
+      <c r="L153" s="2" t="n">
+        <v>15.125</v>
+      </c>
+      <c r="M153" s="2" t="n">
+        <v>24.1021</v>
+      </c>
+      <c r="N153" t="inlineStr">
+        <is>
+          <t>baseline</t>
+        </is>
+      </c>
+    </row>
+    <row r="154">
+      <c r="A154" t="inlineStr">
+        <is>
+          <t>UltraLight</t>
+        </is>
+      </c>
+      <c r="B154" t="inlineStr">
+        <is>
+          <t>Run4</t>
+        </is>
+      </c>
+      <c r="C154" t="inlineStr">
+        <is>
+          <t>R4_2_VIT4_LIGHTDETAIL</t>
+        </is>
+      </c>
+      <c r="D154" t="inlineStr">
+        <is>
+          <t>SYSU-CD-256</t>
+        </is>
+      </c>
+      <c r="E154" s="2" t="n">
+        <v>79.94</v>
+      </c>
+      <c r="F154" s="2" t="n">
+        <v>84.79000000000001</v>
+      </c>
+      <c r="G154" s="2" t="n">
+        <v>91.89</v>
+      </c>
+      <c r="H154" s="2" t="n">
+        <v>82.3</v>
+      </c>
+      <c r="I154" s="2" t="n">
+        <v>69.92</v>
+      </c>
+      <c r="J154" s="2" t="n">
+        <v>77.04000000000001</v>
+      </c>
+      <c r="K154" s="2" t="n">
+        <v>5.492</v>
+      </c>
+      <c r="L154" s="2" t="n">
+        <v>3.515</v>
+      </c>
+      <c r="M154" s="2" t="n">
+        <v>10.7311</v>
+      </c>
+      <c r="N154" t="inlineStr">
+        <is>
+          <t>baseline</t>
+        </is>
+      </c>
+    </row>
+    <row r="155">
+      <c r="A155" t="inlineStr">
+        <is>
+          <t>UltraLight</t>
+        </is>
+      </c>
+      <c r="B155" t="inlineStr">
+        <is>
+          <t>Run4</t>
+        </is>
+      </c>
+      <c r="C155" t="inlineStr">
+        <is>
+          <t>R4_2b_VIT4_LIGHTDETAIL48</t>
+        </is>
+      </c>
+      <c r="D155" t="inlineStr">
+        <is>
+          <t>SYSU-CD-256</t>
+        </is>
+      </c>
+      <c r="E155" s="2" t="n">
+        <v>80.87</v>
+      </c>
+      <c r="F155" s="2" t="n">
+        <v>83.81</v>
+      </c>
+      <c r="G155" s="2" t="n">
+        <v>91.81</v>
+      </c>
+      <c r="H155" s="2" t="n">
+        <v>82.31999999999999</v>
+      </c>
+      <c r="I155" s="2" t="n">
+        <v>69.95</v>
+      </c>
+      <c r="J155" s="2" t="n">
+        <v>76.98999999999999</v>
+      </c>
+      <c r="K155" s="2" t="n">
+        <v>5.533</v>
+      </c>
+      <c r="L155" s="2" t="n">
+        <v>3.556</v>
+      </c>
+      <c r="M155" s="2" t="n">
+        <v>10.9824</v>
+      </c>
+      <c r="N155" t="inlineStr">
+        <is>
+          <t>baseline</t>
+        </is>
+      </c>
+    </row>
+    <row r="156">
+      <c r="A156" t="inlineStr">
+        <is>
+          <t>UltraLight</t>
+        </is>
+      </c>
+      <c r="B156" t="inlineStr">
+        <is>
+          <t>Run4</t>
+        </is>
+      </c>
+      <c r="C156" t="inlineStr">
+        <is>
+          <t>R4_2d_PSD_DETAIL</t>
+        </is>
+      </c>
+      <c r="D156" t="inlineStr">
+        <is>
+          <t>SYSU-CD-256</t>
+        </is>
+      </c>
+      <c r="E156" s="2" t="n">
+        <v>79.78</v>
+      </c>
+      <c r="F156" s="2" t="n">
+        <v>84.39</v>
+      </c>
+      <c r="G156" s="2" t="n">
+        <v>91.75</v>
+      </c>
+      <c r="H156" s="2" t="n">
+        <v>82.02</v>
+      </c>
+      <c r="I156" s="2" t="n">
+        <v>69.52</v>
+      </c>
+      <c r="J156" s="2" t="n">
+        <v>76.68000000000001</v>
+      </c>
+      <c r="K156" s="2" t="n">
+        <v>5.491</v>
+      </c>
+      <c r="L156" s="2" t="n">
+        <v>3.514</v>
+      </c>
+      <c r="M156" s="2" t="n">
+        <v>11.5239</v>
+      </c>
+      <c r="N156" t="inlineStr">
+        <is>
+          <t>baseline</t>
+        </is>
+      </c>
+    </row>
+    <row r="157">
+      <c r="A157" t="inlineStr">
+        <is>
+          <t>baseline</t>
+        </is>
+      </c>
+      <c r="B157" t="inlineStr">
         <is>
           <t>Run1</t>
         </is>
       </c>
-      <c r="C148" t="inlineStr"/>
-      <c r="D148" t="inlineStr">
+      <c r="C157" t="inlineStr"/>
+      <c r="D157" t="inlineStr">
+        <is>
+          <t>CDD-CD-256</t>
+        </is>
+      </c>
+      <c r="E157" s="2" t="n">
+        <v>97.72</v>
+      </c>
+      <c r="F157" s="2" t="n">
+        <v>97.78</v>
+      </c>
+      <c r="G157" s="2" t="n">
+        <v>99.44</v>
+      </c>
+      <c r="H157" s="2" t="n">
+        <v>97.75</v>
+      </c>
+      <c r="I157" s="2" t="n">
+        <v>95.59999999999999</v>
+      </c>
+      <c r="J157" s="2" t="n">
+        <v>97.43000000000001</v>
+      </c>
+      <c r="K157" s="2" t="n">
+        <v>11.754</v>
+      </c>
+      <c r="L157" s="2" t="n">
+        <v>20.661</v>
+      </c>
+      <c r="M157" s="2" t="n">
+        <v>26.3246</v>
+      </c>
+      <c r="N157" t="inlineStr">
+        <is>
+          <t>baseline</t>
+        </is>
+      </c>
+    </row>
+    <row r="158">
+      <c r="A158" t="inlineStr">
+        <is>
+          <t>baseline</t>
+        </is>
+      </c>
+      <c r="B158" t="inlineStr">
+        <is>
+          <t>Run1</t>
+        </is>
+      </c>
+      <c r="C158" t="inlineStr"/>
+      <c r="D158" t="inlineStr">
+        <is>
+          <t>LEVIR-CD-256</t>
+        </is>
+      </c>
+      <c r="E158" s="2" t="n">
+        <v>91.56999999999999</v>
+      </c>
+      <c r="F158" s="2" t="n">
+        <v>92.33</v>
+      </c>
+      <c r="G158" s="2" t="n">
+        <v>99.18000000000001</v>
+      </c>
+      <c r="H158" s="2" t="n">
+        <v>91.95</v>
+      </c>
+      <c r="I158" s="2" t="n">
+        <v>85.09999999999999</v>
+      </c>
+      <c r="J158" s="2" t="n">
+        <v>91.52</v>
+      </c>
+      <c r="K158" s="2" t="n">
+        <v>11.754</v>
+      </c>
+      <c r="L158" s="2" t="n">
+        <v>20.661</v>
+      </c>
+      <c r="M158" s="2" t="n">
+        <v>26.3246</v>
+      </c>
+      <c r="N158" t="inlineStr">
+        <is>
+          <t>baseline</t>
+        </is>
+      </c>
+    </row>
+    <row r="159">
+      <c r="A159" t="inlineStr">
+        <is>
+          <t>baseline</t>
+        </is>
+      </c>
+      <c r="B159" t="inlineStr">
+        <is>
+          <t>Run1</t>
+        </is>
+      </c>
+      <c r="C159" t="inlineStr"/>
+      <c r="D159" t="inlineStr">
+        <is>
+          <t>SYSU-CD-256</t>
+        </is>
+      </c>
+      <c r="E159" s="2" t="n">
+        <v>80.77</v>
+      </c>
+      <c r="F159" s="2" t="n">
+        <v>84.27</v>
+      </c>
+      <c r="G159" s="2" t="n">
+        <v>91.91</v>
+      </c>
+      <c r="H159" s="2" t="n">
+        <v>82.48</v>
+      </c>
+      <c r="I159" s="2" t="n">
+        <v>70.19</v>
+      </c>
+      <c r="J159" s="2" t="n">
+        <v>77.23</v>
+      </c>
+      <c r="K159" s="2" t="n">
+        <v>11.754</v>
+      </c>
+      <c r="L159" s="2" t="n">
+        <v>20.661</v>
+      </c>
+      <c r="M159" s="2" t="n">
+        <v>26.3246</v>
+      </c>
+      <c r="N159" t="inlineStr">
+        <is>
+          <t>baseline</t>
+        </is>
+      </c>
+    </row>
+    <row r="160">
+      <c r="A160" t="inlineStr">
+        <is>
+          <t>baseline</t>
+        </is>
+      </c>
+      <c r="B160" t="inlineStr">
+        <is>
+          <t>Run1</t>
+        </is>
+      </c>
+      <c r="C160" t="inlineStr"/>
+      <c r="D160" t="inlineStr">
         <is>
           <t>WHU-CD-256</t>
         </is>
       </c>
-      <c r="E148" s="2" t="n">
+      <c r="E160" s="2" t="n">
         <v>93.62</v>
       </c>
-      <c r="F148" s="2" t="n">
+      <c r="F160" s="2" t="n">
         <v>96.09</v>
       </c>
-      <c r="G148" s="2" t="n">
+      <c r="G160" s="2" t="n">
         <v>99.59999999999999</v>
       </c>
-      <c r="H148" s="2" t="n">
+      <c r="H160" s="2" t="n">
         <v>94.84</v>
       </c>
-      <c r="I148" s="2" t="n">
+      <c r="I160" s="2" t="n">
         <v>90.18000000000001</v>
       </c>
-      <c r="J148" s="2" t="n">
+      <c r="J160" s="2" t="n">
         <v>94.63</v>
       </c>
-      <c r="K148" s="2" t="n">
+      <c r="K160" s="2" t="n">
         <v>11.754</v>
       </c>
-      <c r="L148" s="2" t="n">
+      <c r="L160" s="2" t="n">
         <v>20.661</v>
       </c>
-      <c r="M148" s="2" t="n">
+      <c r="M160" s="2" t="n">
         <v>26.3246</v>
       </c>
-      <c r="N148" t="inlineStr">
+      <c r="N160" t="inlineStr">
         <is>
           <t>baseline</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:N148"/>
+  <autoFilter ref="A1:N160"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>